<commit_message>
some little changes according to source materilas
</commit_message>
<xml_diff>
--- a/results/Профилирование_лопаток.xlsx
+++ b/results/Профилирование_лопаток.xlsx
@@ -835,61 +835,61 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>66.19676196761966</v>
+        <v>66.53761537615375</v>
       </c>
       <c r="B2" t="n">
-        <v>22.88651637507553</v>
+        <v>23.04332530766255</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5</v>
+        <v>0.8894362943629437</v>
       </c>
       <c r="D2" t="n">
-        <v>1.368779359886178</v>
+        <v>1.413020524194945</v>
       </c>
       <c r="E2" t="n">
-        <v>65.98170981709816</v>
+        <v>67.03742037420375</v>
       </c>
       <c r="F2" t="n">
-        <v>22.78766533241859</v>
+        <v>23.27355074632903</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5</v>
+        <v>0.8830280302803029</v>
       </c>
       <c r="H2" t="n">
-        <v>1.417337707464406</v>
+        <v>1.475261520272945</v>
       </c>
       <c r="I2" t="n">
-        <v>0.921948399715446</v>
+        <v>1.032551310487361</v>
       </c>
       <c r="J2" t="n">
-        <v>-1.456655731338985</v>
+        <v>-1.311846199317638</v>
       </c>
       <c r="K2" t="n">
         <v>0.5</v>
       </c>
       <c r="L2" t="n">
-        <v>0.2776071856747635</v>
+        <v>0.276924768621417</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2780361199516505</v>
+        <v>0.2759255059583664</v>
       </c>
       <c r="N2" t="n">
-        <v>0.2072876043922122</v>
+        <v>0.4428690383644288</v>
       </c>
       <c r="O2" t="n">
-        <v>0.2630780704444102</v>
+        <v>0.4937488175649478</v>
       </c>
       <c r="P2" t="n">
-        <v>0.1036438021961061</v>
+        <v>0.2214345191822144</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.1315390352222051</v>
+        <v>0.2468744087824739</v>
       </c>
       <c r="R2" t="n">
-        <v>57.24146908711621</v>
+        <v>47.29585770116213</v>
       </c>
       <c r="S2" t="n">
-        <v>54.56045233591358</v>
+        <v>45.42106865188677</v>
       </c>
       <c r="T2" t="n">
         <v>3.000000000000001</v>
@@ -898,247 +898,247 @@
         <v>2.2</v>
       </c>
       <c r="V2" t="n">
-        <v>0.06610078313788487</v>
+        <v>0.07927631177856866</v>
       </c>
       <c r="W2" t="n">
-        <v>0.08687345429904655</v>
+        <v>0.09231847708159061</v>
       </c>
       <c r="X2" t="n">
-        <v>18.27074017709954</v>
+        <v>10.25632634966623</v>
       </c>
       <c r="Y2" t="n">
-        <v>18.92018839532619</v>
+        <v>10.7128873763988</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.04829177373289843</v>
+        <v>0.05610414740701351</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.06129340512252493</v>
+        <v>0.06257770287705353</v>
       </c>
       <c r="AB2" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="AC2" t="n">
         <v>26</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.06292779839470038</v>
+        <v>0.0736119838484469</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.07986989796250432</v>
+        <v>0.08210567429249846</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.050422624406509</v>
+        <v>1.076948448255158</v>
       </c>
       <c r="AG2" t="n">
-        <v>1.087687057517341</v>
+        <v>1.124386077784459</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.1260565610162723</v>
+        <v>0.1923711206378953</v>
       </c>
       <c r="AI2" t="n">
-        <v>-2.280782356206648</v>
+        <v>-2.189034805538853</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.3163162157332036</v>
+        <v>0.3250134241483084</v>
       </c>
       <c r="AK2" t="n">
-        <v>0.2660290640444311</v>
+        <v>0.2607302112741996</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.1183450812027955</v>
+        <v>0.229614761635697</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.27493493101266</v>
+        <v>0.5256960683641339</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.03836663424136467</v>
+        <v>0.07744592324816735</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.07628005336885152</v>
+        <v>0.1453395513705724</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.05917254060139774</v>
+        <v>0.1148073808178485</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.13746746550633</v>
+        <v>0.2628480341820669</v>
       </c>
       <c r="AR2" t="n">
-        <v>42.21311649902086</v>
+        <v>33.57241427064274</v>
       </c>
       <c r="AS2" t="n">
-        <v>60.38850677308233</v>
+        <v>52.18370052787058</v>
       </c>
       <c r="AT2" t="n">
-        <v>0.02517111935788015</v>
+        <v>0.02208359515453407</v>
       </c>
       <c r="AU2" t="n">
-        <v>0.03368326620871376</v>
+        <v>0.03302417362647769</v>
       </c>
       <c r="AV2" t="n">
-        <v>2.626056561016272</v>
+        <v>3.589828160850528</v>
       </c>
       <c r="AW2" t="n">
-        <v>2.579127978882661</v>
+        <v>2.795481822672247</v>
       </c>
       <c r="AX2" t="n">
-        <v>4.06514140254068</v>
+        <v>6.47457040212632</v>
       </c>
       <c r="AY2" t="n">
-        <v>1.447819947206652</v>
+        <v>1.988704556680618</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.2408338510608271</v>
+        <v>0.2307422903960569</v>
       </c>
       <c r="BA2" t="n">
-        <v>0.2660290640444311</v>
+        <v>0.2607302112741996</v>
       </c>
       <c r="BB2" t="n">
-        <v>0.09599321327139287</v>
+        <v>0.1688644817957764</v>
       </c>
       <c r="BC2" t="n">
-        <v>0.1674694146200393</v>
+        <v>0.3832906019879738</v>
       </c>
       <c r="BD2" t="n">
-        <v>0.03746365088637753</v>
+        <v>0.07382481050406133</v>
       </c>
       <c r="BE2" t="n">
-        <v>0.0715485826816417</v>
+        <v>0.1670890014736256</v>
       </c>
       <c r="BF2" t="n">
-        <v>0.04799660663569644</v>
+        <v>0.08443224089788821</v>
       </c>
       <c r="BG2" t="n">
-        <v>0.08373470731001965</v>
+        <v>0.1916453009939869</v>
       </c>
       <c r="BH2" t="n">
-        <v>79.94845384048402</v>
+        <v>81.21635254223462</v>
       </c>
       <c r="BI2" t="n">
-        <v>64.06337631829932</v>
+        <v>56.29023715690198</v>
       </c>
       <c r="BJ2" t="n">
-        <v>39.45379272336623</v>
+        <v>26.89849088400845</v>
       </c>
       <c r="BK2" t="n">
-        <v>29.7217498860338</v>
+        <v>13.80015305221628</v>
       </c>
       <c r="BL2" t="n">
-        <v>0.01652519578447122</v>
+        <v>0.01981907794464216</v>
       </c>
       <c r="BM2" t="n">
-        <v>0.02171836357476164</v>
+        <v>0.02307961927039765</v>
       </c>
       <c r="BN2" t="n">
-        <v>0.06508621093476193</v>
+        <v>0.07834655952915857</v>
       </c>
       <c r="BO2" t="n">
-        <v>0.07812342010074105</v>
+        <v>0.07679600846602362</v>
       </c>
       <c r="BP2" t="n">
-        <v>0.05558801256709024</v>
+        <v>0.05825743160560556</v>
       </c>
       <c r="BQ2" t="n">
-        <v>0.07077821485200991</v>
+        <v>0.06575699182726667</v>
       </c>
       <c r="BR2" t="n">
-        <v>0.04441246583947046</v>
+        <v>0.04383904454215617</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.07552741889797941</v>
+        <v>0.07292980784918728</v>
       </c>
       <c r="BT2" t="n">
-        <v>-0.02477372350886577</v>
+        <v>-0.02852424391887475</v>
       </c>
       <c r="BU2" t="n">
-        <v>-0.03208552703561373</v>
+        <v>-0.03120809524078163</v>
       </c>
       <c r="BV2" t="n">
-        <v>-0.002014473848758594</v>
+        <v>0.003589172156867016</v>
       </c>
       <c r="BW2" t="n">
-        <v>-0.005337518024968603</v>
+        <v>-0.01400445825870235</v>
       </c>
       <c r="BX2" t="n">
-        <v>-0.003514633309652028</v>
+        <v>0.001878662409681145</v>
       </c>
       <c r="BY2" t="n">
-        <v>-0.007290522070633522</v>
+        <v>-0.01595658881978716</v>
       </c>
       <c r="BZ2" t="n">
-        <v>-0.0246787902195223</v>
+        <v>-0.02725677001940365</v>
       </c>
       <c r="CA2" t="n">
-        <v>-0.03096979457460348</v>
+        <v>-0.02823444890251725</v>
       </c>
       <c r="CB2" t="n">
-        <v>-0.002656618291165205</v>
+        <v>-0.007052557364857244</v>
       </c>
       <c r="CC2" t="n">
-        <v>-0.009310620844767872</v>
+        <v>-0.0190812107454781</v>
       </c>
       <c r="CD2" t="n">
-        <v>-0.004153174585302284</v>
+        <v>-0.008723851307659148</v>
       </c>
       <c r="CE2" t="n">
-        <v>-0.01121694563097513</v>
+        <v>-0.02090186282059832</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>59.46894468944689</v>
+        <v>57.8930289302893</v>
       </c>
       <c r="B3" t="n">
-        <v>19.82375605342103</v>
+        <v>19.11424852803111</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5</v>
+        <v>0.7026121261212612</v>
       </c>
       <c r="D3" t="n">
-        <v>1.276428655876962</v>
+        <v>1.317664062849037</v>
       </c>
       <c r="E3" t="n">
-        <v>60.64280642806428</v>
+        <v>59.56414564145641</v>
       </c>
       <c r="F3" t="n">
-        <v>20.35396215368517</v>
+        <v>19.86669849423924</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5</v>
+        <v>0.6356117561175612</v>
       </c>
       <c r="H3" t="n">
-        <v>1.298126222011893</v>
+        <v>1.313654812360745</v>
       </c>
       <c r="I3" t="n">
-        <v>0.691071639692406</v>
+        <v>0.7941601571225931</v>
       </c>
       <c r="J3" t="n">
-        <v>-1.754684444970269</v>
+        <v>-1.715862969098137</v>
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
-        <v>0.2910616773572762</v>
+        <v>0.2942137346088875</v>
       </c>
       <c r="M3" t="n">
-        <v>0.288714321685004</v>
+        <v>0.2908711385415155</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1149555807361216</v>
+        <v>0.296542159153081</v>
       </c>
       <c r="O3" t="n">
-        <v>0.159959694681455</v>
+        <v>0.335480397337627</v>
       </c>
       <c r="P3" t="n">
-        <v>0.05747779036806082</v>
+        <v>0.1482710795765405</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.07997984734072749</v>
+        <v>0.1677401986688135</v>
       </c>
       <c r="R3" t="n">
-        <v>54.637003853804</v>
+        <v>45.40560420381076</v>
       </c>
       <c r="S3" t="n">
-        <v>53.8802359192526</v>
+        <v>45.3886497444955</v>
       </c>
       <c r="T3" t="n">
         <v>2.900000000000001</v>
@@ -1147,247 +1147,247 @@
         <v>2.1</v>
       </c>
       <c r="V3" t="n">
-        <v>0.06359223304926613</v>
+        <v>0.07550719441710939</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05658906336071264</v>
+        <v>0.06141055051463777</v>
       </c>
       <c r="X3" t="n">
-        <v>31.69543532666318</v>
+        <v>14.58898257165743</v>
       </c>
       <c r="Y3" t="n">
-        <v>20.26957826222025</v>
+        <v>10.48815494507076</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.04982043669771381</v>
+        <v>0.05730382769478333</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.04359288211049958</v>
+        <v>0.04674785943521798</v>
       </c>
       <c r="AB3" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="AC3" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.0593319242007175</v>
+        <v>0.06886282360015999</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.05191543367562781</v>
+        <v>0.05617756662118316</v>
       </c>
       <c r="AF3" t="n">
-        <v>1.071804663441155</v>
+        <v>1.096487051642389</v>
       </c>
       <c r="AG3" t="n">
-        <v>1.090023897600203</v>
+        <v>1.093150775446393</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.1795116586028872</v>
+        <v>0.2412176291059737</v>
       </c>
       <c r="AI3" t="n">
-        <v>-2.274940255999494</v>
+        <v>-2.267123061384018</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.3166551415459026</v>
+        <v>0.3254229079431258</v>
       </c>
       <c r="AK3" t="n">
-        <v>0.2670379172790708</v>
+        <v>0.262608845959918</v>
       </c>
       <c r="AL3" t="n">
-        <v>0.1456069459885618</v>
+        <v>0.2422538757388784</v>
       </c>
       <c r="AM3" t="n">
-        <v>0.3211555507379597</v>
+        <v>0.5555357608184214</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.04773384935485978</v>
+        <v>0.08255067128748017</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.08953779076227508</v>
+        <v>0.1525321547062393</v>
       </c>
       <c r="AP3" t="n">
-        <v>0.07280347299428092</v>
+        <v>0.1211269378694392</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.1605777753689799</v>
+        <v>0.2777678804092107</v>
       </c>
       <c r="AR3" t="n">
-        <v>40.95429175756146</v>
+        <v>32.84314696125617</v>
       </c>
       <c r="AS3" t="n">
-        <v>57.94720650663606</v>
+        <v>50.13822355247309</v>
       </c>
       <c r="AT3" t="n">
-        <v>0.02622537635491526</v>
+        <v>0.02448106507793388</v>
       </c>
       <c r="AU3" t="n">
-        <v>0.03324855617423588</v>
+        <v>0.03485406335095416</v>
       </c>
       <c r="AV3" t="n">
-        <v>2.424835860833984</v>
+        <v>3.084310023960851</v>
       </c>
       <c r="AW3" t="n">
-        <v>1.702000624152311</v>
+        <v>1.761933749195318</v>
       </c>
       <c r="AX3" t="n">
-        <v>3.562089652084959</v>
+        <v>5.210775059902126</v>
       </c>
       <c r="AY3" t="n">
-        <v>-0.7449984396192233</v>
+        <v>-0.5951656270117062</v>
       </c>
       <c r="AZ3" t="n">
-        <v>0.2733081573119929</v>
+        <v>0.2723046553902756</v>
       </c>
       <c r="BA3" t="n">
-        <v>0.2670379172790708</v>
+        <v>0.262608845959918</v>
       </c>
       <c r="BB3" t="n">
-        <v>-0.1445778452521186</v>
+        <v>-0.1133839041023485</v>
       </c>
       <c r="BC3" t="n">
-        <v>0.2669520320619151</v>
+        <v>0.4822233521235706</v>
       </c>
       <c r="BD3" t="n">
-        <v>-0.0615312184354478</v>
+        <v>-0.05422324265513867</v>
       </c>
       <c r="BE3" t="n">
-        <v>0.09300065788049372</v>
+        <v>0.1680940635442917</v>
       </c>
       <c r="BF3" t="n">
-        <v>-0.07228892262605931</v>
+        <v>-0.05669195205117426</v>
       </c>
       <c r="BG3" t="n">
-        <v>0.1334760160309575</v>
+        <v>0.2411116760617853</v>
       </c>
       <c r="BH3" t="n">
-        <v>75.10342853149074</v>
+        <v>74.28011979665044</v>
       </c>
       <c r="BI3" t="n">
-        <v>59.45004656367831</v>
+        <v>51.77352478249799</v>
       </c>
       <c r="BJ3" t="n">
-        <v>-25.2014236610154</v>
+        <v>-38.15571798437937</v>
       </c>
       <c r="BK3" t="n">
-        <v>12.14569301012065</v>
+        <v>7.296568553904804</v>
       </c>
       <c r="BL3" t="n">
-        <v>0.01589805826231653</v>
+        <v>0.01887679860427735</v>
       </c>
       <c r="BM3" t="n">
-        <v>0.01414726584017816</v>
+        <v>0.01535263762865944</v>
       </c>
       <c r="BN3" t="n">
-        <v>0.06145499120837319</v>
+        <v>0.0726830589950581</v>
       </c>
       <c r="BO3" t="n">
-        <v>0.04873372806083488</v>
+        <v>0.04824235097513396</v>
       </c>
       <c r="BP3" t="n">
-        <v>0.05185957721894627</v>
+        <v>0.05376827457552832</v>
       </c>
       <c r="BQ3" t="n">
-        <v>0.04571188672486447</v>
+        <v>0.04371736864220463</v>
       </c>
       <c r="BR3" t="n">
-        <v>0.04168195799806114</v>
+        <v>0.04095065116298202</v>
       </c>
       <c r="BS3" t="n">
-        <v>0.04796259586305393</v>
+        <v>0.04713830313335133</v>
       </c>
       <c r="BT3" t="n">
-        <v>-0.02442785171493036</v>
+        <v>-0.02817154334759125</v>
       </c>
       <c r="BU3" t="n">
-        <v>-0.03162116649680036</v>
+        <v>-0.0307125006343836</v>
       </c>
       <c r="BV3" t="n">
-        <v>-0.001776580421190908</v>
+        <v>0.003784776917328531</v>
       </c>
       <c r="BW3" t="n">
-        <v>-0.00498166387261515</v>
+        <v>-0.01350262641014433</v>
       </c>
       <c r="BX3" t="n">
-        <v>-0.003658359394066005</v>
+        <v>0.00163913749761288</v>
       </c>
       <c r="BY3" t="n">
-        <v>-0.007431484736914129</v>
+        <v>-0.01595135158764546</v>
       </c>
       <c r="BZ3" t="n">
-        <v>-0.02433021888704212</v>
+        <v>-0.02684847359707806</v>
       </c>
       <c r="CA3" t="n">
-        <v>-0.03049924327619411</v>
+        <v>-0.02776149547790772</v>
       </c>
       <c r="CB3" t="n">
-        <v>-0.002408289603192938</v>
+        <v>-0.006705931273135243</v>
       </c>
       <c r="CC3" t="n">
-        <v>-0.008893864717859346</v>
+        <v>-0.01851344308971568</v>
       </c>
       <c r="CD3" t="n">
-        <v>-0.004285548814259624</v>
+        <v>-0.008802378938228857</v>
       </c>
       <c r="CE3" t="n">
-        <v>-0.01128513177424214</v>
+        <v>-0.0207972434997349</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>57.98057980579806</v>
+        <v>56.07826078260783</v>
       </c>
       <c r="B4" t="n">
-        <v>19.15360340935183</v>
+        <v>18.29986890376677</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5</v>
+        <v>0.7219622196221962</v>
       </c>
       <c r="D4" t="n">
-        <v>1.260990066723166</v>
+        <v>1.296467987594899</v>
       </c>
       <c r="E4" t="n">
-        <v>59.25814258142582</v>
+        <v>57.77912779127792</v>
       </c>
       <c r="F4" t="n">
-        <v>19.72870385158962</v>
+        <v>19.06305907249112</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5</v>
+        <v>0.6455642556425565</v>
       </c>
       <c r="H4" t="n">
-        <v>1.246490272832181</v>
+        <v>1.284174392467016</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6524751668079148</v>
+        <v>0.7411699689872486</v>
       </c>
       <c r="J4" t="n">
-        <v>-1.883774317919548</v>
+        <v>-1.789564018832459</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
-        <v>0.2940392918055511</v>
+        <v>0.297842934908937</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2914835864626361</v>
+        <v>0.2944414577528364</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1356309243852432</v>
+        <v>0.2947554099937199</v>
       </c>
       <c r="O4" t="n">
-        <v>0.180296485776199</v>
+        <v>0.3323850044552822</v>
       </c>
       <c r="P4" t="n">
-        <v>0.06781546219262162</v>
+        <v>0.1473777049968599</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0901482428880995</v>
+        <v>0.1661925022276411</v>
       </c>
       <c r="R4" t="n">
-        <v>52.31193294063381</v>
+        <v>43.75531435107216</v>
       </c>
       <c r="S4" t="n">
-        <v>51.71511865501154</v>
+        <v>43.84944860932053</v>
       </c>
       <c r="T4" t="n">
         <v>2.800000000000001</v>
@@ -1396,247 +1396,247 @@
         <v>2</v>
       </c>
       <c r="V4" t="n">
-        <v>0.06090450081146034</v>
+        <v>0.07146885438697448</v>
       </c>
       <c r="W4" t="n">
-        <v>0.05062623885702998</v>
+        <v>0.05562162566458909</v>
       </c>
       <c r="X4" t="n">
-        <v>25.72843678851818</v>
+        <v>13.89242775427387</v>
       </c>
       <c r="Y4" t="n">
-        <v>16.08833917880933</v>
+        <v>9.587944180220799</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.04829895367037108</v>
+        <v>0.05512581496096761</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.04061502922281204</v>
+        <v>0.04331314032647456</v>
       </c>
       <c r="AB4" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="AC4" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.05612479316284087</v>
+        <v>0.06468931913954425</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.04719584879602528</v>
+        <v>0.05082732218107048</v>
       </c>
       <c r="AF4" t="n">
-        <v>1.085162142776216</v>
+        <v>1.10480146239916</v>
       </c>
       <c r="AG4" t="n">
-        <v>1.072684148045105</v>
+        <v>1.094325321063326</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.2129053569405409</v>
+        <v>0.2620036559979011</v>
       </c>
       <c r="AI4" t="n">
-        <v>-2.318289629887237</v>
+        <v>-2.264186697341684</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0.3170426484150777</v>
+        <v>0.3257241367876161</v>
       </c>
       <c r="AK4" t="n">
-        <v>0.2684165908558657</v>
+        <v>0.2649661865772098</v>
       </c>
       <c r="AL4" t="n">
-        <v>0.1720293078125415</v>
+        <v>0.2565864593668054</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.3672836477746171</v>
+        <v>0.5785254741371562</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.05681558023789944</v>
+        <v>0.08784676964867695</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.1021049696498748</v>
+        <v>0.1603563515071832</v>
       </c>
       <c r="AP4" t="n">
-        <v>0.08601465390627075</v>
+        <v>0.1282932296834027</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0.1836418238873085</v>
+        <v>0.2892627370685781</v>
       </c>
       <c r="AR4" t="n">
-        <v>39.70795886932959</v>
+        <v>32.12069878451009</v>
       </c>
       <c r="AS4" t="n">
-        <v>55.38532393741566</v>
+        <v>48.0549065833119</v>
       </c>
       <c r="AT4" t="n">
-        <v>0.02716565962254116</v>
+        <v>0.02658793258637614</v>
       </c>
       <c r="AU4" t="n">
-        <v>0.03273702878946824</v>
+        <v>0.03418537069834719</v>
       </c>
       <c r="AV4" t="n">
-        <v>2.241966573155611</v>
+        <v>2.688018489395286</v>
       </c>
       <c r="AW4" t="n">
-        <v>1.546451853728303</v>
+        <v>1.62705931011824</v>
       </c>
       <c r="AX4" t="n">
-        <v>3.104916432889027</v>
+        <v>4.220046223488215</v>
       </c>
       <c r="AY4" t="n">
-        <v>-1.133870365679242</v>
+        <v>-0.9323517247043989</v>
       </c>
       <c r="AZ4" t="n">
-        <v>0.2797553671405801</v>
+        <v>0.2802455284145835</v>
       </c>
       <c r="BA4" t="n">
-        <v>0.2684165908558657</v>
+        <v>0.2649661865772098</v>
       </c>
       <c r="BB4" t="n">
-        <v>-0.1155547470558044</v>
+        <v>-0.06582268657612578</v>
       </c>
       <c r="BC4" t="n">
-        <v>0.320631855783804</v>
+        <v>0.5159144546656084</v>
       </c>
       <c r="BD4" t="n">
-        <v>-0.04840394793173008</v>
+        <v>-0.03024338664917521</v>
       </c>
       <c r="BE4" t="n">
-        <v>0.1070247511110088</v>
+        <v>0.1743692274620104</v>
       </c>
       <c r="BF4" t="n">
-        <v>-0.05777737352790221</v>
+        <v>-0.03291134328806289</v>
       </c>
       <c r="BG4" t="n">
-        <v>0.160315927891902</v>
+        <v>0.2579572273328042</v>
       </c>
       <c r="BH4" t="n">
-        <v>70.44832530643828</v>
+        <v>67.97104131334986</v>
       </c>
       <c r="BI4" t="n">
-        <v>56.54641730562825</v>
+        <v>49.35543604621341</v>
       </c>
       <c r="BJ4" t="n">
-        <v>-30.19842568281468</v>
+        <v>-62.21052590211599</v>
       </c>
       <c r="BK4" t="n">
-        <v>9.0467417747618</v>
+        <v>6.177177510168397</v>
       </c>
       <c r="BL4" t="n">
-        <v>0.01522612520286508</v>
+        <v>0.01786721359674362</v>
       </c>
       <c r="BM4" t="n">
-        <v>0.01265655971425749</v>
+        <v>0.01390540641614727</v>
       </c>
       <c r="BN4" t="n">
-        <v>0.057392750309704</v>
+        <v>0.06625122785009492</v>
       </c>
       <c r="BO4" t="n">
-        <v>0.04223912613812685</v>
+        <v>0.04220373798770107</v>
       </c>
       <c r="BP4" t="n">
-        <v>0.04819683019099232</v>
+        <v>0.04942643418892151</v>
       </c>
       <c r="BQ4" t="n">
-        <v>0.03973855408082485</v>
+        <v>0.03853276137609483</v>
       </c>
       <c r="BR4" t="n">
-        <v>0.0389103439215028</v>
+        <v>0.03800031704370419</v>
       </c>
       <c r="BS4" t="n">
-        <v>0.0416649334172539</v>
+        <v>0.04137057047261833</v>
       </c>
       <c r="BT4" t="n">
-        <v>-0.02374619916265513</v>
+        <v>-0.02745254639230837</v>
       </c>
       <c r="BU4" t="n">
-        <v>-0.0307154311331952</v>
+        <v>-0.0297755122158496</v>
       </c>
       <c r="BV4" t="n">
-        <v>-0.001406542965404595</v>
+        <v>0.004055310153288439</v>
       </c>
       <c r="BW4" t="n">
-        <v>-0.0044080937333661</v>
+        <v>-0.01263853048125095</v>
       </c>
       <c r="BX4" t="n">
-        <v>-0.003841012265977273</v>
+        <v>0.001279482931977889</v>
       </c>
       <c r="BY4" t="n">
-        <v>-0.007577442403962681</v>
+        <v>-0.01580646165494122</v>
       </c>
       <c r="BZ4" t="n">
-        <v>-0.02364549377848178</v>
+        <v>-0.02606052724603005</v>
       </c>
       <c r="CA4" t="n">
-        <v>-0.02959537848997569</v>
+        <v>-0.02688772054240456</v>
       </c>
       <c r="CB4" t="n">
-        <v>-0.002017238846675918</v>
+        <v>-0.006131319115623479</v>
       </c>
       <c r="CC4" t="n">
-        <v>-0.008195894532418762</v>
+        <v>-0.01750910469219961</v>
       </c>
       <c r="CD4" t="n">
-        <v>-0.004445860902951003</v>
+        <v>-0.008843506654380953</v>
       </c>
       <c r="CE4" t="n">
-        <v>-0.01128949177319371</v>
+        <v>-0.02046367165621048</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>57.190071900719</v>
+        <v>55.12880128801288</v>
       </c>
       <c r="B5" t="n">
-        <v>18.79849999404022</v>
+        <v>17.87464237590368</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5</v>
+        <v>0.7761102611026111</v>
       </c>
       <c r="D5" t="n">
-        <v>1.247499302547641</v>
+        <v>1.271800132053795</v>
       </c>
       <c r="E5" t="n">
-        <v>58.41493414934149</v>
+        <v>56.74551745517455</v>
       </c>
       <c r="F5" t="n">
-        <v>19.34895253727641</v>
+        <v>18.59902048421408</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5</v>
+        <v>0.7017708177081771</v>
       </c>
       <c r="H5" t="n">
-        <v>1.2127786256096</v>
+        <v>1.253677443896893</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6187482563691027</v>
+        <v>0.6795003301344887</v>
       </c>
       <c r="J5" t="n">
-        <v>-1.968053435976</v>
+        <v>-1.865806390257767</v>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
-        <v>0.2956193867357828</v>
+        <v>0.2997417375895345</v>
       </c>
       <c r="M5" t="n">
-        <v>0.2931696372553508</v>
+        <v>0.2965082465908455</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1724256604042749</v>
+        <v>0.3136206581144917</v>
       </c>
       <c r="O5" t="n">
-        <v>0.2190539113743329</v>
+        <v>0.3541537417428445</v>
       </c>
       <c r="P5" t="n">
-        <v>0.08621283020213744</v>
+        <v>0.1568103290572459</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.1095269556871665</v>
+        <v>0.1770768708714223</v>
       </c>
       <c r="R5" t="n">
-        <v>50.01204967743406</v>
+        <v>42.09280985591618</v>
       </c>
       <c r="S5" t="n">
-        <v>49.31503906181694</v>
+        <v>42.00495229159156</v>
       </c>
       <c r="T5" t="n">
         <v>2.700000000000001</v>
@@ -1645,247 +1645,247 @@
         <v>1.9</v>
       </c>
       <c r="V5" t="n">
-        <v>0.05801767729678004</v>
+        <v>0.06713137805831104</v>
       </c>
       <c r="W5" t="n">
-        <v>0.0478198639467543</v>
+        <v>0.05263902986242827</v>
       </c>
       <c r="X5" t="n">
-        <v>19.27885497348327</v>
+        <v>12.26433698766301</v>
       </c>
       <c r="Y5" t="n">
-        <v>12.50777962622466</v>
+        <v>8.516072808465776</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.04650718215096108</v>
+        <v>0.05278453458713077</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.03943000225842352</v>
+        <v>0.04198769796703584</v>
       </c>
       <c r="AB5" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AC5" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.05324659864166955</v>
+        <v>0.06099278661728457</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.04514385537011114</v>
+        <v>0.04851698935465818</v>
       </c>
       <c r="AF5" t="n">
-        <v>1.089603444667295</v>
+        <v>1.100644548010975</v>
       </c>
       <c r="AG5" t="n">
-        <v>1.059277360223312</v>
+        <v>1.084960764519786</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.2240086116682372</v>
+        <v>0.2516113700274386</v>
       </c>
       <c r="AI5" t="n">
-        <v>-2.351806599441721</v>
+        <v>-2.287598088700534</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.3174587397219557</v>
+        <v>0.3259089294885351</v>
       </c>
       <c r="AK5" t="n">
-        <v>0.270177126695354</v>
+        <v>0.2678422755564227</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.1983865282473615</v>
+        <v>0.2729640504469745</v>
       </c>
       <c r="AM5" t="n">
-        <v>0.4110121897967596</v>
+        <v>0.5999895752827809</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.0657406053703164</v>
+        <v>0.09333085770859355</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.1142899719695283</v>
+        <v>0.1673901302231228</v>
       </c>
       <c r="AP5" t="n">
-        <v>0.09919326412368075</v>
+        <v>0.1364820252234872</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.2055060948983798</v>
+        <v>0.2999947876413904</v>
       </c>
       <c r="AR5" t="n">
-        <v>38.46002095790569</v>
+        <v>31.4008135212329</v>
       </c>
       <c r="AS5" t="n">
-        <v>52.74956603025445</v>
+        <v>45.84170532617449</v>
       </c>
       <c r="AT5" t="n">
-        <v>0.02800950358066696</v>
+        <v>0.02845401523671071</v>
       </c>
       <c r="AU5" t="n">
-        <v>0.03273350696948093</v>
+        <v>0.03423500116988514</v>
       </c>
       <c r="AV5" t="n">
-        <v>2.071356856778628</v>
+        <v>2.35929367085246</v>
       </c>
       <c r="AW5" t="n">
-        <v>1.460884224575727</v>
+        <v>1.537579321268791</v>
       </c>
       <c r="AX5" t="n">
-        <v>2.67839214194657</v>
+        <v>3.398234177131151</v>
       </c>
       <c r="AY5" t="n">
-        <v>-1.347789438560683</v>
+        <v>-1.156051696828022</v>
       </c>
       <c r="AZ5" t="n">
-        <v>0.2831656996869688</v>
+        <v>0.2845679373083452</v>
       </c>
       <c r="BA5" t="n">
-        <v>0.270177126695354</v>
+        <v>0.2678422755564227</v>
       </c>
       <c r="BB5" t="n">
-        <v>-0.05375379889380745</v>
+        <v>0.01321322788305265</v>
       </c>
       <c r="BC5" t="n">
-        <v>0.3678125634901288</v>
+        <v>0.5433162684829774</v>
       </c>
       <c r="BD5" t="n">
-        <v>-0.0219067156310621</v>
+        <v>0.005775450851110768</v>
       </c>
       <c r="BE5" t="n">
-        <v>0.120111070552652</v>
+        <v>0.1804473880604332</v>
       </c>
       <c r="BF5" t="n">
-        <v>-0.02687689944690373</v>
+        <v>0.006606613941526326</v>
       </c>
       <c r="BG5" t="n">
-        <v>0.1839062817450644</v>
+        <v>0.2716581342414887</v>
       </c>
       <c r="BH5" t="n">
-        <v>65.86417764339259</v>
+        <v>62.10583340672036</v>
       </c>
       <c r="BI5" t="n">
-        <v>53.73198337798217</v>
+        <v>46.94491506464711</v>
       </c>
       <c r="BJ5" t="n">
-        <v>-61.84061846002771</v>
+        <v>291.0980328353404</v>
       </c>
       <c r="BK5" t="n">
-        <v>7.449123161261578</v>
+        <v>5.551104805413742</v>
       </c>
       <c r="BL5" t="n">
-        <v>0.01450441932419501</v>
+        <v>0.01678284451457776</v>
       </c>
       <c r="BM5" t="n">
-        <v>0.01195496598668858</v>
+        <v>0.01315975746560707</v>
       </c>
       <c r="BN5" t="n">
-        <v>0.05294569671339285</v>
+        <v>0.05933160252303486</v>
       </c>
       <c r="BO5" t="n">
-        <v>0.03855517787063346</v>
+        <v>0.03846321706612884</v>
       </c>
       <c r="BP5" t="n">
-        <v>0.04445196128421481</v>
+        <v>0.04500041173981374</v>
       </c>
       <c r="BQ5" t="n">
-        <v>0.03626206457835356</v>
+        <v>0.03522576699209243</v>
       </c>
       <c r="BR5" t="n">
-        <v>0.03608516237486031</v>
+        <v>0.03497690814532944</v>
       </c>
       <c r="BS5" t="n">
-        <v>0.03806448822563547</v>
+        <v>0.03776418125425757</v>
       </c>
       <c r="BT5" t="n">
-        <v>-0.02206397520037773</v>
+        <v>-0.02562557897479202</v>
       </c>
       <c r="BU5" t="n">
-        <v>-0.02850070566484374</v>
+        <v>-0.0275478353975069</v>
       </c>
       <c r="BV5" t="n">
-        <v>-0.0007145076088215404</v>
+        <v>0.004465329579521619</v>
       </c>
       <c r="BW5" t="n">
-        <v>-0.003280298876885357</v>
+        <v>-0.01079294460147055</v>
       </c>
       <c r="BX5" t="n">
-        <v>-0.004070127455556853</v>
+        <v>0.0006391893555526829</v>
       </c>
       <c r="BY5" t="n">
-        <v>-0.00764886055797794</v>
+        <v>-0.01515955243547606</v>
       </c>
       <c r="BZ5" t="n">
-        <v>-0.02196059087278938</v>
+        <v>-0.02415210591859589</v>
       </c>
       <c r="CA5" t="n">
-        <v>-0.02741536341520719</v>
+        <v>-0.02485387618831984</v>
       </c>
       <c r="CB5" t="n">
-        <v>-0.001272758794039131</v>
+        <v>-0.004959249515632345</v>
       </c>
       <c r="CC5" t="n">
-        <v>-0.006753886906596965</v>
+        <v>-0.01529765490550886</v>
       </c>
       <c r="CD5" t="n">
-        <v>-0.004620318925661545</v>
+        <v>-0.008697670177162916</v>
       </c>
       <c r="CE5" t="n">
-        <v>-0.01101803445469216</v>
+        <v>-0.01937016612617249</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>56.59676596765968</v>
+        <v>54.44709447094471</v>
       </c>
       <c r="B6" t="n">
-        <v>18.53230501857727</v>
+        <v>17.56957681884398</v>
       </c>
       <c r="C6" t="n">
-        <v>0.5165755657556576</v>
+        <v>0.8429853298532985</v>
       </c>
       <c r="D6" t="n">
-        <v>1.226704595843865</v>
+        <v>1.234605221892104</v>
       </c>
       <c r="E6" t="n">
-        <v>57.71112711127111</v>
+        <v>55.9320593205932</v>
       </c>
       <c r="F6" t="n">
-        <v>19.03250356951729</v>
+        <v>18.23435960335043</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5</v>
+        <v>0.7758775587755877</v>
       </c>
       <c r="H6" t="n">
-        <v>1.202118345086542</v>
+        <v>1.23694702711554</v>
       </c>
       <c r="I6" t="n">
-        <v>0.5667614896096623</v>
+        <v>0.5865130547302611</v>
       </c>
       <c r="J6" t="n">
-        <v>-1.994704137283644</v>
+        <v>-1.907632432211151</v>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
-        <v>0.2968067066336761</v>
+        <v>0.301105328440335</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2945785113922319</v>
+        <v>0.2981364799652667</v>
       </c>
       <c r="N6" t="n">
-        <v>0.2147411878718269</v>
+        <v>0.3405488137280514</v>
       </c>
       <c r="O6" t="n">
-        <v>0.2623709285543007</v>
+        <v>0.382841993754096</v>
       </c>
       <c r="P6" t="n">
-        <v>0.1073705939359134</v>
+        <v>0.1702744068640257</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.1311854642771503</v>
+        <v>0.191420996877048</v>
       </c>
       <c r="R6" t="n">
-        <v>47.69742624025782</v>
+        <v>40.39317361400104</v>
       </c>
       <c r="S6" t="n">
-        <v>46.84810795835929</v>
+        <v>40.06801072794364</v>
       </c>
       <c r="T6" t="n">
         <v>2.600000000000001</v>
@@ -1894,247 +1894,247 @@
         <v>1.8</v>
       </c>
       <c r="V6" t="n">
-        <v>0.05490879043481665</v>
+        <v>0.06246024970436581</v>
       </c>
       <c r="W6" t="n">
-        <v>0.04596123910939658</v>
+        <v>0.05033506110055676</v>
       </c>
       <c r="X6" t="n">
-        <v>14.65039763737286</v>
+        <v>10.5086666549021</v>
       </c>
       <c r="Y6" t="n">
-        <v>10.0368868514775</v>
+        <v>7.533112810843485</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.04476121685762841</v>
+        <v>0.05059127289988442</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.03823353939922426</v>
+        <v>0.04069298037599399</v>
       </c>
       <c r="AB6" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AC6" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.05064920358597835</v>
+        <v>0.05769587923256649</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.04326286139635651</v>
+        <v>0.04640755503489043</v>
       </c>
       <c r="AF6" t="n">
-        <v>1.084099779409315</v>
+        <v>1.082577309422647</v>
       </c>
       <c r="AG6" t="n">
-        <v>1.062371688463198</v>
+        <v>1.08463074735813</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.2102494485232886</v>
+        <v>0.206443273556618</v>
       </c>
       <c r="AI6" t="n">
-        <v>-2.344070778842005</v>
+        <v>-2.288423131604675</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.3178885841314812</v>
+        <v>0.3259683221318029</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.272341466876856</v>
+        <v>0.2712780193320478</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.2253446444659913</v>
+        <v>0.2918360656262429</v>
       </c>
       <c r="AM6" t="n">
-        <v>0.4504023037714934</v>
+        <v>0.616157943408675</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.07458591143326568</v>
+        <v>0.09897917255068914</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.1264307225107155</v>
+        <v>0.1740794931283701</v>
       </c>
       <c r="AP6" t="n">
-        <v>0.1126723222329956</v>
+        <v>0.1459180328131215</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0.2252011518857467</v>
+        <v>0.3080789717043375</v>
       </c>
       <c r="AR6" t="n">
-        <v>37.19902471639204</v>
+        <v>30.67928912767725</v>
       </c>
       <c r="AS6" t="n">
-        <v>50.06697235412246</v>
+        <v>43.56159458442018</v>
       </c>
       <c r="AT6" t="n">
-        <v>0.02877102129897562</v>
+        <v>0.03011835922214425</v>
       </c>
       <c r="AU6" t="n">
-        <v>0.03243349956115919</v>
+        <v>0.03403198700407719</v>
       </c>
       <c r="AV6" t="n">
-        <v>1.908475540865546</v>
+        <v>2.073826440666212</v>
       </c>
       <c r="AW6" t="n">
-        <v>1.417091579116475</v>
+        <v>1.479051490426533</v>
       </c>
       <c r="AX6" t="n">
-        <v>2.271188852163866</v>
+        <v>2.684566101665531</v>
       </c>
       <c r="AY6" t="n">
-        <v>-1.457271052208813</v>
+        <v>-1.302371273933669</v>
       </c>
       <c r="AZ6" t="n">
-        <v>0.2856941808797556</v>
+        <v>0.2878252715628371</v>
       </c>
       <c r="BA6" t="n">
-        <v>0.272341466876856</v>
+        <v>0.2712780193320478</v>
       </c>
       <c r="BB6" t="n">
-        <v>0.01790536441156498</v>
+        <v>0.09765384116005343</v>
       </c>
       <c r="BC6" t="n">
-        <v>0.4096315397831007</v>
+        <v>0.5643317467859383</v>
       </c>
       <c r="BD6" t="n">
-        <v>0.007066882298390071</v>
+        <v>0.0404766403036884</v>
       </c>
       <c r="BE6" t="n">
-        <v>0.1328024597160338</v>
+        <v>0.1861833048655924</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.008952682205782488</v>
+        <v>0.04882692058002672</v>
       </c>
       <c r="BG6" t="n">
-        <v>0.2048157698915503</v>
+        <v>0.2821658733929692</v>
       </c>
       <c r="BH6" t="n">
-        <v>61.34812061914787</v>
+        <v>56.6593288084937</v>
       </c>
       <c r="BI6" t="n">
-        <v>50.93338669876145</v>
+        <v>44.52173334377983</v>
       </c>
       <c r="BJ6" t="n">
-        <v>175.7038779313078</v>
+        <v>36.64688542755982</v>
       </c>
       <c r="BK6" t="n">
-        <v>6.428681326725336</v>
+        <v>5.110466027404137</v>
       </c>
       <c r="BL6" t="n">
-        <v>0.01372719760870416</v>
+        <v>0.01561506242609145</v>
       </c>
       <c r="BM6" t="n">
-        <v>0.01149030977734914</v>
+        <v>0.01258376527513919</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.04818516382129027</v>
+        <v>0.05218038122675305</v>
       </c>
       <c r="BO6" t="n">
-        <v>0.03568493916142309</v>
+        <v>0.03529392620768535</v>
       </c>
       <c r="BP6" t="n">
-        <v>0.04061058874349176</v>
+        <v>0.04047606343487728</v>
       </c>
       <c r="BQ6" t="n">
-        <v>0.03353070693157676</v>
+        <v>0.03240050063979077</v>
       </c>
       <c r="BR6" t="n">
-        <v>0.03319706161156957</v>
+        <v>0.03186922257798593</v>
       </c>
       <c r="BS6" t="n">
-        <v>0.03524286058717162</v>
+        <v>0.0346876007763172</v>
       </c>
       <c r="BT6" t="n">
-        <v>-0.02039150699389587</v>
+        <v>-0.02378555024975349</v>
       </c>
       <c r="BU6" t="n">
-        <v>-0.02630762250488527</v>
+        <v>-0.02536680170512642</v>
       </c>
       <c r="BV6" t="n">
-        <v>-0.0001317036616334838</v>
+        <v>0.004749978820756746</v>
       </c>
       <c r="BW6" t="n">
-        <v>-0.002298588849037125</v>
+        <v>-0.00910566915851245</v>
       </c>
       <c r="BX6" t="n">
-        <v>-0.004197925358265686</v>
+        <v>0.0001135971375947464</v>
       </c>
       <c r="BY6" t="n">
-        <v>-0.007592257709655196</v>
+        <v>-0.01439697041618972</v>
       </c>
       <c r="BZ6" t="n">
-        <v>-0.02028759570880822</v>
+        <v>-0.02226988109245948</v>
       </c>
       <c r="CA6" t="n">
-        <v>-0.02526895005360016</v>
+        <v>-0.02287778298991028</v>
       </c>
       <c r="CB6" t="n">
-        <v>-0.0006381730961425149</v>
+        <v>-0.003915734648662569</v>
       </c>
       <c r="CC6" t="n">
-        <v>-0.005460311729467683</v>
+        <v>-0.01324219003025232</v>
       </c>
       <c r="CD6" t="n">
-        <v>-0.004694628314461441</v>
+        <v>-0.008445820862046673</v>
       </c>
       <c r="CE6" t="n">
-        <v>-0.01062745522892421</v>
+        <v>-0.01817711539176237</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>56.06211062110621</v>
+        <v>53.86993869938699</v>
       </c>
       <c r="B7" t="n">
-        <v>18.29263179368823</v>
+        <v>17.31140569257632</v>
       </c>
       <c r="C7" t="n">
-        <v>0.6192867928679286</v>
+        <v>0.9161075610756108</v>
       </c>
       <c r="D7" t="n">
-        <v>1.195275813492352</v>
+        <v>1.242058297748026</v>
       </c>
       <c r="E7" t="n">
-        <v>57.03112031120311</v>
+        <v>55.18490184901849</v>
       </c>
       <c r="F7" t="n">
-        <v>18.72715861016297</v>
+        <v>17.89975546460377</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5799421994219942</v>
+        <v>0.859220792207922</v>
       </c>
       <c r="H7" t="n">
-        <v>1.197982587212228</v>
+        <v>1.218644224422509</v>
       </c>
       <c r="I7" t="n">
-        <v>0.4881895337308806</v>
+        <v>0.6051457443700653</v>
       </c>
       <c r="J7" t="n">
-        <v>-2.00504353196943</v>
+        <v>-1.953389438943727</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
-        <v>0.2978759353280276</v>
+        <v>0.3022605163655339</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2959384147576039</v>
+        <v>0.2996297694692405</v>
       </c>
       <c r="N7" t="n">
-        <v>0.2600533601097056</v>
+        <v>0.3653101756090399</v>
       </c>
       <c r="O7" t="n">
-        <v>0.3077658985650001</v>
+        <v>0.4152257139917249</v>
       </c>
       <c r="P7" t="n">
-        <v>0.1300266800548528</v>
+        <v>0.18265508780452</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.1538829492825001</v>
+        <v>0.2076128569958625</v>
       </c>
       <c r="R7" t="n">
-        <v>45.35172905253927</v>
+        <v>38.79835109699712</v>
       </c>
       <c r="S7" t="n">
-        <v>44.3188015729954</v>
+        <v>38.05938288014368</v>
       </c>
       <c r="T7" t="n">
         <v>2.500000000000001</v>
@@ -2143,247 +2143,247 @@
         <v>1.7</v>
       </c>
       <c r="V7" t="n">
-        <v>0.05155119262389619</v>
+        <v>0.05741543108210496</v>
       </c>
       <c r="W7" t="n">
-        <v>0.04443442271486049</v>
+        <v>0.04811784881460569</v>
       </c>
       <c r="X7" t="n">
-        <v>11.35793169629945</v>
+        <v>9.005135010387244</v>
       </c>
       <c r="Y7" t="n">
-        <v>8.272222358866033</v>
+        <v>6.639655485049369</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.04312911885439571</v>
+        <v>0.0462260355944683</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.03709104221478032</v>
+        <v>0.03948473873694167</v>
       </c>
       <c r="AB7" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="AC7" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.04829342667500261</v>
+        <v>0.05206701296597464</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.04153234694050225</v>
+        <v>0.04447390690843667</v>
       </c>
       <c r="AF7" t="n">
-        <v>1.067457750944392</v>
+        <v>1.102721815818885</v>
       </c>
       <c r="AG7" t="n">
-        <v>1.069875073000706</v>
+        <v>1.081934378143823</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.1686443773609797</v>
+        <v>0.2568045395472118</v>
       </c>
       <c r="AI7" t="n">
-        <v>-2.325312317498235</v>
+        <v>-2.295164054640443</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.3183209005628527</v>
+        <v>0.3258923112061414</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.2749453897155675</v>
+        <v>0.2753119209400757</v>
       </c>
       <c r="AL7" t="n">
-        <v>0.2535442805579975</v>
+        <v>0.3068333320674511</v>
       </c>
       <c r="AM7" t="n">
-        <v>0.4863739741566267</v>
+        <v>0.6278752788436067</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.08338622640133131</v>
+        <v>0.1050049164886342</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.138319466169391</v>
+        <v>0.17980379794886</v>
       </c>
       <c r="AP7" t="n">
-        <v>0.1267721402789988</v>
+        <v>0.1534166660337255</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0.2431869870783133</v>
+        <v>0.3139376394218034</v>
       </c>
       <c r="AR7" t="n">
-        <v>35.91505917253793</v>
+        <v>30.0829048410905</v>
       </c>
       <c r="AS7" t="n">
-        <v>47.31083673888</v>
+        <v>41.20520690578345</v>
       </c>
       <c r="AT7" t="n">
-        <v>0.02946170015976719</v>
+        <v>0.03006995241838535</v>
       </c>
       <c r="AU7" t="n">
-        <v>0.03203989673471162</v>
+        <v>0.03376626705084224</v>
       </c>
       <c r="AV7" t="n">
-        <v>1.749769780574114</v>
+        <v>1.909395475032413</v>
       </c>
       <c r="AW7" t="n">
-        <v>1.386846626965585</v>
+        <v>1.425027194808183</v>
       </c>
       <c r="AX7" t="n">
-        <v>1.874424451435286</v>
+        <v>2.273488687581033</v>
       </c>
       <c r="AY7" t="n">
-        <v>-1.532883432586036</v>
+        <v>-1.437432012979542</v>
       </c>
       <c r="AZ7" t="n">
-        <v>0.2879042264970392</v>
+        <v>0.290665469079911</v>
       </c>
       <c r="BA7" t="n">
-        <v>0.2749453897155675</v>
+        <v>0.2753119209400757</v>
       </c>
       <c r="BB7" t="n">
-        <v>0.0933388052777987</v>
+        <v>0.1747825224469897</v>
       </c>
       <c r="BC7" t="n">
-        <v>0.4478078248598014</v>
+        <v>0.5806269570148747</v>
       </c>
       <c r="BD7" t="n">
-        <v>0.03554681827996105</v>
+        <v>0.0702003678961831</v>
       </c>
       <c r="BE7" t="n">
-        <v>0.1449947699199788</v>
+        <v>0.1908243483490867</v>
       </c>
       <c r="BF7" t="n">
-        <v>0.04666940263889935</v>
+        <v>0.08739126122349483</v>
       </c>
       <c r="BG7" t="n">
-        <v>0.2239039124299007</v>
+        <v>0.2903134785074373</v>
       </c>
       <c r="BH7" t="n">
-        <v>56.91060833632368</v>
+        <v>51.84687849442006</v>
       </c>
       <c r="BI7" t="n">
-        <v>48.0839825491438</v>
+        <v>42.03931478652999</v>
       </c>
       <c r="BJ7" t="n">
-        <v>31.64456716618857</v>
+        <v>18.8214651522562</v>
       </c>
       <c r="BK7" t="n">
-        <v>5.685276641561827</v>
+        <v>4.748249146754945</v>
       </c>
       <c r="BL7" t="n">
-        <v>0.01288779815597405</v>
+        <v>0.01435385777052624</v>
       </c>
       <c r="BM7" t="n">
-        <v>0.01110860567871512</v>
+        <v>0.01202946220365142</v>
       </c>
       <c r="BN7" t="n">
-        <v>0.04319061057727525</v>
+        <v>0.04514934777977541</v>
       </c>
       <c r="BO7" t="n">
-        <v>0.03306475679172989</v>
+        <v>0.03222165429143534</v>
       </c>
       <c r="BP7" t="n">
-        <v>0.03667528347191585</v>
+        <v>0.03597544019597838</v>
       </c>
       <c r="BQ7" t="n">
-        <v>0.03104411395898945</v>
+        <v>0.0296635884631049</v>
       </c>
       <c r="BR7" t="n">
-        <v>0.03023916877286145</v>
+        <v>0.02877963309788323</v>
       </c>
       <c r="BS7" t="n">
-        <v>0.03266120457429835</v>
+        <v>0.03169800991464296</v>
       </c>
       <c r="BT7" t="n">
-        <v>-0.01872531014111794</v>
+        <v>-0.02193715859326486</v>
       </c>
       <c r="BU7" t="n">
-        <v>-0.02412821865695347</v>
+        <v>-0.02321346453822819</v>
       </c>
       <c r="BV7" t="n">
-        <v>0.0003780581307961395</v>
+        <v>0.004950522426444197</v>
       </c>
       <c r="BW7" t="n">
-        <v>-0.001415843376839104</v>
+        <v>-0.007529509109591303</v>
       </c>
       <c r="BX7" t="n">
-        <v>-0.004260592833808558</v>
+        <v>-0.0003385537655126942</v>
       </c>
       <c r="BY7" t="n">
-        <v>-0.007454737465408263</v>
+        <v>-0.01356570229189304</v>
       </c>
       <c r="BZ7" t="n">
-        <v>-0.01862221610283319</v>
+        <v>-0.02040389572473228</v>
       </c>
       <c r="CA7" t="n">
-        <v>-0.02314317710134851</v>
+        <v>-0.02093411350048825</v>
       </c>
       <c r="CB7" t="n">
-        <v>-7.737837205131935e-05</v>
+        <v>-0.002960436391297258</v>
       </c>
       <c r="CC7" t="n">
-        <v>-0.004269146492106596</v>
+        <v>-0.0112985283060698</v>
       </c>
       <c r="CD7" t="n">
-        <v>-0.004704887965764656</v>
+        <v>-0.008128253188118929</v>
       </c>
       <c r="CE7" t="n">
-        <v>-0.01016370339682642</v>
+        <v>-0.01692817616992836</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>55.52915529155291</v>
+        <v>53.32933329333294</v>
       </c>
       <c r="B8" t="n">
-        <v>18.05388973755599</v>
+        <v>17.06963576463708</v>
       </c>
       <c r="C8" t="n">
-        <v>0.725220052200522</v>
+        <v>0.9927919279192792</v>
       </c>
       <c r="D8" t="n">
-        <v>1.202290324257621</v>
+        <v>1.218415959707605</v>
       </c>
       <c r="E8" t="n">
-        <v>56.32476324763248</v>
+        <v>54.43944439444394</v>
       </c>
       <c r="F8" t="n">
-        <v>18.41034982863581</v>
+        <v>17.56615427257209</v>
       </c>
       <c r="G8" t="n">
-        <v>0.6926238262382624</v>
+        <v>0.9479161791617916</v>
       </c>
       <c r="H8" t="n">
-        <v>1.193399046020158</v>
+        <v>1.191787905311847</v>
       </c>
       <c r="I8" t="n">
-        <v>0.5057258106440515</v>
+        <v>0.5460398992690135</v>
       </c>
       <c r="J8" t="n">
-        <v>-2.016502384949605</v>
+        <v>-2.020530236720382</v>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
-        <v>0.2989418825970642</v>
+        <v>0.3033407810275106</v>
       </c>
       <c r="M8" t="n">
-        <v>0.2973510141360719</v>
+        <v>0.3011203181782858</v>
       </c>
       <c r="N8" t="n">
-        <v>0.3020336970370803</v>
+        <v>0.3947160580853748</v>
       </c>
       <c r="O8" t="n">
-        <v>0.3541419396136146</v>
+        <v>0.450010112160144</v>
       </c>
       <c r="P8" t="n">
-        <v>0.1510168485185401</v>
+        <v>0.1973580290426874</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.1770709698068073</v>
+        <v>0.225005056080072</v>
       </c>
       <c r="R8" t="n">
-        <v>43.09284316171597</v>
+        <v>37.12639334258617</v>
       </c>
       <c r="S8" t="n">
-        <v>41.73374489107451</v>
+        <v>35.99306314365209</v>
       </c>
       <c r="T8" t="n">
         <v>2.400000000000001</v>
@@ -2392,247 +2392,247 @@
         <v>1.6</v>
       </c>
       <c r="V8" t="n">
-        <v>0.047913794995399</v>
+        <v>0.05195021090798905</v>
       </c>
       <c r="W8" t="n">
-        <v>0.04298643398796476</v>
+        <v>0.04573337150644272</v>
       </c>
       <c r="X8" t="n">
-        <v>9.0892554017533</v>
+        <v>7.54094913271603</v>
       </c>
       <c r="Y8" t="n">
-        <v>6.954683670387185</v>
+        <v>5.822837830809024</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.03985210063549699</v>
+        <v>0.0426375003495982</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.03602016788208381</v>
+        <v>0.03837375031463838</v>
       </c>
       <c r="AB8" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AC8" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.04418334780904495</v>
+        <v>0.04743883403566578</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.03993494898125216</v>
+        <v>0.0426949506320992</v>
       </c>
       <c r="AF8" t="n">
-        <v>1.084431066710395</v>
+        <v>1.095098814379196</v>
       </c>
       <c r="AG8" t="n">
-        <v>1.076411391138753</v>
+        <v>1.071165813037834</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.2110776667759873</v>
+        <v>0.2377470359479905</v>
       </c>
       <c r="AI8" t="n">
-        <v>-2.308971522153118</v>
+        <v>-2.322085467405415</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.3187502188632347</v>
+        <v>0.3256692245303652</v>
       </c>
       <c r="AK8" t="n">
-        <v>0.2780420009059285</v>
+        <v>0.2799785999487803</v>
       </c>
       <c r="AL8" t="n">
-        <v>0.2779645601765581</v>
+        <v>0.3263044284596496</v>
       </c>
       <c r="AM8" t="n">
-        <v>0.5188343274131492</v>
+        <v>0.6352091686879894</v>
       </c>
       <c r="AN8" t="n">
-        <v>0.09226583043212078</v>
+        <v>0.1112055192546483</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.1496677569983996</v>
+        <v>0.1840644626597201</v>
       </c>
       <c r="AP8" t="n">
-        <v>0.1389822800882791</v>
+        <v>0.1631522142298248</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0.2594171637065746</v>
+        <v>0.3176045843439947</v>
       </c>
       <c r="AR8" t="n">
-        <v>34.71253028464043</v>
+        <v>29.45096740821688</v>
       </c>
       <c r="AS8" t="n">
-        <v>44.47799188093184</v>
+        <v>38.77895705826994</v>
       </c>
       <c r="AT8" t="n">
-        <v>0.02881051788259528</v>
+        <v>0.03003015126862804</v>
       </c>
       <c r="AU8" t="n">
-        <v>0.03162443419844523</v>
+        <v>0.03349971069939307</v>
       </c>
       <c r="AV8" t="n">
-        <v>1.663066078529057</v>
+        <v>1.729935039063906</v>
       </c>
       <c r="AW8" t="n">
-        <v>1.359279148465465</v>
+        <v>1.365187058384695</v>
       </c>
       <c r="AX8" t="n">
-        <v>1.657665196322642</v>
+        <v>1.824837597659765</v>
       </c>
       <c r="AY8" t="n">
-        <v>-1.601802128836337</v>
+        <v>-1.587032354038263</v>
       </c>
       <c r="AZ8" t="n">
-        <v>0.2900146004734872</v>
+        <v>0.2933260636734031</v>
       </c>
       <c r="BA8" t="n">
-        <v>0.2780420009059285</v>
+        <v>0.2799785999487803</v>
       </c>
       <c r="BB8" t="n">
-        <v>0.1651259558985059</v>
+        <v>0.2498415961746794</v>
       </c>
       <c r="BC8" t="n">
-        <v>0.4825214254360189</v>
+        <v>0.5925278058424351</v>
       </c>
       <c r="BD8" t="n">
-        <v>0.06175753596205705</v>
+        <v>0.09638962654679871</v>
       </c>
       <c r="BE8" t="n">
-        <v>0.1564160573315751</v>
+        <v>0.1938338644374159</v>
       </c>
       <c r="BF8" t="n">
-        <v>0.08256297794925296</v>
+        <v>0.1249207980873397</v>
       </c>
       <c r="BG8" t="n">
-        <v>0.2412607127180095</v>
+        <v>0.2962639029212176</v>
       </c>
       <c r="BH8" t="n">
-        <v>52.74190658390556</v>
+        <v>47.33946282893898</v>
       </c>
       <c r="BI8" t="n">
-        <v>45.16700482326005</v>
+        <v>39.49266949021431</v>
       </c>
       <c r="BJ8" t="n">
-        <v>16.62524325038819</v>
+        <v>11.91366943547293</v>
       </c>
       <c r="BK8" t="n">
-        <v>5.104329864587708</v>
+        <v>4.422308659667107</v>
       </c>
       <c r="BL8" t="n">
-        <v>0.01197844874884975</v>
+        <v>0.01298755272699726</v>
       </c>
       <c r="BM8" t="n">
-        <v>0.01074660849699119</v>
+        <v>0.01143334287661068</v>
       </c>
       <c r="BN8" t="n">
-        <v>0.03813537966596239</v>
+        <v>0.03820322441452783</v>
       </c>
       <c r="BO8" t="n">
-        <v>0.0304844674973273</v>
+        <v>0.02908548638913706</v>
       </c>
       <c r="BP8" t="n">
-        <v>0.03273386929169941</v>
+        <v>0.03135586576250416</v>
       </c>
       <c r="BQ8" t="n">
-        <v>0.02861477860448844</v>
+        <v>0.02687692159774306</v>
       </c>
       <c r="BR8" t="n">
-        <v>0.02728495655990796</v>
+        <v>0.02554280420184993</v>
       </c>
       <c r="BS8" t="n">
-        <v>0.03011781062356645</v>
+        <v>0.02864361286284896</v>
       </c>
       <c r="BT8" t="n">
-        <v>-0.01540666253574766</v>
+        <v>-0.01822211990856982</v>
       </c>
       <c r="BU8" t="n">
-        <v>-0.01979886953088199</v>
+        <v>-0.01896241450890249</v>
       </c>
       <c r="BV8" t="n">
-        <v>0.001231096870508971</v>
+        <v>0.005159318978009496</v>
       </c>
       <c r="BW8" t="n">
-        <v>0.000121311253987004</v>
+        <v>-0.004641656182525272</v>
       </c>
       <c r="BX8" t="n">
-        <v>-0.004243169232400403</v>
+        <v>-0.001082541152072559</v>
       </c>
       <c r="BY8" t="n">
-        <v>-0.00700544035124639</v>
+        <v>-0.01176522033525584</v>
       </c>
       <c r="BZ8" t="n">
-        <v>-0.01530806099016138</v>
+        <v>-0.0167061725017451</v>
       </c>
       <c r="CA8" t="n">
-        <v>-0.01893472276222227</v>
+        <v>-0.01710753955389204</v>
       </c>
       <c r="CB8" t="n">
-        <v>0.0008753572226797093</v>
+        <v>-0.001255767069389537</v>
       </c>
       <c r="CC8" t="n">
-        <v>-0.002127021961492976</v>
+        <v>-0.00768177451602012</v>
       </c>
       <c r="CD8" t="n">
-        <v>-0.004585760482241563</v>
+        <v>-0.007354523913298234</v>
       </c>
       <c r="CE8" t="n">
-        <v>-0.009083435216424742</v>
+        <v>-0.01432555752698511</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>54.96729967299673</v>
+        <v>52.79637796377963</v>
       </c>
       <c r="B9" t="n">
-        <v>17.80235445858203</v>
+        <v>16.83130141101201</v>
       </c>
       <c r="C9" t="n">
-        <v>0.8332118321183213</v>
+        <v>1.071713817138171</v>
       </c>
       <c r="D9" t="n">
-        <v>1.185485916120798</v>
+        <v>1.160611286042853</v>
       </c>
       <c r="E9" t="n">
-        <v>55.56145561455615</v>
+        <v>53.66168661686616</v>
       </c>
       <c r="F9" t="n">
-        <v>18.06835463872141</v>
+        <v>17.21826709079559</v>
       </c>
       <c r="G9" t="n">
-        <v>0.8092076920769208</v>
+        <v>1.039923099230992</v>
       </c>
       <c r="H9" t="n">
-        <v>1.185067690198406</v>
+        <v>1.196826943389362</v>
       </c>
       <c r="I9" t="n">
-        <v>0.4637147903019939</v>
+        <v>0.4015282151071314</v>
       </c>
       <c r="J9" t="n">
-        <v>-2.037330774503985</v>
+        <v>-2.007932641526595</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
-        <v>0.3000654171671014</v>
+        <v>0.3044073355297512</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2988770389532688</v>
+        <v>0.3026769599727747</v>
       </c>
       <c r="N9" t="n">
-        <v>0.3462034947626333</v>
+        <v>0.4290507988180742</v>
       </c>
       <c r="O9" t="n">
-        <v>0.4007764480985715</v>
+        <v>0.4804958028437142</v>
       </c>
       <c r="P9" t="n">
-        <v>0.1731017473813167</v>
+        <v>0.2145253994090371</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.2003882240492858</v>
+        <v>0.2402479014218571</v>
       </c>
       <c r="R9" t="n">
-        <v>40.77105106932142</v>
+        <v>35.37419021270129</v>
       </c>
       <c r="S9" t="n">
-        <v>39.10349931510414</v>
+        <v>33.9882453241072</v>
       </c>
       <c r="T9" t="n">
         <v>2.300000000000001</v>
@@ -2641,247 +2641,247 @@
         <v>1.5</v>
       </c>
       <c r="V9" t="n">
-        <v>0.04396010192094557</v>
+        <v>0.04600975419699348</v>
       </c>
       <c r="W9" t="n">
-        <v>0.04150322700359185</v>
+        <v>0.04305234397454302</v>
       </c>
       <c r="X9" t="n">
-        <v>7.275293799193744</v>
+        <v>6.144192945273719</v>
       </c>
       <c r="Y9" t="n">
-        <v>5.933394047114764</v>
+        <v>5.133707353325343</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.03708192676366318</v>
+        <v>0.03964269066679978</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.03502181972123745</v>
+        <v>0.03597207116061461</v>
       </c>
       <c r="AB9" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="AC9" t="n">
         <v>54</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.04071798719657083</v>
+        <v>0.04356627615520327</v>
       </c>
       <c r="AE9" t="n">
-        <v>0.03845587679676134</v>
+        <v>0.03953236169638815</v>
       </c>
       <c r="AF9" t="n">
-        <v>1.079623649094516</v>
+        <v>1.056086456255417</v>
       </c>
       <c r="AG9" t="n">
-        <v>1.079242770173612</v>
+        <v>1.089040525966767</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.1990591227362892</v>
+        <v>0.1402161406385416</v>
       </c>
       <c r="AI9" t="n">
-        <v>-2.301893074565969</v>
+        <v>-2.277398685083083</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.3191793911653013</v>
+        <v>0.3252866773883619</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.2816987666105443</v>
+        <v>0.2852996322390131</v>
       </c>
       <c r="AL9" t="n">
-        <v>0.305052551658295</v>
+        <v>0.3512902602852533</v>
       </c>
       <c r="AM9" t="n">
-        <v>0.5470722176058072</v>
+        <v>0.6310628418511631</v>
       </c>
       <c r="AN9" t="n">
-        <v>0.1011685903302695</v>
+        <v>0.1174308276773816</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.160099206600355</v>
+        <v>0.1878866146403194</v>
       </c>
       <c r="AP9" t="n">
-        <v>0.1525262758291475</v>
+        <v>0.1756451301426266</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.2735361088029036</v>
+        <v>0.3155314209255816</v>
       </c>
       <c r="AR9" t="n">
-        <v>33.45363832849139</v>
+        <v>28.77582304739979</v>
       </c>
       <c r="AS9" t="n">
-        <v>41.57870966985516</v>
+        <v>36.39342684459161</v>
       </c>
       <c r="AT9" t="n">
-        <v>0.02826148184497974</v>
+        <v>0.02999684826576988</v>
       </c>
       <c r="AU9" t="n">
-        <v>0.03121219718260836</v>
+        <v>0.03201831016581897</v>
       </c>
       <c r="AV9" t="n">
-        <v>1.555477598877373</v>
+        <v>1.533819612959016</v>
       </c>
       <c r="AW9" t="n">
-        <v>1.329711803394531</v>
+        <v>1.344616369557922</v>
       </c>
       <c r="AX9" t="n">
-        <v>1.388693997193434</v>
+        <v>1.334549032397539</v>
       </c>
       <c r="AY9" t="n">
-        <v>-1.675720491513674</v>
+        <v>-1.638459076105195</v>
       </c>
       <c r="AZ9" t="n">
-        <v>0.2921246700062921</v>
+        <v>0.2958972494520846</v>
       </c>
       <c r="BA9" t="n">
-        <v>0.2816987666105443</v>
+        <v>0.2852996322390131</v>
       </c>
       <c r="BB9" t="n">
-        <v>0.2374729594843689</v>
+        <v>0.3230020195306361</v>
       </c>
       <c r="BC9" t="n">
-        <v>0.5131592424392873</v>
+        <v>0.5933804057178184</v>
       </c>
       <c r="BD9" t="n">
-        <v>0.08651955557883524</v>
+        <v>0.1183677273439352</v>
       </c>
       <c r="BE9" t="n">
-        <v>0.1666924242666917</v>
+        <v>0.196306016394569</v>
       </c>
       <c r="BF9" t="n">
-        <v>0.1187364797421845</v>
+        <v>0.161501009765318</v>
       </c>
       <c r="BG9" t="n">
-        <v>0.2565796212196437</v>
+        <v>0.2966902028589092</v>
       </c>
       <c r="BH9" t="n">
-        <v>48.63713775006408</v>
+        <v>43.12784622245556</v>
       </c>
       <c r="BI9" t="n">
-        <v>42.1879257653242</v>
+        <v>37.01352523550283</v>
       </c>
       <c r="BJ9" t="n">
-        <v>10.60638699803229</v>
+        <v>8.16146049665082</v>
       </c>
       <c r="BK9" t="n">
-        <v>4.633976151520757</v>
+        <v>4.157078002409932</v>
       </c>
       <c r="BL9" t="n">
-        <v>0.01099002548023639</v>
+        <v>0.01150243854924837</v>
       </c>
       <c r="BM9" t="n">
-        <v>0.01037580675089796</v>
+        <v>0.01076308599363575</v>
       </c>
       <c r="BN9" t="n">
-        <v>0.03299379548812491</v>
+        <v>0.03145358190977478</v>
       </c>
       <c r="BO9" t="n">
-        <v>0.02787209226584079</v>
+        <v>0.02591766314192321</v>
       </c>
       <c r="BP9" t="n">
-        <v>0.02870761904748252</v>
+        <v>0.02663568745548795</v>
       </c>
       <c r="BQ9" t="n">
-        <v>0.02617704826870411</v>
+        <v>0.02406724222746321</v>
       </c>
       <c r="BR9" t="n">
-        <v>0.02423353609937522</v>
+        <v>0.02214835299703139</v>
       </c>
       <c r="BS9" t="n">
-        <v>0.02754354584839037</v>
+        <v>0.02554409840569221</v>
       </c>
       <c r="BT9" t="n">
-        <v>-0.01210201446215303</v>
+        <v>-0.0144885769843099</v>
       </c>
       <c r="BU9" t="n">
-        <v>-0.01549891121350449</v>
+        <v>-0.01476216961707945</v>
       </c>
       <c r="BV9" t="n">
-        <v>0.001907123456374202</v>
+        <v>0.005163005897729704</v>
       </c>
       <c r="BW9" t="n">
-        <v>0.001412597128783765</v>
+        <v>-0.002047345690203576</v>
       </c>
       <c r="BX9" t="n">
-        <v>-0.004080355093682926</v>
+        <v>-0.001664028619547709</v>
       </c>
       <c r="BY9" t="n">
-        <v>-0.006382287439440257</v>
+        <v>-0.00983874398225263</v>
       </c>
       <c r="BZ9" t="n">
-        <v>-0.01201071312741437</v>
+        <v>-0.01304176511527865</v>
       </c>
       <c r="CA9" t="n">
-        <v>-0.01476766499687218</v>
+        <v>-0.01333115247966061</v>
       </c>
       <c r="CB9" t="n">
-        <v>0.001647819851323551</v>
+        <v>0.0002245442505444473</v>
       </c>
       <c r="CC9" t="n">
-        <v>-0.0002478344608667846</v>
+        <v>-0.004369794505968703</v>
       </c>
       <c r="CD9" t="n">
-        <v>-0.004325277638434089</v>
+        <v>-0.00644597104748069</v>
       </c>
       <c r="CE9" t="n">
-        <v>-0.007856411458448405</v>
+        <v>-0.01163643217421166</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>54.3510435104351</v>
+        <v>52.24982249822499</v>
       </c>
       <c r="B10" t="n">
-        <v>17.52660604857688</v>
+        <v>16.58686326801209</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9424208242082421</v>
+        <v>1.152139321393214</v>
       </c>
       <c r="D10" t="n">
-        <v>1.142168148013268</v>
+        <v>1.145589697774146</v>
       </c>
       <c r="E10" t="n">
-        <v>54.71314713147132</v>
+        <v>52.82442824428244</v>
       </c>
       <c r="F10" t="n">
-        <v>17.68861655360206</v>
+        <v>16.84384553128256</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9284228842288423</v>
+        <v>1.133952739527395</v>
       </c>
       <c r="H10" t="n">
-        <v>1.170713129957772</v>
+        <v>1.1787111173992</v>
       </c>
       <c r="I10" t="n">
-        <v>0.3554203700331693</v>
+        <v>0.3639742444353639</v>
       </c>
       <c r="J10" t="n">
-        <v>-2.07321717510557</v>
+        <v>-2.053222206502001</v>
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
-        <v>0.3012979485857906</v>
+        <v>0.3055000331116358</v>
       </c>
       <c r="M10" t="n">
-        <v>0.3005738580002413</v>
+        <v>0.3043516411954972</v>
       </c>
       <c r="N10" t="n">
-        <v>0.3928260242759346</v>
+        <v>0.457874147785971</v>
       </c>
       <c r="O10" t="n">
-        <v>0.446983288399684</v>
+        <v>0.513005877734807</v>
       </c>
       <c r="P10" t="n">
-        <v>0.1964130121379673</v>
+        <v>0.2289370738929855</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.223491644199842</v>
+        <v>0.2565029388674035</v>
       </c>
       <c r="R10" t="n">
-        <v>38.3854928611384</v>
+        <v>33.73265795644888</v>
       </c>
       <c r="S10" t="n">
-        <v>36.44073292442602</v>
+        <v>31.9274156360846</v>
       </c>
       <c r="T10" t="n">
         <v>2.200000000000001</v>
@@ -2890,247 +2890,247 @@
         <v>1.4</v>
       </c>
       <c r="V10" t="n">
-        <v>0.03964698220335999</v>
+        <v>0.03952925596681648</v>
       </c>
       <c r="W10" t="n">
-        <v>0.03991216099801174</v>
+        <v>0.03997088668477335</v>
       </c>
       <c r="X10" t="n">
-        <v>5.782736019140004</v>
+        <v>4.946480537978068</v>
       </c>
       <c r="Y10" t="n">
-        <v>5.116084280558865</v>
+        <v>4.46421933885594</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.03471203629021131</v>
+        <v>0.03450559658804624</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.03409217849931468</v>
+        <v>0.033910672508942</v>
       </c>
       <c r="AB10" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="AC10" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.03775667903682022</v>
+        <v>0.03745171108078877</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.03708245262544844</v>
+        <v>0.03680599192422345</v>
       </c>
       <c r="AF10" t="n">
-        <v>1.050065398090132</v>
+        <v>1.055472629315818</v>
       </c>
       <c r="AG10" t="n">
-        <v>1.076308554915307</v>
+        <v>1.085988574008977</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.1251634952253311</v>
+        <v>0.1386815732895452</v>
       </c>
       <c r="AI10" t="n">
-        <v>-2.309228612711732</v>
+        <v>-2.285028564977558</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.3196190440644869</v>
+        <v>0.3247291395463486</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.285999593254318</v>
+        <v>0.2912793316098631</v>
       </c>
       <c r="AL10" t="n">
-        <v>0.3355233597888996</v>
+        <v>0.3724104997574471</v>
       </c>
       <c r="AM10" t="n">
-        <v>0.5700085911613973</v>
+        <v>0.6230774982541682</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.1098913690955634</v>
+        <v>0.124241494408256</v>
       </c>
       <c r="AO10" t="n">
-        <v>0.1691278830880716</v>
+        <v>0.1891317168130878</v>
       </c>
       <c r="AP10" t="n">
-        <v>0.1677616798944498</v>
+        <v>0.1862052498787236</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.2850042955806987</v>
+        <v>0.3115387491270841</v>
       </c>
       <c r="AR10" t="n">
-        <v>32.13028103198103</v>
+        <v>28.22847012139814</v>
       </c>
       <c r="AS10" t="n">
-        <v>38.62940725248131</v>
+        <v>33.95058109956111</v>
       </c>
       <c r="AT10" t="n">
-        <v>0.02779230559465374</v>
+        <v>0.02786551443784538</v>
       </c>
       <c r="AU10" t="n">
-        <v>0.0308130650364361</v>
+        <v>0.03074388359481325</v>
       </c>
       <c r="AV10" t="n">
-        <v>1.426545274134675</v>
+        <v>1.418572625134459</v>
       </c>
       <c r="AW10" t="n">
-        <v>1.295299930429384</v>
+        <v>1.300124838213893</v>
       </c>
       <c r="AX10" t="n">
-        <v>1.066363185336688</v>
+        <v>1.046431562836147</v>
       </c>
       <c r="AY10" t="n">
-        <v>-1.761750173926541</v>
+        <v>-1.749687904465267</v>
       </c>
       <c r="AZ10" t="n">
-        <v>0.2943026421172626</v>
+        <v>0.2984252504044027</v>
       </c>
       <c r="BA10" t="n">
-        <v>0.285999593254318</v>
+        <v>0.291279331609863</v>
       </c>
       <c r="BB10" t="n">
-        <v>0.3100197096945663</v>
+        <v>0.3852946276159027</v>
       </c>
       <c r="BC10" t="n">
-        <v>0.5386837005468235</v>
+        <v>0.5903991336056188</v>
       </c>
       <c r="BD10" t="n">
-        <v>0.1089748414833468</v>
+        <v>0.1369475628295694</v>
       </c>
       <c r="BE10" t="n">
-        <v>0.1753413804793136</v>
+        <v>0.1960865965241824</v>
       </c>
       <c r="BF10" t="n">
-        <v>0.1550098548472831</v>
+        <v>0.1926473138079514</v>
       </c>
       <c r="BG10" t="n">
-        <v>0.2693418502734117</v>
+        <v>0.2951995668028094</v>
       </c>
       <c r="BH10" t="n">
-        <v>44.61773455342048</v>
+        <v>39.43554253770483</v>
       </c>
       <c r="BI10" t="n">
-        <v>39.16122324595921</v>
+        <v>34.46958257774912</v>
       </c>
       <c r="BJ10" t="n">
-        <v>7.32730033209903</v>
+        <v>5.87826468197291</v>
       </c>
       <c r="BK10" t="n">
-        <v>4.245175409233017</v>
+        <v>3.879025412218591</v>
       </c>
       <c r="BL10" t="n">
-        <v>0.009911745550839996</v>
+        <v>0.00988231399170412</v>
       </c>
       <c r="BM10" t="n">
-        <v>0.009978040249502936</v>
+        <v>0.009992721671193337</v>
       </c>
       <c r="BN10" t="n">
-        <v>0.02784698609345244</v>
+        <v>0.02510936857073795</v>
       </c>
       <c r="BO10" t="n">
-        <v>0.02520471683649925</v>
+        <v>0.02262226843980155</v>
       </c>
       <c r="BP10" t="n">
-        <v>0.02461876708615066</v>
+        <v>0.02195132878504805</v>
       </c>
       <c r="BQ10" t="n">
-        <v>0.02370746261244674</v>
+        <v>0.0211383836361574</v>
       </c>
       <c r="BR10" t="n">
-        <v>0.02108609731638256</v>
+        <v>0.01869688838230594</v>
       </c>
       <c r="BS10" t="n">
-        <v>0.02491638911394102</v>
+        <v>0.02232284614362525</v>
       </c>
       <c r="BT10" t="n">
-        <v>-0.008805474602091868</v>
+        <v>-0.01074447326061525</v>
       </c>
       <c r="BU10" t="n">
-        <v>-0.01121488494239979</v>
+        <v>-0.01058086380550657</v>
       </c>
       <c r="BV10" t="n">
-        <v>0.002467335705785564</v>
+        <v>0.005031367330393595</v>
       </c>
       <c r="BW10" t="n">
-        <v>0.002537725485563792</v>
+        <v>0.0003336487722948069</v>
       </c>
       <c r="BX10" t="n">
-        <v>-0.00383333402996686</v>
+        <v>-0.002152773607787418</v>
       </c>
       <c r="BY10" t="n">
-        <v>-0.005664891506228872</v>
+        <v>-0.00786529958426143</v>
       </c>
       <c r="BZ10" t="n">
-        <v>-0.00872291595106355</v>
+        <v>-0.009393859643506558</v>
       </c>
       <c r="CA10" t="n">
-        <v>-0.0106201303458191</v>
+        <v>-0.009562721319563268</v>
       </c>
       <c r="CB10" t="n">
-        <v>0.002301066543546217</v>
+        <v>0.001548796853391142</v>
       </c>
       <c r="CC10" t="n">
-        <v>0.001446388069457849</v>
+        <v>-0.001286854560478048</v>
       </c>
       <c r="CD10" t="n">
-        <v>-0.003984469891829517</v>
+        <v>-0.005470637706376848</v>
       </c>
       <c r="CE10" t="n">
-        <v>-0.006560176032612657</v>
+        <v>-0.008933593275982947</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>53.65148651486515</v>
+        <v>51.67436674366743</v>
       </c>
       <c r="B11" t="n">
-        <v>17.21370535381967</v>
+        <v>16.32943318866563</v>
       </c>
       <c r="C11" t="n">
-        <v>1.052005720057201</v>
+        <v>1.233549335493355</v>
       </c>
       <c r="D11" t="n">
-        <v>1.141697593771103</v>
+        <v>1.156120230094621</v>
       </c>
       <c r="E11" t="n">
-        <v>53.7449874498745</v>
+        <v>51.90386903869039</v>
       </c>
       <c r="F11" t="n">
-        <v>17.25552177816727</v>
+        <v>16.43211214370189</v>
       </c>
       <c r="G11" t="n">
-        <v>1.049070090700907</v>
+        <v>1.229092190921909</v>
       </c>
       <c r="H11" t="n">
-        <v>1.148435776024146</v>
+        <v>1.13265938343887</v>
       </c>
       <c r="I11" t="n">
-        <v>0.3542439844277573</v>
+        <v>0.3903005752365529</v>
       </c>
       <c r="J11" t="n">
-        <v>-2.128910559939634</v>
+        <v>-2.168351541402824</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>0.3026969765980049</v>
+        <v>0.3066506859009309</v>
       </c>
       <c r="M11" t="n">
-        <v>0.3025100422224595</v>
+        <v>0.3061918749229294</v>
       </c>
       <c r="N11" t="n">
-        <v>0.4323641986415384</v>
+        <v>0.4823024245877988</v>
       </c>
       <c r="O11" t="n">
-        <v>0.4919785618848414</v>
+        <v>0.5480007802894514</v>
       </c>
       <c r="P11" t="n">
-        <v>0.2161820993207692</v>
+        <v>0.2411512122938994</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2459892809424207</v>
+        <v>0.2740003901447257</v>
       </c>
       <c r="R11" t="n">
-        <v>36.11291320652701</v>
+        <v>32.16297277546646</v>
       </c>
       <c r="S11" t="n">
-        <v>33.759780926605</v>
+        <v>29.81325963152542</v>
       </c>
       <c r="T11" t="n">
         <v>2.100000000000001</v>
@@ -3139,247 +3139,247 @@
         <v>1.3</v>
       </c>
       <c r="V11" t="n">
-        <v>0.03492308917933769</v>
+        <v>0.0324315674290036</v>
       </c>
       <c r="W11" t="n">
-        <v>0.03815758112915708</v>
+        <v>0.0363857159299894</v>
       </c>
       <c r="X11" t="n">
-        <v>4.62792796321876</v>
+        <v>3.852764008996989</v>
       </c>
       <c r="Y11" t="n">
-        <v>4.443842152816631</v>
+        <v>3.804293677225718</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.03058873853275315</v>
+        <v>0.02805207156209807</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.03322569875109394</v>
+        <v>0.03212414646627359</v>
       </c>
       <c r="AB11" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="AC11" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="AD11" t="n">
-        <v>0.03296218011150972</v>
+        <v>0.03006686664232338</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.03580374736250194</v>
+        <v>0.03443141180008</v>
       </c>
       <c r="AF11" t="n">
-        <v>1.059489665464915</v>
+        <v>1.078648061828683</v>
       </c>
       <c r="AG11" t="n">
-        <v>1.065742664945747</v>
+        <v>1.056759337701769</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.1487241636622866</v>
+        <v>0.1966201545717078</v>
       </c>
       <c r="AI11" t="n">
-        <v>-2.335643337635632</v>
+        <v>-2.358101655745578</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.3200916643726608</v>
+        <v>0.323978722868547</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.2910404655911204</v>
+        <v>0.2978965808409578</v>
       </c>
       <c r="AL11" t="n">
-        <v>0.3606121557949996</v>
+        <v>0.3914262527658048</v>
       </c>
       <c r="AM11" t="n">
-        <v>0.5863054520552046</v>
+        <v>0.6118742466506846</v>
       </c>
       <c r="AN11" t="n">
-        <v>0.1188127612786513</v>
+        <v>0.131706231355893</v>
       </c>
       <c r="AO11" t="n">
-        <v>0.1761584520240767</v>
+        <v>0.187376766413773</v>
       </c>
       <c r="AP11" t="n">
-        <v>0.1803060778974998</v>
+        <v>0.1957131263829024</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.2931527260276023</v>
+        <v>0.3059371233253423</v>
       </c>
       <c r="AR11" t="n">
-        <v>30.89815403352284</v>
+        <v>27.77526954612507</v>
       </c>
       <c r="AS11" t="n">
-        <v>35.65061071166728</v>
+        <v>31.45909953228723</v>
       </c>
       <c r="AT11" t="n">
-        <v>0.02564790541774515</v>
+        <v>0.02403976170269928</v>
       </c>
       <c r="AU11" t="n">
-        <v>0.03043001462042086</v>
+        <v>0.02963780447041426</v>
       </c>
       <c r="AV11" t="n">
-        <v>1.361635135911538</v>
+        <v>1.349080237569994</v>
       </c>
       <c r="AW11" t="n">
-        <v>1.25394554045171</v>
+        <v>1.22767919487124</v>
       </c>
       <c r="AX11" t="n">
-        <v>0.9040878397788449</v>
+        <v>0.872700593924986</v>
       </c>
       <c r="AY11" t="n">
-        <v>-1.865136148870724</v>
+        <v>-1.930802012821901</v>
       </c>
       <c r="AZ11" t="n">
-        <v>0.2966123914753207</v>
+        <v>0.3009379475647944</v>
       </c>
       <c r="BA11" t="n">
-        <v>0.2910404655911204</v>
+        <v>0.2978965808409578</v>
       </c>
       <c r="BB11" t="n">
-        <v>0.3736905323870252</v>
+        <v>0.4380678125758646</v>
       </c>
       <c r="BC11" t="n">
-        <v>0.5577684224927152</v>
+        <v>0.5841599580950033</v>
       </c>
       <c r="BD11" t="n">
-        <v>0.1293396734556361</v>
+        <v>0.1531218575928276</v>
       </c>
       <c r="BE11" t="n">
-        <v>0.1817802253948383</v>
+        <v>0.1928145268596413</v>
       </c>
       <c r="BF11" t="n">
-        <v>0.1868452661935126</v>
+        <v>0.2190339062879323</v>
       </c>
       <c r="BG11" t="n">
-        <v>0.2788842112463576</v>
+        <v>0.2920799790475017</v>
       </c>
       <c r="BH11" t="n">
-        <v>40.912199093214</v>
+        <v>36.15374741201552</v>
       </c>
       <c r="BI11" t="n">
-        <v>36.10684938565095</v>
+        <v>31.87254203093307</v>
       </c>
       <c r="BJ11" t="n">
-        <v>5.354562105928948</v>
+        <v>4.241800948077484</v>
       </c>
       <c r="BK11" t="n">
-        <v>3.919685840665101</v>
+        <v>3.568811860388671</v>
       </c>
       <c r="BL11" t="n">
-        <v>0.008730772294834424</v>
+        <v>0.008107891857250899</v>
       </c>
       <c r="BM11" t="n">
-        <v>0.009539395282289271</v>
+        <v>0.009096428982497351</v>
       </c>
       <c r="BN11" t="n">
-        <v>0.02287119155261808</v>
+        <v>0.01913313450431633</v>
       </c>
       <c r="BO11" t="n">
-        <v>0.02248599331011248</v>
+        <v>0.01921280123878312</v>
       </c>
       <c r="BP11" t="n">
-        <v>0.02058291601286048</v>
+        <v>0.01726427407567146</v>
       </c>
       <c r="BQ11" t="n">
-        <v>0.02120463200442455</v>
+        <v>0.01809005993667558</v>
       </c>
       <c r="BR11" t="n">
-        <v>0.01793348147428795</v>
+        <v>0.01511326567593507</v>
       </c>
       <c r="BS11" t="n">
-        <v>0.02223980175138366</v>
+        <v>0.01898933314764943</v>
       </c>
       <c r="BT11" t="n">
-        <v>-0.005513685726175858</v>
+        <v>-0.006994335225418097</v>
       </c>
       <c r="BU11" t="n">
-        <v>-0.006939122954581783</v>
+        <v>-0.006400401441992176</v>
       </c>
       <c r="BV11" t="n">
-        <v>0.002946611752252228</v>
+        <v>0.004804176412740136</v>
       </c>
       <c r="BW11" t="n">
-        <v>0.00354213667192158</v>
+        <v>0.00254720781938023</v>
       </c>
       <c r="BX11" t="n">
-        <v>-0.003536972163381061</v>
+        <v>-0.002588526678826034</v>
       </c>
       <c r="BY11" t="n">
-        <v>-0.004898609760526717</v>
+        <v>-0.00588976347401003</v>
       </c>
       <c r="BZ11" t="n">
-        <v>-0.005440534435186682</v>
+        <v>-0.005752882585058473</v>
       </c>
       <c r="CA11" t="n">
-        <v>-0.0064796696823008</v>
+        <v>-0.00577839975703551</v>
       </c>
       <c r="CB11" t="n">
-        <v>0.002869896899613586</v>
+        <v>0.002755948895993138</v>
       </c>
       <c r="CC11" t="n">
-        <v>0.003000139435017994</v>
+        <v>0.001610585966491807</v>
       </c>
       <c r="CD11" t="n">
-        <v>-0.003598114382152544</v>
+        <v>-0.004467266241011224</v>
       </c>
       <c r="CE11" t="n">
-        <v>-0.005238862513791816</v>
+        <v>-0.006258144537119853</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>52.83632836328363</v>
+        <v>51.05811058110581</v>
       </c>
       <c r="B12" t="n">
-        <v>16.84916726326217</v>
+        <v>16.05362174798062</v>
       </c>
       <c r="C12" t="n">
-        <v>1.161268412684127</v>
+        <v>1.315639556395564</v>
       </c>
       <c r="D12" t="n">
-        <v>1.146311542434053</v>
+        <v>1.135330707305273</v>
       </c>
       <c r="E12" t="n">
-        <v>52.61617616176162</v>
+        <v>50.87875878758788</v>
       </c>
       <c r="F12" t="n">
-        <v>16.75071335307731</v>
+        <v>15.97331751056624</v>
       </c>
       <c r="G12" t="n">
-        <v>1.170111101111011</v>
+        <v>1.324750747507475</v>
       </c>
       <c r="H12" t="n">
-        <v>1.15394361601452</v>
+        <v>1.116892394771442</v>
       </c>
       <c r="I12" t="n">
-        <v>0.3657788560851316</v>
+        <v>0.3383267682631835</v>
       </c>
       <c r="J12" t="n">
-        <v>-2.115140959963699</v>
+        <v>-2.207769013071395</v>
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
-        <v>0.3043274728037851</v>
+        <v>0.307884515849925</v>
       </c>
       <c r="M12" t="n">
-        <v>0.3047677796775575</v>
+        <v>0.3082423340772001</v>
       </c>
       <c r="N12" t="n">
-        <v>0.4681978047415705</v>
+        <v>0.5101273927942181</v>
       </c>
       <c r="O12" t="n">
-        <v>0.5291231367300102</v>
+        <v>0.5757950802160927</v>
       </c>
       <c r="P12" t="n">
-        <v>0.2340989023707852</v>
+        <v>0.2550636963971091</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.2645615683650051</v>
+        <v>0.2878975401080464</v>
       </c>
       <c r="R12" t="n">
-        <v>33.86963915032388</v>
+        <v>30.53020906418184</v>
       </c>
       <c r="S12" t="n">
-        <v>31.16529161854619</v>
+        <v>27.79836502850665</v>
       </c>
       <c r="T12" t="n">
         <v>2.000000000000001</v>
@@ -3388,247 +3388,247 @@
         <v>1.2</v>
       </c>
       <c r="V12" t="n">
-        <v>0.02972680685291317</v>
+        <v>0.02462411003740946</v>
       </c>
       <c r="W12" t="n">
-        <v>0.03619926550666276</v>
+        <v>0.03218358363804736</v>
       </c>
       <c r="X12" t="n">
-        <v>3.637832755054713</v>
+        <v>2.765705702787438</v>
       </c>
       <c r="Y12" t="n">
-        <v>3.919829546754229</v>
+        <v>3.202513072784972</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.02593257221312796</v>
+        <v>0.02168893158527809</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.03137004703200962</v>
+        <v>0.02881529482044089</v>
       </c>
       <c r="AB12" t="n">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="AC12" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.02768823129366816</v>
+        <v>0.02295427453338667</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.03349382817782439</v>
+        <v>0.03049639330864229</v>
       </c>
       <c r="AF12" t="n">
-        <v>1.073626066527088</v>
+        <v>1.072746167673216</v>
       </c>
       <c r="AG12" t="n">
-        <v>1.080774204563144</v>
+        <v>1.055324257932067</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.184065166317719</v>
+        <v>0.181865419183041</v>
       </c>
       <c r="AI12" t="n">
-        <v>-2.298064488592141</v>
+        <v>-2.361689355169834</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.3206343010747352</v>
+        <v>0.3230141601888347</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.2969236624079362</v>
+        <v>0.3050978024555132</v>
       </c>
       <c r="AL12" t="n">
-        <v>0.3841530494362852</v>
+        <v>0.416217589808362</v>
       </c>
       <c r="AM12" t="n">
-        <v>0.5883887444590241</v>
+        <v>0.5877965600682342</v>
       </c>
       <c r="AN12" t="n">
-        <v>0.127626479425474</v>
+        <v>0.1392484844436202</v>
       </c>
       <c r="AO12" t="n">
-        <v>0.1816254278438135</v>
+        <v>0.1842294604561899</v>
       </c>
       <c r="AP12" t="n">
-        <v>0.1920765247181426</v>
+        <v>0.208108794904181</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0.2941943722295121</v>
+        <v>0.2938982800341171</v>
       </c>
       <c r="AR12" t="n">
-        <v>29.67556963750726</v>
+        <v>27.2908317911367</v>
       </c>
       <c r="AS12" t="n">
-        <v>32.74879726962968</v>
+        <v>29.06894087365446</v>
       </c>
       <c r="AT12" t="n">
-        <v>0.02270745699906578</v>
+        <v>0.0196270090196356</v>
       </c>
       <c r="AU12" t="n">
-        <v>0.02909163411662137</v>
+        <v>0.02702984325412289</v>
       </c>
       <c r="AV12" t="n">
-        <v>1.309120913633621</v>
+        <v>1.254603287376827</v>
       </c>
       <c r="AW12" t="n">
-        <v>1.244318739935633</v>
+        <v>1.190668526467994</v>
       </c>
       <c r="AX12" t="n">
-        <v>0.7728022840840537</v>
+        <v>0.6365082184420673</v>
       </c>
       <c r="AY12" t="n">
-        <v>-1.889203150160919</v>
+        <v>-2.023328683830014</v>
       </c>
       <c r="AZ12" t="n">
-        <v>0.2991177666482132</v>
+        <v>0.3034507227748294</v>
       </c>
       <c r="BA12" t="n">
-        <v>0.2969236624079362</v>
+        <v>0.3050978024555132</v>
       </c>
       <c r="BB12" t="n">
-        <v>0.4312442481487284</v>
+        <v>0.4891740038365265</v>
       </c>
       <c r="BC12" t="n">
-        <v>0.5630846462013438</v>
+        <v>0.565410860115356</v>
       </c>
       <c r="BD12" t="n">
-        <v>0.1475894810031996</v>
+        <v>0.1662665005217774</v>
       </c>
       <c r="BE12" t="n">
-        <v>0.1865023528533712</v>
+        <v>0.1882342562596729</v>
       </c>
       <c r="BF12" t="n">
-        <v>0.2156221240743642</v>
+        <v>0.2445870019182633</v>
       </c>
       <c r="BG12" t="n">
-        <v>0.2815423231006719</v>
+        <v>0.282705430057678</v>
       </c>
       <c r="BH12" t="n">
-        <v>37.40775413810024</v>
+        <v>33.08475205451941</v>
       </c>
       <c r="BI12" t="n">
-        <v>33.14500655893206</v>
+        <v>29.39610869501784</v>
       </c>
       <c r="BJ12" t="n">
-        <v>3.949558976646094</v>
+        <v>2.884171794450784</v>
       </c>
       <c r="BK12" t="n">
-        <v>3.683413312174367</v>
+        <v>3.261329281688954</v>
       </c>
       <c r="BL12" t="n">
-        <v>0.007431701713228291</v>
+        <v>0.006156027509352365</v>
       </c>
       <c r="BM12" t="n">
-        <v>0.00904981637666569</v>
+        <v>0.00804589590951184</v>
       </c>
       <c r="BN12" t="n">
-        <v>0.01805854010641287</v>
+        <v>0.01344178461809785</v>
       </c>
       <c r="BO12" t="n">
-        <v>0.01979230429456191</v>
+        <v>0.0157971376919532</v>
       </c>
       <c r="BP12" t="n">
-        <v>0.01656690433131804</v>
+        <v>0.01250886529474235</v>
       </c>
       <c r="BQ12" t="n">
-        <v>0.01873343684650764</v>
+        <v>0.01500918106032717</v>
       </c>
       <c r="BR12" t="n">
-        <v>0.01471739270514461</v>
+        <v>0.01129033559063781</v>
       </c>
       <c r="BS12" t="n">
-        <v>0.01958223942776331</v>
+        <v>0.01563676908255854</v>
       </c>
       <c r="BT12" t="n">
-        <v>-0.002228612307986443</v>
+        <v>-0.003235513507737744</v>
       </c>
       <c r="BU12" t="n">
-        <v>-0.002676120018033163</v>
+        <v>-0.002231649350291192</v>
       </c>
       <c r="BV12" t="n">
-        <v>0.003324559601741529</v>
+        <v>0.004458185441687315</v>
       </c>
       <c r="BW12" t="n">
-        <v>0.00439931063721822</v>
+        <v>0.004567196420364833</v>
       </c>
       <c r="BX12" t="n">
-        <v>-0.003170867678056709</v>
+        <v>-0.002948021674198894</v>
       </c>
       <c r="BY12" t="n">
-        <v>-0.00405685424822217</v>
+        <v>-0.003885186430086625</v>
       </c>
       <c r="BZ12" t="n">
-        <v>-0.002165989052420206</v>
+        <v>-0.002124470866564396</v>
       </c>
       <c r="CA12" t="n">
-        <v>-0.002353635661473123</v>
+        <v>-0.001993117610687891</v>
       </c>
       <c r="CB12" t="n">
-        <v>0.003333972185365974</v>
+        <v>0.003823364606156455</v>
       </c>
       <c r="CC12" t="n">
-        <v>0.004387646980845651</v>
+        <v>0.004298752523734298</v>
       </c>
       <c r="CD12" t="n">
-        <v>-0.003145854014511765</v>
+        <v>-0.003413044956712133</v>
       </c>
       <c r="CE12" t="n">
-        <v>-0.003866404900486849</v>
+        <v>-0.00358435154889147</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>51.86476864768647</v>
+        <v>50.38745387453875</v>
       </c>
       <c r="B13" t="n">
-        <v>16.41461985525426</v>
+        <v>15.75324061915245</v>
       </c>
       <c r="C13" t="n">
-        <v>1.269564495644957</v>
+        <v>1.398392083920839</v>
       </c>
       <c r="D13" t="n">
-        <v>1.112026976677277</v>
+        <v>1.103987837784548</v>
       </c>
       <c r="E13" t="n">
-        <v>51.27316273162732</v>
+        <v>49.72529725297252</v>
       </c>
       <c r="F13" t="n">
-        <v>16.14988924487325</v>
+        <v>15.45636084504887</v>
       </c>
       <c r="G13" t="n">
-        <v>1.290776207762078</v>
+        <v>1.420767307673077</v>
       </c>
       <c r="H13" t="n">
-        <v>1.143435201699411</v>
+        <v>1.119394038287382</v>
       </c>
       <c r="I13" t="n">
-        <v>0.2800674416931914</v>
+        <v>0.2599695944613711</v>
       </c>
       <c r="J13" t="n">
-        <v>-2.141411995751472</v>
+        <v>-2.201514904281546</v>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
-        <v>0.3062712781906106</v>
+        <v>0.3092243246578802</v>
       </c>
       <c r="M13" t="n">
-        <v>0.3074530132251371</v>
+        <v>0.3105488432985803</v>
       </c>
       <c r="N13" t="n">
-        <v>0.5057039368807671</v>
+        <v>0.5383961351376184</v>
       </c>
       <c r="O13" t="n">
-        <v>0.5631107426843625</v>
+        <v>0.5968960171726396</v>
       </c>
       <c r="P13" t="n">
-        <v>0.2528519684403835</v>
+        <v>0.2691980675688092</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.2815553713421812</v>
+        <v>0.2984480085863198</v>
       </c>
       <c r="R13" t="n">
-        <v>31.55777234267475</v>
+        <v>28.88775074060709</v>
       </c>
       <c r="S13" t="n">
-        <v>28.56779238809923</v>
+        <v>25.86269368846262</v>
       </c>
       <c r="T13" t="n">
         <v>1.900000000000001</v>
@@ -3637,439 +3637,299 @@
         <v>1.1</v>
       </c>
       <c r="V13" t="n">
-        <v>0.02398354743949658</v>
+        <v>0.01599481502564746</v>
       </c>
       <c r="W13" t="n">
-        <v>0.0340022074499291</v>
+        <v>0.0272231107021466</v>
       </c>
       <c r="X13" t="n">
-        <v>2.717322144859494</v>
+        <v>1.702164460260683</v>
       </c>
       <c r="Y13" t="n">
-        <v>3.459693936139531</v>
+        <v>2.613145936716569</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.02156741512796671</v>
+        <v>0.01448821669788084</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.02973689055522683</v>
+        <v>0.02431950660001426</v>
       </c>
       <c r="AB13" t="n">
-        <v>91</v>
+        <v>141</v>
       </c>
       <c r="AC13" t="n">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="AD13" t="n">
-        <v>0.02281997084642981</v>
+        <v>0.01514005341563801</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.03146389919735019</v>
+        <v>0.02541366109053524</v>
       </c>
       <c r="AF13" t="n">
-        <v>1.05098939875503</v>
+        <v>1.056456974526032</v>
       </c>
       <c r="AG13" t="n">
-        <v>1.080673671011274</v>
+        <v>1.071199879669649</v>
       </c>
       <c r="AH13" t="n">
-        <v>0.1274734968875757</v>
+        <v>0.1411424363150804</v>
       </c>
       <c r="AI13" t="n">
-        <v>-2.298315822471815</v>
+        <v>-2.322000300825877</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.3213045762969667</v>
+        <v>0.3218099308454808</v>
       </c>
       <c r="AK13" t="n">
-        <v>0.3037398893257064</v>
+        <v>0.3123374127771664</v>
       </c>
       <c r="AL13" t="n">
-        <v>0.4115183566688427</v>
+        <v>0.4444630324663207</v>
       </c>
       <c r="AM13" t="n">
-        <v>0.5811678748802481</v>
+        <v>0.5583113288574335</v>
       </c>
       <c r="AN13" t="n">
-        <v>0.1355518007873978</v>
+        <v>0.1470147786408094</v>
       </c>
       <c r="AO13" t="n">
-        <v>0.183506188808452</v>
+        <v>0.1804827528325299</v>
       </c>
       <c r="AP13" t="n">
-        <v>0.2057591783344213</v>
+        <v>0.2222315162331603</v>
       </c>
       <c r="AQ13" t="n">
-        <v>0.2905839374401241</v>
+        <v>0.2791556644287168</v>
       </c>
       <c r="AR13" t="n">
-        <v>28.36495331839544</v>
+        <v>26.82459465325925</v>
       </c>
       <c r="AS13" t="n">
-        <v>29.85140973351764</v>
+        <v>26.77513366787684</v>
       </c>
       <c r="AT13" t="n">
-        <v>0.01967363196199914</v>
+        <v>0.01378581983518137</v>
       </c>
       <c r="AU13" t="n">
-        <v>0.02790319635966574</v>
+        <v>0.02317374877985195</v>
       </c>
       <c r="AV13" t="n">
-        <v>1.21907065689865</v>
+        <v>1.160236766247934</v>
       </c>
       <c r="AW13" t="n">
-        <v>1.218577506736093</v>
+        <v>1.174739182717614</v>
       </c>
       <c r="AX13" t="n">
-        <v>0.5476766422466262</v>
+        <v>0.400591915619834</v>
       </c>
       <c r="AY13" t="n">
-        <v>-1.953556233159768</v>
+        <v>-2.063152043205964</v>
       </c>
       <c r="AZ13" t="n">
-        <v>0.3018960018499668</v>
+        <v>0.3059745553868967</v>
       </c>
       <c r="BA13" t="n">
-        <v>0.3037398893257064</v>
+        <v>0.3123374127771664</v>
       </c>
       <c r="BB13" t="n">
-        <v>0.4877256404027732</v>
+        <v>0.5367220658383516</v>
       </c>
       <c r="BC13" t="n">
-        <v>0.559212939786063</v>
+        <v>0.5412930952861537</v>
       </c>
       <c r="BD13" t="n">
-        <v>0.1625726137365685</v>
+        <v>0.1768919520879173</v>
       </c>
       <c r="BE13" t="n">
-        <v>0.1875018776712611</v>
+        <v>0.1832429281975233</v>
       </c>
       <c r="BF13" t="n">
-        <v>0.2438628202013866</v>
+        <v>0.2683610329191758</v>
       </c>
       <c r="BG13" t="n">
-        <v>0.2796064698930315</v>
+        <v>0.2706465476430768</v>
       </c>
       <c r="BH13" t="n">
-        <v>33.99208179069541</v>
+        <v>30.26460008371505</v>
       </c>
       <c r="BI13" t="n">
-        <v>30.1851918552826</v>
+        <v>27.02547280871111</v>
       </c>
       <c r="BJ13" t="n">
-        <v>2.817486064065559</v>
+        <v>1.70747357742092</v>
       </c>
       <c r="BK13" t="n">
-        <v>3.483808358250308</v>
+        <v>2.881572225092967</v>
       </c>
       <c r="BL13" t="n">
-        <v>0.005995886859874146</v>
+        <v>0.003998703756411864</v>
       </c>
       <c r="BM13" t="n">
-        <v>0.008500551862482275</v>
+        <v>0.006805777675536649</v>
       </c>
       <c r="BN13" t="n">
-        <v>0.01340868155675388</v>
+        <v>0.008061292129149612</v>
       </c>
       <c r="BO13" t="n">
-        <v>0.01709619284466626</v>
+        <v>0.01236981623545321</v>
       </c>
       <c r="BP13" t="n">
-        <v>0.01255198216524143</v>
+        <v>0.007727018471452724</v>
       </c>
       <c r="BQ13" t="n">
-        <v>0.01625979585239639</v>
+        <v>0.01187515584780896</v>
       </c>
       <c r="BR13" t="n">
-        <v>0.01139424897868896</v>
+        <v>0.007217830600366845</v>
       </c>
       <c r="BS13" t="n">
-        <v>0.01692467968382138</v>
+        <v>0.01226374231326723</v>
       </c>
       <c r="BT13" t="n">
-        <v>0.001061465934277512</v>
+        <v>0.000516188217643537</v>
       </c>
       <c r="BU13" t="n">
-        <v>0.001600908772048477</v>
+        <v>0.00198913649199365</v>
       </c>
       <c r="BV13" t="n">
-        <v>0.003722906537125982</v>
+        <v>0.004132192950783035</v>
       </c>
       <c r="BW13" t="n">
-        <v>0.005267741184923131</v>
+        <v>0.006552325458838363</v>
       </c>
       <c r="BX13" t="n">
-        <v>-0.002856740221178555</v>
+        <v>-0.003370042782489039</v>
       </c>
       <c r="BY13" t="n">
-        <v>-0.003298066032905465</v>
+        <v>-0.002009650686270488</v>
       </c>
       <c r="BZ13" t="n">
-        <v>0.001115157590801716</v>
+        <v>0.001524868665391059</v>
       </c>
       <c r="CA13" t="n">
-        <v>0.00180157150144587</v>
+        <v>0.001878393563504645</v>
       </c>
       <c r="CB13" t="n">
-        <v>0.003814730638905047</v>
+        <v>0.00488672157508899</v>
       </c>
       <c r="CC13" t="n">
-        <v>0.00576370421903165</v>
+        <v>0.006926125273800484</v>
       </c>
       <c r="CD13" t="n">
-        <v>-0.00274911275643302</v>
+        <v>-0.002443515016147425</v>
       </c>
       <c r="CE13" t="n">
-        <v>-0.002597369404684416</v>
+        <v>-0.001059190845147822</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>51.59191591915919</v>
-      </c>
-      <c r="B14" t="n">
-        <v>16.29254050725435</v>
-      </c>
-      <c r="C14" t="n">
-        <v>1.397944579445795</v>
-      </c>
-      <c r="D14" t="n">
-        <v>1.109958846819295</v>
-      </c>
-      <c r="E14" t="n">
-        <v>51.63611636116362</v>
-      </c>
-      <c r="F14" t="n">
-        <v>16.31231833016527</v>
-      </c>
-      <c r="G14" t="n">
-        <v>1.396942169421694</v>
-      </c>
-      <c r="H14" t="n">
-        <v>1.117752681781864</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0.2748971170482384</v>
-      </c>
-      <c r="J14" t="n">
-        <v>-2.205618295545339</v>
-      </c>
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="n">
-        <v>0.3068164075095842</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0.3067272093184099</v>
-      </c>
-      <c r="N14" t="n">
-        <v>0.5540789810891333</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0.6144872002276871</v>
-      </c>
-      <c r="P14" t="n">
-        <v>0.2770394905445667</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>0.3072436001138436</v>
-      </c>
-      <c r="R14" t="n">
-        <v>29.36771543248367</v>
-      </c>
-      <c r="S14" t="n">
-        <v>26.95056414569196</v>
-      </c>
-      <c r="T14" t="n">
-        <v>1.800000000000001</v>
-      </c>
-      <c r="U14" t="n">
-        <v>1</v>
-      </c>
-      <c r="V14" t="n">
-        <v>0.01760214809125594</v>
-      </c>
-      <c r="W14" t="n">
-        <v>0.03077386402799354</v>
-      </c>
-      <c r="X14" t="n">
-        <v>1.82019668723767</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>2.869418562049467</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>0.01585837902161576</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>0.02753190802363848</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>125</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>72</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>0.0166129387762009</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>0.02884190759757101</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>1.059544510961067</v>
-      </c>
-      <c r="AG14" t="n">
-        <v>1.066984349904277</v>
-      </c>
-      <c r="AH14" t="n">
-        <v>0.1488612774026687</v>
-      </c>
-      <c r="AI14" t="n">
-        <v>-2.332539125239307</v>
-      </c>
-      <c r="AJ14" t="n">
-        <v>0.3199640955313294</v>
-      </c>
-      <c r="AK14" t="n">
-        <v>0.3037398893257064</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>0.4583692419546027</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>0.6298048730849896</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>0.1509650160319608</v>
-      </c>
-      <c r="AO14" t="n">
-        <v>0.1975999688184572</v>
-      </c>
-      <c r="AP14" t="n">
-        <v>0.2291846209773013</v>
-      </c>
-      <c r="AQ14" t="n">
-        <v>0.3149024365424948</v>
-      </c>
-      <c r="AR14" t="n">
-        <v>27.1480767441945</v>
-      </c>
-      <c r="AS14" t="n">
-        <v>27.97067789111671</v>
-      </c>
-      <c r="AT14" t="n">
-        <v>0.01502033393723129</v>
-      </c>
-      <c r="AU14" t="n">
-        <v>0.02615638134332335</v>
-      </c>
-      <c r="AV14" t="n">
-        <v>1.171887933038895</v>
-      </c>
-      <c r="AW14" t="n">
-        <v>1.176533696464432</v>
-      </c>
-      <c r="AX14" t="n">
-        <v>0.4297198325972368</v>
-      </c>
-      <c r="AY14" t="n">
-        <v>-2.058665758838919</v>
-      </c>
-      <c r="AZ14" t="n">
-        <v>0.3033699598030959</v>
-      </c>
-      <c r="BA14" t="n">
-        <v>0.3037398893257064</v>
-      </c>
-      <c r="BB14" t="n">
-        <v>0.5508418774718791</v>
-      </c>
-      <c r="BC14" t="n">
-        <v>0.6108978575460861</v>
-      </c>
-      <c r="BD14" t="n">
-        <v>0.1809016654021944</v>
-      </c>
-      <c r="BE14" t="n">
-        <v>0.2012670204887022</v>
-      </c>
-      <c r="BF14" t="n">
-        <v>0.2754209387359395</v>
-      </c>
-      <c r="BG14" t="n">
-        <v>0.305448928773043</v>
-      </c>
-      <c r="BH14" t="n">
-        <v>30.87414498544942</v>
-      </c>
-      <c r="BI14" t="n">
-        <v>28.23509774974764</v>
-      </c>
-      <c r="BJ14" t="n">
-        <v>1.83089325867946</v>
-      </c>
-      <c r="BK14" t="n">
-        <v>2.886277727548924</v>
-      </c>
-      <c r="BL14" t="n">
-        <v>0.004400537022813985</v>
-      </c>
-      <c r="BM14" t="n">
-        <v>0.007693466006998384</v>
-      </c>
-      <c r="BN14" t="n">
-        <v>0.009032612588833809</v>
-      </c>
-      <c r="BO14" t="n">
-        <v>0.01455882386994705</v>
-      </c>
-      <c r="BP14" t="n">
-        <v>0.008632318223110683</v>
-      </c>
-      <c r="BQ14" t="n">
-        <v>0.0139473784773552</v>
-      </c>
-      <c r="BR14" t="n">
-        <v>0.008031714465142028</v>
-      </c>
-      <c r="BS14" t="n">
-        <v>0.01443354655343122</v>
-      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="inlineStr"/>
+      <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr"/>
+      <c r="AQ14" t="inlineStr"/>
+      <c r="AR14" t="inlineStr"/>
+      <c r="AS14" t="inlineStr"/>
+      <c r="AT14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr"/>
+      <c r="AW14" t="inlineStr"/>
+      <c r="AX14" t="inlineStr"/>
+      <c r="AY14" t="inlineStr"/>
+      <c r="AZ14" t="inlineStr"/>
+      <c r="BA14" t="inlineStr"/>
+      <c r="BB14" t="inlineStr"/>
+      <c r="BC14" t="inlineStr"/>
+      <c r="BD14" t="inlineStr"/>
+      <c r="BE14" t="inlineStr"/>
+      <c r="BF14" t="inlineStr"/>
+      <c r="BG14" t="inlineStr"/>
+      <c r="BH14" t="inlineStr"/>
+      <c r="BI14" t="inlineStr"/>
+      <c r="BJ14" t="inlineStr"/>
+      <c r="BK14" t="inlineStr"/>
+      <c r="BL14" t="inlineStr"/>
+      <c r="BM14" t="inlineStr"/>
+      <c r="BN14" t="inlineStr"/>
+      <c r="BO14" t="inlineStr"/>
+      <c r="BP14" t="inlineStr"/>
+      <c r="BQ14" t="inlineStr"/>
+      <c r="BR14" t="inlineStr"/>
+      <c r="BS14" t="inlineStr"/>
       <c r="BT14" t="n">
-        <v>0.00762907658124304</v>
+        <v>0.008035395703107122</v>
       </c>
       <c r="BU14" t="n">
-        <v>0.01013404125875495</v>
+        <v>0.01043630286365026</v>
       </c>
       <c r="BV14" t="n">
-        <v>0.004294592845140329</v>
+        <v>0.0032138745886835</v>
       </c>
       <c r="BW14" t="n">
-        <v>0.006665827142929006</v>
+        <v>0.01004636225816696</v>
       </c>
       <c r="BX14" t="n">
-        <v>-0.002098191945228358</v>
+        <v>-0.00407529764976355</v>
       </c>
       <c r="BY14" t="n">
-        <v>-0.001656711149913256</v>
+        <v>0.001727546235579196</v>
       </c>
       <c r="BZ14" t="n">
-        <v>0.007663303098571872</v>
+        <v>0.008807494124215269</v>
       </c>
       <c r="CA14" t="n">
-        <v>0.01009682928324908</v>
+        <v>0.009677472420787099</v>
       </c>
       <c r="CB14" t="n">
-        <v>0.004540788198835494</v>
+        <v>0.006682568978678978</v>
       </c>
       <c r="CC14" t="n">
-        <v>0.008118052397757185</v>
+        <v>0.01165303954821195</v>
       </c>
       <c r="CD14" t="n">
-        <v>-0.001836642044074973</v>
+        <v>-0.0004394888933663219</v>
       </c>
       <c r="CE14" t="n">
-        <v>-5.566735045341685e-06</v>
+        <v>0.003894506407041777</v>
       </c>
     </row>
     <row r="15">
@@ -4145,40 +4005,40 @@
       <c r="BR15" t="inlineStr"/>
       <c r="BS15" t="inlineStr"/>
       <c r="BT15" t="n">
-        <v>0.01418540743804711</v>
+        <v>0.01556832944782732</v>
       </c>
       <c r="BU15" t="n">
-        <v>0.01865172069746427</v>
+        <v>0.01892044073400895</v>
       </c>
       <c r="BV15" t="n">
-        <v>0.004622859482402207</v>
+        <v>0.002004974518019791</v>
       </c>
       <c r="BW15" t="n">
-        <v>0.007685916462648274</v>
+        <v>0.0129795151541851</v>
       </c>
       <c r="BX15" t="n">
-        <v>-0.001222498697675543</v>
+        <v>-0.004660011707418921</v>
       </c>
       <c r="BY15" t="n">
-        <v>7.605333032934892e-05</v>
+        <v>0.005373055546870394</v>
       </c>
       <c r="BZ15" t="n">
-        <v>0.01419929552195498</v>
+        <v>0.01608426841341041</v>
       </c>
       <c r="CA15" t="n">
-        <v>0.01839211567646852</v>
+        <v>0.01759052216944542</v>
       </c>
       <c r="CB15" t="n">
-        <v>0.005009359199770165</v>
+        <v>0.00810039811715026</v>
       </c>
       <c r="CC15" t="n">
-        <v>0.01001411231116784</v>
+        <v>0.015745907786902</v>
       </c>
       <c r="CD15" t="n">
-        <v>-0.0008219592726481739</v>
+        <v>0.001588215929495831</v>
       </c>
       <c r="CE15" t="n">
-        <v>0.002586134503858488</v>
+        <v>0.008651752946828323</v>
       </c>
     </row>
     <row r="16">
@@ -4254,40 +4114,40 @@
       <c r="BR16" t="inlineStr"/>
       <c r="BS16" t="inlineStr"/>
       <c r="BT16" t="n">
-        <v>0.02073242334523521</v>
+        <v>0.02311233926609982</v>
       </c>
       <c r="BU16" t="n">
-        <v>0.02715844629000115</v>
+        <v>0.02745254011488848</v>
       </c>
       <c r="BV16" t="n">
-        <v>0.004728094631881426</v>
+        <v>0.0005287332871603502</v>
       </c>
       <c r="BW16" t="n">
-        <v>0.008354502967161949</v>
+        <v>0.01537761367686739</v>
       </c>
       <c r="BX16" t="n">
-        <v>-0.0002500661054517859</v>
+        <v>-0.005147458268633167</v>
       </c>
       <c r="BY16" t="n">
-        <v>0.001873613226152834</v>
+        <v>0.008899622525478037</v>
       </c>
       <c r="BZ16" t="n">
-        <v>0.0207255561796886</v>
+        <v>0.02336084512573884</v>
       </c>
       <c r="CA16" t="n">
-        <v>0.02669481492934405</v>
+        <v>0.02563288594643249</v>
       </c>
       <c r="CB16" t="n">
-        <v>0.005240775259836876</v>
+        <v>0.009162777317660225</v>
       </c>
       <c r="CC16" t="n">
-        <v>0.01147754461314398</v>
+        <v>0.01922779210756178</v>
       </c>
       <c r="CD16" t="n">
-        <v>0.000274571346924094</v>
+        <v>0.003616720312730754</v>
       </c>
       <c r="CE16" t="n">
-        <v>0.005151556309440402</v>
+        <v>0.01318610193196549</v>
       </c>
     </row>
     <row r="17">
@@ -4363,40 +4223,40 @@
       <c r="BR17" t="inlineStr"/>
       <c r="BS17" t="inlineStr"/>
       <c r="BT17" t="n">
-        <v>0.02726816282275107</v>
+        <v>0.03067006787802389</v>
       </c>
       <c r="BU17" t="n">
-        <v>0.03564975957122629</v>
+        <v>0.03602276667661294</v>
       </c>
       <c r="BV17" t="n">
-        <v>0.004589875210631285</v>
+        <v>-0.00123815521346641</v>
       </c>
       <c r="BW17" t="n">
-        <v>0.008644851863192842</v>
+        <v>0.01721196225785935</v>
       </c>
       <c r="BX17" t="n">
-        <v>0.0008394765583976994</v>
+        <v>-0.00551442958143164</v>
       </c>
       <c r="BY17" t="n">
-        <v>0.003762341749030543</v>
+        <v>0.0123316358551473</v>
       </c>
       <c r="BZ17" t="n">
-        <v>0.02723967150771641</v>
+        <v>0.03063172461391239</v>
       </c>
       <c r="CA17" t="n">
-        <v>0.03499783548539535</v>
+        <v>0.03379318836606342</v>
       </c>
       <c r="CB17" t="n">
-        <v>0.005214639541091025</v>
+        <v>0.009846515261591053</v>
       </c>
       <c r="CC17" t="n">
-        <v>0.01248165102412013</v>
+        <v>0.02206879121142657</v>
       </c>
       <c r="CD17" t="n">
-        <v>0.001473248805748327</v>
+        <v>0.005668280404586297</v>
       </c>
       <c r="CE17" t="n">
-        <v>0.007715839058601974</v>
+        <v>0.01751716102362604</v>
       </c>
     </row>
     <row r="18">
@@ -4472,40 +4332,40 @@
       <c r="BR18" t="inlineStr"/>
       <c r="BS18" t="inlineStr"/>
       <c r="BT18" t="n">
-        <v>0.03379763510963812</v>
+        <v>0.03823475699305898</v>
       </c>
       <c r="BU18" t="n">
-        <v>0.04413715140473402</v>
+        <v>0.04465986356366604</v>
       </c>
       <c r="BV18" t="n">
-        <v>0.004260136757832303</v>
+        <v>-0.003236505391651533</v>
       </c>
       <c r="BW18" t="n">
-        <v>0.008624330863706318</v>
+        <v>0.0185465584484208</v>
       </c>
       <c r="BX18" t="n">
-        <v>0.001994106414272221</v>
+        <v>-0.005820275378190133</v>
       </c>
       <c r="BY18" t="n">
-        <v>0.005674266857886149</v>
+        <v>0.01559781386404531</v>
       </c>
       <c r="BZ18" t="n">
-        <v>0.03374781673420876</v>
+        <v>0.03791141026265075</v>
       </c>
       <c r="CA18" t="n">
-        <v>0.0433201783049494</v>
+        <v>0.04211314296289681</v>
       </c>
       <c r="CB18" t="n">
-        <v>0.004982724753069155</v>
+        <v>0.01020873692671188</v>
       </c>
       <c r="CC18" t="n">
-        <v>0.01309117593489559</v>
+        <v>0.02432317180783913</v>
       </c>
       <c r="CD18" t="n">
-        <v>0.002722137087714725</v>
+        <v>0.007684203444690054</v>
       </c>
       <c r="CE18" t="n">
-        <v>0.01021162217888778</v>
+        <v>0.02157302893647334</v>
       </c>
     </row>
     <row r="19">
@@ -4581,40 +4441,40 @@
       <c r="BR19" t="inlineStr"/>
       <c r="BS19" t="inlineStr"/>
       <c r="BT19" t="n">
-        <v>0.03705483565328305</v>
+        <v>0.04202670234571454</v>
       </c>
       <c r="BU19" t="n">
-        <v>0.0483675423003745</v>
+        <v>0.04897585218343851</v>
       </c>
       <c r="BV19" t="n">
-        <v>0.003969558592422028</v>
+        <v>-0.004383937843225719</v>
       </c>
       <c r="BW19" t="n">
-        <v>0.008427233688676466</v>
+        <v>0.01895478352797825</v>
       </c>
       <c r="BX19" t="n">
-        <v>0.002649681452706138</v>
+        <v>-0.005888886331320044</v>
       </c>
       <c r="BY19" t="n">
-        <v>0.00670893276078005</v>
+        <v>0.01723725111326942</v>
       </c>
       <c r="BZ19" t="n">
-        <v>0.03699326476467638</v>
+        <v>0.04153980726794487</v>
       </c>
       <c r="CA19" t="n">
-        <v>0.04746944265161113</v>
+        <v>0.04629729304236604</v>
       </c>
       <c r="CB19" t="n">
-        <v>0.004735824233164489</v>
+        <v>0.01020892973103858</v>
       </c>
       <c r="CC19" t="n">
-        <v>0.01317895700534213</v>
+        <v>0.02516115087731458</v>
       </c>
       <c r="CD19" t="n">
-        <v>0.003419117248059672</v>
+        <v>0.008738484270836552</v>
       </c>
       <c r="CE19" t="n">
-        <v>0.01150172563642469</v>
+        <v>0.02355929646385355</v>
       </c>
     </row>
     <row r="20">
@@ -4690,40 +4550,40 @@
       <c r="BR20" t="inlineStr"/>
       <c r="BS20" t="inlineStr"/>
       <c r="BT20" t="n">
-        <v>0.04029556751117</v>
+        <v>0.04584047994611924</v>
       </c>
       <c r="BU20" t="n">
-        <v>0.05256291546760771</v>
+        <v>0.05322817914864099</v>
       </c>
       <c r="BV20" t="n">
-        <v>0.003476290144943738</v>
+        <v>-0.005765771573148123</v>
       </c>
       <c r="BW20" t="n">
-        <v>0.007950739445927505</v>
+        <v>0.01903456632786238</v>
       </c>
       <c r="BX20" t="n">
-        <v>0.003476290144943738</v>
+        <v>-0.005765771573148123</v>
       </c>
       <c r="BY20" t="n">
-        <v>0.007950739445927505</v>
+        <v>0.01903456632786238</v>
       </c>
       <c r="BZ20" t="n">
-        <v>0.04021886570395366</v>
+        <v>0.04512790272181015</v>
       </c>
       <c r="CA20" t="n">
-        <v>0.05156826259938208</v>
+        <v>0.05041537327571449</v>
       </c>
       <c r="CB20" t="n">
-        <v>0.004283018989172565</v>
+        <v>0.009955858702121708</v>
       </c>
       <c r="CC20" t="n">
-        <v>0.01297066024396581</v>
+        <v>0.02565944805568296</v>
       </c>
       <c r="CD20" t="n">
-        <v>0.004283018989172565</v>
+        <v>0.009955858702121708</v>
       </c>
       <c r="CE20" t="n">
-        <v>0.01297066024396581</v>
+        <v>0.02565944805568296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new commit with little fixes in input data
</commit_message>
<xml_diff>
--- a/results/Профилирование_лопаток.xlsx
+++ b/results/Профилирование_лопаток.xlsx
@@ -835,2992 +835,2852 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>66.53761537615375</v>
+        <v>64.71094710947109</v>
       </c>
       <c r="B2" t="n">
-        <v>23.04332530766255</v>
+        <v>22.20486627069856</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8894362943629437</v>
+        <v>0.8614941149411495</v>
       </c>
       <c r="D2" t="n">
-        <v>1.413020524194945</v>
+        <v>1.343470347883344</v>
       </c>
       <c r="E2" t="n">
-        <v>67.03742037420375</v>
+        <v>65.10110101101012</v>
       </c>
       <c r="F2" t="n">
-        <v>23.27355074632903</v>
+        <v>22.3835587120456</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8830280302803029</v>
+        <v>0.8574665746657466</v>
       </c>
       <c r="H2" t="n">
-        <v>1.475261520272945</v>
+        <v>1.386708868839728</v>
       </c>
       <c r="I2" t="n">
-        <v>1.032551310487361</v>
+        <v>0.8586758697083607</v>
       </c>
       <c r="J2" t="n">
-        <v>-1.311846199317638</v>
+        <v>-1.53322782790068</v>
       </c>
       <c r="K2" t="n">
         <v>0.5</v>
       </c>
       <c r="L2" t="n">
-        <v>0.276924768621417</v>
+        <v>0.2805780275618496</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2759255059583664</v>
+        <v>0.2797974550671152</v>
       </c>
       <c r="N2" t="n">
-        <v>0.4428690383644288</v>
+        <v>0.420727598857796</v>
       </c>
       <c r="O2" t="n">
-        <v>0.4937488175649478</v>
+        <v>0.4744794689706583</v>
       </c>
       <c r="P2" t="n">
-        <v>0.2214345191822144</v>
+        <v>0.210363799428898</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.2468744087824739</v>
+        <v>0.2372397344853292</v>
       </c>
       <c r="R2" t="n">
-        <v>47.29585770116213</v>
+        <v>46.6507350952965</v>
       </c>
       <c r="S2" t="n">
-        <v>45.42106865188677</v>
+        <v>44.61222616554168</v>
       </c>
       <c r="T2" t="n">
-        <v>3.000000000000001</v>
+        <v>2.3</v>
       </c>
       <c r="U2" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="V2" t="n">
-        <v>0.07927631177856866</v>
+        <v>0.08809094646749863</v>
       </c>
       <c r="W2" t="n">
-        <v>0.09231847708159061</v>
+        <v>0.08767872315935056</v>
       </c>
       <c r="X2" t="n">
-        <v>10.25632634966623</v>
+        <v>11.99648133201724</v>
       </c>
       <c r="Y2" t="n">
-        <v>10.7128873763988</v>
+        <v>10.58767654539239</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.05610414740701351</v>
+        <v>0.06556969910522187</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.06257770287705353</v>
+        <v>0.06322792413717823</v>
       </c>
       <c r="AB2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="AC2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.0736119838484469</v>
+        <v>0.08271806388838863</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.08210567429249846</v>
+        <v>0.07976384732094619</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.076948448255158</v>
+        <v>1.064954162688813</v>
       </c>
       <c r="AG2" t="n">
-        <v>1.124386077784459</v>
+        <v>1.099228862501545</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.1923711206378953</v>
+        <v>0.1623854067220315</v>
       </c>
       <c r="AI2" t="n">
-        <v>-2.189034805538853</v>
+        <v>-2.251927843746138</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.3250134241483084</v>
+        <v>0.3228070637905909</v>
       </c>
       <c r="AK2" t="n">
-        <v>0.2607302112741996</v>
+        <v>0.2657315072231888</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.229614761635697</v>
+        <v>0.2393527695658109</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.5256960683641339</v>
+        <v>0.5121947927975168</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.07744592324816735</v>
+        <v>0.0797346228595819</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.1453395513705724</v>
+        <v>0.1426994408343503</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.1148073808178485</v>
+        <v>0.1196763847829054</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.2628480341820669</v>
+        <v>0.2560973963987584</v>
       </c>
       <c r="AR2" t="n">
-        <v>33.57241427064274</v>
+        <v>34.29205694531353</v>
       </c>
       <c r="AS2" t="n">
-        <v>52.18370052787058</v>
+        <v>50.48175425748313</v>
       </c>
       <c r="AT2" t="n">
-        <v>0.02208359515453407</v>
+        <v>0.03556876747200711</v>
       </c>
       <c r="AU2" t="n">
-        <v>0.03302417362647769</v>
+        <v>0.0404137283847249</v>
       </c>
       <c r="AV2" t="n">
-        <v>3.589828160850528</v>
+        <v>2.476637587648402</v>
       </c>
       <c r="AW2" t="n">
-        <v>2.795481822672247</v>
+        <v>2.169528194099763</v>
       </c>
       <c r="AX2" t="n">
-        <v>6.47457040212632</v>
+        <v>3.691593969121004</v>
       </c>
       <c r="AY2" t="n">
-        <v>1.988704556680618</v>
+        <v>0.4238204852494087</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.2307422903960569</v>
+        <v>0.2474271985205285</v>
       </c>
       <c r="BA2" t="n">
-        <v>0.2607302112741996</v>
+        <v>0.2657315072231888</v>
       </c>
       <c r="BB2" t="n">
-        <v>0.1688644817957764</v>
+        <v>0.2587207385462206</v>
       </c>
       <c r="BC2" t="n">
-        <v>0.3832906019879738</v>
+        <v>0.409566208189467</v>
       </c>
       <c r="BD2" t="n">
-        <v>0.07382481050406133</v>
+        <v>0.1007418472750847</v>
       </c>
       <c r="BE2" t="n">
-        <v>0.1670890014736256</v>
+        <v>0.1603060146952187</v>
       </c>
       <c r="BF2" t="n">
-        <v>0.08443224089788821</v>
+        <v>0.1293603692731103</v>
       </c>
       <c r="BG2" t="n">
-        <v>0.1916453009939869</v>
+        <v>0.2047831040947335</v>
       </c>
       <c r="BH2" t="n">
-        <v>81.21635254223462</v>
+        <v>68.92276727815506</v>
       </c>
       <c r="BI2" t="n">
-        <v>56.29023715690198</v>
+        <v>53.10618829417465</v>
       </c>
       <c r="BJ2" t="n">
-        <v>26.89849088400845</v>
+        <v>19.50846214460636</v>
       </c>
       <c r="BK2" t="n">
-        <v>13.80015305221628</v>
+        <v>12.26573722484221</v>
       </c>
       <c r="BL2" t="n">
-        <v>0.01981907794464216</v>
+        <v>0.02202273661687466</v>
       </c>
       <c r="BM2" t="n">
-        <v>0.02307961927039765</v>
+        <v>0.02191968078983764</v>
       </c>
       <c r="BN2" t="n">
-        <v>0.07834655952915857</v>
+        <v>0.08219735479291895</v>
       </c>
       <c r="BO2" t="n">
-        <v>0.07679600846602362</v>
+        <v>0.07012101525937343</v>
       </c>
       <c r="BP2" t="n">
-        <v>0.05825743160560556</v>
+        <v>0.06405822095022083</v>
       </c>
       <c r="BQ2" t="n">
-        <v>0.06575699182726667</v>
+        <v>0.06157720338866012</v>
       </c>
       <c r="BR2" t="n">
-        <v>0.04383904454215617</v>
+        <v>0.04963145400225756</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.07292980784918728</v>
+        <v>0.06763729477145963</v>
       </c>
       <c r="BT2" t="n">
-        <v>-0.02852424391887475</v>
+        <v>-0.03175313042359209</v>
       </c>
       <c r="BU2" t="n">
-        <v>-0.03120809524078163</v>
+        <v>-0.02917686407068444</v>
       </c>
       <c r="BV2" t="n">
-        <v>0.003589172156867016</v>
+        <v>-0.0004265776232835885</v>
       </c>
       <c r="BW2" t="n">
-        <v>-0.01400445825870235</v>
+        <v>-0.01421966510978654</v>
       </c>
       <c r="BX2" t="n">
-        <v>0.001878662409681145</v>
+        <v>-0.002343648423975944</v>
       </c>
       <c r="BY2" t="n">
-        <v>-0.01595658881978716</v>
+        <v>-0.01605340381042088</v>
       </c>
       <c r="BZ2" t="n">
-        <v>-0.02725677001940365</v>
+        <v>-0.03024295581060679</v>
       </c>
       <c r="CA2" t="n">
-        <v>-0.02823444890251725</v>
+        <v>-0.02711578569644493</v>
       </c>
       <c r="CB2" t="n">
-        <v>-0.007052557364857244</v>
+        <v>-0.008276644027908587</v>
       </c>
       <c r="CC2" t="n">
-        <v>-0.0190812107454781</v>
+        <v>-0.01768313750147933</v>
       </c>
       <c r="CD2" t="n">
-        <v>-0.008723851307659148</v>
+        <v>-0.01013352970601998</v>
       </c>
       <c r="CE2" t="n">
-        <v>-0.02090186282059832</v>
+        <v>-0.01942567302533631</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>57.8930289302893</v>
+        <v>57.22832228322283</v>
       </c>
       <c r="B3" t="n">
-        <v>19.11424852803111</v>
+        <v>18.81567062072647</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7026121261212612</v>
+        <v>0.7110431104311044</v>
       </c>
       <c r="D3" t="n">
-        <v>1.317664062849037</v>
+        <v>1.276261555027143</v>
       </c>
       <c r="E3" t="n">
-        <v>59.56414564145641</v>
+        <v>58.60958609586096</v>
       </c>
       <c r="F3" t="n">
-        <v>19.86669849423924</v>
+        <v>19.43655408659217</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6356117561175612</v>
+        <v>0.6575573755737557</v>
       </c>
       <c r="H3" t="n">
-        <v>1.313654812360745</v>
+        <v>1.243016434060997</v>
       </c>
       <c r="I3" t="n">
-        <v>0.7941601571225931</v>
+        <v>0.6906538875678575</v>
       </c>
       <c r="J3" t="n">
-        <v>-1.715862969098137</v>
+        <v>-1.892458914847508</v>
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
-        <v>0.2942137346088875</v>
+        <v>0.2955426512428469</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2908711385415155</v>
+        <v>0.2927804127314371</v>
       </c>
       <c r="N3" t="n">
-        <v>0.296542159153081</v>
+        <v>0.2999085555356453</v>
       </c>
       <c r="O3" t="n">
-        <v>0.335480397337627</v>
+        <v>0.3472958171817123</v>
       </c>
       <c r="P3" t="n">
-        <v>0.1482710795765405</v>
+        <v>0.1499542777678227</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.1677401986688135</v>
+        <v>0.1736479085908562</v>
       </c>
       <c r="R3" t="n">
-        <v>45.40560420381076</v>
+        <v>44.69046656841657</v>
       </c>
       <c r="S3" t="n">
-        <v>45.3886497444955</v>
+        <v>44.11033190632091</v>
       </c>
       <c r="T3" t="n">
-        <v>2.900000000000001</v>
+        <v>2.2</v>
       </c>
       <c r="U3" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="V3" t="n">
-        <v>0.07550719441710939</v>
+        <v>0.08414191042415915</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06141055051463777</v>
+        <v>0.05941383124246263</v>
       </c>
       <c r="X3" t="n">
-        <v>14.58898257165743</v>
+        <v>16.07483935423091</v>
       </c>
       <c r="Y3" t="n">
-        <v>10.48815494507076</v>
+        <v>9.801923368690177</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.05730382769478333</v>
+        <v>0.06592842203287214</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.04674785943521798</v>
+        <v>0.04779810597383229</v>
       </c>
       <c r="AB3" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="AC3" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.06886282360015999</v>
+        <v>0.07701336982712045</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.05617756662118316</v>
+        <v>0.05583469312466233</v>
       </c>
       <c r="AF3" t="n">
-        <v>1.096487051642389</v>
+        <v>1.092562377325403</v>
       </c>
       <c r="AG3" t="n">
-        <v>1.093150775446393</v>
+        <v>1.064102405108758</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.2412176291059737</v>
+        <v>0.2314059433135063</v>
       </c>
       <c r="AI3" t="n">
-        <v>-2.267123061384018</v>
+        <v>-2.339743987228105</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.3254229079431258</v>
+        <v>0.323074478994441</v>
       </c>
       <c r="AK3" t="n">
-        <v>0.262608845959918</v>
+        <v>0.2680887534788575</v>
       </c>
       <c r="AL3" t="n">
-        <v>0.2422538757388784</v>
+        <v>0.2539937444186274</v>
       </c>
       <c r="AM3" t="n">
-        <v>0.5555357608184214</v>
+        <v>0.5434140918325888</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.08255067128748017</v>
+        <v>0.08577264324703658</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.1525321547062393</v>
+        <v>0.150280006146969</v>
       </c>
       <c r="AP3" t="n">
-        <v>0.1211269378694392</v>
+        <v>0.1269968722093137</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.2777678804092107</v>
+        <v>0.2717070459162944</v>
       </c>
       <c r="AR3" t="n">
-        <v>32.84314696125617</v>
+        <v>33.53504718272685</v>
       </c>
       <c r="AS3" t="n">
-        <v>50.13822355247309</v>
+        <v>48.18370821953807</v>
       </c>
       <c r="AT3" t="n">
-        <v>0.02448106507793388</v>
+        <v>0.03690667073576822</v>
       </c>
       <c r="AU3" t="n">
-        <v>0.03485406335095416</v>
+        <v>0.03810255782813261</v>
       </c>
       <c r="AV3" t="n">
-        <v>3.084310023960851</v>
+        <v>2.279856425592264</v>
       </c>
       <c r="AW3" t="n">
-        <v>1.761933749195318</v>
+        <v>1.55931345896666</v>
       </c>
       <c r="AX3" t="n">
-        <v>5.210775059902126</v>
+        <v>3.199641063980661</v>
       </c>
       <c r="AY3" t="n">
-        <v>-0.5951656270117062</v>
+        <v>-1.101716352583351</v>
       </c>
       <c r="AZ3" t="n">
-        <v>0.2723046553902756</v>
+        <v>0.2790202819545599</v>
       </c>
       <c r="BA3" t="n">
-        <v>0.262608845959918</v>
+        <v>0.2680887534788575</v>
       </c>
       <c r="BB3" t="n">
-        <v>-0.1133839041023485</v>
+        <v>0.03772200787821538</v>
       </c>
       <c r="BC3" t="n">
-        <v>0.4822233521235706</v>
+        <v>0.4846231861043642</v>
       </c>
       <c r="BD3" t="n">
-        <v>-0.05422324265513867</v>
+        <v>0.01589221104361284</v>
       </c>
       <c r="BE3" t="n">
-        <v>0.1680940635442917</v>
+        <v>0.1622368470732864</v>
       </c>
       <c r="BF3" t="n">
-        <v>-0.05669195205117426</v>
+        <v>0.01886100393910769</v>
       </c>
       <c r="BG3" t="n">
-        <v>0.2411116760617853</v>
+        <v>0.2423115930521821</v>
       </c>
       <c r="BH3" t="n">
-        <v>74.28011979665044</v>
+        <v>63.74680026925577</v>
       </c>
       <c r="BI3" t="n">
-        <v>51.77352478249799</v>
+        <v>49.3923404013187</v>
       </c>
       <c r="BJ3" t="n">
-        <v>-38.15571798437937</v>
+        <v>127.8027524437847</v>
       </c>
       <c r="BK3" t="n">
-        <v>7.296568553904804</v>
+        <v>7.024368664345802</v>
       </c>
       <c r="BL3" t="n">
-        <v>0.01887679860427735</v>
+        <v>0.02103547760603979</v>
       </c>
       <c r="BM3" t="n">
-        <v>0.01535263762865944</v>
+        <v>0.01485345781061566</v>
       </c>
       <c r="BN3" t="n">
-        <v>0.0726830589950581</v>
+        <v>0.07546250745856779</v>
       </c>
       <c r="BO3" t="n">
-        <v>0.04824235097513396</v>
+        <v>0.04510604798065593</v>
       </c>
       <c r="BP3" t="n">
-        <v>0.05376827457552832</v>
+        <v>0.05917502181382855</v>
       </c>
       <c r="BQ3" t="n">
-        <v>0.04371736864220463</v>
+        <v>0.04135453867823583</v>
       </c>
       <c r="BR3" t="n">
-        <v>0.04095065116298202</v>
+        <v>0.0464839426715804</v>
       </c>
       <c r="BS3" t="n">
-        <v>0.04713830313335133</v>
+        <v>0.0442803230249816</v>
       </c>
       <c r="BT3" t="n">
-        <v>-0.02817154334759125</v>
+        <v>-0.03132380954186157</v>
       </c>
       <c r="BU3" t="n">
-        <v>-0.0307125006343836</v>
+        <v>-0.02870878976301185</v>
       </c>
       <c r="BV3" t="n">
-        <v>0.003784776917328531</v>
+        <v>-0.0001591414503246175</v>
       </c>
       <c r="BW3" t="n">
-        <v>-0.01350262641014433</v>
+        <v>-0.01373050623955496</v>
       </c>
       <c r="BX3" t="n">
-        <v>0.00163913749761288</v>
+        <v>-0.002563888156456257</v>
       </c>
       <c r="BY3" t="n">
-        <v>-0.01595135158764546</v>
+        <v>-0.01603072232894716</v>
       </c>
       <c r="BZ3" t="n">
-        <v>-0.02684847359707806</v>
+        <v>-0.02978758592278062</v>
       </c>
       <c r="CA3" t="n">
-        <v>-0.02776149547790772</v>
+        <v>-0.02666379557088615</v>
       </c>
       <c r="CB3" t="n">
-        <v>-0.006705931273135243</v>
+        <v>-0.007884074647287425</v>
       </c>
       <c r="CC3" t="n">
-        <v>-0.01851344308971568</v>
+        <v>-0.01714925142425885</v>
       </c>
       <c r="CD3" t="n">
-        <v>-0.008802378938228857</v>
+        <v>-0.01021332598035699</v>
       </c>
       <c r="CE3" t="n">
-        <v>-0.0207972434997349</v>
+        <v>-0.01933506352874612</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>56.07826078260783</v>
+        <v>55.64475644756448</v>
       </c>
       <c r="B4" t="n">
-        <v>18.29986890376677</v>
+        <v>18.10566130567151</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7219622196221962</v>
+        <v>0.7476310763107631</v>
       </c>
       <c r="D4" t="n">
-        <v>1.296467987594899</v>
+        <v>1.266616501556358</v>
       </c>
       <c r="E4" t="n">
-        <v>57.77912779127792</v>
+        <v>57.0149701497015</v>
       </c>
       <c r="F4" t="n">
-        <v>19.06305907249112</v>
+        <v>18.71991109733465</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6455642556425565</v>
+        <v>0.6892585925859258</v>
       </c>
       <c r="H4" t="n">
-        <v>1.284174392467016</v>
+        <v>1.20943424583362</v>
       </c>
       <c r="I4" t="n">
-        <v>0.7411699689872486</v>
+        <v>0.6665412538908938</v>
       </c>
       <c r="J4" t="n">
-        <v>-1.789564018832459</v>
+        <v>-1.976414385415951</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
-        <v>0.297842934908937</v>
+        <v>0.2987103941889569</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2944414577528364</v>
+        <v>0.29597009572608</v>
       </c>
       <c r="N4" t="n">
-        <v>0.2947554099937199</v>
+        <v>0.3057816916136074</v>
       </c>
       <c r="O4" t="n">
-        <v>0.3323850044552822</v>
+        <v>0.3553164973311553</v>
       </c>
       <c r="P4" t="n">
-        <v>0.1473777049968599</v>
+        <v>0.1528908458068037</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.1661925022276411</v>
+        <v>0.1776582486655776</v>
       </c>
       <c r="R4" t="n">
-        <v>43.75531435107216</v>
+        <v>42.92778890381278</v>
       </c>
       <c r="S4" t="n">
-        <v>43.84944860932053</v>
+        <v>42.31339151253506</v>
       </c>
       <c r="T4" t="n">
-        <v>2.800000000000001</v>
+        <v>2.1</v>
       </c>
       <c r="U4" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="V4" t="n">
-        <v>0.07146885438697448</v>
+        <v>0.07981677571002545</v>
       </c>
       <c r="W4" t="n">
-        <v>0.05562162566458909</v>
+        <v>0.05369580001542452</v>
       </c>
       <c r="X4" t="n">
-        <v>13.89242775427387</v>
+        <v>14.9556691432101</v>
       </c>
       <c r="Y4" t="n">
-        <v>9.587944180220799</v>
+        <v>8.658611889585416</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.05512581496096761</v>
+        <v>0.06301573965912367</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.04331314032647456</v>
+        <v>0.04439745294165532</v>
       </c>
       <c r="AB4" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="AC4" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.06468931913954425</v>
+        <v>0.07204476532214493</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.05082732218107048</v>
+        <v>0.05075881193151121</v>
       </c>
       <c r="AF4" t="n">
-        <v>1.10480146239916</v>
+        <v>1.107877516890066</v>
       </c>
       <c r="AG4" t="n">
-        <v>1.094325321063326</v>
+        <v>1.05786163962774</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.2620036559979011</v>
+        <v>0.2696937922251647</v>
       </c>
       <c r="AI4" t="n">
-        <v>-2.264186697341684</v>
+        <v>-2.355345900930651</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0.3257241367876161</v>
+        <v>0.3232596062489652</v>
       </c>
       <c r="AK4" t="n">
-        <v>0.2649661865772098</v>
+        <v>0.2708961631488436</v>
       </c>
       <c r="AL4" t="n">
-        <v>0.2565864593668054</v>
+        <v>0.2704232733200921</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.5785254741371562</v>
+        <v>0.5678093528231558</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.08784676964867695</v>
+        <v>0.0920113450601408</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.1603563515071832</v>
+        <v>0.158204863460758</v>
       </c>
       <c r="AP4" t="n">
-        <v>0.1282932296834027</v>
+        <v>0.135211636660046</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0.2892627370685781</v>
+        <v>0.2839046764115779</v>
       </c>
       <c r="AR4" t="n">
-        <v>32.12069878451009</v>
+        <v>32.7698202562645</v>
       </c>
       <c r="AS4" t="n">
-        <v>48.0549065833119</v>
+        <v>45.87141709504831</v>
       </c>
       <c r="AT4" t="n">
-        <v>0.02658793258637614</v>
+        <v>0.03807194132033433</v>
       </c>
       <c r="AU4" t="n">
-        <v>0.03418537069834719</v>
+        <v>0.03695687577047703</v>
       </c>
       <c r="AV4" t="n">
-        <v>2.688018489395286</v>
+        <v>2.096472439859406</v>
       </c>
       <c r="AW4" t="n">
-        <v>1.62705931011824</v>
+        <v>1.452931258283455</v>
       </c>
       <c r="AX4" t="n">
-        <v>4.220046223488215</v>
+        <v>2.741181099648514</v>
       </c>
       <c r="AY4" t="n">
-        <v>-0.9323517247043989</v>
+        <v>-1.367671854291363</v>
       </c>
       <c r="AZ4" t="n">
-        <v>0.2802455284145835</v>
+        <v>0.2854359292291072</v>
       </c>
       <c r="BA4" t="n">
-        <v>0.2649661865772098</v>
+        <v>0.2708961631488436</v>
       </c>
       <c r="BB4" t="n">
-        <v>-0.06582268657612578</v>
+        <v>0.07401070235359011</v>
       </c>
       <c r="BC4" t="n">
-        <v>0.5159144546656084</v>
+        <v>0.5172711206614387</v>
       </c>
       <c r="BD4" t="n">
-        <v>-0.03024338664917521</v>
+        <v>0.03058776489424033</v>
       </c>
       <c r="BE4" t="n">
-        <v>0.1743692274620104</v>
+        <v>0.168905433241024</v>
       </c>
       <c r="BF4" t="n">
-        <v>-0.03291134328806289</v>
+        <v>0.03700535117679506</v>
       </c>
       <c r="BG4" t="n">
-        <v>0.2579572273328042</v>
+        <v>0.2586355603307193</v>
       </c>
       <c r="BH4" t="n">
-        <v>67.97104131334986</v>
+        <v>58.91449161643909</v>
       </c>
       <c r="BI4" t="n">
-        <v>49.35543604621341</v>
+        <v>46.83382202560673</v>
       </c>
       <c r="BJ4" t="n">
-        <v>-62.21052590211599</v>
+        <v>61.79058642926131</v>
       </c>
       <c r="BK4" t="n">
-        <v>6.177177510168397</v>
+        <v>5.947660798823581</v>
       </c>
       <c r="BL4" t="n">
-        <v>0.01786721359674362</v>
+        <v>0.01995419392750636</v>
       </c>
       <c r="BM4" t="n">
-        <v>0.01390540641614727</v>
+        <v>0.01342395000385613</v>
       </c>
       <c r="BN4" t="n">
-        <v>0.06625122785009492</v>
+        <v>0.06835490331001551</v>
       </c>
       <c r="BO4" t="n">
-        <v>0.04220373798770107</v>
+        <v>0.03916424486105904</v>
       </c>
       <c r="BP4" t="n">
-        <v>0.04942643418892151</v>
+        <v>0.05436129655519698</v>
       </c>
       <c r="BQ4" t="n">
-        <v>0.03853276137609483</v>
+        <v>0.03614722679314573</v>
       </c>
       <c r="BR4" t="n">
-        <v>0.03800031704370419</v>
+        <v>0.0432020573194755</v>
       </c>
       <c r="BS4" t="n">
-        <v>0.04137057047261833</v>
+        <v>0.03854171985818369</v>
       </c>
       <c r="BT4" t="n">
-        <v>-0.02745254639230837</v>
+        <v>-0.03047023599544833</v>
       </c>
       <c r="BU4" t="n">
-        <v>-0.0297755122158496</v>
+        <v>-0.02782737475496434</v>
       </c>
       <c r="BV4" t="n">
-        <v>0.004055310153288439</v>
+        <v>0.0002409616260022956</v>
       </c>
       <c r="BW4" t="n">
-        <v>-0.01263853048125095</v>
+        <v>-0.01288347460431978</v>
       </c>
       <c r="BX4" t="n">
-        <v>0.001279482931977889</v>
+        <v>-0.002870074322489686</v>
       </c>
       <c r="BY4" t="n">
-        <v>-0.01580646165494122</v>
+        <v>-0.01585927863605094</v>
       </c>
       <c r="BZ4" t="n">
-        <v>-0.02606052724603005</v>
+        <v>-0.02891026322160087</v>
       </c>
       <c r="CA4" t="n">
-        <v>-0.02688772054240456</v>
+        <v>-0.02582677688731723</v>
       </c>
       <c r="CB4" t="n">
-        <v>-0.006131319115623479</v>
+        <v>-0.007230826380267347</v>
       </c>
       <c r="CC4" t="n">
-        <v>-0.01750910469219961</v>
+        <v>-0.01620694862055892</v>
       </c>
       <c r="CD4" t="n">
-        <v>-0.008843506654380953</v>
+        <v>-0.01024419348948321</v>
       </c>
       <c r="CE4" t="n">
-        <v>-0.02046367165621048</v>
+        <v>-0.01903474749699349</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>55.12880128801288</v>
+        <v>54.76839768397684</v>
       </c>
       <c r="B5" t="n">
-        <v>17.87464237590368</v>
+        <v>17.71334018699288</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7761102611026111</v>
+        <v>0.8133784337843379</v>
       </c>
       <c r="D5" t="n">
-        <v>1.271800132053795</v>
+        <v>1.249735220329377</v>
       </c>
       <c r="E5" t="n">
-        <v>56.74551745517455</v>
+        <v>56.02216022160222</v>
       </c>
       <c r="F5" t="n">
-        <v>18.59902048421408</v>
+        <v>18.27473013364838</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7017708177081771</v>
+        <v>0.7591587915879159</v>
       </c>
       <c r="H5" t="n">
-        <v>1.253677443896893</v>
+        <v>1.223742124628993</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6795003301344887</v>
+        <v>0.624338050823442</v>
       </c>
       <c r="J5" t="n">
-        <v>-1.865806390257767</v>
+        <v>-1.940644688427518</v>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
-        <v>0.2997417375895345</v>
+        <v>0.3004637537005771</v>
       </c>
       <c r="M5" t="n">
-        <v>0.2965082465908455</v>
+        <v>0.2979554985504871</v>
       </c>
       <c r="N5" t="n">
-        <v>0.3136206581144917</v>
+        <v>0.3289842006785773</v>
       </c>
       <c r="O5" t="n">
-        <v>0.3541537417428445</v>
+        <v>0.3777546745912216</v>
       </c>
       <c r="P5" t="n">
-        <v>0.1568103290572459</v>
+        <v>0.1644921003392887</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.1770768708714223</v>
+        <v>0.1888773372956108</v>
       </c>
       <c r="R5" t="n">
-        <v>42.09280985591618</v>
+        <v>41.14939067960899</v>
       </c>
       <c r="S5" t="n">
-        <v>42.00495229159156</v>
+        <v>40.3969818341203</v>
       </c>
       <c r="T5" t="n">
-        <v>2.700000000000001</v>
+        <v>2</v>
       </c>
       <c r="U5" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="V5" t="n">
-        <v>0.06713137805831104</v>
+        <v>0.07505912752447835</v>
       </c>
       <c r="W5" t="n">
-        <v>0.05263902986242827</v>
+        <v>0.05052986232852519</v>
       </c>
       <c r="X5" t="n">
-        <v>12.26433698766301</v>
+        <v>13.07229076636349</v>
       </c>
       <c r="Y5" t="n">
-        <v>8.516072808465776</v>
+        <v>7.6641092465475</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.05278453458713077</v>
+        <v>0.06006002415831409</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.04198769796703584</v>
+        <v>0.04129126660884094</v>
       </c>
       <c r="AB5" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="AC5" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.06099278661728457</v>
+        <v>0.06767841590868161</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.04851698935465818</v>
+        <v>0.04652891093721861</v>
       </c>
       <c r="AF5" t="n">
-        <v>1.100644548010975</v>
+        <v>1.109055620122013</v>
       </c>
       <c r="AG5" t="n">
-        <v>1.084960764519786</v>
+        <v>1.08598850286234</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.2516113700274386</v>
+        <v>0.2726390503050313</v>
       </c>
       <c r="AI5" t="n">
-        <v>-2.287598088700534</v>
+        <v>-2.28502874284415</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.3259089294885351</v>
+        <v>0.3233557544476356</v>
       </c>
       <c r="AK5" t="n">
-        <v>0.2678422755564227</v>
+        <v>0.2741937413115497</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.2729640504469745</v>
+        <v>0.2890375618319029</v>
       </c>
       <c r="AM5" t="n">
-        <v>0.5999895752827809</v>
+        <v>0.5832000152692201</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.09333085770859355</v>
+        <v>0.0984263868106539</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.1673901302231228</v>
+        <v>0.1666432311688638</v>
       </c>
       <c r="AP5" t="n">
-        <v>0.1364820252234872</v>
+        <v>0.1445187809159515</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.2999947876413904</v>
+        <v>0.29160000763461</v>
       </c>
       <c r="AR5" t="n">
-        <v>31.4008135212329</v>
+        <v>31.99089078020046</v>
       </c>
       <c r="AS5" t="n">
-        <v>45.84170532617449</v>
+        <v>43.5717772983281</v>
       </c>
       <c r="AT5" t="n">
-        <v>0.02845401523671071</v>
+        <v>0.03909596698555911</v>
       </c>
       <c r="AU5" t="n">
-        <v>0.03423500116988514</v>
+        <v>0.03528452696751289</v>
       </c>
       <c r="AV5" t="n">
-        <v>2.35929367085246</v>
+        <v>1.919868807752037</v>
       </c>
       <c r="AW5" t="n">
-        <v>1.537579321268791</v>
+        <v>1.432068577114523</v>
       </c>
       <c r="AX5" t="n">
-        <v>3.398234177131151</v>
+        <v>2.299672019380092</v>
       </c>
       <c r="AY5" t="n">
-        <v>-1.156051696828022</v>
+        <v>-1.419828557213693</v>
       </c>
       <c r="AZ5" t="n">
-        <v>0.2845679373083452</v>
+        <v>0.2891204224269057</v>
       </c>
       <c r="BA5" t="n">
-        <v>0.2678422755564227</v>
+        <v>0.2741937413115497</v>
       </c>
       <c r="BB5" t="n">
-        <v>0.01321322788305265</v>
+        <v>0.1363696986133681</v>
       </c>
       <c r="BC5" t="n">
-        <v>0.5433162684829774</v>
+        <v>0.5378976972816791</v>
       </c>
       <c r="BD5" t="n">
-        <v>0.005775450851110768</v>
+        <v>0.05463015425008073</v>
       </c>
       <c r="BE5" t="n">
-        <v>0.1804473880604332</v>
+        <v>0.1764977324823939</v>
       </c>
       <c r="BF5" t="n">
-        <v>0.006606613941526326</v>
+        <v>0.06818484930668407</v>
       </c>
       <c r="BG5" t="n">
-        <v>0.2716581342414887</v>
+        <v>0.2689488486408396</v>
       </c>
       <c r="BH5" t="n">
-        <v>62.10583340672036</v>
+        <v>54.32492543270619</v>
       </c>
       <c r="BI5" t="n">
-        <v>46.94491506464711</v>
+        <v>44.41432632496479</v>
       </c>
       <c r="BJ5" t="n">
-        <v>291.0980328353404</v>
+        <v>31.53612774617817</v>
       </c>
       <c r="BK5" t="n">
-        <v>5.551104805413742</v>
+        <v>5.382358945626046</v>
       </c>
       <c r="BL5" t="n">
-        <v>0.01678284451457776</v>
+        <v>0.01876478188111959</v>
       </c>
       <c r="BM5" t="n">
-        <v>0.01315975746560707</v>
+        <v>0.0126324655821313</v>
       </c>
       <c r="BN5" t="n">
-        <v>0.05933160252303486</v>
+        <v>0.06097332963005083</v>
       </c>
       <c r="BO5" t="n">
-        <v>0.03846321706612884</v>
+        <v>0.035362918218419</v>
       </c>
       <c r="BP5" t="n">
-        <v>0.04500041173981374</v>
+        <v>0.04939075204307926</v>
       </c>
       <c r="BQ5" t="n">
-        <v>0.03522576699209243</v>
+        <v>0.0327473822968867</v>
       </c>
       <c r="BR5" t="n">
-        <v>0.03497690814532944</v>
+        <v>0.03976515708176084</v>
       </c>
       <c r="BS5" t="n">
-        <v>0.03776418125425757</v>
+        <v>0.03482835177406542</v>
       </c>
       <c r="BT5" t="n">
-        <v>-0.02562557897479202</v>
+        <v>-0.02834735611040769</v>
       </c>
       <c r="BU5" t="n">
-        <v>-0.0275478353975069</v>
+        <v>-0.02573946916751957</v>
       </c>
       <c r="BV5" t="n">
-        <v>0.004465329579521619</v>
+        <v>0.0009455439222736328</v>
       </c>
       <c r="BW5" t="n">
-        <v>-0.01079294460147055</v>
+        <v>-0.01106252337007117</v>
       </c>
       <c r="BX5" t="n">
-        <v>0.0006391893555526829</v>
+        <v>-0.003342640763485584</v>
       </c>
       <c r="BY5" t="n">
-        <v>-0.01515955243547606</v>
+        <v>-0.0151643073057006</v>
       </c>
       <c r="BZ5" t="n">
-        <v>-0.02415210591859589</v>
+        <v>-0.02678856129391288</v>
       </c>
       <c r="CA5" t="n">
-        <v>-0.02485387618831984</v>
+        <v>-0.02387423139481638</v>
       </c>
       <c r="CB5" t="n">
-        <v>-0.004959249515632345</v>
+        <v>-0.0058919751161406</v>
       </c>
       <c r="CC5" t="n">
-        <v>-0.01529765490550886</v>
+        <v>-0.01413717610845646</v>
       </c>
       <c r="CD5" t="n">
-        <v>-0.008697670177162916</v>
+        <v>-0.01004553518560031</v>
       </c>
       <c r="CE5" t="n">
-        <v>-0.01937016612617249</v>
+        <v>-0.01803495293813654</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>54.44709447094471</v>
+        <v>54.09349093490935</v>
       </c>
       <c r="B6" t="n">
-        <v>17.56957681884398</v>
+        <v>17.41139532448921</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8429853298532985</v>
+        <v>0.8892393923939239</v>
       </c>
       <c r="D6" t="n">
-        <v>1.234605221892104</v>
+        <v>1.217356601623034</v>
       </c>
       <c r="E6" t="n">
-        <v>55.9320593205932</v>
+        <v>55.18490184901849</v>
       </c>
       <c r="F6" t="n">
-        <v>18.23435960335043</v>
+        <v>17.89975546460377</v>
       </c>
       <c r="G6" t="n">
-        <v>0.7758775587755877</v>
+        <v>0.8430569305693056</v>
       </c>
       <c r="H6" t="n">
-        <v>1.23694702711554</v>
+        <v>1.195035017839403</v>
       </c>
       <c r="I6" t="n">
-        <v>0.5865130547302611</v>
+        <v>0.5433915040575843</v>
       </c>
       <c r="J6" t="n">
-        <v>-1.907632432211151</v>
+        <v>-2.012412455401493</v>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
-        <v>0.301105328440335</v>
+        <v>0.3018128905830701</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2981364799652667</v>
+        <v>0.2996301905837089</v>
       </c>
       <c r="N6" t="n">
-        <v>0.3405488137280514</v>
+        <v>0.358928187961907</v>
       </c>
       <c r="O6" t="n">
-        <v>0.382841993754096</v>
+        <v>0.4112113896333193</v>
       </c>
       <c r="P6" t="n">
-        <v>0.1702744068640257</v>
+        <v>0.1794640939809535</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.191420996877048</v>
+        <v>0.2056056948166596</v>
       </c>
       <c r="R6" t="n">
-        <v>40.39317361400104</v>
+        <v>39.33342189079472</v>
       </c>
       <c r="S6" t="n">
-        <v>40.06801072794364</v>
+        <v>38.28760996860306</v>
       </c>
       <c r="T6" t="n">
-        <v>2.600000000000001</v>
+        <v>1.9</v>
       </c>
       <c r="U6" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="V6" t="n">
-        <v>0.06246024970436581</v>
+        <v>0.06980067426676839</v>
       </c>
       <c r="W6" t="n">
-        <v>0.05033506110055676</v>
+        <v>0.04796456102876087</v>
       </c>
       <c r="X6" t="n">
-        <v>10.5086666549021</v>
+        <v>11.14231402335541</v>
       </c>
       <c r="Y6" t="n">
-        <v>7.533112810843485</v>
+        <v>6.68311452600924</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.05059127289988442</v>
+        <v>0.05733790261104021</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.04069298037599399</v>
+        <v>0.04013653182772815</v>
       </c>
       <c r="AB6" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="AC6" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.05769587923256649</v>
+        <v>0.06381107785675695</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.04640755503489043</v>
+        <v>0.04466775449972986</v>
       </c>
       <c r="AF6" t="n">
-        <v>1.082577309422647</v>
+        <v>1.093864523389761</v>
       </c>
       <c r="AG6" t="n">
-        <v>1.08463074735813</v>
+        <v>1.073807303858334</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.206443273556618</v>
+        <v>0.2346613084744031</v>
       </c>
       <c r="AI6" t="n">
-        <v>-2.288423131604675</v>
+        <v>-2.315481740354166</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.3259683221318029</v>
+        <v>0.323357043621327</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.2712780193320478</v>
+        <v>0.2780209936980219</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.2918360656262429</v>
+        <v>0.3103510664937243</v>
       </c>
       <c r="AM6" t="n">
-        <v>0.616157943408675</v>
+        <v>0.6003567640730721</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.09897917255068914</v>
+        <v>0.1049584325580039</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.1740794931283701</v>
+        <v>0.1729617919774725</v>
       </c>
       <c r="AP6" t="n">
-        <v>0.1459180328131215</v>
+        <v>0.1551755332468621</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0.3080789717043375</v>
+        <v>0.3001783820365361</v>
       </c>
       <c r="AR6" t="n">
-        <v>30.67928912767725</v>
+        <v>31.19248913774425</v>
       </c>
       <c r="AS6" t="n">
-        <v>43.56159458442018</v>
+        <v>41.12059868663862</v>
       </c>
       <c r="AT6" t="n">
-        <v>0.03011835922214425</v>
+        <v>0.04000296114618677</v>
       </c>
       <c r="AU6" t="n">
-        <v>0.03403198700407719</v>
+        <v>0.03502390729585054</v>
       </c>
       <c r="AV6" t="n">
-        <v>2.073826440666212</v>
+        <v>1.744887684981342</v>
       </c>
       <c r="AW6" t="n">
-        <v>1.479051490426533</v>
+        <v>1.369480584321998</v>
       </c>
       <c r="AX6" t="n">
-        <v>2.684566101665531</v>
+        <v>1.862219212453354</v>
       </c>
       <c r="AY6" t="n">
-        <v>-1.302371273933669</v>
+        <v>-1.576298539195006</v>
       </c>
       <c r="AZ6" t="n">
-        <v>0.2878252715628371</v>
+        <v>0.2920127510737035</v>
       </c>
       <c r="BA6" t="n">
-        <v>0.2712780193320478</v>
+        <v>0.2780209936980219</v>
       </c>
       <c r="BB6" t="n">
-        <v>0.09765384116005343</v>
+        <v>0.2043459560127115</v>
       </c>
       <c r="BC6" t="n">
-        <v>0.5643317467859383</v>
+        <v>0.5592443222309613</v>
       </c>
       <c r="BD6" t="n">
-        <v>0.0404766403036884</v>
+        <v>0.07882275352738675</v>
       </c>
       <c r="BE6" t="n">
-        <v>0.1861833048655924</v>
+        <v>0.1819521176839946</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.04882692058002672</v>
+        <v>0.1021729780063558</v>
       </c>
       <c r="BG6" t="n">
-        <v>0.2821658733929692</v>
+        <v>0.2796221611154807</v>
       </c>
       <c r="BH6" t="n">
-        <v>56.6593288084937</v>
+        <v>49.97588978525735</v>
       </c>
       <c r="BI6" t="n">
-        <v>44.52173334377983</v>
+        <v>41.83922566687674</v>
       </c>
       <c r="BJ6" t="n">
-        <v>36.64688542755982</v>
+        <v>19.57115394064573</v>
       </c>
       <c r="BK6" t="n">
-        <v>5.110466027404137</v>
+        <v>4.914091592980399</v>
       </c>
       <c r="BL6" t="n">
-        <v>0.01561506242609145</v>
+        <v>0.0174501685666921</v>
       </c>
       <c r="BM6" t="n">
-        <v>0.01258376527513919</v>
+        <v>0.01199114025719022</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.05218038122675305</v>
+        <v>0.05345153375920686</v>
       </c>
       <c r="BO6" t="n">
-        <v>0.03529392620768535</v>
+        <v>0.03199440931343411</v>
       </c>
       <c r="BP6" t="n">
-        <v>0.04047606343487728</v>
+        <v>0.04424191234172514</v>
       </c>
       <c r="BQ6" t="n">
-        <v>0.03240050063979077</v>
+        <v>0.02971928865428763</v>
       </c>
       <c r="BR6" t="n">
-        <v>0.03186922257798593</v>
+        <v>0.03615080754648143</v>
       </c>
       <c r="BS6" t="n">
-        <v>0.0346876007763172</v>
+        <v>0.03154370748566083</v>
       </c>
       <c r="BT6" t="n">
-        <v>-0.02378555024975349</v>
+        <v>-0.02622947858270684</v>
       </c>
       <c r="BU6" t="n">
-        <v>-0.02536680170512642</v>
+        <v>-0.02369808632938877</v>
       </c>
       <c r="BV6" t="n">
-        <v>0.004749978820756746</v>
+        <v>0.001513611854500646</v>
       </c>
       <c r="BW6" t="n">
-        <v>-0.00910566915851245</v>
+        <v>-0.009391772232274562</v>
       </c>
       <c r="BX6" t="n">
-        <v>0.0001135971375947464</v>
+        <v>-0.003682659000007582</v>
       </c>
       <c r="BY6" t="n">
-        <v>-0.01439697041618972</v>
+        <v>-0.01436216923662553</v>
       </c>
       <c r="BZ6" t="n">
-        <v>-0.02226988109245948</v>
+        <v>-0.02469727369418137</v>
       </c>
       <c r="CA6" t="n">
-        <v>-0.02287778298991028</v>
+        <v>-0.02197569805238161</v>
       </c>
       <c r="CB6" t="n">
-        <v>-0.003915734648662569</v>
+        <v>-0.004696581147643412</v>
       </c>
       <c r="CC6" t="n">
-        <v>-0.01324219003025232</v>
+        <v>-0.01221590462526304</v>
       </c>
       <c r="CD6" t="n">
-        <v>-0.008445820862046673</v>
+        <v>-0.009729718643576938</v>
       </c>
       <c r="CE6" t="n">
-        <v>-0.01817711539176237</v>
+        <v>-0.01693909301887539</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>53.86993869938699</v>
+        <v>53.48318483184832</v>
       </c>
       <c r="B7" t="n">
-        <v>17.31140569257632</v>
+        <v>17.1384383428834</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9161075610756108</v>
+        <v>0.9698259982599826</v>
       </c>
       <c r="D7" t="n">
-        <v>1.242058297748026</v>
+        <v>1.165437426353791</v>
       </c>
       <c r="E7" t="n">
-        <v>55.18490184901849</v>
+        <v>54.37569375693757</v>
       </c>
       <c r="F7" t="n">
-        <v>17.89975546460377</v>
+        <v>17.53763370054599</v>
       </c>
       <c r="G7" t="n">
-        <v>0.859220792207922</v>
+        <v>0.9337750377503775</v>
       </c>
       <c r="H7" t="n">
-        <v>1.218644224422509</v>
+        <v>1.164040719255348</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6051457443700653</v>
+        <v>0.4135935658844764</v>
       </c>
       <c r="J7" t="n">
-        <v>-1.953389438943727</v>
+        <v>-2.089898201861629</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
-        <v>0.3022605163655339</v>
+        <v>0.3030330710459859</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2996297694692405</v>
+        <v>0.3012485544041718</v>
       </c>
       <c r="N7" t="n">
-        <v>0.3653101756090399</v>
+        <v>0.3932664755724555</v>
       </c>
       <c r="O7" t="n">
-        <v>0.4152257139917249</v>
+        <v>0.4471428201622599</v>
       </c>
       <c r="P7" t="n">
-        <v>0.18265508780452</v>
+        <v>0.1966332377862277</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.2076128569958625</v>
+        <v>0.2235714100811299</v>
       </c>
       <c r="R7" t="n">
-        <v>38.79835109699712</v>
+        <v>37.47250943835508</v>
       </c>
       <c r="S7" t="n">
-        <v>38.05938288014368</v>
+        <v>36.13325278834031</v>
       </c>
       <c r="T7" t="n">
-        <v>2.500000000000001</v>
+        <v>1.8</v>
       </c>
       <c r="U7" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="V7" t="n">
-        <v>0.05741543108210496</v>
+        <v>0.06395794842486846</v>
       </c>
       <c r="W7" t="n">
-        <v>0.04811784881460569</v>
+        <v>0.0454540009599275</v>
       </c>
       <c r="X7" t="n">
-        <v>9.005135010387244</v>
+        <v>9.318179738409766</v>
       </c>
       <c r="Y7" t="n">
-        <v>6.639655485049369</v>
+        <v>5.824378494947632</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.0462260355944683</v>
+        <v>0.05487892097730936</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.03948473873694167</v>
+        <v>0.0390484630030855</v>
       </c>
       <c r="AB7" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="AC7" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.05206701296597464</v>
+        <v>0.06036183040504035</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.04447390690843667</v>
+        <v>0.04294976394204794</v>
       </c>
       <c r="AF7" t="n">
-        <v>1.102721815818885</v>
+        <v>1.05957602669928</v>
       </c>
       <c r="AG7" t="n">
-        <v>1.081934378143823</v>
+        <v>1.058306188161093</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.2568045395472118</v>
+        <v>0.1489400667482005</v>
       </c>
       <c r="AI7" t="n">
-        <v>-2.295164054640443</v>
+        <v>-2.354234529597268</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.3258923112061414</v>
+        <v>0.3232570383862633</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.2753119209400757</v>
+        <v>0.2824179838032992</v>
       </c>
       <c r="AL7" t="n">
-        <v>0.3068333320674511</v>
+        <v>0.3351190207521428</v>
       </c>
       <c r="AM7" t="n">
-        <v>0.6278752788436067</v>
+        <v>0.6127960838682518</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.1050049164886342</v>
+        <v>0.1115098238674079</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.17980379794886</v>
+        <v>0.178038528953999</v>
       </c>
       <c r="AP7" t="n">
-        <v>0.1534166660337255</v>
+        <v>0.1675595103760714</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0.3139376394218034</v>
+        <v>0.3063980419341259</v>
       </c>
       <c r="AR7" t="n">
-        <v>30.0829048410905</v>
+        <v>30.3679449448747</v>
       </c>
       <c r="AS7" t="n">
-        <v>41.20520690578345</v>
+        <v>38.62562843696337</v>
       </c>
       <c r="AT7" t="n">
-        <v>0.03006995241838535</v>
+        <v>0.04081190188404387</v>
       </c>
       <c r="AU7" t="n">
-        <v>0.03376626705084224</v>
+        <v>0.03471142035597266</v>
       </c>
       <c r="AV7" t="n">
-        <v>1.909395475032413</v>
+        <v>1.567139620363391</v>
       </c>
       <c r="AW7" t="n">
-        <v>1.425027194808183</v>
+        <v>1.309482599495713</v>
       </c>
       <c r="AX7" t="n">
-        <v>2.273488687581033</v>
+        <v>1.417849050908477</v>
       </c>
       <c r="AY7" t="n">
-        <v>-1.437432012979542</v>
+        <v>-1.726293501260717</v>
       </c>
       <c r="AZ7" t="n">
-        <v>0.290665469079911</v>
+        <v>0.294608132753876</v>
       </c>
       <c r="BA7" t="n">
-        <v>0.2753119209400757</v>
+        <v>0.2824179838032992</v>
       </c>
       <c r="BB7" t="n">
-        <v>0.1747825224469897</v>
+        <v>0.2731692930271788</v>
       </c>
       <c r="BC7" t="n">
-        <v>0.5806269570148747</v>
+        <v>0.5756849101511206</v>
       </c>
       <c r="BD7" t="n">
-        <v>0.0702003678961831</v>
+        <v>0.100746613225767</v>
       </c>
       <c r="BE7" t="n">
-        <v>0.1908243483490867</v>
+        <v>0.1860488800495158</v>
       </c>
       <c r="BF7" t="n">
-        <v>0.08739126122349483</v>
+        <v>0.1365846465135894</v>
       </c>
       <c r="BG7" t="n">
-        <v>0.2903134785074373</v>
+        <v>0.2878424550755603</v>
       </c>
       <c r="BH7" t="n">
-        <v>51.84687849442006</v>
+        <v>45.86444111702144</v>
       </c>
       <c r="BI7" t="n">
-        <v>42.03931478652999</v>
+        <v>39.23501387844136</v>
       </c>
       <c r="BJ7" t="n">
-        <v>18.8214651522562</v>
+        <v>13.41484594118216</v>
       </c>
       <c r="BK7" t="n">
-        <v>4.748249146754945</v>
+        <v>4.523886810275879</v>
       </c>
       <c r="BL7" t="n">
-        <v>0.01435385777052624</v>
+        <v>0.01598948710621712</v>
       </c>
       <c r="BM7" t="n">
-        <v>0.01202946220365142</v>
+        <v>0.01136350023998187</v>
       </c>
       <c r="BN7" t="n">
-        <v>0.04514934777977541</v>
+        <v>0.0459022526180675</v>
       </c>
       <c r="BO7" t="n">
-        <v>0.03222165429143534</v>
+        <v>0.02874978101379696</v>
       </c>
       <c r="BP7" t="n">
-        <v>0.03597544019597838</v>
+        <v>0.0389107819048984</v>
       </c>
       <c r="BQ7" t="n">
-        <v>0.0296635884631049</v>
+        <v>0.02680264218980146</v>
       </c>
       <c r="BR7" t="n">
-        <v>0.02877963309788323</v>
+        <v>0.03233401358859338</v>
       </c>
       <c r="BS7" t="n">
-        <v>0.03169800991464296</v>
+        <v>0.02837371051366916</v>
       </c>
       <c r="BT7" t="n">
-        <v>-0.02193715859326486</v>
+        <v>-0.02411485812882431</v>
       </c>
       <c r="BU7" t="n">
-        <v>-0.02321346453822819</v>
+        <v>-0.02168407538745187</v>
       </c>
       <c r="BV7" t="n">
-        <v>0.004950522426444197</v>
+        <v>0.001991410644251035</v>
       </c>
       <c r="BW7" t="n">
-        <v>-0.007529509109591303</v>
+        <v>-0.007826865984237201</v>
       </c>
       <c r="BX7" t="n">
-        <v>-0.0003385537655126942</v>
+        <v>-0.003936374068416118</v>
       </c>
       <c r="BY7" t="n">
-        <v>-0.01356570229189304</v>
+        <v>-0.01349697907172495</v>
       </c>
       <c r="BZ7" t="n">
-        <v>-0.02040389572473228</v>
+        <v>-0.02262477933347893</v>
       </c>
       <c r="CA7" t="n">
-        <v>-0.02093411350048825</v>
+        <v>-0.02010767303653961</v>
       </c>
       <c r="CB7" t="n">
-        <v>-0.002960436391297258</v>
+        <v>-0.00359982317809619</v>
       </c>
       <c r="CC7" t="n">
-        <v>-0.0112985283060698</v>
+        <v>-0.01040086809235825</v>
       </c>
       <c r="CD7" t="n">
-        <v>-0.008128253188118929</v>
+        <v>-0.00934150915646696</v>
       </c>
       <c r="CE7" t="n">
-        <v>-0.01692817616992836</v>
+        <v>-0.01578897135691602</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>53.32933329333294</v>
+        <v>52.87627876278763</v>
       </c>
       <c r="B8" t="n">
-        <v>17.06963576463708</v>
+        <v>16.86703301445201</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9927919279192792</v>
+        <v>1.05270382703827</v>
       </c>
       <c r="D8" t="n">
-        <v>1.218415959707605</v>
+        <v>1.146317521157504</v>
       </c>
       <c r="E8" t="n">
-        <v>54.43944439444394</v>
+        <v>53.53418534185342</v>
       </c>
       <c r="F8" t="n">
-        <v>17.56615427257209</v>
+        <v>17.16124622760632</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9479161791617916</v>
+        <v>1.0280015800158</v>
       </c>
       <c r="H8" t="n">
-        <v>1.191787905311847</v>
+        <v>1.165410083416179</v>
       </c>
       <c r="I8" t="n">
-        <v>0.5460398992690135</v>
+        <v>0.3657938028937596</v>
       </c>
       <c r="J8" t="n">
-        <v>-2.020530236720382</v>
+        <v>-2.086474791459553</v>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
-        <v>0.3033407810275106</v>
+        <v>0.3042473633251507</v>
       </c>
       <c r="M8" t="n">
-        <v>0.3011203181782858</v>
+        <v>0.3029324564797469</v>
       </c>
       <c r="N8" t="n">
-        <v>0.3947160580853748</v>
+        <v>0.4240047443827742</v>
       </c>
       <c r="O8" t="n">
-        <v>0.450010112160144</v>
+        <v>0.4786319094543319</v>
       </c>
       <c r="P8" t="n">
-        <v>0.1973580290426874</v>
+        <v>0.2120023721913871</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.225005056080072</v>
+        <v>0.239315954727166</v>
       </c>
       <c r="R8" t="n">
-        <v>37.12639334258617</v>
+        <v>35.69811256907244</v>
       </c>
       <c r="S8" t="n">
-        <v>35.99306314365209</v>
+        <v>34.04489055790832</v>
       </c>
       <c r="T8" t="n">
-        <v>2.400000000000001</v>
+        <v>1.7</v>
       </c>
       <c r="U8" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="V8" t="n">
-        <v>0.05195021090798905</v>
+        <v>0.05742784307215678</v>
       </c>
       <c r="W8" t="n">
-        <v>0.04573337150644272</v>
+        <v>0.04274567461434009</v>
       </c>
       <c r="X8" t="n">
-        <v>7.54094913271603</v>
+        <v>7.760244634706289</v>
       </c>
       <c r="Y8" t="n">
-        <v>5.822837830809024</v>
+        <v>5.11698827599242</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.0426375003495982</v>
+        <v>0.05009767539291254</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.03837375031463838</v>
+        <v>0.03667865519838239</v>
       </c>
       <c r="AB8" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="AC8" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.04743883403566578</v>
+        <v>0.05447287134113397</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.0426949506320992</v>
+        <v>0.03988192366047309</v>
       </c>
       <c r="AF8" t="n">
-        <v>1.095098814379196</v>
+        <v>1.054246667345979</v>
       </c>
       <c r="AG8" t="n">
-        <v>1.071165813037834</v>
+        <v>1.071805737813627</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.2377470359479905</v>
+        <v>0.1356166683649473</v>
       </c>
       <c r="AI8" t="n">
-        <v>-2.322085467405415</v>
+        <v>-2.320485655465934</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.3256692245303652</v>
+        <v>0.3230510312222958</v>
       </c>
       <c r="AK8" t="n">
-        <v>0.2799785999487803</v>
+        <v>0.2874184716703982</v>
       </c>
       <c r="AL8" t="n">
-        <v>0.3263044284596496</v>
+        <v>0.3569796019119958</v>
       </c>
       <c r="AM8" t="n">
-        <v>0.6352091686879894</v>
+        <v>0.61400621058755</v>
       </c>
       <c r="AN8" t="n">
-        <v>0.1112055192546483</v>
+        <v>0.1184092556419938</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.1840644626597201</v>
+        <v>0.1827029158544624</v>
       </c>
       <c r="AP8" t="n">
-        <v>0.1631522142298248</v>
+        <v>0.1784898009559979</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0.3176045843439947</v>
+        <v>0.307003105293775</v>
       </c>
       <c r="AR8" t="n">
-        <v>29.45096740821688</v>
+        <v>29.63480886447563</v>
       </c>
       <c r="AS8" t="n">
-        <v>38.77895705826994</v>
+        <v>36.18459693358399</v>
       </c>
       <c r="AT8" t="n">
-        <v>0.03003015126862804</v>
+        <v>0.03951163656835877</v>
       </c>
       <c r="AU8" t="n">
-        <v>0.03349971069939307</v>
+        <v>0.03316744879341556</v>
       </c>
       <c r="AV8" t="n">
-        <v>1.729935039063906</v>
+        <v>1.453441265911659</v>
       </c>
       <c r="AW8" t="n">
-        <v>1.365187058384695</v>
+        <v>1.288783918250173</v>
       </c>
       <c r="AX8" t="n">
-        <v>1.824837597659765</v>
+        <v>1.133603164779148</v>
       </c>
       <c r="AY8" t="n">
-        <v>-1.587032354038263</v>
+        <v>-1.778040204374567</v>
       </c>
       <c r="AZ8" t="n">
-        <v>0.2933260636734031</v>
+        <v>0.2971037363289566</v>
       </c>
       <c r="BA8" t="n">
-        <v>0.2799785999487803</v>
+        <v>0.2874184716703982</v>
       </c>
       <c r="BB8" t="n">
-        <v>0.2498415961746794</v>
+        <v>0.3348930312282813</v>
       </c>
       <c r="BC8" t="n">
-        <v>0.5925278058424351</v>
+        <v>0.581230308546366</v>
       </c>
       <c r="BD8" t="n">
-        <v>0.09638962654679871</v>
+        <v>0.1199535118183713</v>
       </c>
       <c r="BE8" t="n">
-        <v>0.1938338644374159</v>
+        <v>0.1896500591756478</v>
       </c>
       <c r="BF8" t="n">
-        <v>0.1249207980873397</v>
+        <v>0.1674465156141407</v>
       </c>
       <c r="BG8" t="n">
-        <v>0.2962639029212176</v>
+        <v>0.290615154273183</v>
       </c>
       <c r="BH8" t="n">
-        <v>47.33946282893898</v>
+        <v>42.15628134070876</v>
       </c>
       <c r="BI8" t="n">
-        <v>39.49266949021431</v>
+        <v>36.71065443365476</v>
       </c>
       <c r="BJ8" t="n">
-        <v>11.91366943547293</v>
+        <v>9.825160309660243</v>
       </c>
       <c r="BK8" t="n">
-        <v>4.422308659667107</v>
+        <v>4.213746622370513</v>
       </c>
       <c r="BL8" t="n">
-        <v>0.01298755272699726</v>
+        <v>0.01435696076803919</v>
       </c>
       <c r="BM8" t="n">
-        <v>0.01143334287661068</v>
+        <v>0.01068641865358502</v>
       </c>
       <c r="BN8" t="n">
-        <v>0.03820322441452783</v>
+        <v>0.03854299173146317</v>
       </c>
       <c r="BO8" t="n">
-        <v>0.02908548638913706</v>
+        <v>0.02555226276216753</v>
       </c>
       <c r="BP8" t="n">
-        <v>0.03135586576250416</v>
+        <v>0.03350997680924203</v>
       </c>
       <c r="BQ8" t="n">
-        <v>0.02687692159774306</v>
+        <v>0.02393083562823278</v>
       </c>
       <c r="BR8" t="n">
-        <v>0.02554280420184993</v>
+        <v>0.02839634665716753</v>
       </c>
       <c r="BS8" t="n">
-        <v>0.02864361286284896</v>
+        <v>0.02523656359666101</v>
       </c>
       <c r="BT8" t="n">
-        <v>-0.01822211990856982</v>
+        <v>-0.01989284985619742</v>
       </c>
       <c r="BU8" t="n">
-        <v>-0.01896241450890249</v>
+        <v>-0.01771042926372345</v>
       </c>
       <c r="BV8" t="n">
-        <v>0.005159318978009496</v>
+        <v>0.002743466782374377</v>
       </c>
       <c r="BW8" t="n">
-        <v>-0.004641656182525272</v>
+        <v>-0.004949804610491677</v>
       </c>
       <c r="BX8" t="n">
-        <v>-0.001082541152072559</v>
+        <v>-0.004252159999099484</v>
       </c>
       <c r="BY8" t="n">
-        <v>-0.01176522033525584</v>
+        <v>-0.01164134232508715</v>
       </c>
       <c r="BZ8" t="n">
-        <v>-0.0167061725017451</v>
+        <v>-0.01851928324003799</v>
       </c>
       <c r="CA8" t="n">
-        <v>-0.01710753955389204</v>
+        <v>-0.01642924602092173</v>
       </c>
       <c r="CB8" t="n">
-        <v>-0.001255767069389537</v>
+        <v>-0.001636957783799632</v>
       </c>
       <c r="CC8" t="n">
-        <v>-0.00768177451602012</v>
+        <v>-0.007027514307615145</v>
       </c>
       <c r="CD8" t="n">
-        <v>-0.007354523913298234</v>
+        <v>-0.008412961661820173</v>
       </c>
       <c r="CE8" t="n">
-        <v>-0.01432555752698511</v>
+        <v>-0.01338624042975992</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>52.79637796377963</v>
+        <v>52.24217242172422</v>
       </c>
       <c r="B9" t="n">
-        <v>16.83130141101201</v>
+        <v>16.58344155447169</v>
       </c>
       <c r="C9" t="n">
-        <v>1.071713817138171</v>
+        <v>1.136888368883689</v>
       </c>
       <c r="D9" t="n">
-        <v>1.160611286042853</v>
+        <v>1.132969949813204</v>
       </c>
       <c r="E9" t="n">
-        <v>53.66168661686616</v>
+        <v>52.62552625526256</v>
       </c>
       <c r="F9" t="n">
-        <v>17.21826709079559</v>
+        <v>16.75489488904788</v>
       </c>
       <c r="G9" t="n">
-        <v>1.039923099230992</v>
+        <v>1.12419714197142</v>
       </c>
       <c r="H9" t="n">
-        <v>1.196826943389362</v>
+        <v>1.146622940113251</v>
       </c>
       <c r="I9" t="n">
-        <v>0.4015282151071314</v>
+        <v>0.3324248745330105</v>
       </c>
       <c r="J9" t="n">
-        <v>-2.007932641526595</v>
+        <v>-2.133442649716872</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
-        <v>0.3044073355297512</v>
+        <v>0.3055150624609416</v>
       </c>
       <c r="M9" t="n">
-        <v>0.3026769599727747</v>
+        <v>0.3047490474010108</v>
       </c>
       <c r="N9" t="n">
-        <v>0.4290507988180742</v>
+        <v>0.4533875879227014</v>
       </c>
       <c r="O9" t="n">
-        <v>0.4804958028437142</v>
+        <v>0.5115789341276044</v>
       </c>
       <c r="P9" t="n">
-        <v>0.2145253994090371</v>
+        <v>0.2266937939613507</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.2402479014218571</v>
+        <v>0.2557894670638022</v>
       </c>
       <c r="R9" t="n">
-        <v>35.37419021270129</v>
+        <v>33.94813538194801</v>
       </c>
       <c r="S9" t="n">
-        <v>33.9882453241072</v>
+        <v>31.91189708010511</v>
       </c>
       <c r="T9" t="n">
-        <v>2.300000000000001</v>
+        <v>1.6</v>
       </c>
       <c r="U9" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="V9" t="n">
-        <v>0.04600975419699348</v>
+        <v>0.05008147455035611</v>
       </c>
       <c r="W9" t="n">
-        <v>0.04305234397454302</v>
+        <v>0.03970324010460867</v>
       </c>
       <c r="X9" t="n">
-        <v>6.144192945273719</v>
+        <v>6.328943902613379</v>
       </c>
       <c r="Y9" t="n">
-        <v>5.133707353325343</v>
+        <v>4.446695310720652</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.03964269066679978</v>
+        <v>0.04420370951463733</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.03597207116061461</v>
+        <v>0.03462623911979924</v>
       </c>
       <c r="AB9" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="AC9" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.04356627615520327</v>
+        <v>0.04751888776567006</v>
       </c>
       <c r="AE9" t="n">
-        <v>0.03953236169638815</v>
+        <v>0.03722312874977488</v>
       </c>
       <c r="AF9" t="n">
-        <v>1.056086456255417</v>
+        <v>1.053927751788361</v>
       </c>
       <c r="AG9" t="n">
-        <v>1.089040525966767</v>
+        <v>1.066628234598597</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.1402161406385416</v>
+        <v>0.1348193794709029</v>
       </c>
       <c r="AI9" t="n">
-        <v>-2.277398685083083</v>
+        <v>-2.333429413503507</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.3252866773883619</v>
+        <v>0.3227348281599319</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.2852996322390131</v>
+        <v>0.2930447408362419</v>
       </c>
       <c r="AL9" t="n">
-        <v>0.3512902602852533</v>
+        <v>0.3789438236241698</v>
       </c>
       <c r="AM9" t="n">
-        <v>0.6310628418511631</v>
+        <v>0.6111630122576944</v>
       </c>
       <c r="AN9" t="n">
-        <v>0.1174308276773816</v>
+        <v>0.1255527091495957</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.1878866146403194</v>
+        <v>0.1849683967517839</v>
       </c>
       <c r="AP9" t="n">
-        <v>0.1756451301426266</v>
+        <v>0.1894719118120849</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.3155314209255816</v>
+        <v>0.3055815061288472</v>
       </c>
       <c r="AR9" t="n">
-        <v>28.77582304739979</v>
+        <v>28.93572964698342</v>
       </c>
       <c r="AS9" t="n">
-        <v>36.39342684459161</v>
+        <v>33.70204707950448</v>
       </c>
       <c r="AT9" t="n">
-        <v>0.02999684826576988</v>
+        <v>0.03680667721054885</v>
       </c>
       <c r="AU9" t="n">
-        <v>0.03201831016581897</v>
+        <v>0.03181810109419971</v>
       </c>
       <c r="AV9" t="n">
-        <v>1.533819612959016</v>
+        <v>1.360662747790846</v>
       </c>
       <c r="AW9" t="n">
-        <v>1.344616369557922</v>
+        <v>1.247819283340148</v>
       </c>
       <c r="AX9" t="n">
-        <v>1.334549032397539</v>
+        <v>0.9016568694771154</v>
       </c>
       <c r="AY9" t="n">
-        <v>-1.638459076105195</v>
+        <v>-1.880451791649629</v>
       </c>
       <c r="AZ9" t="n">
-        <v>0.2958972494520846</v>
+        <v>0.299579042801456</v>
       </c>
       <c r="BA9" t="n">
-        <v>0.2852996322390131</v>
+        <v>0.2930447408362419</v>
       </c>
       <c r="BB9" t="n">
-        <v>0.3230020195306361</v>
+        <v>0.3913960639445379</v>
       </c>
       <c r="BC9" t="n">
-        <v>0.5933804057178184</v>
+        <v>0.5827083999874485</v>
       </c>
       <c r="BD9" t="n">
-        <v>0.1183677273439352</v>
+        <v>0.1367738683324493</v>
       </c>
       <c r="BE9" t="n">
-        <v>0.196306016394569</v>
+        <v>0.1907484671793578</v>
       </c>
       <c r="BF9" t="n">
-        <v>0.161501009765318</v>
+        <v>0.1956980319722689</v>
       </c>
       <c r="BG9" t="n">
-        <v>0.2966902028589092</v>
+        <v>0.2913541999937242</v>
       </c>
       <c r="BH9" t="n">
-        <v>43.12784622245556</v>
+        <v>38.7402078659939</v>
       </c>
       <c r="BI9" t="n">
-        <v>37.01352523550283</v>
+        <v>34.14079739522325</v>
       </c>
       <c r="BJ9" t="n">
-        <v>8.16146049665082</v>
+        <v>7.331352987738656</v>
       </c>
       <c r="BK9" t="n">
-        <v>4.157078002409932</v>
+        <v>3.903904414062849</v>
       </c>
       <c r="BL9" t="n">
-        <v>0.01150243854924837</v>
+        <v>0.01252036863758903</v>
       </c>
       <c r="BM9" t="n">
-        <v>0.01076308599363575</v>
+        <v>0.009925810026152167</v>
       </c>
       <c r="BN9" t="n">
-        <v>0.03145358190977478</v>
+        <v>0.03134049481839025</v>
       </c>
       <c r="BO9" t="n">
-        <v>0.02591766314192321</v>
+        <v>0.02228258877003633</v>
       </c>
       <c r="BP9" t="n">
-        <v>0.02663568745548795</v>
+        <v>0.0279676099658938</v>
       </c>
       <c r="BQ9" t="n">
-        <v>0.02406724222746321</v>
+        <v>0.02098771264639267</v>
       </c>
       <c r="BR9" t="n">
-        <v>0.02214835299703139</v>
+        <v>0.02423083113304251</v>
       </c>
       <c r="BS9" t="n">
-        <v>0.02554409840569221</v>
+        <v>0.02203030166014159</v>
       </c>
       <c r="BT9" t="n">
-        <v>-0.0144885769843099</v>
+        <v>-0.01567831672982289</v>
       </c>
       <c r="BU9" t="n">
-        <v>-0.01476216961707945</v>
+        <v>-0.01378571248240011</v>
       </c>
       <c r="BV9" t="n">
-        <v>0.005163005897729704</v>
+        <v>0.003281590921554414</v>
       </c>
       <c r="BW9" t="n">
-        <v>-0.002047345690203576</v>
+        <v>-0.002354125795174246</v>
       </c>
       <c r="BX9" t="n">
-        <v>-0.001664028619547709</v>
+        <v>-0.00436987587068262</v>
       </c>
       <c r="BY9" t="n">
-        <v>-0.00983874398225263</v>
+        <v>-0.009672995170513045</v>
       </c>
       <c r="BZ9" t="n">
-        <v>-0.01304176511527865</v>
+        <v>-0.01445203711680873</v>
       </c>
       <c r="CA9" t="n">
-        <v>-0.01333115247966061</v>
+        <v>-0.01279899079310491</v>
       </c>
       <c r="CB9" t="n">
-        <v>0.0002245442505444473</v>
+        <v>7.418178537552198e-05</v>
       </c>
       <c r="CC9" t="n">
-        <v>-0.004369794505968703</v>
+        <v>-0.003942975044175599</v>
       </c>
       <c r="CD9" t="n">
-        <v>-0.00644597104748069</v>
+        <v>-0.007337072456209444</v>
       </c>
       <c r="CE9" t="n">
-        <v>-0.01163643217421166</v>
+        <v>-0.01089783174027144</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>52.24982249822499</v>
+        <v>51.55706557065571</v>
       </c>
       <c r="B10" t="n">
-        <v>16.58686326801209</v>
+        <v>16.27694594702777</v>
       </c>
       <c r="C10" t="n">
-        <v>1.152139321393214</v>
+        <v>1.221627816278163</v>
       </c>
       <c r="D10" t="n">
-        <v>1.145589697774146</v>
+        <v>1.132626605955138</v>
       </c>
       <c r="E10" t="n">
-        <v>52.82442824428244</v>
+        <v>51.619966199662</v>
       </c>
       <c r="F10" t="n">
-        <v>16.84384553128256</v>
+        <v>16.30509190018539</v>
       </c>
       <c r="G10" t="n">
-        <v>1.133952739527395</v>
+        <v>1.221287712877129</v>
       </c>
       <c r="H10" t="n">
-        <v>1.1787111173992</v>
+        <v>1.13681283173414</v>
       </c>
       <c r="I10" t="n">
-        <v>0.3639742444353639</v>
+        <v>0.3315665148878455</v>
       </c>
       <c r="J10" t="n">
-        <v>-2.053222206502001</v>
+        <v>-2.157967920664649</v>
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
-        <v>0.3055000331116358</v>
+        <v>0.3068865758055554</v>
       </c>
       <c r="M10" t="n">
-        <v>0.3043516411954972</v>
+        <v>0.3067603790283607</v>
       </c>
       <c r="N10" t="n">
-        <v>0.457874147785971</v>
+        <v>0.4795377968307512</v>
       </c>
       <c r="O10" t="n">
-        <v>0.513005877734807</v>
+        <v>0.5408096523449138</v>
       </c>
       <c r="P10" t="n">
-        <v>0.2289370738929855</v>
+        <v>0.2397688984153756</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2565029388674035</v>
+        <v>0.2704048261724569</v>
       </c>
       <c r="R10" t="n">
-        <v>33.73265795644888</v>
+        <v>32.24381274424297</v>
       </c>
       <c r="S10" t="n">
-        <v>31.9274156360846</v>
+        <v>29.81911500434607</v>
       </c>
       <c r="T10" t="n">
-        <v>2.200000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="U10" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="V10" t="n">
-        <v>0.03952925596681648</v>
+        <v>0.0417555902256487</v>
       </c>
       <c r="W10" t="n">
-        <v>0.03997088668477335</v>
+        <v>0.03619493115286361</v>
       </c>
       <c r="X10" t="n">
-        <v>4.946480537978068</v>
+        <v>4.989025035319954</v>
       </c>
       <c r="Y10" t="n">
-        <v>4.46421933885594</v>
+        <v>3.834666197790785</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.03450559658804624</v>
+        <v>0.0368661569542033</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.033910672508942</v>
+        <v>0.03183895373317558</v>
       </c>
       <c r="AB10" t="n">
         <v>57</v>
       </c>
       <c r="AC10" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.03745171108078877</v>
+        <v>0.03918224078923672</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.03680599192422345</v>
+        <v>0.0338392079543408</v>
       </c>
       <c r="AF10" t="n">
-        <v>1.055472629315818</v>
+        <v>1.065676423414734</v>
       </c>
       <c r="AG10" t="n">
-        <v>1.085988574008977</v>
+        <v>1.069615199082123</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.1386815732895452</v>
+        <v>0.1641910585368361</v>
       </c>
       <c r="AI10" t="n">
-        <v>-2.285028564977558</v>
+        <v>-2.325962002294691</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.3247291395463486</v>
+        <v>0.3223054666341844</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.2912793316098631</v>
+        <v>0.2993002966190627</v>
       </c>
       <c r="AL10" t="n">
-        <v>0.3724104997574471</v>
+        <v>0.3998730226111253</v>
       </c>
       <c r="AM10" t="n">
-        <v>0.6230774982541682</v>
+        <v>0.5989875099944068</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.124241494408256</v>
+        <v>0.1330461941971205</v>
       </c>
       <c r="AO10" t="n">
-        <v>0.1891317168130878</v>
+        <v>0.1854123663402281</v>
       </c>
       <c r="AP10" t="n">
-        <v>0.1862052498787236</v>
+        <v>0.1999365113055626</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.3115387491270841</v>
+        <v>0.2994937549972034</v>
       </c>
       <c r="AR10" t="n">
-        <v>28.22847012139814</v>
+        <v>28.2893561625286</v>
       </c>
       <c r="AS10" t="n">
-        <v>33.95058109956111</v>
+        <v>31.26182173763126</v>
       </c>
       <c r="AT10" t="n">
-        <v>0.02786551443784538</v>
+        <v>0.03227807997348915</v>
       </c>
       <c r="AU10" t="n">
-        <v>0.03074388359481325</v>
+        <v>0.02970430868863082</v>
       </c>
       <c r="AV10" t="n">
-        <v>1.418572625134459</v>
+        <v>1.293620632328307</v>
       </c>
       <c r="AW10" t="n">
-        <v>1.300124838213893</v>
+        <v>1.218507777180388</v>
       </c>
       <c r="AX10" t="n">
-        <v>1.046431562836147</v>
+        <v>0.7340515808207676</v>
       </c>
       <c r="AY10" t="n">
-        <v>-1.749687904465267</v>
+        <v>-1.953730557049031</v>
       </c>
       <c r="AZ10" t="n">
-        <v>0.2984252504044027</v>
+        <v>0.3020909267446344</v>
       </c>
       <c r="BA10" t="n">
-        <v>0.291279331609863</v>
+        <v>0.2993002966190627</v>
       </c>
       <c r="BB10" t="n">
-        <v>0.3852946276159027</v>
+        <v>0.4410138577094522</v>
       </c>
       <c r="BC10" t="n">
-        <v>0.5903991336056188</v>
+        <v>0.5750702554717844</v>
       </c>
       <c r="BD10" t="n">
-        <v>0.1369475628295694</v>
+        <v>0.1515281721869352</v>
       </c>
       <c r="BE10" t="n">
-        <v>0.1960865965241824</v>
+        <v>0.1899950144359695</v>
       </c>
       <c r="BF10" t="n">
-        <v>0.1926473138079514</v>
+        <v>0.2205069288547261</v>
       </c>
       <c r="BG10" t="n">
-        <v>0.2951995668028094</v>
+        <v>0.2875351277358922</v>
       </c>
       <c r="BH10" t="n">
-        <v>39.43554253770483</v>
+        <v>35.61814836726003</v>
       </c>
       <c r="BI10" t="n">
-        <v>34.46958257774912</v>
+        <v>31.62209455561561</v>
       </c>
       <c r="BJ10" t="n">
-        <v>5.87826468197291</v>
+        <v>5.424829526517995</v>
       </c>
       <c r="BK10" t="n">
-        <v>3.879025412218591</v>
+        <v>3.606212423363169</v>
       </c>
       <c r="BL10" t="n">
-        <v>0.00988231399170412</v>
+        <v>0.01043889755641218</v>
       </c>
       <c r="BM10" t="n">
-        <v>0.009992721671193337</v>
+        <v>0.009048732788215903</v>
       </c>
       <c r="BN10" t="n">
-        <v>0.02510936857073795</v>
+        <v>0.02431764107959863</v>
       </c>
       <c r="BO10" t="n">
-        <v>0.02262226843980155</v>
+        <v>0.01897752043537419</v>
       </c>
       <c r="BP10" t="n">
-        <v>0.02195132878504805</v>
+        <v>0.02227757546207935</v>
       </c>
       <c r="BQ10" t="n">
-        <v>0.0211383836361574</v>
+        <v>0.0179984158695632</v>
       </c>
       <c r="BR10" t="n">
-        <v>0.01869688838230594</v>
+        <v>0.019789002839435</v>
       </c>
       <c r="BS10" t="n">
-        <v>0.02232284614362525</v>
+        <v>0.01878334647649972</v>
       </c>
       <c r="BT10" t="n">
-        <v>-0.01074447326061525</v>
+        <v>-0.01146830764878171</v>
       </c>
       <c r="BU10" t="n">
-        <v>-0.01058086380550657</v>
+        <v>-0.009877753811690915</v>
       </c>
       <c r="BV10" t="n">
-        <v>0.005031367330393595</v>
+        <v>0.003683979920929735</v>
       </c>
       <c r="BW10" t="n">
-        <v>0.0003336487722948069</v>
+        <v>3.565740570789233e-05</v>
       </c>
       <c r="BX10" t="n">
-        <v>-0.002152773607787418</v>
+        <v>-0.00436771744197816</v>
       </c>
       <c r="BY10" t="n">
-        <v>-0.00786529958426143</v>
+        <v>-0.007666045136956321</v>
       </c>
       <c r="BZ10" t="n">
-        <v>-0.009393859643506558</v>
+        <v>-0.01040342108122155</v>
       </c>
       <c r="CA10" t="n">
-        <v>-0.009562721319563268</v>
+        <v>-0.009177675042699229</v>
       </c>
       <c r="CB10" t="n">
-        <v>0.001548796853391142</v>
+        <v>0.001609501071360295</v>
       </c>
       <c r="CC10" t="n">
-        <v>-0.001286854560478048</v>
+        <v>-0.001074874203591695</v>
       </c>
       <c r="CD10" t="n">
-        <v>-0.005470637706376848</v>
+        <v>-0.006189418776707579</v>
       </c>
       <c r="CE10" t="n">
-        <v>-0.008933593275982947</v>
+        <v>-0.008393523403791014</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>51.67436674366743</v>
+        <v>50.7980079800798</v>
       </c>
       <c r="B11" t="n">
-        <v>16.32943318866563</v>
+        <v>15.93715581087307</v>
       </c>
       <c r="C11" t="n">
-        <v>1.233549335493355</v>
+        <v>1.30659996599966</v>
       </c>
       <c r="D11" t="n">
-        <v>1.156120230094621</v>
+        <v>1.107336598538291</v>
       </c>
       <c r="E11" t="n">
-        <v>51.90386903869039</v>
+        <v>50.48775487754877</v>
       </c>
       <c r="F11" t="n">
-        <v>16.43211214370189</v>
+        <v>15.79818232696347</v>
       </c>
       <c r="G11" t="n">
-        <v>1.229092190921909</v>
+        <v>1.318682586825868</v>
       </c>
       <c r="H11" t="n">
-        <v>1.13265938343887</v>
+        <v>1.117062330807713</v>
       </c>
       <c r="I11" t="n">
-        <v>0.3903005752365529</v>
+        <v>0.2683414963457287</v>
       </c>
       <c r="J11" t="n">
-        <v>-2.168351541402824</v>
+        <v>-2.207344172980718</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>0.3066506859009309</v>
+        <v>0.3084042689634705</v>
       </c>
       <c r="M11" t="n">
-        <v>0.3061918749229294</v>
+        <v>0.3090242915738176</v>
       </c>
       <c r="N11" t="n">
-        <v>0.4823024245877988</v>
+        <v>0.5074876956603916</v>
       </c>
       <c r="O11" t="n">
-        <v>0.5480007802894514</v>
+        <v>0.5682845795127031</v>
       </c>
       <c r="P11" t="n">
-        <v>0.2411512122938994</v>
+        <v>0.2537438478301958</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2740003901447257</v>
+        <v>0.2841422897563515</v>
       </c>
       <c r="R11" t="n">
-        <v>32.16297277546646</v>
+        <v>30.49645456396367</v>
       </c>
       <c r="S11" t="n">
-        <v>29.81325963152542</v>
+        <v>27.73180847627293</v>
       </c>
       <c r="T11" t="n">
-        <v>2.100000000000001</v>
+        <v>1.4</v>
       </c>
       <c r="U11" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="V11" t="n">
-        <v>0.0324315674290036</v>
+        <v>0.0322402938545545</v>
       </c>
       <c r="W11" t="n">
-        <v>0.0363857159299894</v>
+        <v>0.0320839539886808</v>
       </c>
       <c r="X11" t="n">
-        <v>3.852764008996989</v>
+        <v>3.639967672630804</v>
       </c>
       <c r="Y11" t="n">
-        <v>3.804293677225718</v>
+        <v>3.234792487743701</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.02805207156209807</v>
+        <v>0.02911517048846068</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.03212414646627359</v>
+        <v>0.02872172223861662</v>
       </c>
       <c r="AB11" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="AC11" t="n">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="AD11" t="n">
-        <v>0.03006686664232338</v>
+        <v>0.03059435239707525</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.03443141180008</v>
+        <v>0.03018091520252018</v>
       </c>
       <c r="AF11" t="n">
-        <v>1.078648061828683</v>
+        <v>1.053798865755256</v>
       </c>
       <c r="AG11" t="n">
-        <v>1.056759337701769</v>
+        <v>1.063054376363037</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.1966201545717078</v>
+        <v>0.1344971643881404</v>
       </c>
       <c r="AI11" t="n">
-        <v>-2.358101655745578</v>
+        <v>-2.342364059092406</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.323978722868547</v>
+        <v>0.3217617658612484</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.2978965808409578</v>
+        <v>0.3061617641109472</v>
       </c>
       <c r="AL11" t="n">
-        <v>0.3914262527658048</v>
+        <v>0.4250546433436606</v>
       </c>
       <c r="AM11" t="n">
-        <v>0.6118742466506846</v>
+        <v>0.580168085289523</v>
       </c>
       <c r="AN11" t="n">
-        <v>0.131706231355893</v>
+        <v>0.1403970766254894</v>
       </c>
       <c r="AO11" t="n">
-        <v>0.187376766413773</v>
+        <v>0.1831397117635581</v>
       </c>
       <c r="AP11" t="n">
-        <v>0.1957131263829024</v>
+        <v>0.2125273216718303</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.3059371233253423</v>
+        <v>0.2900840426447615</v>
       </c>
       <c r="AR11" t="n">
-        <v>27.77526954612507</v>
+        <v>27.61129426905793</v>
       </c>
       <c r="AS11" t="n">
-        <v>31.45909953228723</v>
+        <v>28.8387585302718</v>
       </c>
       <c r="AT11" t="n">
-        <v>0.02403976170269928</v>
+        <v>0.02670941490523244</v>
       </c>
       <c r="AU11" t="n">
-        <v>0.02963780447041426</v>
+        <v>0.02718431559268645</v>
       </c>
       <c r="AV11" t="n">
-        <v>1.349080237569994</v>
+        <v>1.207076005556323</v>
       </c>
       <c r="AW11" t="n">
-        <v>1.22767919487124</v>
+        <v>1.180237695493519</v>
       </c>
       <c r="AX11" t="n">
-        <v>0.872700593924986</v>
+        <v>0.517690013890808</v>
       </c>
       <c r="AY11" t="n">
-        <v>-1.930802012821901</v>
+        <v>-2.049405761266202</v>
       </c>
       <c r="AZ11" t="n">
-        <v>0.3009379475647944</v>
+        <v>0.3046789745696233</v>
       </c>
       <c r="BA11" t="n">
-        <v>0.2978965808409578</v>
+        <v>0.3061617641109472</v>
       </c>
       <c r="BB11" t="n">
-        <v>0.4380678125758646</v>
+        <v>0.4887623023636871</v>
       </c>
       <c r="BC11" t="n">
-        <v>0.5841599580950033</v>
+        <v>0.5608288468685019</v>
       </c>
       <c r="BD11" t="n">
-        <v>0.1531218575928276</v>
+        <v>0.1636091150959681</v>
       </c>
       <c r="BE11" t="n">
-        <v>0.1928145268596413</v>
+        <v>0.1865374503102971</v>
       </c>
       <c r="BF11" t="n">
-        <v>0.2190339062879323</v>
+        <v>0.2443811511818435</v>
       </c>
       <c r="BG11" t="n">
-        <v>0.2920799790475017</v>
+        <v>0.2804144234342509</v>
       </c>
       <c r="BH11" t="n">
-        <v>36.15374741201552</v>
+        <v>32.66684322498656</v>
       </c>
       <c r="BI11" t="n">
-        <v>31.87254203093307</v>
+        <v>29.12204720888749</v>
       </c>
       <c r="BJ11" t="n">
-        <v>4.241800948077484</v>
+        <v>3.779420712565006</v>
       </c>
       <c r="BK11" t="n">
-        <v>3.568811860388671</v>
+        <v>3.277795895402487</v>
       </c>
       <c r="BL11" t="n">
-        <v>0.008107891857250899</v>
+        <v>0.008060073463638625</v>
       </c>
       <c r="BM11" t="n">
-        <v>0.009096428982497351</v>
+        <v>0.008020988497170201</v>
       </c>
       <c r="BN11" t="n">
-        <v>0.01913313450431633</v>
+        <v>0.01740180345513065</v>
       </c>
       <c r="BO11" t="n">
-        <v>0.01921280123878312</v>
+        <v>0.01561434822108594</v>
       </c>
       <c r="BP11" t="n">
-        <v>0.01726427407567146</v>
+        <v>0.01636146697048647</v>
       </c>
       <c r="BQ11" t="n">
-        <v>0.01809005993667558</v>
+        <v>0.01492973897330453</v>
       </c>
       <c r="BR11" t="n">
-        <v>0.01511326567593507</v>
+        <v>0.01494243209295661</v>
       </c>
       <c r="BS11" t="n">
-        <v>0.01898933314764943</v>
+        <v>0.01547557821945856</v>
       </c>
       <c r="BT11" t="n">
-        <v>-0.006994335225418097</v>
+        <v>-0.007261140808606898</v>
       </c>
       <c r="BU11" t="n">
-        <v>-0.006400401441992176</v>
+        <v>-0.005968298650680107</v>
       </c>
       <c r="BV11" t="n">
-        <v>0.004804176412740136</v>
+        <v>0.003995197733883896</v>
       </c>
       <c r="BW11" t="n">
-        <v>0.00254720781938023</v>
+        <v>0.002262747660908318</v>
       </c>
       <c r="BX11" t="n">
-        <v>-0.002588526678826034</v>
+        <v>-0.004290247735424206</v>
       </c>
       <c r="BY11" t="n">
-        <v>-0.00588976347401003</v>
+        <v>-0.005662542319815694</v>
       </c>
       <c r="BZ11" t="n">
-        <v>-0.005752882585058473</v>
+        <v>-0.00636226550829627</v>
       </c>
       <c r="CA11" t="n">
-        <v>-0.00577839975703551</v>
+        <v>-0.00554313025847813</v>
       </c>
       <c r="CB11" t="n">
-        <v>0.002755948895993138</v>
+        <v>0.003012302749138648</v>
       </c>
       <c r="CC11" t="n">
-        <v>0.001610585966491807</v>
+        <v>0.001618372183190402</v>
       </c>
       <c r="CD11" t="n">
-        <v>-0.004467266241011224</v>
+        <v>-0.005013026843891929</v>
       </c>
       <c r="CE11" t="n">
-        <v>-0.006258144537119853</v>
+        <v>-0.005912744067724811</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>51.05811058110581</v>
+        <v>49.94544945449454</v>
       </c>
       <c r="B12" t="n">
-        <v>16.05362174798062</v>
+        <v>15.55510550409931</v>
       </c>
       <c r="C12" t="n">
-        <v>1.315639556395564</v>
+        <v>1.391679516795168</v>
       </c>
       <c r="D12" t="n">
-        <v>1.135330707305273</v>
+        <v>1.097855557873013</v>
       </c>
       <c r="E12" t="n">
-        <v>50.87875878758788</v>
+        <v>49.19999199992</v>
       </c>
       <c r="F12" t="n">
-        <v>15.97331751056624</v>
+        <v>15.22056748382437</v>
       </c>
       <c r="G12" t="n">
-        <v>1.324750747507475</v>
+        <v>1.416238562385624</v>
       </c>
       <c r="H12" t="n">
-        <v>1.116892394771442</v>
+        <v>1.113574975338442</v>
       </c>
       <c r="I12" t="n">
-        <v>0.3383267682631835</v>
+        <v>0.2446388946825329</v>
       </c>
       <c r="J12" t="n">
-        <v>-2.207769013071395</v>
+        <v>-2.216062561653895</v>
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
-        <v>0.307884515849925</v>
+        <v>0.3101091080320683</v>
       </c>
       <c r="M12" t="n">
-        <v>0.3082423340772001</v>
+        <v>0.3116003651206804</v>
       </c>
       <c r="N12" t="n">
-        <v>0.5101273927942181</v>
+        <v>0.5305893879082068</v>
       </c>
       <c r="O12" t="n">
-        <v>0.5757950802160927</v>
+        <v>0.5887487885570706</v>
       </c>
       <c r="P12" t="n">
-        <v>0.2550636963971091</v>
+        <v>0.2652946939541034</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.2878975401080464</v>
+        <v>0.2943743942785353</v>
       </c>
       <c r="R12" t="n">
-        <v>30.53020906418184</v>
+        <v>28.80773411960175</v>
       </c>
       <c r="S12" t="n">
-        <v>27.79836502850665</v>
+        <v>25.72209457356125</v>
       </c>
       <c r="T12" t="n">
-        <v>2.000000000000001</v>
+        <v>1.3</v>
       </c>
       <c r="U12" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="V12" t="n">
-        <v>0.02462411003740946</v>
+        <v>0.02126110573406127</v>
       </c>
       <c r="W12" t="n">
-        <v>0.03218358363804736</v>
+        <v>0.02720197341586789</v>
       </c>
       <c r="X12" t="n">
-        <v>2.765705702787438</v>
+        <v>2.295892090794215</v>
       </c>
       <c r="Y12" t="n">
-        <v>3.202513072784972</v>
+        <v>2.647249825987519</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.02168893158527809</v>
+        <v>0.01936603188059873</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.02881529482044089</v>
+        <v>0.02442760839484612</v>
       </c>
       <c r="AB12" t="n">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="AC12" t="n">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.02295427453338667</v>
+        <v>0.02012061013501345</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.03049639330864229</v>
+        <v>0.0253794059657556</v>
       </c>
       <c r="AF12" t="n">
-        <v>1.072746167673216</v>
+        <v>1.056682953021546</v>
       </c>
       <c r="AG12" t="n">
-        <v>1.055324257932067</v>
+        <v>1.071812849070284</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.181865419183041</v>
+        <v>0.1417073825538662</v>
       </c>
       <c r="AI12" t="n">
-        <v>-2.361689355169834</v>
+        <v>-2.320467877324289</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.3230141601888347</v>
+        <v>0.3211051539846675</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.3050978024555132</v>
+        <v>0.3131469769879968</v>
       </c>
       <c r="AL12" t="n">
-        <v>0.416217589808362</v>
+        <v>0.448606653189455</v>
       </c>
       <c r="AM12" t="n">
-        <v>0.5877965600682342</v>
+        <v>0.5553155812795485</v>
       </c>
       <c r="AN12" t="n">
-        <v>0.1392484844436202</v>
+        <v>0.1480762260451801</v>
       </c>
       <c r="AO12" t="n">
-        <v>0.1842294604561899</v>
+        <v>0.1800311113172217</v>
       </c>
       <c r="AP12" t="n">
-        <v>0.208108794904181</v>
+        <v>0.2243033265947275</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0.2938982800341171</v>
+        <v>0.2776577906397742</v>
       </c>
       <c r="AR12" t="n">
-        <v>27.2908317911367</v>
+        <v>26.99749191655454</v>
       </c>
       <c r="AS12" t="n">
-        <v>29.06894087365446</v>
+        <v>26.51083315967323</v>
       </c>
       <c r="AT12" t="n">
-        <v>0.0196270090196356</v>
+        <v>0.01855607223130679</v>
       </c>
       <c r="AU12" t="n">
-        <v>0.02702984325412289</v>
+        <v>0.02343718960560934</v>
       </c>
       <c r="AV12" t="n">
-        <v>1.254603287376827</v>
+        <v>1.145776189542456</v>
       </c>
       <c r="AW12" t="n">
-        <v>1.190668526467994</v>
+        <v>1.160632903245255</v>
       </c>
       <c r="AX12" t="n">
-        <v>0.6365082184420673</v>
+        <v>0.3644404738561396</v>
       </c>
       <c r="AY12" t="n">
-        <v>-2.023328683830014</v>
+        <v>-2.098417741886863</v>
       </c>
       <c r="AZ12" t="n">
-        <v>0.3034507227748294</v>
+        <v>0.3073774277821744</v>
       </c>
       <c r="BA12" t="n">
-        <v>0.3050978024555132</v>
+        <v>0.3131469769879969</v>
       </c>
       <c r="BB12" t="n">
-        <v>0.4891740038365265</v>
+        <v>0.528739714390285</v>
       </c>
       <c r="BC12" t="n">
-        <v>0.565410860115356</v>
+        <v>0.5406108429184538</v>
       </c>
       <c r="BD12" t="n">
-        <v>0.1662665005217774</v>
+        <v>0.1739657687450305</v>
       </c>
       <c r="BE12" t="n">
-        <v>0.1882342562596729</v>
+        <v>0.1823813452398087</v>
       </c>
       <c r="BF12" t="n">
-        <v>0.2445870019182633</v>
+        <v>0.2643698571951425</v>
       </c>
       <c r="BG12" t="n">
-        <v>0.282705430057678</v>
+        <v>0.2703054214592269</v>
       </c>
       <c r="BH12" t="n">
-        <v>33.08475205451941</v>
+        <v>29.98044858403659</v>
       </c>
       <c r="BI12" t="n">
-        <v>29.39610869501784</v>
+        <v>26.72553092593011</v>
       </c>
       <c r="BJ12" t="n">
-        <v>2.884171794450784</v>
+        <v>2.303923680608885</v>
       </c>
       <c r="BK12" t="n">
-        <v>3.261329281688954</v>
+        <v>2.882968540175306</v>
       </c>
       <c r="BL12" t="n">
-        <v>0.006156027509352365</v>
+        <v>0.005315276433515318</v>
       </c>
       <c r="BM12" t="n">
-        <v>0.00804589590951184</v>
+        <v>0.006800493353966972</v>
       </c>
       <c r="BN12" t="n">
-        <v>0.01344178461809785</v>
+        <v>0.01062426917585756</v>
       </c>
       <c r="BO12" t="n">
-        <v>0.0157971376919532</v>
+        <v>0.0122331909433647</v>
       </c>
       <c r="BP12" t="n">
-        <v>0.01250886529474235</v>
+        <v>0.01024513066453868</v>
       </c>
       <c r="BQ12" t="n">
-        <v>0.01500918106032717</v>
+        <v>0.01180583404810668</v>
       </c>
       <c r="BR12" t="n">
-        <v>0.01129033559063781</v>
+        <v>0.009651510756827819</v>
       </c>
       <c r="BS12" t="n">
-        <v>0.01563676908255854</v>
+        <v>0.01214206365467917</v>
       </c>
       <c r="BT12" t="n">
-        <v>-0.003235513507737744</v>
+        <v>-0.003057799930897423</v>
       </c>
       <c r="BU12" t="n">
-        <v>-0.002231649350291192</v>
+        <v>-0.002068373106626384</v>
       </c>
       <c r="BV12" t="n">
-        <v>0.004458185441687315</v>
+        <v>0.004189179304898662</v>
       </c>
       <c r="BW12" t="n">
-        <v>0.004567196420364833</v>
+        <v>0.004302679159995472</v>
       </c>
       <c r="BX12" t="n">
-        <v>-0.002948021674198894</v>
+        <v>-0.004111400933888591</v>
       </c>
       <c r="BY12" t="n">
-        <v>-0.003885186430086625</v>
+        <v>-0.003637087705207234</v>
       </c>
       <c r="BZ12" t="n">
-        <v>-0.002124470866564396</v>
+        <v>-0.002335153805042054</v>
       </c>
       <c r="CA12" t="n">
-        <v>-0.001993117610687891</v>
+        <v>-0.001909165039167516</v>
       </c>
       <c r="CB12" t="n">
-        <v>0.003823364606156455</v>
+        <v>0.004257452329189768</v>
       </c>
       <c r="CC12" t="n">
-        <v>0.004298752523734298</v>
+        <v>0.004113939185833794</v>
       </c>
       <c r="CD12" t="n">
-        <v>-0.003413044956712133</v>
+        <v>-0.003782536887615375</v>
       </c>
       <c r="CE12" t="n">
-        <v>-0.00358435154889147</v>
+        <v>-0.003430933924480291</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>50.38745387453875</v>
-      </c>
-      <c r="B13" t="n">
-        <v>15.75324061915245</v>
-      </c>
-      <c r="C13" t="n">
-        <v>1.398392083920839</v>
-      </c>
-      <c r="D13" t="n">
-        <v>1.103987837784548</v>
-      </c>
-      <c r="E13" t="n">
-        <v>49.72529725297252</v>
-      </c>
-      <c r="F13" t="n">
-        <v>15.45636084504887</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1.420767307673077</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1.119394038287382</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.2599695944613711</v>
-      </c>
-      <c r="J13" t="n">
-        <v>-2.201514904281546</v>
-      </c>
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="n">
-        <v>0.3092243246578802</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.3105488432985803</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0.5383961351376184</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0.5968960171726396</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0.2691980675688092</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0.2984480085863198</v>
-      </c>
-      <c r="R13" t="n">
-        <v>28.88775074060709</v>
-      </c>
-      <c r="S13" t="n">
-        <v>25.86269368846262</v>
-      </c>
-      <c r="T13" t="n">
-        <v>1.900000000000001</v>
-      </c>
-      <c r="U13" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="V13" t="n">
-        <v>0.01599481502564746</v>
-      </c>
-      <c r="W13" t="n">
-        <v>0.0272231107021466</v>
-      </c>
-      <c r="X13" t="n">
-        <v>1.702164460260683</v>
-      </c>
-      <c r="Y13" t="n">
-        <v>2.613145936716569</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>0.01448821669788084</v>
-      </c>
-      <c r="AA13" t="n">
-        <v>0.02431950660001426</v>
-      </c>
-      <c r="AB13" t="n">
-        <v>141</v>
-      </c>
-      <c r="AC13" t="n">
-        <v>84</v>
-      </c>
-      <c r="AD13" t="n">
-        <v>0.01514005341563801</v>
-      </c>
-      <c r="AE13" t="n">
-        <v>0.02541366109053524</v>
-      </c>
-      <c r="AF13" t="n">
-        <v>1.056456974526032</v>
-      </c>
-      <c r="AG13" t="n">
-        <v>1.071199879669649</v>
-      </c>
-      <c r="AH13" t="n">
-        <v>0.1411424363150804</v>
-      </c>
-      <c r="AI13" t="n">
-        <v>-2.322000300825877</v>
-      </c>
-      <c r="AJ13" t="n">
-        <v>0.3218099308454808</v>
-      </c>
-      <c r="AK13" t="n">
-        <v>0.3123374127771664</v>
-      </c>
-      <c r="AL13" t="n">
-        <v>0.4444630324663207</v>
-      </c>
-      <c r="AM13" t="n">
-        <v>0.5583113288574335</v>
-      </c>
-      <c r="AN13" t="n">
-        <v>0.1470147786408094</v>
-      </c>
-      <c r="AO13" t="n">
-        <v>0.1804827528325299</v>
-      </c>
-      <c r="AP13" t="n">
-        <v>0.2222315162331603</v>
-      </c>
-      <c r="AQ13" t="n">
-        <v>0.2791556644287168</v>
-      </c>
-      <c r="AR13" t="n">
-        <v>26.82459465325925</v>
-      </c>
-      <c r="AS13" t="n">
-        <v>26.77513366787684</v>
-      </c>
-      <c r="AT13" t="n">
-        <v>0.01378581983518137</v>
-      </c>
-      <c r="AU13" t="n">
-        <v>0.02317374877985195</v>
-      </c>
-      <c r="AV13" t="n">
-        <v>1.160236766247934</v>
-      </c>
-      <c r="AW13" t="n">
-        <v>1.174739182717614</v>
-      </c>
-      <c r="AX13" t="n">
-        <v>0.400591915619834</v>
-      </c>
-      <c r="AY13" t="n">
-        <v>-2.063152043205964</v>
-      </c>
-      <c r="AZ13" t="n">
-        <v>0.3059745553868967</v>
-      </c>
-      <c r="BA13" t="n">
-        <v>0.3123374127771664</v>
-      </c>
-      <c r="BB13" t="n">
-        <v>0.5367220658383516</v>
-      </c>
-      <c r="BC13" t="n">
-        <v>0.5412930952861537</v>
-      </c>
-      <c r="BD13" t="n">
-        <v>0.1768919520879173</v>
-      </c>
-      <c r="BE13" t="n">
-        <v>0.1832429281975233</v>
-      </c>
-      <c r="BF13" t="n">
-        <v>0.2683610329191758</v>
-      </c>
-      <c r="BG13" t="n">
-        <v>0.2706465476430768</v>
-      </c>
-      <c r="BH13" t="n">
-        <v>30.26460008371505</v>
-      </c>
-      <c r="BI13" t="n">
-        <v>27.02547280871111</v>
-      </c>
-      <c r="BJ13" t="n">
-        <v>1.70747357742092</v>
-      </c>
-      <c r="BK13" t="n">
-        <v>2.881572225092967</v>
-      </c>
-      <c r="BL13" t="n">
-        <v>0.003998703756411864</v>
-      </c>
-      <c r="BM13" t="n">
-        <v>0.006805777675536649</v>
-      </c>
-      <c r="BN13" t="n">
-        <v>0.008061292129149612</v>
-      </c>
-      <c r="BO13" t="n">
-        <v>0.01236981623545321</v>
-      </c>
-      <c r="BP13" t="n">
-        <v>0.007727018471452724</v>
-      </c>
-      <c r="BQ13" t="n">
-        <v>0.01187515584780896</v>
-      </c>
-      <c r="BR13" t="n">
-        <v>0.007217830600366845</v>
-      </c>
-      <c r="BS13" t="n">
-        <v>0.01226374231326723</v>
-      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="inlineStr"/>
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr"/>
+      <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr"/>
+      <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
+      <c r="AZ13" t="inlineStr"/>
+      <c r="BA13" t="inlineStr"/>
+      <c r="BB13" t="inlineStr"/>
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr"/>
+      <c r="BE13" t="inlineStr"/>
+      <c r="BF13" t="inlineStr"/>
+      <c r="BG13" t="inlineStr"/>
+      <c r="BH13" t="inlineStr"/>
+      <c r="BI13" t="inlineStr"/>
+      <c r="BJ13" t="inlineStr"/>
+      <c r="BK13" t="inlineStr"/>
+      <c r="BL13" t="inlineStr"/>
+      <c r="BM13" t="inlineStr"/>
+      <c r="BN13" t="inlineStr"/>
+      <c r="BO13" t="inlineStr"/>
+      <c r="BP13" t="inlineStr"/>
+      <c r="BQ13" t="inlineStr"/>
+      <c r="BR13" t="inlineStr"/>
+      <c r="BS13" t="inlineStr"/>
       <c r="BT13" t="n">
-        <v>0.000516188217643537</v>
+        <v>0.001147585484042551</v>
       </c>
       <c r="BU13" t="n">
-        <v>0.00198913649199365</v>
+        <v>0.001886458724673981</v>
       </c>
       <c r="BV13" t="n">
-        <v>0.004132192950783035</v>
+        <v>0.004421476727561352</v>
       </c>
       <c r="BW13" t="n">
-        <v>0.006552325458838363</v>
+        <v>0.006304602004577764</v>
       </c>
       <c r="BX13" t="n">
-        <v>-0.003370042782489039</v>
+        <v>-0.003986728538633191</v>
       </c>
       <c r="BY13" t="n">
-        <v>-0.002009650686270488</v>
+        <v>-0.001738111594695642</v>
       </c>
       <c r="BZ13" t="n">
-        <v>0.001524868665391059</v>
+        <v>0.001717004926768318</v>
       </c>
       <c r="CA13" t="n">
-        <v>0.001878393563504645</v>
+        <v>0.001803341793740059</v>
       </c>
       <c r="CB13" t="n">
-        <v>0.00488672157508899</v>
+        <v>0.005495705494631966</v>
       </c>
       <c r="CC13" t="n">
-        <v>0.006926125273800484</v>
+        <v>0.006553882715624301</v>
       </c>
       <c r="CD13" t="n">
-        <v>-0.002443515016147425</v>
+        <v>-0.002648529935681185</v>
       </c>
       <c r="CE13" t="n">
-        <v>-0.001059190845147822</v>
+        <v>-0.001088816950415088</v>
       </c>
     </row>
     <row r="14">
@@ -3896,40 +3756,40 @@
       <c r="BR14" t="inlineStr"/>
       <c r="BS14" t="inlineStr"/>
       <c r="BT14" t="n">
-        <v>0.008035395703107122</v>
+        <v>0.00955068626320011</v>
       </c>
       <c r="BU14" t="n">
-        <v>0.01043630286365026</v>
+        <v>0.00980856344415993</v>
       </c>
       <c r="BV14" t="n">
-        <v>0.0032138745886835</v>
+        <v>0.004635262960266697</v>
       </c>
       <c r="BW14" t="n">
-        <v>0.01004636225816696</v>
+        <v>0.00984548276080586</v>
       </c>
       <c r="BX14" t="n">
-        <v>-0.00407529764976355</v>
+        <v>-0.003534149276367921</v>
       </c>
       <c r="BY14" t="n">
-        <v>0.001727546235579196</v>
+        <v>0.00203118222775182</v>
       </c>
       <c r="BZ14" t="n">
-        <v>0.008807494124215269</v>
+        <v>0.009804435594725235</v>
       </c>
       <c r="CA14" t="n">
-        <v>0.009677472420787099</v>
+        <v>0.00927610565731205</v>
       </c>
       <c r="CB14" t="n">
-        <v>0.006682568978678978</v>
+        <v>0.007597472296685035</v>
       </c>
       <c r="CC14" t="n">
-        <v>0.01165303954821195</v>
+        <v>0.01093613606588819</v>
       </c>
       <c r="CD14" t="n">
-        <v>-0.0004394888933663219</v>
+        <v>-0.0003154668474072216</v>
       </c>
       <c r="CE14" t="n">
-        <v>0.003894506407041777</v>
+        <v>0.003510489070364321</v>
       </c>
     </row>
     <row r="15">
@@ -4005,40 +3865,40 @@
       <c r="BR15" t="inlineStr"/>
       <c r="BS15" t="inlineStr"/>
       <c r="BT15" t="n">
-        <v>0.01556832944782732</v>
+        <v>0.01794628928633898</v>
       </c>
       <c r="BU15" t="n">
-        <v>0.01892044073400895</v>
+        <v>0.01777706205585864</v>
       </c>
       <c r="BV15" t="n">
-        <v>0.002004974518019791</v>
+        <v>0.004586948697817221</v>
       </c>
       <c r="BW15" t="n">
-        <v>0.0129795151541851</v>
+        <v>0.01283875289979368</v>
       </c>
       <c r="BX15" t="n">
-        <v>-0.004660011707418921</v>
+        <v>-0.002882900860670011</v>
       </c>
       <c r="BY15" t="n">
-        <v>0.005373055546870394</v>
+        <v>0.005693606138199185</v>
       </c>
       <c r="BZ15" t="n">
-        <v>0.01608426841341041</v>
+        <v>0.01788750080773875</v>
       </c>
       <c r="CA15" t="n">
-        <v>0.01759052216944542</v>
+        <v>0.01684896516405627</v>
       </c>
       <c r="CB15" t="n">
-        <v>0.00810039811715026</v>
+        <v>0.009269751052096015</v>
       </c>
       <c r="CC15" t="n">
-        <v>0.015745907786902</v>
+        <v>0.01472154056754115</v>
       </c>
       <c r="CD15" t="n">
-        <v>0.001588215929495831</v>
+        <v>0.002034412295805811</v>
       </c>
       <c r="CE15" t="n">
-        <v>0.008651752946828323</v>
+        <v>0.007931766184231758</v>
       </c>
     </row>
     <row r="16">
@@ -4114,40 +3974,40 @@
       <c r="BR16" t="inlineStr"/>
       <c r="BS16" t="inlineStr"/>
       <c r="BT16" t="n">
-        <v>0.02311233926609982</v>
+        <v>0.02633537828623222</v>
       </c>
       <c r="BU16" t="n">
-        <v>0.02745254011488848</v>
+        <v>0.02580313190364955</v>
       </c>
       <c r="BV16" t="n">
-        <v>0.0005287332871603502</v>
+        <v>0.00430259869965029</v>
       </c>
       <c r="BW16" t="n">
-        <v>0.01537761367686739</v>
+        <v>0.01530852985326219</v>
       </c>
       <c r="BX16" t="n">
-        <v>-0.005147458268633167</v>
+        <v>-0.002059049404752501</v>
       </c>
       <c r="BY16" t="n">
-        <v>0.008899622525478037</v>
+        <v>0.009223412744051933</v>
       </c>
       <c r="BZ16" t="n">
-        <v>0.02336084512573884</v>
+        <v>0.02597280636219234</v>
       </c>
       <c r="CA16" t="n">
-        <v>0.02563288594643249</v>
+        <v>0.02453608471346371</v>
       </c>
       <c r="CB16" t="n">
-        <v>0.009162777317660225</v>
+        <v>0.01053759000486187</v>
       </c>
       <c r="CC16" t="n">
-        <v>0.01922779210756178</v>
+        <v>0.01793228832795921</v>
       </c>
       <c r="CD16" t="n">
-        <v>0.003616720312730754</v>
+        <v>0.004375661478286942</v>
       </c>
       <c r="CE16" t="n">
-        <v>0.01318610193196549</v>
+        <v>0.0121498217606338</v>
       </c>
     </row>
     <row r="17">
@@ -4223,40 +4083,40 @@
       <c r="BR17" t="inlineStr"/>
       <c r="BS17" t="inlineStr"/>
       <c r="BT17" t="n">
-        <v>0.03067006787802389</v>
+        <v>0.03471696963229506</v>
       </c>
       <c r="BU17" t="n">
-        <v>0.03602276667661294</v>
+        <v>0.03387701969654561</v>
       </c>
       <c r="BV17" t="n">
-        <v>-0.00123815521346641</v>
+        <v>0.003756145498629917</v>
       </c>
       <c r="BW17" t="n">
-        <v>0.01721196225785935</v>
+        <v>0.0172274158351154</v>
       </c>
       <c r="BX17" t="n">
-        <v>-0.00551442958143164</v>
+        <v>-0.001036531503100972</v>
       </c>
       <c r="BY17" t="n">
-        <v>0.0123316358551473</v>
+        <v>0.01264306908352956</v>
       </c>
       <c r="BZ17" t="n">
-        <v>0.03063172461391239</v>
+        <v>0.03405395348403976</v>
       </c>
       <c r="CA17" t="n">
-        <v>0.03379318836606342</v>
+        <v>0.03232670696120247</v>
       </c>
       <c r="CB17" t="n">
-        <v>0.009846515261591053</v>
+        <v>0.01137514344564886</v>
       </c>
       <c r="CC17" t="n">
-        <v>0.02206879121142657</v>
+        <v>0.02054012749244327</v>
       </c>
       <c r="CD17" t="n">
-        <v>0.005668280404586297</v>
+        <v>0.006732929250370362</v>
       </c>
       <c r="CE17" t="n">
-        <v>0.01751716102362604</v>
+        <v>0.01618378868280081</v>
       </c>
     </row>
     <row r="18">
@@ -4332,40 +4192,40 @@
       <c r="BR18" t="inlineStr"/>
       <c r="BS18" t="inlineStr"/>
       <c r="BT18" t="n">
-        <v>0.03823475699305898</v>
+        <v>0.04309357031908856</v>
       </c>
       <c r="BU18" t="n">
-        <v>0.04465986356366604</v>
+        <v>0.04202812187832328</v>
       </c>
       <c r="BV18" t="n">
-        <v>-0.003236505391651533</v>
+        <v>0.003014010531194258</v>
       </c>
       <c r="BW18" t="n">
-        <v>0.0185465584484208</v>
+        <v>0.0186547700100353</v>
       </c>
       <c r="BX18" t="n">
-        <v>-0.005820275378190133</v>
+        <v>0.0001182246375168578</v>
       </c>
       <c r="BY18" t="n">
-        <v>0.01559781386404531</v>
+        <v>0.01588485944644554</v>
       </c>
       <c r="BZ18" t="n">
-        <v>0.03791141026265075</v>
+        <v>0.04214790538443931</v>
       </c>
       <c r="CA18" t="n">
-        <v>0.04211314296289681</v>
+        <v>0.04025916432930614</v>
       </c>
       <c r="CB18" t="n">
-        <v>0.01020873692671188</v>
+        <v>0.01184574675172044</v>
       </c>
       <c r="CC18" t="n">
-        <v>0.02432317180783913</v>
+        <v>0.02259763513098226</v>
       </c>
       <c r="CD18" t="n">
-        <v>0.007684203444690054</v>
+        <v>0.009040872069520593</v>
       </c>
       <c r="CE18" t="n">
-        <v>0.02157302893647334</v>
+        <v>0.01996548936599829</v>
       </c>
     </row>
     <row r="19">
@@ -4441,40 +4301,40 @@
       <c r="BR19" t="inlineStr"/>
       <c r="BS19" t="inlineStr"/>
       <c r="BT19" t="n">
-        <v>0.04202670234571454</v>
+        <v>0.04727740112144834</v>
       </c>
       <c r="BU19" t="n">
-        <v>0.04897585218343851</v>
+        <v>0.0461048232567489</v>
       </c>
       <c r="BV19" t="n">
-        <v>-0.004383937843225719</v>
+        <v>0.0025007187760862</v>
       </c>
       <c r="BW19" t="n">
-        <v>0.01895478352797825</v>
+        <v>0.01911647324937043</v>
       </c>
       <c r="BX19" t="n">
-        <v>-0.005888886331320044</v>
+        <v>0.0008140327996875746</v>
       </c>
       <c r="BY19" t="n">
-        <v>0.01723725111326942</v>
+        <v>0.01750310490135618</v>
       </c>
       <c r="BZ19" t="n">
-        <v>0.04153980726794487</v>
+        <v>0.0461824835761678</v>
       </c>
       <c r="CA19" t="n">
-        <v>0.04629729304236604</v>
+        <v>0.04424531037938278</v>
       </c>
       <c r="CB19" t="n">
-        <v>0.01020892973103858</v>
+        <v>0.01187633418792981</v>
       </c>
       <c r="CC19" t="n">
-        <v>0.02516115087731458</v>
+        <v>0.02335404047297559</v>
       </c>
       <c r="CD19" t="n">
-        <v>0.008738484270836552</v>
+        <v>0.01024260056060899</v>
       </c>
       <c r="CE19" t="n">
-        <v>0.02355929646385355</v>
+        <v>0.02182091491996809</v>
       </c>
     </row>
     <row r="20">
@@ -4550,40 +4410,40 @@
       <c r="BR20" t="inlineStr"/>
       <c r="BS20" t="inlineStr"/>
       <c r="BT20" t="n">
-        <v>0.04584047994611924</v>
+        <v>0.05145251926151809</v>
       </c>
       <c r="BU20" t="n">
-        <v>0.05322817914864099</v>
+        <v>0.05011973338663249</v>
       </c>
       <c r="BV20" t="n">
-        <v>-0.005765771573148123</v>
+        <v>0.001740701666978982</v>
       </c>
       <c r="BW20" t="n">
-        <v>0.01903456632786238</v>
+        <v>0.01926368860337439</v>
       </c>
       <c r="BX20" t="n">
-        <v>-0.005765771573148123</v>
+        <v>0.001740701666978982</v>
       </c>
       <c r="BY20" t="n">
-        <v>0.01903456632786238</v>
+        <v>0.01926368860337439</v>
       </c>
       <c r="BZ20" t="n">
-        <v>0.04512790272181015</v>
+        <v>0.05017067209093633</v>
       </c>
       <c r="CA20" t="n">
-        <v>0.05041537327571449</v>
+        <v>0.04816839271303663</v>
       </c>
       <c r="CB20" t="n">
-        <v>0.009955858702121708</v>
+        <v>0.01162302551437479</v>
       </c>
       <c r="CC20" t="n">
-        <v>0.02565944805568296</v>
+        <v>0.02378850484138425</v>
       </c>
       <c r="CD20" t="n">
-        <v>0.009955858702121708</v>
+        <v>0.01162302551437479</v>
       </c>
       <c r="CE20" t="n">
-        <v>0.02565944805568296</v>
+        <v>0.02378850484138425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adiabatic index calculations added
</commit_message>
<xml_diff>
--- a/results/Профилирование_лопаток.xlsx
+++ b/results/Профилирование_лопаток.xlsx
@@ -430,13 +430,13 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -514,37 +514,37 @@
       </c>
       <c r="B2" s="1" t="inlineStr"/>
       <c r="C2" s="2" t="n">
-        <v>64.71094710947109</v>
+        <v>64.77384773847739</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>57.22492224922249</v>
+        <v>57.16372163721637</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>55.63965639656396</v>
+        <v>55.55550555505555</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>54.76159761597616</v>
+        <v>54.6629966299663</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>54.08499084990849</v>
+        <v>53.97363973639736</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>53.4729847298473</v>
+        <v>53.34803348033481</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>52.86437864378644</v>
+        <v>52.72327723277233</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>52.22772227722277</v>
+        <v>52.06962069620696</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>51.53836538365384</v>
+        <v>51.36241362413624</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>50.77590775907759</v>
+        <v>50.57870578705787</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>49.91909919099191</v>
+        <v>49.69724697246973</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
@@ -555,37 +555,37 @@
       </c>
       <c r="B3" s="1" t="inlineStr"/>
       <c r="C3" s="2" t="n">
-        <v>22.20486627069856</v>
+        <v>22.23366067928492</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>18.81414429643773</v>
+        <v>18.78667200347058</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>18.10337712128646</v>
+        <v>18.06569001223161</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>17.71029722059282</v>
+        <v>17.66617600981681</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>17.40759325460909</v>
+        <v>17.35778752225922</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>17.13387679317958</v>
+        <v>17.07799842963868</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>16.86171131101422</v>
+        <v>16.79861039153258</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>16.5769782848382</v>
+        <v>16.50625949507566</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>16.26857794552883</v>
+        <v>16.18983586580151</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>15.92725827195502</v>
+        <v>15.83892876207851</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>15.5432887962779</v>
+        <v>15.44377647190229</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
@@ -596,37 +596,37 @@
       </c>
       <c r="B4" s="1" t="inlineStr"/>
       <c r="C4" s="2" t="n">
-        <v>0.8614941149411495</v>
+        <v>0.8631946319463195</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.7108999089990899</v>
+        <v>0.7088234882348824</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.7474341743417434</v>
+        <v>0.744659646596466</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.8131278312783128</v>
+        <v>0.8100669006690067</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.8889529895298953</v>
+        <v>0.8857309573095731</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.9694858948589486</v>
+        <v>0.9661564615646157</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>1.052310023100231</v>
+        <v>1.048926889268893</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>1.136422964229642</v>
+        <v>1.133021930219302</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>1.221144511445114</v>
+        <v>1.217707677076771</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>1.306045060450605</v>
+        <v>1.302608226082261</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1.391053010530105</v>
+        <v>1.38759827598276</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -637,37 +637,37 @@
       </c>
       <c r="B5" s="1" t="inlineStr"/>
       <c r="C5" s="2" t="n">
-        <v>1.343470347883344</v>
+        <v>1.341371646014791</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.276216055321003</v>
+        <v>1.279071438452971</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1.266554808711321</v>
+        <v>1.217728103341536</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1.249660274931126</v>
+        <v>1.200562235727506</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>1.217269844939181</v>
+        <v>1.205662142741908</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.165340464237523</v>
+        <v>1.177835429668613</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>1.146207216339745</v>
+        <v>1.146552488128985</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1.132844612450705</v>
+        <v>1.147086980315868</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>1.132482955930341</v>
+        <v>1.125673335068041</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>1.107175675100259</v>
+        <v>1.10117963536189</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>1.097672504434753</v>
+        <v>1.096041329849556</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -678,37 +678,37 @@
       </c>
       <c r="B6" s="1" t="inlineStr"/>
       <c r="C6" s="2" t="n">
-        <v>65.10110101101012</v>
+        <v>65.15210152101521</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>58.60618606186062</v>
+        <v>58.54838548385484</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>57.00987009870099</v>
+        <v>56.92911929119291</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>56.01621016210162</v>
+        <v>55.91845918459185</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>55.17725177251772</v>
+        <v>55.06505065050651</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>54.36634366343664</v>
+        <v>54.23884238842388</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>53.52228522285223</v>
+        <v>53.37863378633786</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>52.61192611926119</v>
+        <v>52.45042450424504</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>51.60381603816038</v>
+        <v>51.42446424464245</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>50.4690546905469</v>
+        <v>50.27015270152701</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>49.17874178741788</v>
+        <v>48.95773957739577</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -719,37 +719,37 @@
       </c>
       <c r="B7" s="1" t="inlineStr"/>
       <c r="C7" s="2" t="n">
-        <v>22.3835587120456</v>
+        <v>22.40693294537645</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>19.43502361372193</v>
+        <v>19.40900729747304</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>18.71762244984242</v>
+        <v>18.68138812067616</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>18.27206400949141</v>
+        <v>18.22826634488273</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>17.89633087263101</v>
+        <v>17.84610639440173</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>17.53345077857043</v>
+        <v>17.47641324513817</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>17.15592436668552</v>
+        <v>17.09168283200835</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>16.74881265158745</v>
+        <v>16.67658426996932</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>16.29786537577372</v>
+        <v>16.21760625413955</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>15.78980388031258</v>
+        <v>15.70067280769886</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>15.21102317753028</v>
+        <v>15.11173387104089</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -760,37 +760,37 @@
       </c>
       <c r="B8" s="1" t="inlineStr"/>
       <c r="C8" s="2" t="n">
-        <v>0.8574665746657466</v>
+        <v>0.8595429954299543</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.6573783737837379</v>
+        <v>0.6547291472914729</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.6890079900799009</v>
+        <v>0.6854279542795428</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.7588365883658836</v>
+        <v>0.7549522495224952</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.8426631266312663</v>
+        <v>0.8386534865348654</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.9333275332753328</v>
+        <v>0.9292641926419265</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1.02750037500375</v>
+        <v>1.023419134191342</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>1.123642236422364</v>
+        <v>1.11959679596796</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>1.220661206612066</v>
+        <v>1.216687366873669</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>1.3180023800238</v>
+        <v>1.314118041180412</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1.415468854688547</v>
+        <v>1.411763517635176</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
@@ -801,37 +801,37 @@
       </c>
       <c r="B9" s="1" t="inlineStr"/>
       <c r="C9" s="2" t="n">
-        <v>1.386708868839728</v>
+        <v>1.362960719157583</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1.242672434326975</v>
+        <v>1.243175370640397</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1.208920074676587</v>
+        <v>1.217846027693225</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1.223038041151503</v>
+        <v>1.203343778173821</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>1.194137516578516</v>
+        <v>1.188751970858458</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.162911161304894</v>
+        <v>1.161060963730647</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1.163943155104231</v>
+        <v>1.153012993973322</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>1.144727538137692</v>
+        <v>1.12973797875404</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>1.134288878699166</v>
+        <v>1.124170385155504</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>1.113612371112979</v>
+        <v>1.101330071021851</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1.108521885047528</v>
+        <v>1.08790969082936</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
@@ -842,37 +842,37 @@
       </c>
       <c r="B10" s="1" t="inlineStr"/>
       <c r="C10" s="2" t="n">
-        <v>0.8586758697083607</v>
+        <v>0.8534291150369783</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.6905401383025078</v>
+        <v>0.6976785961324267</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.666387021778303</v>
+        <v>0.5443202583538403</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.6241506873278152</v>
+        <v>0.5014055893187652</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.5431746123479514</v>
+        <v>0.5141553568547702</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0.4133511605938073</v>
+        <v>0.4445885741715316</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.3655180408493613</v>
+        <v>0.3663812203224615</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0.3321115311267625</v>
+        <v>0.3677174507896691</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0.3312073898258527</v>
+        <v>0.3141833376701036</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>0.2679391877506465</v>
+        <v>0.2529490884047253</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0.2441812610868815</v>
+        <v>0.2401033246238898</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
@@ -883,37 +883,37 @@
       </c>
       <c r="B11" s="1" t="inlineStr"/>
       <c r="C11" s="2" t="n">
-        <v>-1.53322782790068</v>
+        <v>-1.592598202106044</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>-1.893318914182562</v>
+        <v>-1.892061573399007</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-1.977699813308532</v>
+        <v>-1.955384930766939</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-1.942404897121243</v>
+        <v>-1.991640554565447</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-2.014656208553709</v>
+        <v>-2.028120072853854</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>-2.092722096737766</v>
+        <v>-2.097347590673383</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>-2.090142112239421</v>
+        <v>-2.117467515066696</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>-2.13818115465577</v>
+        <v>-2.175655053114901</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>-2.164277803252084</v>
+        <v>-2.189574037111239</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>-2.215969072217554</v>
+        <v>-2.246674822445373</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>-2.22869528738118</v>
+        <v>-2.280225772926599</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -945,37 +945,37 @@
       </c>
       <c r="B13" s="1" t="inlineStr"/>
       <c r="C13" s="2" t="n">
-        <v>0.2805780275618496</v>
+        <v>0.2804526037547906</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.2955501222767397</v>
+        <v>0.2956724194296661</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.2987208415105116</v>
+        <v>0.2988884788824699</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.3004771224953454</v>
+        <v>0.3006735859023923</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.3018294964074096</v>
+        <v>0.3020528891766766</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>0.3030533927479625</v>
+        <v>0.3033044283879892</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.3042720407536296</v>
+        <v>0.3045535063250858</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>0.3055448779081271</v>
+        <v>0.3058599617351919</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>0.3069225100380258</v>
+        <v>0.3072743401601156</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>0.3084475442871231</v>
+        <v>0.308841767907909</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0.3101612505719784</v>
+        <v>0.3106056762622871</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
@@ -986,37 +986,37 @@
       </c>
       <c r="B14" s="1" t="inlineStr"/>
       <c r="C14" s="2" t="n">
-        <v>0.2797974550671152</v>
+        <v>0.2796962690770293</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.2927873051524886</v>
+        <v>0.292902472557148</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.2959799055217359</v>
+        <v>0.2961425517452044</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.2979680737285447</v>
+        <v>0.2981625981921411</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.2996457346074712</v>
+        <v>0.2998702804560274</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>0.3012673960851999</v>
+        <v>0.3015225351993011</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.3029550207105427</v>
+        <v>0.3032430724758871</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>0.3047758064976246</v>
+        <v>0.3050989684454197</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>0.3067918634590923</v>
+        <v>0.3071516686220299</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>0.3090610725140273</v>
+        <v>0.3094602850926037</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0.3116430333523839</v>
+        <v>0.3120847789933427</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -1027,37 +1027,37 @@
       </c>
       <c r="B15" s="1" t="inlineStr"/>
       <c r="C15" s="2" t="n">
-        <v>0.420727598857796</v>
+        <v>0.4223376568031352</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.2998275271987845</v>
+        <v>0.2981993690575462</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.3056677973852782</v>
+        <v>0.308983278457205</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.3288381289455449</v>
+        <v>0.3321736925204204</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.3587461654119073</v>
+        <v>0.3577791331188592</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>0.3930424783949269</v>
+        <v>0.3889077998816547</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0.4237323656626913</v>
+        <v>0.4208401454858027</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>0.4530582134209176</v>
+        <v>0.4479027457180903</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>0.4791410012183553</v>
+        <v>0.4766401314196184</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>0.5070081862184586</v>
+        <v>0.5040200801505635</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0.5300104596754484</v>
+        <v>0.5258355692086617</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -1068,37 +1068,37 @@
       </c>
       <c r="B16" s="1" t="inlineStr"/>
       <c r="C16" s="2" t="n">
-        <v>0.4744794689706583</v>
+        <v>0.4786002320540451</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.3472304666519005</v>
+        <v>0.3455986140250983</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.3552289083652951</v>
+        <v>0.3520978053349409</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.377651635661902</v>
+        <v>0.3775720228264185</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.411096476572654</v>
+        <v>0.4091411257835789</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>0.4470219933759244</v>
+        <v>0.444405744654935</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0.4785151284134683</v>
+        <v>0.4769415485356119</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0.5114829101224904</v>
+        <v>0.5103324860175888</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0.5407642322756867</v>
+        <v>0.538636476382473</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>0.5683468758339792</v>
+        <v>0.5663103666617944</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0.5890317907894089</v>
+        <v>0.5881185676044323</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
@@ -1109,37 +1109,37 @@
       </c>
       <c r="B17" s="1" t="inlineStr"/>
       <c r="C17" s="2" t="n">
-        <v>0.210363799428898</v>
+        <v>0.2111688284015676</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.1499137635993922</v>
+        <v>0.1490996845287731</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.1528338986926391</v>
+        <v>0.1544916392286025</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0.1644190644727725</v>
+        <v>0.1660868462602102</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.1793730827059536</v>
+        <v>0.1788895665594296</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>0.1965212391974634</v>
+        <v>0.1944538999408274</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.2118661828313457</v>
+        <v>0.2104200727429013</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>0.2265291067104588</v>
+        <v>0.2239513728590452</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>0.2395705006091776</v>
+        <v>0.2383200657098092</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>0.2535040931092293</v>
+        <v>0.2520100400752818</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0.2650052298377242</v>
+        <v>0.2629177846043309</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1150,37 +1150,37 @@
       </c>
       <c r="B18" s="1" t="inlineStr"/>
       <c r="C18" s="2" t="n">
-        <v>0.2372397344853292</v>
+        <v>0.2393001160270225</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.1736152333259503</v>
+        <v>0.1727993070125491</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.1776144541826475</v>
+        <v>0.1760489026674704</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.188825817830951</v>
+        <v>0.1887860114132092</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.205548238286327</v>
+        <v>0.2045705628917895</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>0.2235109966879622</v>
+        <v>0.2222028723274675</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.2392575642067341</v>
+        <v>0.2384707742678059</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0.2557414550612452</v>
+        <v>0.2551662430087944</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0.2703821161378434</v>
+        <v>0.2693182381912365</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>0.2841734379169896</v>
+        <v>0.2831551833308972</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0.2945158953947045</v>
+        <v>0.2940592838022161</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -1191,37 +1191,37 @@
       </c>
       <c r="B19" s="1" t="inlineStr"/>
       <c r="C19" s="2" t="n">
-        <v>46.6507350952965</v>
+        <v>46.64629336959779</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>44.6903123049828</v>
+        <v>44.69408619850299</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>42.92757772458603</v>
+        <v>42.80184761491208</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>41.14913028024685</v>
+        <v>41.01979183410091</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>39.33311398781009</v>
+        <v>39.29228501686831</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>37.47215503447565</v>
+        <v>37.48684935179171</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>35.697700617668</v>
+        <v>35.67944400938476</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>33.94765735129087</v>
+        <v>33.95979880847663</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>32.24325522137479</v>
+        <v>32.20089641861436</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>30.49581250064761</v>
+        <v>30.45209030999562</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>28.80698702188971</v>
+        <v>28.77050047964588</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
@@ -1232,37 +1232,37 @@
       </c>
       <c r="B20" s="1" t="inlineStr"/>
       <c r="C20" s="2" t="n">
-        <v>44.61222616554168</v>
+        <v>44.53901660782599</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>44.11046014096319</v>
+        <v>44.12199484808684</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>42.31345700234485</v>
+        <v>42.34470977155496</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>40.39687964631737</v>
+        <v>40.35424983295096</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>38.28732061675203</v>
+        <v>38.274755076396</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>36.13268124092896</v>
+        <v>36.12352072192418</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>34.04378351675329</v>
+        <v>34.00742910129591</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>31.91004045234901</v>
+        <v>31.85898732639359</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>29.81603189698111</v>
+        <v>29.77225115163278</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>27.72679526811413</v>
+        <v>27.67386610097276</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>25.71353038406959</v>
+        <v>25.63735255569113</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -1273,37 +1273,37 @@
       </c>
       <c r="B21" s="1" t="inlineStr"/>
       <c r="C21" s="2" t="n">
-        <v>2.3</v>
+        <v>3.5</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>2.2</v>
+        <v>3.4</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>2.1</v>
+        <v>3.3</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>2</v>
+        <v>3.2</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>1.9</v>
+        <v>3.1</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>1.7</v>
+        <v>2.9</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>1.6</v>
+        <v>2.8</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>1.5</v>
+        <v>2.7</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>1.4</v>
+        <v>2.6</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -1314,37 +1314,37 @@
       </c>
       <c r="B22" s="1" t="inlineStr"/>
       <c r="C22" s="2" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>1.9</v>
+        <v>3.4</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>1.8</v>
+        <v>3.3</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1.7</v>
+        <v>3.2</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>1.6</v>
+        <v>3.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>1.4</v>
+        <v>2.9</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>1.3</v>
+        <v>2.8</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>1.2</v>
+        <v>2.7</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>1.1</v>
+        <v>2.6</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
@@ -1355,37 +1355,37 @@
       </c>
       <c r="B23" s="1" t="inlineStr"/>
       <c r="C23" s="2" t="n">
-        <v>0.08809094646749863</v>
+        <v>0.05788847985244956</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.08414191042415915</v>
+        <v>0.05438441135141131</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.07981677571002545</v>
+        <v>0.05066797506243135</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.07505912752447835</v>
+        <v>0.04671926150539013</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.06980067426676839</v>
+        <v>0.04251579223499142</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>0.06395794842486846</v>
+        <v>0.03803209167989946</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0.05742784307215678</v>
+        <v>0.03323917039687013</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>0.05008147455035611</v>
+        <v>0.02810389759362441</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>0.0417555902256487</v>
+        <v>0.0225882342123605</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>0.0322402938545545</v>
+        <v>0.01664828903253782</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0.02126110573406127</v>
+        <v>0.01023314823832933</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
@@ -1396,37 +1396,37 @@
       </c>
       <c r="B24" s="1" t="inlineStr"/>
       <c r="C24" s="2" t="n">
-        <v>0.08767872315935056</v>
+        <v>0.05024223865310477</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.05939950634481234</v>
+        <v>0.0330363490196371</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.0536755864920891</v>
+        <v>0.0290442126994289</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.05050381849451652</v>
+        <v>0.0265355854855908</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.04793195438108674</v>
+        <v>0.02438173920314907</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0.04541367178683042</v>
+        <v>0.02228205825779598</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0.04269597809250796</v>
+        <v>0.02011253337541212</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0.03964199494790194</v>
+        <v>0.01782349740153451</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0.03611915208888455</v>
+        <v>0.01538050594622177</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>0.03198951407341378</v>
+        <v>0.01275939913358668</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0.02708305425958041</v>
+        <v>0.009942032001660861</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
@@ -1437,37 +1437,37 @@
       </c>
       <c r="B25" s="1" t="inlineStr"/>
       <c r="C25" s="2" t="n">
-        <v>11.99648133201724</v>
+        <v>7.8533681131314</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>16.07918356684138</v>
+        <v>10.44938749683246</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>14.96124173007902</v>
+        <v>9.395539654564837</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>13.07809753496442</v>
+        <v>8.058495646426026</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>11.14796745181253</v>
+        <v>6.80861232521248</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>9.323490201994993</v>
+        <v>5.603082589732964</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>7.765232962313869</v>
+        <v>4.525396352380644</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>6.333545037322579</v>
+        <v>3.595063516661203</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>4.993156620152052</v>
+        <v>2.715285880504606</v>
       </c>
       <c r="L25" s="2" t="n">
-        <v>3.643410195866711</v>
+        <v>1.892543195920661</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>2.29839986631614</v>
+        <v>1.115022066201138</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
@@ -1478,37 +1478,37 @@
       </c>
       <c r="B26" s="1" t="inlineStr"/>
       <c r="C26" s="2" t="n">
-        <v>10.58767654539239</v>
+        <v>6.014783120593119</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>9.80140440930618</v>
+        <v>5.477007609425855</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>8.657486544798552</v>
+        <v>4.72628173264571</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>7.662249051449331</v>
+        <v>4.026727920356604</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>6.680438138550452</v>
+        <v>3.414405528039143</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>5.820783683216979</v>
+        <v>2.872760113081014</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>5.112286553190208</v>
+        <v>2.416158978708918</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>4.440669471090175</v>
+        <v>2.001076907645014</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>3.826959202955183</v>
+        <v>1.636059496977638</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>3.224917277717041</v>
+        <v>1.290922325166725</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>2.634410507467362</v>
+        <v>0.9685784561464872</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
@@ -1519,37 +1519,37 @@
       </c>
       <c r="B27" s="1" t="inlineStr"/>
       <c r="C27" s="2" t="n">
-        <v>0.06556969910522187</v>
+        <v>0.04315618272119882</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.06593077251562642</v>
+        <v>0.04251866605448475</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.06301880910407379</v>
+        <v>0.04160861108764319</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.06006362611519773</v>
+        <v>0.0389144853261852</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.05734198917106659</v>
+        <v>0.03526343801282697</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>0.05488348717618406</v>
+        <v>0.03228981801863431</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.05010249652374787</v>
+        <v>0.02899053531435954</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.04420860019099519</v>
+        <v>0.0245002323937855</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0.03687083324918233</v>
+        <v>0.0200664202559219</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0.02911940225893694</v>
+        <v>0.01511859509376647</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0.01936926145837068</v>
+        <v>0.00933646201072905</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -1560,37 +1560,37 @@
       </c>
       <c r="B28" s="1" t="inlineStr"/>
       <c r="C28" s="2" t="n">
-        <v>0.06322792413717823</v>
+        <v>0.036862572741024</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.04779981007382915</v>
+        <v>0.02657416628405297</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.04439961550514289</v>
+        <v>0.02384883806242963</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.04129374295419844</v>
+        <v>0.02205154168483828</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.04013939241974662</v>
+        <v>0.02051036700746059</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>0.03905171202920788</v>
+        <v>0.01919111825635813</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0.03668218495488684</v>
+        <v>0.01744345768914854</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.0346300701496129</v>
+        <v>0.01577666479902854</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0.03184299235156655</v>
+        <v>0.0136816501744922</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0.02872589682300536</v>
+        <v>0.01158544515337539</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0.02443168206680847</v>
+        <v>0.009138655612196653</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -1601,37 +1601,37 @@
       </c>
       <c r="B29" s="1" t="inlineStr"/>
       <c r="C29" s="2" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>37</v>
+        <v>63</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>47</v>
+        <v>85</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>57</v>
+        <v>105</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>73</v>
+        <v>141</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>111</v>
+        <v>231</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -1642,37 +1642,37 @@
       </c>
       <c r="B30" s="1" t="inlineStr"/>
       <c r="C30" s="2" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>52</v>
+        <v>106</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>60</v>
+        <v>132</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>66</v>
+        <v>154</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>74</v>
+        <v>184</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>88</v>
+        <v>236</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -1683,37 +1683,37 @@
       </c>
       <c r="B31" s="1" t="inlineStr"/>
       <c r="C31" s="2" t="n">
-        <v>0.08271806388838863</v>
+        <v>0.054473006470841</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.07701336982712045</v>
+        <v>0.04963096145121069</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.07204476532214493</v>
+        <v>0.04751900564477619</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.06767841590868161</v>
+        <v>0.04379202480989178</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.06381107785675695</v>
+        <v>0.03918233798779791</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>0.06036183040504035</v>
+        <v>0.03545068675086478</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.05447287134113397</v>
+        <v>0.03145624317330255</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.04751888776567006</v>
+        <v>0.02627521488593507</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>0.03918224078923672</v>
+        <v>0.02127041205051887</v>
       </c>
       <c r="L31" s="2" t="n">
-        <v>0.03059435239707525</v>
+        <v>0.01583966854825873</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>0.02012061013501345</v>
+        <v>0.009668369113872212</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -1724,37 +1724,37 @@
       </c>
       <c r="B32" s="1" t="inlineStr"/>
       <c r="C32" s="2" t="n">
-        <v>0.07976384732094619</v>
+        <v>0.04652902636051002</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.05583469312466233</v>
+        <v>0.03101935090700668</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.05075881193151121</v>
+        <v>0.0272365032354205</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.04652891093721861</v>
+        <v>0.02481548072560534</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.04466775449972986</v>
+        <v>0.0227897271969845</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>0.04294976394204794</v>
+        <v>0.02106974778589133</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.03988192366047309</v>
+        <v>0.01892706157037696</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.03722312874977488</v>
+        <v>0.01691964594927637</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>0.0338392079543408</v>
+        <v>0.01450255367080832</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>0.03018091520252018</v>
+        <v>0.01213800687665479</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>0.0253794059657556</v>
+        <v>0.00946353078518848</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -1765,37 +1765,37 @@
       </c>
       <c r="B33" s="1" t="inlineStr"/>
       <c r="C33" s="2" t="n">
-        <v>1.064954162688813</v>
+        <v>1.062700291445027</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>1.092562377325403</v>
+        <v>1.095775897971944</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1.107877516890066</v>
+        <v>1.066267578096961</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1.109055620122013</v>
+        <v>1.066844059122773</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>1.093864523389761</v>
+        <v>1.085075429859025</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>1.05957602669928</v>
+        <v>1.072816782004137</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>1.054246667345979</v>
+        <v>1.056679598188025</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>1.053927751788361</v>
+        <v>1.069597250322326</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>1.065676423414734</v>
+        <v>1.061955648001163</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>1.053798865755256</v>
+        <v>1.051050341224974</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>1.056682953021546</v>
+        <v>1.058415138872467</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -1806,37 +1806,37 @@
       </c>
       <c r="B34" s="1" t="inlineStr"/>
       <c r="C34" s="2" t="n">
-        <v>1.099228862501545</v>
+        <v>1.07980421218842</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>1.063845846026069</v>
+        <v>1.065023865866091</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1.057463412747199</v>
+        <v>1.066370835065843</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>1.08542876842016</v>
+        <v>1.069315794402911</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>1.073077322061861</v>
+        <v>1.069856562669834</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>1.05736720341716</v>
+        <v>1.057537967906594</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>1.070559646420062</v>
+        <v>1.062633695179106</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1.064982882400547</v>
+        <v>1.053420234381252</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>1.067375812625995</v>
+        <v>1.060537771163754</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>1.059925249408692</v>
+        <v>1.051193928562277</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>1.067127193446668</v>
+        <v>1.050562652284208</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -1847,37 +1847,37 @@
       </c>
       <c r="B35" s="1" t="inlineStr"/>
       <c r="C35" s="2" t="n">
-        <v>0.1623854067220315</v>
+        <v>0.1567507286125669</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.2314059433135063</v>
+        <v>0.2394397449298591</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.2696937922251647</v>
+        <v>0.1656689452424037</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.2726390503050313</v>
+        <v>0.1671101478069326</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.2346613084744031</v>
+        <v>0.2126885746475621</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>0.1489400667482005</v>
+        <v>0.1820419550103436</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.1356166683649473</v>
+        <v>0.1416989954700615</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.1348193794709029</v>
+        <v>0.1739931258058158</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>0.1641910585368361</v>
+        <v>0.1548891200029068</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>0.1344971643881404</v>
+        <v>0.1276258530624341</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>0.1417073825538662</v>
+        <v>0.1460378471811669</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -1888,37 +1888,37 @@
       </c>
       <c r="B36" s="1" t="inlineStr"/>
       <c r="C36" s="2" t="n">
-        <v>-2.251927843746138</v>
+        <v>-2.300489469528949</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>-2.340385384934827</v>
+        <v>-2.337440335334771</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>-2.356341468132002</v>
+        <v>-2.334072912335392</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>-2.286428078949599</v>
+        <v>-2.326710513992722</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>-2.317306694845348</v>
+        <v>-2.325358593325415</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>-2.356581991457099</v>
+        <v>-2.356155080233514</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>-2.323600883949846</v>
+        <v>-2.343415762052236</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>-2.337542793998631</v>
+        <v>-2.366449414046871</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>-2.331560468435012</v>
+        <v>-2.348655572090615</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>-2.35018687647827</v>
+        <v>-2.372015178594308</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>-2.33218201638333</v>
+        <v>-2.37359336928948</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -1932,34 +1932,34 @@
         <v>0.3228070637905909</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.323074478994441</v>
+        <v>0.3230602849731979</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.3232596062489652</v>
+        <v>0.3232271641850702</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.3233557544476356</v>
+        <v>0.3233004513239806</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0.3233570436213269</v>
+        <v>0.3232735693609198</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>0.3232570383862633</v>
+        <v>0.3231392117085626</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0.3230510312222958</v>
+        <v>0.3228915853001034</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.3227348281599319</v>
+        <v>0.3225251404601913</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>0.3223054666341843</v>
+        <v>0.3220352205216633</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>0.3217617658612484</v>
+        <v>0.321418525355042</v>
       </c>
       <c r="M37" s="2" t="n">
-        <v>0.3211051539846675</v>
+        <v>0.3206738288787304</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -1970,37 +1970,37 @@
       </c>
       <c r="B38" s="1" t="inlineStr"/>
       <c r="C38" s="2" t="n">
-        <v>0.2657315072231888</v>
+        <v>0.2657581721488756</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.2680887534788575</v>
+        <v>0.2681490133793929</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.2708961631488436</v>
+        <v>0.2709971595477912</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.2741937413115497</v>
+        <v>0.2743426149901204</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.2780209936980219</v>
+        <v>0.278224559371095</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>0.2824179838032992</v>
+        <v>0.2826822550061147</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.2874184716703982</v>
+        <v>0.2877480200199637</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.2930447408362419</v>
+        <v>0.2934418950502328</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>0.2993002966190627</v>
+        <v>0.299764244528729</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>0.3061617641109473</v>
+        <v>0.3066877019372144</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>0.313136364925779</v>
+        <v>0.3137134970048904</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2011,37 +2011,37 @@
       </c>
       <c r="B39" s="1" t="inlineStr"/>
       <c r="C39" s="2" t="n">
-        <v>0.2393527695658109</v>
+        <v>0.2396114809554285</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.2539937444186276</v>
+        <v>0.2536872140695393</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.2704232733200921</v>
+        <v>0.2755565742579111</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.2890375618319029</v>
+        <v>0.2945285051957288</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.3103510664937246</v>
+        <v>0.3119135649896195</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>0.3351190207521426</v>
+        <v>0.3339942131437232</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.3569796019119958</v>
+        <v>0.3575800721371906</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.3789438236241698</v>
+        <v>0.3779752735744971</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>0.3998730226111254</v>
+        <v>0.4021769585974781</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>0.4250546433436606</v>
+        <v>0.4278004452516717</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0.4486066531894552</v>
+        <v>0.4513487749732895</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
@@ -2052,37 +2052,37 @@
       </c>
       <c r="B40" s="1" t="inlineStr"/>
       <c r="C40" s="2" t="n">
-        <v>0.5121947927975168</v>
+        <v>0.5146005039945204</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.5434522265643476</v>
+        <v>0.5428186242758158</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0.5678711704934101</v>
+        <v>0.5658241595770125</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.5832868523719804</v>
+        <v>0.584868898865598</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.6004751721066423</v>
+        <v>0.599718682561613</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>0.6129555265157987</v>
+        <v>0.6112377646359372</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.6142188180752061</v>
+        <v>0.6134172831338576</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.6114502866981669</v>
+        <v>0.6107938920581668</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>0.5993809462997995</v>
+        <v>0.5973384487598037</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>0.5807240704758313</v>
+        <v>0.5784764029561554</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>0.5562622638940381</v>
+        <v>0.554915040243403</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
@@ -2093,37 +2093,37 @@
       </c>
       <c r="B41" s="1" t="inlineStr"/>
       <c r="C41" s="2" t="n">
-        <v>0.0797346228595819</v>
+        <v>0.07973629514112802</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.08577264324703664</v>
+        <v>0.08579125537495753</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.0920113450601408</v>
+        <v>0.09197117412752559</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.0984263868106539</v>
+        <v>0.09835220832820595</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.104958432558004</v>
+        <v>0.105035093325436</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>0.1115098238674079</v>
+        <v>0.1117870209523802</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0.1184092556419938</v>
+        <v>0.1186866019840878</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.1255527091495957</v>
+        <v>0.1260773587401199</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>0.1330461941971205</v>
+        <v>0.1334669535142987</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>0.1403970766254894</v>
+        <v>0.1409690896831756</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0.1480762260451801</v>
+        <v>0.1489031231639316</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
@@ -2134,37 +2134,37 @@
       </c>
       <c r="B42" s="1" t="inlineStr"/>
       <c r="C42" s="2" t="n">
-        <v>0.1426994408343503</v>
+        <v>0.1421115394167231</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.1502724333253288</v>
+        <v>0.1502140699975936</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.1581923035266436</v>
+        <v>0.1583435419166321</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.1666250868356817</v>
+        <v>0.1659223127444531</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.1729370932197975</v>
+        <v>0.1725861016572397</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>0.1780058319350655</v>
+        <v>0.1776874317051405</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.1826599053372731</v>
+        <v>0.1819533867043754</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.1849125545235307</v>
+        <v>0.1839575564929344</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>0.185339829389197</v>
+        <v>0.1844010414978863</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>0.1830452224621802</v>
+        <v>0.1818961183039974</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>0.1799372994768778</v>
+        <v>0.1784311516647284</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
@@ -2175,37 +2175,37 @@
       </c>
       <c r="B43" s="1" t="inlineStr"/>
       <c r="C43" s="2" t="n">
-        <v>0.1196763847829054</v>
+        <v>0.1198057404777143</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0.1269968722093138</v>
+        <v>0.1268436070347697</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.135211636660046</v>
+        <v>0.1377782871289555</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0.1445187809159515</v>
+        <v>0.1472642525978644</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.1551755332468623</v>
+        <v>0.1559567824948097</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>0.1675595103760713</v>
+        <v>0.1669971065718616</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.1784898009559979</v>
+        <v>0.1787900360685953</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.1894719118120849</v>
+        <v>0.1889876367872485</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>0.1999365113055627</v>
+        <v>0.201088479298739</v>
       </c>
       <c r="L43" s="2" t="n">
-        <v>0.2125273216718303</v>
+        <v>0.2139002226258358</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>0.2243033265947276</v>
+        <v>0.2256743874866448</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
@@ -2216,37 +2216,37 @@
       </c>
       <c r="B44" s="1" t="inlineStr"/>
       <c r="C44" s="2" t="n">
-        <v>0.2560973963987584</v>
+        <v>0.2573002519972602</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0.2717261132821738</v>
+        <v>0.2714093121379079</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.283935585246705</v>
+        <v>0.2829120797885062</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.2916434261859902</v>
+        <v>0.292434449432799</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.3002375860533211</v>
+        <v>0.2998593412808065</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>0.3064777632578993</v>
+        <v>0.3056188823179686</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.307109409037603</v>
+        <v>0.3067086415669288</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.3057251433490835</v>
+        <v>0.3053969460290834</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0.2996904731498998</v>
+        <v>0.2986692243799018</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>0.2903620352379156</v>
+        <v>0.2892382014780777</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0.2781311319470191</v>
+        <v>0.2774575201217015</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
@@ -2257,37 +2257,37 @@
       </c>
       <c r="B45" s="1" t="inlineStr"/>
       <c r="C45" s="2" t="n">
-        <v>34.29205694531353</v>
+        <v>34.28655162289887</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>33.53504718272685</v>
+        <v>33.54733580484677</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>32.7698202562645</v>
+        <v>32.67802913005254</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>31.99089078020046</v>
+        <v>31.90388839665297</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>31.19248913774424</v>
+        <v>31.19406171394414</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>30.3679449448747</v>
+        <v>30.43112663436511</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>29.63480886447563</v>
+        <v>29.68064932108195</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>28.93572964698342</v>
+        <v>29.02369356777023</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>28.2893561625286</v>
+        <v>28.3413892797471</v>
       </c>
       <c r="L45" s="2" t="n">
-        <v>27.61129426905793</v>
+        <v>27.67810841176009</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>26.99749191655454</v>
+        <v>27.08903621811739</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
@@ -2298,37 +2298,37 @@
       </c>
       <c r="B46" s="1" t="inlineStr"/>
       <c r="C46" s="2" t="n">
-        <v>50.48175425748313</v>
+        <v>50.43439548729882</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>48.18308588919722</v>
+        <v>48.17685013838984</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>45.87045243668208</v>
+        <v>45.87274619652885</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>43.57042138077403</v>
+        <v>43.50101038814033</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>41.11883293616422</v>
+        <v>41.06901622001109</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>38.62336069642733</v>
+        <v>38.56997876919348</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>36.1815880088439</v>
+        <v>36.09715909624808</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>33.6980773362296</v>
+        <v>33.59403292626152</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>31.25641998964364</v>
+        <v>31.15388054193205</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>28.83121370547909</v>
+        <v>28.71545735840479</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>26.49959236192144</v>
+        <v>26.35773025165374</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
@@ -2339,37 +2339,37 @@
       </c>
       <c r="B47" s="1" t="inlineStr"/>
       <c r="C47" s="2" t="n">
-        <v>0.03556876747200711</v>
+        <v>0.02342339278246163</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0.03690667073576822</v>
+        <v>0.0238130739675326</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.03807194132033433</v>
+        <v>0.02516633091482993</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.03909596698555911</v>
+        <v>0.02537346622460876</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.04000296114618677</v>
+        <v>0.02465396494584363</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>0.04081190188404387</v>
+        <v>0.02407151152970043</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.03951163656835877</v>
+        <v>0.02292583733562207</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.03680667721054885</v>
+        <v>0.0204583961798495</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0.03227807997348915</v>
+        <v>0.01762088475947854</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>0.02670941490523244</v>
+        <v>0.01391079520711551</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0.01855607223130679</v>
+        <v>0.008972516660871545</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
@@ -2380,37 +2380,37 @@
       </c>
       <c r="B48" s="1" t="inlineStr"/>
       <c r="C48" s="2" t="n">
-        <v>0.0404137283847249</v>
+        <v>0.02351059854868724</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0.03810683311248867</v>
+        <v>0.02121726883208532</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.03696207144236543</v>
+        <v>0.01989238661807359</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.03529032248834239</v>
+        <v>0.01888737402905523</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.03503046325135718</v>
+        <v>0.01794376336916201</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>0.03471872984639153</v>
+        <v>0.01710741851063369</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.0331752551048104</v>
+        <v>0.01582133915373127</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.03182643874535608</v>
+        <v>0.01454413577057599</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0.029712965668656</v>
+        <v>0.01280824109781234</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>0.02719313615804887</v>
+        <v>0.01100517459498121</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0.02344568041351307</v>
+        <v>0.008801797422939064</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
@@ -2421,37 +2421,37 @@
       </c>
       <c r="B49" s="1" t="inlineStr"/>
       <c r="C49" s="2" t="n">
-        <v>2.476637587648402</v>
+        <v>2.471396026616342</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>2.279856425592264</v>
+        <v>2.283804746315428</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>2.096472439859406</v>
+        <v>2.013323882369118</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>1.919868807752037</v>
+        <v>1.84126445680799</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>1.744887684981342</v>
+        <v>1.72450120410182</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>1.567139620363391</v>
+        <v>1.579962755266693</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>1.453441265911659</v>
+        <v>1.449856330665979</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1.360662747790846</v>
+        <v>1.373709715393299</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>1.293620632328307</v>
+        <v>1.281901250742245</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>1.207076005556323</v>
+        <v>1.196789168747309</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>1.145776189542456</v>
+        <v>1.140499218346988</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
@@ -2462,37 +2462,37 @@
       </c>
       <c r="B50" s="1" t="inlineStr"/>
       <c r="C50" s="2" t="n">
-        <v>2.169528194099763</v>
+        <v>2.137003809114428</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>1.558762602220688</v>
+        <v>1.557050027554849</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>1.452180151098536</v>
+        <v>1.460066771125404</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>1.431095408980739</v>
+        <v>1.404937787792523</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>1.368293477512882</v>
+        <v>1.358786264705836</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>1.30804531121263</v>
+        <v>1.302479286629121</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>1.286982660950723</v>
+        <v>1.271228255711137</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>1.245568040617999</v>
+        <v>1.225476555134541</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>1.21560239027188</v>
+        <v>1.200828890459344</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>1.176381932833637</v>
+        <v>1.159399973482062</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>1.155140468602947</v>
+        <v>1.129545651181444</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
@@ -2503,37 +2503,37 @@
       </c>
       <c r="B51" s="1" t="inlineStr"/>
       <c r="C51" s="2" t="n">
-        <v>3.691593969121004</v>
+        <v>3.678490066540854</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>3.199641063980661</v>
+        <v>3.20951186578857</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>2.741181099648514</v>
+        <v>2.533309705922794</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>2.299672019380092</v>
+        <v>2.103161142019975</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>1.862219212453354</v>
+        <v>1.811253010254551</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>1.417849050908477</v>
+        <v>1.449906888166733</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>1.133603164779148</v>
+        <v>1.124640826664948</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.9016568694771154</v>
+        <v>0.9342742884832472</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0.7340515808207676</v>
+        <v>0.7047531268556118</v>
       </c>
       <c r="L51" s="2" t="n">
-        <v>0.517690013890808</v>
+        <v>0.4919729218682728</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>0.3644404738561396</v>
+        <v>0.3512480458674705</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
@@ -2544,37 +2544,37 @@
       </c>
       <c r="B52" s="1" t="inlineStr"/>
       <c r="C52" s="2" t="n">
-        <v>0.4238204852494087</v>
+        <v>0.3425095227860697</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>-1.103093494448279</v>
+        <v>-1.107374931112877</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>-1.369549622253661</v>
+        <v>-1.34983307218649</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>-1.422261477548152</v>
+        <v>-1.487655530518692</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>-1.579266306217794</v>
+        <v>-1.603034338235409</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>-1.729886721968426</v>
+        <v>-1.743801783427199</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>-1.782543347623192</v>
+        <v>-1.821929360722159</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>-1.886079898455002</v>
+        <v>-1.936308612163648</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>-1.960994024320299</v>
+        <v>-1.997927773851639</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>-2.059045167915908</v>
+        <v>-2.101500066294844</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>-2.112148828492634</v>
+        <v>-2.17613587204639</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
@@ -2585,37 +2585,37 @@
       </c>
       <c r="B53" s="1" t="inlineStr"/>
       <c r="C53" s="2" t="n">
-        <v>0.2474271985205285</v>
+        <v>0.2471465010949953</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>0.279033987290496</v>
+        <v>0.2792786854553043</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.2854539513780725</v>
+        <v>0.2857811351935611</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0.2891424595675562</v>
+        <v>0.289522149012689</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.2920390361881434</v>
+        <v>0.2924660637659758</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>0.2946390881086</v>
+        <v>0.2951116756352958</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.297139956884392</v>
+        <v>0.2976586518274703</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.2996212554865067</v>
+        <v>0.3001864148364644</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0.3021400529060791</v>
+        <v>0.3027512429645513</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>0.3047361677903553</v>
+        <v>0.3053957126985964</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0.3074441322625881</v>
+        <v>0.3081563553984701</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
@@ -2626,37 +2626,37 @@
       </c>
       <c r="B54" s="1" t="inlineStr"/>
       <c r="C54" s="2" t="n">
-        <v>0.2657315072231888</v>
+        <v>0.2657581721488756</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>0.2680887534788575</v>
+        <v>0.2681490133793929</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.2708961631488436</v>
+        <v>0.2709971595477912</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>0.2741937413115497</v>
+        <v>0.2743426149901204</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.2780209936980219</v>
+        <v>0.278224559371095</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>0.2824179838032992</v>
+        <v>0.2826822550061147</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.2874184716703982</v>
+        <v>0.2877480200199637</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.2930447408362419</v>
+        <v>0.2934418950502328</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0.2993002966190627</v>
+        <v>0.2997642445287291</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>0.3061617641109473</v>
+        <v>0.3066877019372144</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0.313136364925779</v>
+        <v>0.3137134970048904</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
@@ -2667,37 +2667,37 @@
       </c>
       <c r="B55" s="1" t="inlineStr"/>
       <c r="C55" s="2" t="n">
-        <v>0.2587207385462206</v>
+        <v>0.2618949270690872</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>0.03757571334013546</v>
+        <v>0.03550209488243607</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.07381595707773488</v>
+        <v>0.07658956610249039</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>0.1361294154214472</v>
+        <v>0.1390315873175538</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.2040566890803394</v>
+        <v>0.2031812135733084</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>0.2728248403034224</v>
+        <v>0.2691432391962249</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>0.3344869132545552</v>
+        <v>0.3318558856581675</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.3909194222906661</v>
+        <v>0.3860843391407</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>0.4404560087331414</v>
+        <v>0.4379161103630089</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>0.488106834907179</v>
+        <v>0.4849335474476257</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>0.527969269269892</v>
+        <v>0.5234505100335498</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
@@ -2708,37 +2708,37 @@
       </c>
       <c r="B56" s="1" t="inlineStr"/>
       <c r="C56" s="2" t="n">
-        <v>0.409566208189467</v>
+        <v>0.4117100293844798</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>0.4846772033561549</v>
+        <v>0.4844023222038345</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.5173521751173826</v>
+        <v>0.515849069111718</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.5380071429589364</v>
+        <v>0.5400559429492678</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.5593878562373842</v>
+        <v>0.5592863517090041</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>0.575871813144094</v>
+        <v>0.5749382624348064</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.5814734453221611</v>
+        <v>0.581489969945292</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.5830288538880268</v>
+        <v>0.5832676489139323</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0.5754998784313891</v>
+        <v>0.574496497919317</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>0.5614238467896036</v>
+        <v>0.5603075811629855</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>0.5415987240447843</v>
+        <v>0.5414478465154466</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
@@ -2749,37 +2749,37 @@
       </c>
       <c r="B57" s="1" t="inlineStr"/>
       <c r="C57" s="2" t="n">
-        <v>0.1007418472750847</v>
+        <v>0.1017542891489504</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>0.01583135501959349</v>
+        <v>0.01498377550446164</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.03050920513055261</v>
+        <v>0.03105703480736935</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.05453805265085377</v>
+        <v>0.05462020926452753</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.07871825911935569</v>
+        <v>0.07803524190948873</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>0.1006301492182104</v>
+        <v>0.09983740671436131</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.119822652688742</v>
+        <v>0.1189407080495123</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.1366265541611752</v>
+        <v>0.1358378204073504</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0.1513611109871712</v>
+        <v>0.1501081052555216</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>0.163420373733545</v>
+        <v>0.1620145393657782</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>0.173749974728821</v>
+        <v>0.172263890888112</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
@@ -2790,37 +2790,37 @@
       </c>
       <c r="B58" s="1" t="inlineStr"/>
       <c r="C58" s="2" t="n">
-        <v>0.1603060146952187</v>
+        <v>0.1599487030376185</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>0.1622262680463858</v>
+        <v>0.1620815954847321</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.1688882289395252</v>
+        <v>0.1689171512790251</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0.1764736520771516</v>
+        <v>0.1756145803795007</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.1819199188647715</v>
+        <v>0.1813866244173785</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>0.1860071182149297</v>
+        <v>0.1854834528812329</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.1895967592981207</v>
+        <v>0.1886541402137852</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.1906811261688446</v>
+        <v>0.1894708969514859</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>0.1899101409719913</v>
+        <v>0.188715589976583</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0.1864300775242289</v>
+        <v>0.1850288727577945</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>0.1822756005209552</v>
+        <v>0.1805268185451869</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
@@ -2831,37 +2831,37 @@
       </c>
       <c r="B59" s="1" t="inlineStr"/>
       <c r="C59" s="2" t="n">
-        <v>0.1293603692731103</v>
+        <v>0.1309474635345436</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>0.01878785667006773</v>
+        <v>0.01775104744121804</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.03690797853886744</v>
+        <v>0.03829478305124519</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.06806470771072362</v>
+        <v>0.06951579365877691</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.1020283445401697</v>
+        <v>0.1015906067866542</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>0.1364124201517112</v>
+        <v>0.1345716195981125</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.1672434566272776</v>
+        <v>0.1659279428290838</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.1954597111453331</v>
+        <v>0.19304216957035</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0.2202280043665707</v>
+        <v>0.2189580551815044</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>0.2440534174535895</v>
+        <v>0.2424667737238129</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>0.263984634634946</v>
+        <v>0.2617252550167749</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
@@ -2872,37 +2872,37 @@
       </c>
       <c r="B60" s="1" t="inlineStr"/>
       <c r="C60" s="2" t="n">
-        <v>0.2047831040947335</v>
+        <v>0.2058550146922399</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0.2423386016780775</v>
+        <v>0.2422011611019173</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>0.2586760875586913</v>
+        <v>0.257924534555859</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.2690035714794682</v>
+        <v>0.2700279714746339</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.2796939281186921</v>
+        <v>0.279643175854502</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>0.287935906572047</v>
+        <v>0.2874691312174032</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.2907367226610805</v>
+        <v>0.290744984972646</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.2915144269440134</v>
+        <v>0.2916338244569662</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0.2877499392156945</v>
+        <v>0.2872482489596585</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>0.2807119233948018</v>
+        <v>0.2801537905814928</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>0.2707993620223921</v>
+        <v>0.2707239232577233</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
@@ -2913,37 +2913,37 @@
       </c>
       <c r="B61" s="1" t="inlineStr"/>
       <c r="C61" s="2" t="n">
-        <v>68.92276727815506</v>
+        <v>68.91125046983635</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>63.74672712198674</v>
+        <v>63.72019901913738</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>58.91439424380116</v>
+        <v>58.64329877649394</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>54.32480529111023</v>
+        <v>54.04216938205894</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>49.97574515179116</v>
+        <v>49.81981864350208</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>45.86426889065956</v>
+        <v>45.77846647037669</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>42.15607828172189</v>
+        <v>42.02298856503295</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>38.73996954516696</v>
+        <v>38.64446364461252</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>35.61786944277189</v>
+        <v>35.46181431465674</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>32.66651549125832</v>
+        <v>32.51634293361779</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>29.98006336147639</v>
+        <v>29.84614221799288</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
@@ -2954,37 +2954,37 @@
       </c>
       <c r="B62" s="1" t="inlineStr"/>
       <c r="C62" s="2" t="n">
-        <v>53.10618829417465</v>
+        <v>53.02594924230883</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>49.39099026807968</v>
+        <v>49.37770739157574</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>46.83198478487241</v>
+        <v>46.83199849144511</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>44.41194812746895</v>
+        <v>44.31765889365619</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>41.83632966685715</v>
+        <v>41.7711243096748</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>39.23151410923014</v>
+        <v>39.16418231489922</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>36.70627285879404</v>
+        <v>36.60268184098388</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>34.13532951536816</v>
+        <v>34.01041060657262</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>31.61504589982413</v>
+        <v>31.49318736475078</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>29.11270530219834</v>
+        <v>28.97688805980768</v>
       </c>
       <c r="M62" s="2" t="n">
-        <v>26.7122937798875</v>
+        <v>26.54845415203285</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
@@ -2995,37 +2995,37 @@
       </c>
       <c r="B63" s="1" t="inlineStr"/>
       <c r="C63" s="2" t="n">
-        <v>19.50846214460636</v>
+        <v>12.66450061683238</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>128.3003303284896</v>
+        <v>87.76939225433988</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>61.95360569507856</v>
+        <v>37.90413618231608</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>31.59179240791338</v>
+        <v>19.25330217834851</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>19.59889761174122</v>
+        <v>11.98918291346836</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>13.43178271083509</v>
+        <v>8.096359207438532</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>9.837089514317523</v>
+        <v>5.738837015131057</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>7.340291951712707</v>
+        <v>4.170689155746326</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>5.431700180127948</v>
+        <v>2.955391698416143</v>
       </c>
       <c r="L63" s="2" t="n">
-        <v>3.784495979067797</v>
+        <v>1.96703146191539</v>
       </c>
       <c r="M63" s="2" t="n">
-        <v>2.307285683424119</v>
+        <v>1.120102536913406</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
@@ -3036,37 +3036,37 @@
       </c>
       <c r="B64" s="1" t="inlineStr"/>
       <c r="C64" s="2" t="n">
-        <v>12.26573722484221</v>
+        <v>6.991994889379535</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>7.02189239056047</v>
+        <v>3.90759688772624</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>5.944490357632755</v>
+        <v>3.225975439455065</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>5.378490448946372</v>
+        <v>2.815231835392211</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>4.909490913253908</v>
+        <v>2.497783640747444</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>4.518406038454767</v>
+        <v>2.220539728792237</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>4.2070878124316</v>
+        <v>1.981750817528045</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>3.895739955796507</v>
+        <v>1.750852440969198</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>3.595975866141877</v>
+        <v>1.533937582335717</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>3.264684049564287</v>
+        <v>1.304752348750222</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>2.865129502236727</v>
+        <v>1.0520654884007</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
@@ -3077,37 +3077,37 @@
       </c>
       <c r="B65" s="1" t="inlineStr"/>
       <c r="C65" s="2" t="n">
-        <v>0.02202273661687466</v>
+        <v>0.01447211996311239</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0.02103547760603979</v>
+        <v>0.01359610283785283</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.01995419392750636</v>
+        <v>0.01266699376560784</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.01876478188111959</v>
+        <v>0.01167981537634753</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.0174501685666921</v>
+        <v>0.01062894805874785</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>0.01598948710621712</v>
+        <v>0.009508022919974865</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>0.01435696076803919</v>
+        <v>0.008309792599217531</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.01252036863758903</v>
+        <v>0.007025974398406101</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>0.01043889755641218</v>
+        <v>0.005647058553090126</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>0.008060073463638625</v>
+        <v>0.004162072258134456</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>0.005315276433515318</v>
+        <v>0.002558287059582331</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
@@ -3118,37 +3118,37 @@
       </c>
       <c r="B66" s="1" t="inlineStr"/>
       <c r="C66" s="2" t="n">
-        <v>0.02191968078983764</v>
+        <v>0.01256055966327619</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0.01484987658620308</v>
+        <v>0.008259087254909274</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>0.01341889662302227</v>
+        <v>0.007261053174857226</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0.01262595462362913</v>
+        <v>0.006633896371397701</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.01198298859527169</v>
+        <v>0.006095434800787267</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>0.01135341794670761</v>
+        <v>0.005570514564448996</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>0.01067399452312699</v>
+        <v>0.005028133343853029</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.009910498736975484</v>
+        <v>0.004455874350383628</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>0.009029788022221139</v>
+        <v>0.003845126486555443</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>0.007997378518353445</v>
+        <v>0.00318984978339667</v>
       </c>
       <c r="M66" s="2" t="n">
-        <v>0.006770763564895102</v>
+        <v>0.002485508000415215</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
@@ -3159,37 +3159,37 @@
       </c>
       <c r="B67" s="1" t="inlineStr"/>
       <c r="C67" s="2" t="n">
-        <v>0.08219735479291895</v>
+        <v>0.05401135289295622</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>0.07546245994217911</v>
+        <v>0.04876337861864726</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0.06835483327337574</v>
+        <v>0.04326762767249133</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>0.06097323784258143</v>
+        <v>0.03781687735148853</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.05345142044310348</v>
+        <v>0.0324828835743967</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>0.04590211874137408</v>
+        <v>0.02725564300495917</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.03854284085319139</v>
+        <v>0.02225125534678672</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.03134033233572431</v>
+        <v>0.01755048771446508</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>0.02431747583577096</v>
+        <v>0.01310479552914998</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>0.01740164820955814</v>
+        <v>0.008949123846660013</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>0.01062414535553529</v>
+        <v>0.005092757904332724</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
@@ -3200,37 +3200,37 @@
       </c>
       <c r="B68" s="1" t="inlineStr"/>
       <c r="C68" s="2" t="n">
-        <v>0.07012101525937343</v>
+        <v>0.04013892589465536</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>0.04509426169605621</v>
+        <v>0.02507518511351156</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0.03914832417950787</v>
+        <v>0.02118342031733042</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.03534319425123329</v>
+        <v>0.0185387108681091</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.03197085428227402</v>
+        <v>0.01624205853048202</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>0.02872212403794324</v>
+        <v>0.01407211653503559</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0.02551993788422295</v>
+        <v>0.01199234846140843</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.02224508499006836</v>
+        <v>0.009969457950614847</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>0.01893400452833329</v>
+        <v>0.008034732927449811</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>0.01556383035184584</v>
+        <v>0.006181377383190171</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>0.01217412203468798</v>
+        <v>0.004443635798839883</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
@@ -3241,37 +3241,37 @@
       </c>
       <c r="B69" s="1" t="inlineStr"/>
       <c r="C69" s="2" t="n">
-        <v>0.06405822095022083</v>
+        <v>0.04209242610150406</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>0.05917486075968466</v>
+        <v>0.03824971672294817</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0.05436108114774698</v>
+        <v>0.03442711387548201</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.04939049517237393</v>
+        <v>0.03066277128379772</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.04424162220970736</v>
+        <v>0.02692425923818854</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>0.03891046792788381</v>
+        <v>0.02314554452478348</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0.03350964149039595</v>
+        <v>0.01938674024497689</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.02796726334832917</v>
+        <v>0.01569914851205892</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>0.02227723181218233</v>
+        <v>0.01203703317602205</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>0.01636115566134978</v>
+        <v>0.008437647672236199</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>0.01024488774297561</v>
+        <v>0.004925239131243734</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
@@ -3282,37 +3282,37 @@
       </c>
       <c r="B70" s="1" t="inlineStr"/>
       <c r="C70" s="2" t="n">
-        <v>0.06157720338866012</v>
+        <v>0.03523964506601306</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0.04134466339688302</v>
+        <v>0.02299952367411574</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0.03613366471312308</v>
+        <v>0.01956387574848632</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>0.03273043521643305</v>
+        <v>0.01718209975939567</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.02969889527346289</v>
+        <v>0.01510285858147681</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>0.02677849559923044</v>
+        <v>0.01313589721585449</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0.02390232985638472</v>
+        <v>0.0112489478345701</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.02095424712855832</v>
+        <v>0.009407785548860381</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>0.01795904743207712</v>
+        <v>0.007637246156388489</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>0.01488331537713343</v>
+        <v>0.005925951720486575</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>0.01175057516963411</v>
+        <v>0.004301654620225066</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
@@ -3323,37 +3323,37 @@
       </c>
       <c r="B71" s="1" t="inlineStr"/>
       <c r="C71" s="2" t="n">
-        <v>0.04963145400225756</v>
+        <v>0.03261044082545702</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>0.0464839426715804</v>
+        <v>0.03005422473505339</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>0.04320205731947549</v>
+        <v>0.02735653106991717</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>0.03976515708176084</v>
+        <v>0.02469094045728014</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.03615080754648142</v>
+        <v>0.02202055946526221</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>0.03233401358859338</v>
+        <v>0.01926334040912139</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>0.02839634665716753</v>
+        <v>0.01645888293710986</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.02423083113304251</v>
+        <v>0.01363520343291549</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>0.019789002839435</v>
+        <v>0.0107231796952561</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>0.01494243209295661</v>
+        <v>0.007733192193019188</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>0.009651510756827819</v>
+        <v>0.004659915305130723</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
@@ -3364,37 +3364,37 @@
       </c>
       <c r="B72" s="1" t="inlineStr"/>
       <c r="C72" s="2" t="n">
-        <v>0.06763729477145963</v>
+        <v>0.0387315286892632</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.04426921669989489</v>
+        <v>0.02461890639280539</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>0.03852658178430277</v>
+        <v>0.02084779625039499</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>0.03480953479501307</v>
+        <v>0.01826623111977542</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.03152115103980984</v>
+        <v>0.01601801380947973</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>0.02834713160373665</v>
+        <v>0.01389219527050886</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>0.02520541356878222</v>
+        <v>0.01184942562573182</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.0219940332629067</v>
+        <v>0.009861826693401032</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0.01874111004961566</v>
+        <v>0.007956925227012038</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>0.01542633531748339</v>
+        <v>0.006130382413758983</v>
       </c>
       <c r="M72" s="2" t="n">
-        <v>0.01208422714149282</v>
+        <v>0.004414006203627959</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
again edit export files
</commit_message>
<xml_diff>
--- a/results/Профилирование_лопаток.xlsx
+++ b/results/Профилирование_лопаток.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:N87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -515,3126 +515,3742 @@
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>ε_РК_x</t>
+          <t>D_к1_i</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr"/>
       <c r="C2" s="2" t="n">
-        <v>65.86015860158602</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>58.74728747287473</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>57.1790217902179</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>56.3120131201312</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>55.63880638806388</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>55.01830018300183</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>54.38759387593876</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>53.71013710137102</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>52.95277952779528</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>52.0789707897079</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>51.04876048760488</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>49.81624816248163</v>
+        <v>0.6807728945329433</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>ε_РК_i</t>
+          <t>D_к2_i</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr"/>
       <c r="C3" s="2" t="n">
-        <v>22.73182157254356</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>19.49854778014516</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>18.79353980328821</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>18.40463436665847</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>18.10299642520362</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>17.82518107529433</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>17.54295745421819</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>17.23993552100599</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>16.90124379958324</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>16.51044195220687</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>16.0494356894103</v>
+        <v>0.6807728945329433</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>15.49715997861603</v>
+        <v>0.6807728945329433</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>bt_1_x</t>
+          <t>D_ср1_i</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr"/>
       <c r="C4" s="2" t="n">
-        <v>0.5959449594495945</v>
+        <v>0.4867526195910545</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.5</v>
+        <v>0.501832502447439</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.5</v>
+        <v>0.5169123853038237</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.5740172401724017</v>
+        <v>0.5319922681602083</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.6678857788577885</v>
+        <v>0.5470721510165928</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.7672317723177232</v>
+        <v>0.5621520338729775</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.8694954949549496</v>
+        <v>0.577231916729362</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0.9732449324493245</v>
+        <v>0.5923117995857468</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>1.07749557495575</v>
+        <v>0.6073916824421313</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>1.181531415314153</v>
+        <v>0.6224715652985159</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1.284725947259473</v>
+        <v>0.6375514481549005</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1.386882268822688</v>
+        <v>0.652631331011285</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>bt_1ср_i</t>
+          <t>D_ср2_i</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr"/>
       <c r="C5" s="2" t="n">
-        <v>1.361459495072957</v>
+        <v>0.499513600828743</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.244749296801998</v>
+        <v>0.5675288881640966</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1.254119507037462</v>
+        <v>0.5844542258540137</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1.206436006567531</v>
+        <v>0.5949265769048206</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>1.196017453808264</v>
+        <v>0.6034225179525432</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.166365032040376</v>
+        <v>0.6111218150628972</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>1.151847098547373</v>
+        <v>0.6184683559077462</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1.168887338473666</v>
+        <v>0.6256246358243144</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>1.131683349016788</v>
+        <v>0.6326628619275969</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>1.124773200734969</v>
+        <v>0.6396082573033322</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>1.113603383524838</v>
+        <v>0.6464562235743894</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1.101858787170988</v>
+        <v>0.6531775376318343</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>ε_НА_x</t>
+          <t>D_вт1_i</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr"/>
       <c r="C6" s="2" t="n">
-        <v>65.79555795557955</v>
+        <v>0.2927323446491656</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>59.92709927099271</v>
+        <v>0.3228921103619348</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>58.41323413234132</v>
+        <v>0.3530518760747041</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>57.46292462924629</v>
+        <v>0.3832116417874732</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>56.65286652866529</v>
+        <v>0.4133714075002424</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>55.86150861508615</v>
+        <v>0.4435311732130116</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>55.02850028500285</v>
+        <v>0.4736909389257808</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>54.11559115591156</v>
+        <v>0.5038507046385501</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>53.08538085380854</v>
+        <v>0.5340104703513192</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>51.89536895368954</v>
+        <v>0.5641702360640884</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>50.49370493704937</v>
+        <v>0.5943300017768577</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>48.82258822588226</v>
+        <v>0.6244897674896268</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>ε_НА_i</t>
+          <t>D_вт2_i</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr"/>
       <c r="C7" s="2" t="n">
-        <v>22.70215077764346</v>
+        <v>0.3182543071245426</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>20.03050783437985</v>
+        <v>0.45428488179525</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>19.34818761846924</v>
+        <v>0.4881355571750841</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>18.92100922637824</v>
+        <v>0.5090802592766979</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>18.55746447090211</v>
+        <v>0.526072141372143</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>18.20275196411341</v>
+        <v>0.5414707355928511</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>17.82974652363652</v>
+        <v>0.5561638172825492</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>17.42128077964202</v>
+        <v>0.5704763771156854</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>16.96054205221007</v>
+        <v>0.5845528293222505</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>16.42830951051472</v>
+        <v>0.598443620073721</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>15.8008481474968</v>
+        <v>0.6121395526158354</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>15.05098807453122</v>
+        <v>0.6255821807307252</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>bt_2_x</t>
+          <t>S_в_РК_i</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr"/>
       <c r="C8" s="2" t="n">
-        <v>0.6018162181621817</v>
+        <v>0.05348065161085038</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.5</v>
+        <v>0.04935244672483962</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.5</v>
+        <v>0.04502393831156841</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.5268323683236832</v>
+        <v>0.0403932297369132</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.6249074490744908</v>
+        <v>0.03570359291219267</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.7312524125241253</v>
+        <v>0.03095986565509889</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0.8424483244832448</v>
+        <v>0.02629641552912036</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0.9565619656196562</v>
+        <v>0.02179981936945496</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>1.072215022150222</v>
+        <v>0.0174220548346053</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>1.188261882618826</v>
+        <v>0.01330970194045197</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1.304022340223402</v>
+        <v>0.009454337808190653</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>1.419406894068941</v>
+        <v>0.005880451855633163</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>bt_2ср_i</t>
+          <t>S_в_НА_i</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr"/>
       <c r="C9" s="2" t="n">
-        <v>1.364981334382785</v>
+        <v>0.04465635870911464</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1.245745100108579</v>
+        <v>0.02741770449389811</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1.223409472435786</v>
+        <v>0.02318550569353218</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1.193336115742473</v>
+        <v>0.0204784656919946</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>1.174986203758765</v>
+        <v>0.01822035692341738</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.177477160218605</v>
+        <v>0.01614278537928499</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1.1661853217552</v>
+        <v>0.01412746963743333</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>1.157943254299948</v>
+        <v>0.0121706120674842</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>1.14421483298957</v>
+        <v>0.01027183699361799</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>1.116548947947683</v>
+        <v>0.008444034212239363</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1.106901430168325</v>
+        <v>0.00672959614882052</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>1.097267445213182</v>
+        <v>0.00514094589581024</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>i_рк_i</t>
+          <t>S_ср_РК_i</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr"/>
       <c r="C10" s="2" t="n">
-        <v>0.9036487376823932</v>
+        <v>0.04448146661709266</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.6118732420049944</v>
+        <v>0.04080380248333932</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.6352987675936544</v>
+        <v>0.0372905260295658</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.516090016418827</v>
+        <v>0.03366047207473166</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.4900436345206605</v>
+        <v>0.0300558749697196</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0.4159125801009395</v>
+        <v>0.02641565437523911</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.379617746368433</v>
+        <v>0.02280380767342325</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0.4222183461841644</v>
+        <v>0.01925557442008509</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0.3292083725419703</v>
+        <v>0.01570097082549171</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>0.3119330018374228</v>
+        <v>0.01225179121567093</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0.284008458812095</v>
+        <v>0.008895152825414362</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.2546469679274699</v>
+        <v>0.005656269385850665</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>i_на_i</t>
+          <t>S_ср_НА_i</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr"/>
       <c r="C11" s="2" t="n">
-        <v>-1.587546664043038</v>
+        <v>0.04008746233962627</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>-1.885637249728552</v>
+        <v>0.0255432593625421</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-1.941476318910534</v>
+        <v>0.02168935847875152</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-2.016659710643817</v>
+        <v>0.0191741161370407</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-2.062534490603087</v>
+        <v>0.01706723427804866</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>-2.056307099453487</v>
+        <v>0.01513339634946587</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>-2.084536695612</v>
+        <v>0.0132654841102659</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>-2.10514186425013</v>
+        <v>0.0114580375728913</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>-2.139462917526076</v>
+        <v>0.009706961431880611</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>-2.208627630130793</v>
+        <v>0.008019610838336058</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>-2.232746424579187</v>
+        <v>0.006431329457920825</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-2.256831386967044</v>
+        <v>0.004949255210666078</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>X_f_отн</t>
+          <t>S_к_РК_i</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr"/>
       <c r="C12" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D12" s="1" t="inlineStr"/>
-      <c r="E12" s="1" t="inlineStr"/>
-      <c r="F12" s="1" t="inlineStr"/>
-      <c r="G12" s="1" t="inlineStr"/>
-      <c r="H12" s="1" t="inlineStr"/>
-      <c r="I12" s="1" t="inlineStr"/>
-      <c r="J12" s="1" t="inlineStr"/>
-      <c r="K12" s="1" t="inlineStr"/>
-      <c r="L12" s="1" t="inlineStr"/>
-      <c r="M12" s="1" t="inlineStr"/>
-      <c r="N12" s="1" t="inlineStr"/>
+        <v>0.03529297818838117</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>0.0326517455312112</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0.03006171193335206</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0.02735388853024765</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0.02467509740809998</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0.02194795422776095</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0.01921914512347143</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>0.01650314711364222</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>0.01370996279618971</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>0.01092945770959476</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>0.008128018298888534</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0.005309553953316647</v>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>m_рк_i</t>
+          <t>S_к_НА_i</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr"/>
       <c r="C13" s="2" t="n">
-        <v>0.278280383393174</v>
+        <v>0.04323053019914518</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.2925060337085559</v>
+        <v>0.02698397035490908</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.2956423088465648</v>
+        <v>0.02286398367976868</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.2973763371712121</v>
+        <v>0.02021385051689902</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.2987231567492909</v>
+        <v>0.01799499497206569</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>0.2999634266313577</v>
+        <v>0.01594775050048612</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.3012241705710921</v>
+        <v>0.01396300280667979</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>0.302579389711173</v>
+        <v>0.01203470518695078</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>0.304094923198526</v>
+        <v>0.01016347391261594</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>0.3058415916829391</v>
+        <v>0.008362116810762451</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0.3079016558590607</v>
+        <v>0.006669958596379822</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.3103677360799227</v>
+        <v>0.005100603145579266</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>m_на_i</t>
+          <t>S_1_i</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr"/>
       <c r="C14" s="2" t="n">
-        <v>0.2784088862773235</v>
+        <v>0.01385859106727777</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.290145758525186</v>
+        <v>0.01315738177099296</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.2931740075161676</v>
+        <v>0.01241367494159997</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.2950743805877517</v>
+        <v>0.01162348643536992</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.2966941167788055</v>
+        <v>0.01078231802551213</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>0.2982774621942075</v>
+        <v>0.009885071721663821</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.2999430459044465</v>
+        <v>0.008925946362377693</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>0.3017683087548075</v>
+        <v>0.007898312048856842</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>0.3038284072773666</v>
+        <v>0.00679455667507519</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>0.306208816044133</v>
+        <v>0.005605897041771868</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0.3090118087713087</v>
+        <v>0.004322144637804282</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.3123553769535541</v>
+        <v>0.002931412866839401</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>θ_рк_i</t>
+          <t>S_2_i</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr"/>
       <c r="C15" s="2" t="n">
-        <v>0.2897752077348815</v>
+        <v>0.01294709240744288</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.1894596498726411</v>
+        <v>0.008326765174179901</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.204032939286868</v>
+        <v>0.007296868839312849</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.2404874621568816</v>
+        <v>0.006706743564697088</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.2785555181894611</v>
+        <v>0.006237933595193562</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>0.3204358653219178</v>
+        <v>0.005804256622503843</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0.3608863595821978</v>
+        <v>0.005371080915965266</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>0.3964156754475768</v>
+        <v>0.004923951670413299</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>0.4370220505788445</v>
+        <v>0.004454632648643186</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>0.4707937585285812</v>
+        <v>0.00395813819515492</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0.5011293448307715</v>
+        <v>0.003431667095855395</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.5262816246511876</v>
+        <v>0.002874516343865525</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>θ_на_i</t>
+          <t>ε_РК_x</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr"/>
       <c r="C16" s="2" t="n">
-        <v>0.3494339757321023</v>
+        <v>65.86015860158602</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.235090332136063</v>
+        <v>58.74728747287473</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.2503395106870253</v>
+        <v>57.1790217902179</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.2865856164178282</v>
+        <v>56.3120131201312</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.3282430011756985</v>
+        <v>55.63880638806388</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>0.3698767712696619</v>
+        <v>55.01830018300183</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0.4133462955498508</v>
+        <v>54.38759387593876</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0.4552656912836749</v>
+        <v>53.71013710137102</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0.4954632889968579</v>
+        <v>52.95277952779528</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>0.5340049796103393</v>
+        <v>52.0789707897079</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0.5643430223457975</v>
+        <v>51.04876048760488</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.5874142888999352</v>
+        <v>49.81624816248163</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>χ_рк_i</t>
+          <t>ε_РК_i</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr"/>
       <c r="C17" s="2" t="n">
-        <v>0.1448876038674407</v>
+        <v>22.73182157254356</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.09472982493632053</v>
+        <v>19.49854778014516</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.102016469643434</v>
+        <v>18.79353980328821</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0.1202437310784408</v>
+        <v>18.40463436665847</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.1392777590947306</v>
+        <v>18.10299642520362</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>0.1602179326609589</v>
+        <v>17.82518107529433</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.1804431797910989</v>
+        <v>17.54295745421819</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>0.1982078377237884</v>
+        <v>17.23993552100599</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>0.2185110252894223</v>
+        <v>16.90124379958324</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>0.2353968792642906</v>
+        <v>16.51044195220687</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0.2505646724153858</v>
+        <v>16.0494356894103</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.2631408123255938</v>
+        <v>15.49715997861603</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>χ_на_i</t>
+          <t>bt_1_x</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr"/>
       <c r="C18" s="2" t="n">
-        <v>0.1747169878660511</v>
+        <v>0.5959449594495945</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.1175451660680315</v>
+        <v>0.5</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.1251697553435127</v>
+        <v>0.5</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.1432928082089141</v>
+        <v>0.5740172401724017</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.1641215005878493</v>
+        <v>0.6678857788577885</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>0.1849383856348309</v>
+        <v>0.7672317723177232</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.2066731477749254</v>
+        <v>0.8694954949549496</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0.2276328456418374</v>
+        <v>0.9732449324493245</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0.247731644498429</v>
+        <v>1.07749557495575</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>0.2670024898051697</v>
+        <v>1.181531415314153</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0.2821715111728987</v>
+        <v>1.284725947259473</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.2937071444499676</v>
+        <v>1.386882268822688</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>v_рк_i</t>
+          <t>bt_1ср_i</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr"/>
       <c r="C19" s="2" t="n">
-        <v>53.36151595490971</v>
+        <v>1.361459495072957</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>50.83246384023893</v>
+        <v>1.244749296801998</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>48.67680714295572</v>
+        <v>1.254119507037462</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>46.38367820929632</v>
+        <v>1.206436006567531</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>44.17712222971348</v>
+        <v>1.196017453808264</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>41.91823182418606</v>
+        <v>1.166365032040376</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>39.69453263128516</v>
+        <v>1.151847098547373</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>37.55219102641462</v>
+        <v>1.168887338473666</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>35.28921715191872</v>
+        <v>1.131683349016788</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>33.11899142444339</v>
+        <v>1.124773200734969</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>30.96473257991795</v>
+        <v>1.113603383524838</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>28.84123613160006</v>
+        <v>1.101858787170988</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>v_на_i</t>
+          <t>ε_НА_x</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr"/>
       <c r="C20" s="2" t="n">
-        <v>50.72016075131927</v>
+        <v>65.79555795557955</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>50.07652160407117</v>
+        <v>59.92709927099271</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>47.99658880520145</v>
+        <v>58.41323413234132</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>45.62129843758604</v>
+        <v>57.46292462924629</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>43.15779401816041</v>
+        <v>56.65286652866529</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>40.6792043031489</v>
+        <v>55.86150861508615</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>38.13011904016454</v>
+        <v>55.02850028500285</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>35.5737299611924</v>
+        <v>54.11559115591156</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>33.00879625441686</v>
+        <v>53.08538085380854</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>30.43275117827625</v>
+        <v>51.89536895368954</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>27.93879278458221</v>
+        <v>50.49370493704937</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>25.49564119157854</v>
+        <v>48.82258822588226</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>h_рк_i_отн</t>
+          <t>ε_НА_i</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr"/>
       <c r="C21" s="2" t="n">
-        <v>3.5</v>
+        <v>22.70215077764346</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>3.4</v>
+        <v>20.03050783437985</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>3.3</v>
+        <v>19.34818761846924</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>3.2</v>
+        <v>18.92100922637824</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>3.1</v>
+        <v>18.55746447090211</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>3</v>
+        <v>18.20275196411341</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>2.9</v>
+        <v>17.82974652363652</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>2.8</v>
+        <v>17.42128077964202</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>2.7</v>
+        <v>16.96054205221007</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>2.6</v>
+        <v>16.42830951051472</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>2.5</v>
+        <v>15.8008481474968</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>2.4</v>
+        <v>15.05098807453122</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>h_на_i_отн</t>
+          <t>bt_2_x</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr"/>
       <c r="C22" s="2" t="n">
-        <v>3.5</v>
+        <v>0.6018162181621817</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>3.4</v>
+        <v>0.5</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>3.3</v>
+        <v>0.5</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>3.2</v>
+        <v>0.5268323683236832</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>3.1</v>
+        <v>0.6249074490744908</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>3</v>
+        <v>0.7312524125241253</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>2.9</v>
+        <v>0.8424483244832448</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>2.8</v>
+        <v>0.9565619656196562</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>2.7</v>
+        <v>1.072215022150222</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>2.6</v>
+        <v>1.188261882618826</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>2.5</v>
+        <v>1.304022340223402</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>2.4</v>
+        <v>1.419406894068941</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>b_рк_i</t>
+          <t>bt_2ср_i</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr"/>
       <c r="C23" s="2" t="n">
-        <v>0.05543436426911109</v>
+        <v>1.364981334382785</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.05262952708397184</v>
+        <v>1.245745100108579</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.04965469976639989</v>
+        <v>1.223409472435786</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.0464939457414797</v>
+        <v>1.193336115742473</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.04312927210204854</v>
+        <v>1.174986203758765</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>0.03954028688665528</v>
+        <v>1.177477160218605</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0.03570378544951077</v>
+        <v>1.1661853217552</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>0.03159324819542737</v>
+        <v>1.157943254299948</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>0.02717822670030076</v>
+        <v>1.14421483298957</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>0.02242358816708747</v>
+        <v>1.116548947947683</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0.01728857855121713</v>
+        <v>1.106901430168325</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.01172565146735761</v>
+        <v>1.097267445213182</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>b_на_i</t>
+          <t>i_рк_i</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr"/>
       <c r="C24" s="2" t="n">
-        <v>0.05178836962977153</v>
+        <v>0.9036487376823932</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.03330706069671961</v>
+        <v>0.6118732420049944</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.0291874753572514</v>
+        <v>0.6352987675936544</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.02682697425878835</v>
+        <v>0.516090016418827</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.02495173438077425</v>
+        <v>0.4900436345206605</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0.02321702649001537</v>
+        <v>0.4159125801009395</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0.02148432366386106</v>
+        <v>0.379617746368433</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0.0196958066816532</v>
+        <v>0.4222183461841644</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0.01781853059457274</v>
+        <v>0.3292083725419703</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>0.01583255278061968</v>
+        <v>0.3119330018374228</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0.01372666838342158</v>
+        <v>0.284008458812095</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.0114980653754621</v>
+        <v>0.2546469679274699</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>R_сл_рк_i</t>
+          <t>i_на_i</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr"/>
       <c r="C25" s="2" t="n">
-        <v>10.96076687343545</v>
+        <v>-1.587546664043038</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>15.91605999233117</v>
+        <v>-1.885637249728552</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>13.94385751038012</v>
+        <v>-1.941476318910534</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>11.07712142437331</v>
+        <v>-2.016659710643817</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>8.871221488099128</v>
+        <v>-2.062534490603087</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>7.070040395000136</v>
+        <v>-2.056307099453487</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>5.668486896713686</v>
+        <v>-2.084536695612</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>4.566326473150806</v>
+        <v>-2.10514186425013</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>3.563210271245665</v>
+        <v>-2.139462917526076</v>
       </c>
       <c r="L25" s="2" t="n">
-        <v>2.728966887552488</v>
+        <v>-2.208627630130793</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>1.976666807396439</v>
+        <v>-2.232746424579187</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>1.276565001395402</v>
+        <v>-2.256831386967044</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>R_сл_на_i</t>
+          <t>X_f_отн</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr"/>
       <c r="C26" s="2" t="n">
-        <v>8.491617336491974</v>
-      </c>
-      <c r="D26" s="2" t="n">
-        <v>8.117540722471976</v>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>6.680209920670077</v>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>5.363402475178872</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>4.355404445733249</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>3.596440879550598</v>
-      </c>
-      <c r="I26" s="2" t="n">
-        <v>2.978044691105112</v>
-      </c>
-      <c r="J26" s="2" t="n">
-        <v>2.4787494144602</v>
-      </c>
-      <c r="K26" s="2" t="n">
-        <v>2.060555855203703</v>
-      </c>
-      <c r="L26" s="2" t="n">
-        <v>1.698751455831154</v>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>1.393626417287184</v>
-      </c>
-      <c r="N26" s="2" t="n">
-        <v>1.121514263891278</v>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="D26" s="1" t="inlineStr"/>
+      <c r="E26" s="1" t="inlineStr"/>
+      <c r="F26" s="1" t="inlineStr"/>
+      <c r="G26" s="1" t="inlineStr"/>
+      <c r="H26" s="1" t="inlineStr"/>
+      <c r="I26" s="1" t="inlineStr"/>
+      <c r="J26" s="1" t="inlineStr"/>
+      <c r="K26" s="1" t="inlineStr"/>
+      <c r="L26" s="1" t="inlineStr"/>
+      <c r="M26" s="1" t="inlineStr"/>
+      <c r="N26" s="1" t="inlineStr"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>t_ср_рк_i</t>
+          <t>m_рк_i</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr"/>
       <c r="C27" s="2" t="n">
-        <v>0.04071686632597211</v>
+        <v>0.278280383393174</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.04228122660457596</v>
+        <v>0.2925060337085559</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.0395932759898588</v>
+        <v>0.2956423088465648</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.03853826103363832</v>
+        <v>0.2973763371712121</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.03606073804752575</v>
+        <v>0.2987231567492909</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>0.03390043922826257</v>
+        <v>0.2999634266313577</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.03099698344905137</v>
+        <v>0.3012241705710921</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.02702848012425377</v>
+        <v>0.302579389711173</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0.02401575204222394</v>
+        <v>0.304094923198526</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0.01993609747497101</v>
+        <v>0.3058415916829391</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0.0155248976493717</v>
+        <v>0.3079016558590607</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.01064170073686403</v>
+        <v>0.3103677360799227</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>t_ср_на_i</t>
+          <t>m_на_i</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr"/>
       <c r="C28" s="2" t="n">
-        <v>0.03794071634920129</v>
+        <v>0.2784088862773235</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.02673665799995244</v>
+        <v>0.290145758525186</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.0238574868144021</v>
+        <v>0.2931740075161676</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.02248065226962235</v>
+        <v>0.2950743805877517</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.02123576796132072</v>
+        <v>0.2966941167788055</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>0.01971760240827517</v>
+        <v>0.2982774621942075</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0.01842273544613431</v>
+        <v>0.2999430459044465</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.0170093021471597</v>
+        <v>0.3017683087548075</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0.01557271421487959</v>
+        <v>0.3038284072773666</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0.01417990031670473</v>
+        <v>0.306208816044133</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0.01240098531748593</v>
+        <v>0.3090118087713087</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.01047881756232019</v>
+        <v>0.3123553769535541</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>Z_рк_i</t>
+          <t>θ_рк_i</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr"/>
       <c r="C29" s="2" t="n">
-        <v>41</v>
+        <v>0.2897752077348815</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>43</v>
+        <v>0.1894596498726411</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>47</v>
+        <v>0.204032939286868</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>49</v>
+        <v>0.2404874621568816</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>53</v>
+        <v>0.2785555181894611</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>57</v>
+        <v>0.3204358653219178</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>63</v>
+        <v>0.3608863595821978</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>73</v>
+        <v>0.3964156754475768</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>83</v>
+        <v>0.4370220505788445</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>101</v>
+        <v>0.4707937585285812</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>131</v>
+        <v>0.5011293448307715</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>193</v>
+        <v>0.5262816246511876</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>Z_на_i</t>
+          <t>θ_на_i</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr"/>
       <c r="C30" s="2" t="n">
-        <v>44</v>
+        <v>0.3494339757321023</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>68</v>
+        <v>0.235090332136063</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>78</v>
+        <v>0.2503395106870253</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>84</v>
+        <v>0.2865856164178282</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>90</v>
+        <v>0.3282430011756985</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>98</v>
+        <v>0.3698767712696619</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>106</v>
+        <v>0.4133462955498508</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>116</v>
+        <v>0.4552656912836749</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>128</v>
+        <v>0.4954632889968579</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>142</v>
+        <v>0.5340049796103393</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>164</v>
+        <v>0.5643430223457975</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>196</v>
+        <v>0.5874142888999352</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>t_к_рк_i</t>
+          <t>χ_рк_i</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr"/>
       <c r="C31" s="2" t="n">
-        <v>0.05216368595677448</v>
+        <v>0.1448876038674407</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.0497374680052966</v>
+        <v>0.09472982493632053</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.04550449200484583</v>
+        <v>0.102016469643434</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.0436471658005664</v>
+        <v>0.1202437310784408</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.04035304007976893</v>
+        <v>0.1392777590947306</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>0.03752124779346936</v>
+        <v>0.1602179326609589</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.03394779562266276</v>
+        <v>0.1804431797910989</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.02929741266065416</v>
+        <v>0.1982078377237884</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>0.02576760390635848</v>
+        <v>0.2185110252894223</v>
       </c>
       <c r="L31" s="2" t="n">
-        <v>0.02117535766562132</v>
+        <v>0.2353968792642906</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>0.01632603911624239</v>
+        <v>0.2505646724153858</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.01108140478874484</v>
+        <v>0.2631408123255938</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>t_к_на_i</t>
+          <t>χ_на_i</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr"/>
       <c r="C32" s="2" t="n">
-        <v>0.04860707100517622</v>
+        <v>0.1747169878660511</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.03145163417981991</v>
+        <v>0.1175451660680315</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.0274193733875353</v>
+        <v>0.1251697553435127</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.02546084671699707</v>
+        <v>0.1432928082089141</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.02376345693586393</v>
+        <v>0.1641215005878493</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>0.0218235829002832</v>
+        <v>0.1849383856348309</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.02017652003988447</v>
+        <v>0.2066731477749254</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.01843716486403236</v>
+        <v>0.2276328456418374</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>0.01670868065802933</v>
+        <v>0.247731644498429</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>0.01506134594526587</v>
+        <v>0.2670024898051697</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>0.01304092148919362</v>
+        <v>0.2821715111728987</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.0109117914501416</v>
+        <v>0.2937071444499676</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>bt_1к_i_отн</t>
+          <t>v_рк_i</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr"/>
       <c r="C33" s="2" t="n">
-        <v>1.062700291445027</v>
+        <v>53.36151595490971</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>1.05814648784227</v>
+        <v>50.83246384023893</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1.091204353212252</v>
+        <v>48.67680714295572</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1.065222561160577</v>
+        <v>46.38367820929632</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>1.068798584116379</v>
+        <v>44.17712222971348</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>1.053810553004512</v>
+        <v>41.91823182418606</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>1.05172618117436</v>
+        <v>39.69453263128516</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>1.078363081455874</v>
+        <v>37.55219102641462</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>1.054744042134014</v>
+        <v>35.28921715191872</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>1.058947316082065</v>
+        <v>33.11899142444339</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>1.058957315250894</v>
+        <v>30.96473257991795</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>1.058137636057399</v>
+        <v>28.84123613160006</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>bt_2к_i_отн</t>
+          <t>v_на_i</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr"/>
       <c r="C34" s="2" t="n">
-        <v>1.065449296960447</v>
+        <v>50.72016075131927</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>1.058993008321653</v>
+        <v>50.07652160407117</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1.064483675273187</v>
+        <v>47.99658880520145</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>1.053656013760111</v>
+        <v>45.62129843758604</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>1.050004401637245</v>
+        <v>43.15779401816041</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>1.063850358398945</v>
+        <v>40.6792043031489</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>1.064818096549423</v>
+        <v>38.13011904016454</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1.06826655979392</v>
+        <v>35.5737299611924</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>1.066423553077489</v>
+        <v>33.00879625441686</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>1.05120437696315</v>
+        <v>30.43275117827625</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>1.052584236075357</v>
+        <v>27.93879278458221</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>1.053728476025162</v>
+        <v>25.49564119157854</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>i_рк_к_i</t>
+          <t>h_рк_i_отн</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr"/>
       <c r="C35" s="2" t="n">
-        <v>0.1567507286125669</v>
+        <v>3.5</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.1453662196056738</v>
+        <v>3.4</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.2280108830306304</v>
+        <v>3.3</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0.1630564029014431</v>
+        <v>3.2</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.171996460290948</v>
+        <v>3.1</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>0.1345263825112808</v>
+        <v>3</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.1293154529359009</v>
+        <v>2.9</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.1959077036396861</v>
+        <v>2.8</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>0.136860105335036</v>
+        <v>2.7</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>0.1473682902051615</v>
+        <v>2.6</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>0.1473932881272355</v>
+        <v>2.5</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.1453440901434977</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>i_на_к_i</t>
+          <t>h_на_i_отн</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr"/>
       <c r="C36" s="2" t="n">
-        <v>-2.336376757598883</v>
+        <v>3.5</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>-2.352517479195868</v>
+        <v>3.4</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>-2.338790811817033</v>
+        <v>3.3</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>-2.365859965599721</v>
+        <v>3.2</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>-2.374988995906887</v>
+        <v>3.1</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>-2.340374104002637</v>
+        <v>3</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>-2.337954758626443</v>
+        <v>2.9</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>-2.329333600515199</v>
+        <v>2.8</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>-2.333941117306279</v>
+        <v>2.7</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>-2.371989057592124</v>
+        <v>2.6</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>-2.368539409811606</v>
+        <v>2.5</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-2.365678809937095</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>m_рк_к_i</t>
+          <t>b_рк_i</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr"/>
       <c r="C37" s="2" t="n">
-        <v>0.3178629028527515</v>
+        <v>0.05543436426911109</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.3182693391553421</v>
+        <v>0.05262952708397184</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.3186733604517634</v>
+        <v>0.04965469976639989</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.3190622263745982</v>
+        <v>0.0464939457414797</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0.3194282596558449</v>
+        <v>0.04312927210204854</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>0.3197672862786282</v>
+        <v>0.03954028688665528</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0.320080883052504</v>
+        <v>0.03570378544951077</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.3203790126430688</v>
+        <v>0.03159324819542737</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>0.3206797736966317</v>
+        <v>0.02717822670030076</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>0.321013506631057</v>
+        <v>0.02242358816708747</v>
       </c>
       <c r="M37" s="2" t="n">
-        <v>0.3214276603523565</v>
+        <v>0.01728857855121713</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.3219900612567497</v>
+        <v>0.01172565146735761</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>m_на_к_i</t>
+          <t>b_на_i</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr"/>
       <c r="C38" s="2" t="n">
-        <v>0.2663549579009676</v>
+        <v>0.05178836962977153</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.2679208643185232</v>
+        <v>0.03330706069671961</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.2698777984725082</v>
+        <v>0.0291874753572514</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.2722579294732932</v>
+        <v>0.02682697425878835</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.2751034993137159</v>
+        <v>0.02495173438077425</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>0.2784695412248092</v>
+        <v>0.02321702649001537</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.2824253772273643</v>
+        <v>0.02148432366386106</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.2870486147946897</v>
+        <v>0.0196958066816532</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>0.2924220028884709</v>
+        <v>0.01781853059457274</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>0.2986248932311759</v>
+        <v>0.01583255278061968</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>0.3057143940942084</v>
+        <v>0.01372666838342158</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.3131505681731241</v>
+        <v>0.0114980653754621</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>θ_рк_к_i</t>
+          <t>R_сл_рк_i</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr"/>
       <c r="C39" s="2" t="n">
-        <v>0.1667599944012234</v>
+        <v>10.96076687343545</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.1924686654491106</v>
+        <v>15.91605999233117</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.2137657550545313</v>
+        <v>13.94385751038012</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.241282643529005</v>
+        <v>11.07712142437331</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.2657197985404201</v>
+        <v>8.871221488099128</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>0.2927016711094964</v>
+        <v>7.070040395000136</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.3184515338798583</v>
+        <v>5.668486896713686</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.3404895453615822</v>
+        <v>4.566326473150806</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>0.3692420520132633</v>
+        <v>3.563210271245665</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>0.3936771331507258</v>
+        <v>2.728966887552488</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0.4175626941829056</v>
+        <v>1.976666807396439</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.4395275561706619</v>
+        <v>1.276565001395402</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>θ_на_к_i</t>
+          <t>R_сл_на_i</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr"/>
       <c r="C40" s="2" t="n">
-        <v>0.3625801184371908</v>
+        <v>8.491617336491974</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.4042201245857512</v>
+        <v>8.117540722471976</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0.4423218195602118</v>
+        <v>6.680209920670077</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.4802396404625832</v>
+        <v>5.363402475178872</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.5142115779108413</v>
+        <v>4.355404445733249</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>0.5415388590697533</v>
+        <v>3.596440879550598</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.5655473968687256</v>
+        <v>2.978044691105112</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.5824327305322247</v>
+        <v>2.4787494144602</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>0.5918384384581661</v>
+        <v>2.060555855203703</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>0.593559948826178</v>
+        <v>1.698751455831154</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>0.580788660528019</v>
+        <v>1.393626417287184</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.561858264375525</v>
+        <v>1.121514263891278</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>δ_рк_к_i</t>
+          <t>t_ср_рк_i</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr"/>
       <c r="C41" s="2" t="n">
-        <v>0.05464332487589616</v>
+        <v>0.04071686632597211</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.06301264861872663</v>
+        <v>0.04228122660457596</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.07116016364560376</v>
+        <v>0.0395932759898588</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.07945507680302193</v>
+        <v>0.03853826103363832</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.08774960793556263</v>
+        <v>0.03606073804752575</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>0.09608166157996206</v>
+        <v>0.03390043922826257</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0.1045332430485577</v>
+        <v>0.03099698344905137</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.1132792449756882</v>
+        <v>0.02702848012425377</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>0.1216063531781603</v>
+        <v>0.02401575204222394</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>0.1300471000174254</v>
+        <v>0.01993609747497101</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0.1381160551386239</v>
+        <v>0.0155248976493717</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.1455793097611287</v>
+        <v>0.01064170073686403</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>δ_на_к_i</t>
+          <t>t_ср_на_i</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr"/>
       <c r="C42" s="2" t="n">
-        <v>0.09968531032359713</v>
+        <v>0.03794071634920129</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.1114476752146032</v>
+        <v>0.02673665799995244</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.1231615157120472</v>
+        <v>0.0238574868144021</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.1342109553210837</v>
+        <v>0.02248065226962235</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.1449551085172039</v>
+        <v>0.02123576796132072</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>0.1555419706860113</v>
+        <v>0.01971760240827517</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.1648202000435461</v>
+        <v>0.01842273544613431</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.1727989284543775</v>
+        <v>0.0170093021471597</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>0.1787220262908049</v>
+        <v>0.01557271421487959</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>0.1817331592612706</v>
+        <v>0.01417990031670473</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>0.1821639549180084</v>
+        <v>0.01240098531748593</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.180611057551283</v>
+        <v>0.01047881756232019</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>χ_рк_к_i</t>
+          <t>Z_рк_i</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr"/>
       <c r="C43" s="2" t="n">
-        <v>0.08337999720061171</v>
+        <v>41</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0.09623433272455532</v>
+        <v>43</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.1068828775272656</v>
+        <v>47</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0.1206413217645025</v>
+        <v>49</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.1328598992702101</v>
+        <v>53</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>0.1463508355547482</v>
+        <v>57</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.1592257669399292</v>
+        <v>63</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.1702447726807911</v>
+        <v>73</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>0.1846210260066317</v>
+        <v>83</v>
       </c>
       <c r="L43" s="2" t="n">
-        <v>0.1968385665753629</v>
+        <v>101</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>0.2087813470914528</v>
+        <v>131</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.219763778085331</v>
+        <v>193</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>χ_на_к_i</t>
+          <t>Z_на_i</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr"/>
       <c r="C44" s="2" t="n">
-        <v>0.1812900592185954</v>
+        <v>44</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0.2021100622928756</v>
+        <v>68</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.2211609097801059</v>
+        <v>78</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.2401198202312916</v>
+        <v>84</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.2571057889554206</v>
+        <v>90</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>0.2707694295348766</v>
+        <v>98</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.2827736984343628</v>
+        <v>106</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.2912163652661123</v>
+        <v>116</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0.295919219229083</v>
+        <v>128</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>0.296779974413089</v>
+        <v>142</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0.2903943302640095</v>
+        <v>164</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.2809291321877625</v>
+        <v>196</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>v_рк_к_i</t>
+          <t>t_к_рк_i</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr"/>
       <c r="C45" s="2" t="n">
-        <v>39.54339464197052</v>
+        <v>0.05216368595677448</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>38.34588757448704</v>
+        <v>0.0497374680052966</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>37.2587280915807</v>
+        <v>0.04550449200484583</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>36.03874995978816</v>
+        <v>0.0436471658005664</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>34.89815727748316</v>
+        <v>0.04035304007976893</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>33.71610631975087</v>
+        <v>0.03752124779346936</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>32.56760154310536</v>
+        <v>0.03394779562266276</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>31.49089757502536</v>
+        <v>0.02929741266065416</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>30.29462025863446</v>
+        <v>0.02576760390635848</v>
       </c>
       <c r="L45" s="2" t="n">
-        <v>29.17042160359454</v>
+        <v>0.02117535766562132</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>28.0432568729264</v>
+        <v>0.01632603911624239</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>26.92445228005211</v>
+        <v>0.01108140478874484</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>v_на_к_i</t>
+          <t>t_к_на_i</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr"/>
       <c r="C46" s="2" t="n">
-        <v>56.59019450008793</v>
+        <v>0.04860707100517622</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>54.1113380830797</v>
+        <v>0.03145163417981991</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>51.56825052584809</v>
+        <v>0.0274193733875353</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>48.89358313125041</v>
+        <v>0.02546084671699707</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>46.15299448472333</v>
+        <v>0.02376345693586393</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>43.38513031450641</v>
+        <v>0.0218235829002832</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>40.53525878638788</v>
+        <v>0.02017652003988447</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>37.66392937342557</v>
+        <v>0.01843716486403236</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>34.77727832185135</v>
+        <v>0.01670868065802933</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>31.88119935810246</v>
+        <v>0.01506134594526587</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>29.07226872304961</v>
+        <v>0.01304092148919362</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>26.33414299342228</v>
+        <v>0.0109117914501416</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>t_вт_рк_i</t>
+          <t>bt_1к_i_отн</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr"/>
       <c r="C47" s="2" t="n">
-        <v>0.02243038496141303</v>
+        <v>1.062700291445027</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0.02359059260035254</v>
+        <v>1.05814648784227</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.02359883362154009</v>
+        <v>1.091204353212252</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.0245692832369308</v>
+        <v>1.065222561160577</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.02450272786805347</v>
+        <v>1.068798584116379</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>0.02444551360357999</v>
+        <v>1.053810553004512</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.02362133291748071</v>
+        <v>1.05172618117436</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.02168347496162342</v>
+        <v>1.078363081455874</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0.02021257073006909</v>
+        <v>1.054744042134014</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>0.01754844622765307</v>
+        <v>1.058947316082065</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0.01425299822435255</v>
+        <v>1.058957315250894</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.01016524593672233</v>
+        <v>1.058137636057399</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>t_вт_на_i</t>
+          <t>bt_2к_i_отн</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr"/>
       <c r="C48" s="2" t="n">
-        <v>0.02272330439172211</v>
+        <v>1.065449296960447</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0.02098791246007154</v>
+        <v>1.058993008321653</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.01966055231252826</v>
+        <v>1.064483675273187</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.01903955717418168</v>
+        <v>1.053656013760111</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.01836338193992195</v>
+        <v>1.050004401637245</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>0.01735796413339145</v>
+        <v>1.063850358398945</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.01648339776006898</v>
+        <v>1.064818096549423</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.01545003789132032</v>
+        <v>1.06826655979392</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0.01434708495495242</v>
+        <v>1.066423553077489</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>0.01323990197472734</v>
+        <v>1.05120437696315</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0.0117261775699369</v>
+        <v>1.052584236075357</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.01002716522040984</v>
+        <v>1.053728476025162</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>bt_1вт_i_отн</t>
+          <t>i_рк_к_i</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr"/>
       <c r="C49" s="2" t="n">
-        <v>2.471396026616342</v>
+        <v>0.1567507286125669</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>2.230954006775791</v>
+        <v>0.1453662196056738</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>2.10411669333848</v>
+        <v>0.2280108830306304</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>1.892360688471095</v>
+        <v>0.1630564029014431</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>1.760182471694519</v>
+        <v>0.171996460290948</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>1.617486444664623</v>
+        <v>0.1345263825112808</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>1.511505958374118</v>
+        <v>0.1293154529359009</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1.457019608311988</v>
+        <v>0.1959077036396861</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>1.344619992343144</v>
+        <v>0.136860105335036</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>1.277810461176449</v>
+        <v>0.1473682902051615</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>1.212978369819622</v>
+        <v>0.1473932881272355</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>1.15350396245685</v>
+        <v>0.1453440901434977</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>bt_2вт_i_отн</t>
+          <t>i_на_к_i</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr"/>
       <c r="C50" s="2" t="n">
-        <v>2.279086207578047</v>
+        <v>-2.336376757598883</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>1.586963961284126</v>
+        <v>-2.352517479195868</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>1.484570468483345</v>
+        <v>-2.338790811817033</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>1.409012510814416</v>
+        <v>-2.365859965599721</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>1.358776638334208</v>
+        <v>-2.374988995906887</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>1.337543176814893</v>
+        <v>-2.340374104002637</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>1.303391690025634</v>
+        <v>-2.337954758626443</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>1.274806367479403</v>
+        <v>-2.329333600515199</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>1.241961739999457</v>
+        <v>-2.333941117306279</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>1.195820997076961</v>
+        <v>-2.371989057592124</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>1.170600419578624</v>
+        <v>-2.368539409811606</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>1.14669152474503</v>
+        <v>-2.365678809937095</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>i_рк_вт_i</t>
+          <t>m_рк_к_i</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr"/>
       <c r="C51" s="2" t="n">
-        <v>3.678490066540854</v>
+        <v>0.3178629028527515</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>3.077385016939478</v>
+        <v>0.3182693391553421</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>2.760291733346201</v>
+        <v>0.3186733604517634</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>2.230901721177736</v>
+        <v>0.3190622263745982</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>1.900456179236298</v>
+        <v>0.3194282596558449</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>1.543716111661558</v>
+        <v>0.3197672862786282</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>1.278764895935294</v>
+        <v>0.320080883052504</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>1.142549020779971</v>
+        <v>0.3203790126430688</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0.8615499808578603</v>
+        <v>0.3206797736966317</v>
       </c>
       <c r="L51" s="2" t="n">
-        <v>0.6945261529411217</v>
+        <v>0.321013506631057</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>0.5324459245490543</v>
+        <v>0.3214276603523565</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.383759906142126</v>
+        <v>0.3219900612567497</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>i_на_вт_i</t>
+          <t>m_на_к_i</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr"/>
       <c r="C52" s="2" t="n">
-        <v>0.6977155189451179</v>
+        <v>0.2663549579009676</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>-1.032590096789685</v>
+        <v>0.2679208643185232</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>-1.288573828791638</v>
+        <v>0.2698777984725082</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>-1.477468722963961</v>
+        <v>0.2722579294732932</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>-1.603058404164481</v>
+        <v>0.2751034993137159</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>-1.656142057962767</v>
+        <v>0.2784695412248092</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>-1.741520774935915</v>
+        <v>0.2824253772273643</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>-1.812984081301493</v>
+        <v>0.2870486147946897</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>-1.895095650001357</v>
+        <v>0.2924220028884709</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>-2.010447507307597</v>
+        <v>0.2986248932311759</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>-2.07349895105344</v>
+        <v>0.3057143940942084</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-2.133271188137424</v>
+        <v>0.3131505681731241</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>m_рк_вт_i</t>
+          <t>θ_рк_к_i</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr"/>
       <c r="C53" s="2" t="n">
-        <v>0.2444953355682234</v>
+        <v>0.1667599944012234</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>0.2760752532782931</v>
+        <v>0.1924686654491106</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.2824543186837005</v>
+        <v>0.2137657550545313</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0.2859874013401232</v>
+        <v>0.241282643529005</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.288707758774392</v>
+        <v>0.2657197985404201</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>0.2911450660861047</v>
+        <v>0.2927016711094964</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.2935143251639874</v>
+        <v>0.3184515338798583</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.2959195017249108</v>
+        <v>0.3404895453615822</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0.2984378036069403</v>
+        <v>0.3692420520132633</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>0.3011421125314475</v>
+        <v>0.3936771331507258</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0.3041113325474636</v>
+        <v>0.4175626941829056</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.3074309813694824</v>
+        <v>0.4395275561706619</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>m_на_вт_i</t>
+          <t>θ_на_к_i</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr"/>
       <c r="C54" s="2" t="n">
-        <v>0.2663549579009676</v>
+        <v>0.3625801184371908</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>0.2679208643185232</v>
+        <v>0.4042201245857512</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.2698777984725082</v>
+        <v>0.4423218195602118</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>0.2722579294732932</v>
+        <v>0.4802396404625832</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.275103499313716</v>
+        <v>0.5142115779108413</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>0.2784695412248092</v>
+        <v>0.5415388590697533</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.2824253772273643</v>
+        <v>0.5655473968687256</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.2870486147946897</v>
+        <v>0.5824327305322247</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0.2924220028884709</v>
+        <v>0.5918384384581661</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>0.2986248932311759</v>
+        <v>0.593559948826178</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0.3057143940942084</v>
+        <v>0.580788660528019</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.3131505681731242</v>
+        <v>0.561858264375525</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>θ_рк_вт_i</t>
+          <t>δ_рк_к_i</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr"/>
       <c r="C55" s="2" t="n">
-        <v>0.1672572324564189</v>
+        <v>0.05464332487589616</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>-0.05869201149797553</v>
+        <v>0.06301264861872663</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>-0.02817582100459576</v>
+        <v>0.07116016364560376</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>0.03762070947421998</v>
+        <v>0.07945507680302193</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.1076060234669587</v>
+        <v>0.08774960793556263</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>0.1806753866817011</v>
+        <v>0.09608166157996206</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>0.2506516675510275</v>
+        <v>0.1045332430485577</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.3136636635194889</v>
+        <v>0.1132792449756882</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>0.378419898898765</v>
+        <v>0.1216063531781603</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>0.4338586330293461</v>
+        <v>0.1300471000174254</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>0.4830472253713849</v>
+        <v>0.1381160551386239</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.5244444381950567</v>
+        <v>0.1455793097611287</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>θ_на_вт_i</t>
+          <t>δ_на_к_i</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr"/>
       <c r="C56" s="2" t="n">
-        <v>0.2623508740600435</v>
+        <v>0.09968531032359713</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>0.3504840813915654</v>
+        <v>0.1114476752146032</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.3960050825107493</v>
+        <v>0.1231615157120472</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.4377648462680688</v>
+        <v>0.1342109553210837</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.474724530418023</v>
+        <v>0.1449551085172039</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>0.5049802154841083</v>
+        <v>0.1555419706860113</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.5319430436560044</v>
+        <v>0.1648202000435461</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.5520019168150699</v>
+        <v>0.1727989284543775</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0.5647862669665616</v>
+        <v>0.1787220262908049</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>0.5700352755623559</v>
+        <v>0.1817331592612706</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>0.5611284693331983</v>
+        <v>0.1821639549180084</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.5460986545811601</v>
+        <v>0.180611057551283</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>δ_рк_вт_i</t>
+          <t>χ_рк_к_i</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr"/>
       <c r="C57" s="2" t="n">
-        <v>0.06428751765653345</v>
+        <v>0.08337999720061171</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>-0.02420202926285983</v>
+        <v>0.09623433272455532</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>-0.01154409016165329</v>
+        <v>0.1068828775272656</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.0148004814087846</v>
+        <v>0.1206413217645025</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.04121676326293985</v>
+        <v>0.1328598992702101</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>0.06690040585460004</v>
+        <v>0.1463508355547482</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.0904492212768311</v>
+        <v>0.1592257669399292</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.1120393281474088</v>
+        <v>0.1702447726807911</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0.1309566577428124</v>
+        <v>0.1846210260066317</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>0.1476906343689841</v>
+        <v>0.1968385665753629</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>0.1617889007592458</v>
+        <v>0.2087813470914528</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.1731636218328381</v>
+        <v>0.219763778085331</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>δ_на_вт_i</t>
+          <t>χ_на_к_i</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr"/>
       <c r="C58" s="2" t="n">
-        <v>0.1054930082770162</v>
+        <v>0.1812900592185954</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>0.1182928146079504</v>
+        <v>0.2021100622928756</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.1302171923699162</v>
+        <v>0.2211609097801059</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0.1414747208230928</v>
+        <v>0.2401198202312916</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.1522340578875385</v>
+        <v>0.2571057889554206</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>0.1626319868588671</v>
+        <v>0.2707694295348766</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.1715166656621255</v>
+        <v>0.2827736984343628</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.1789032183371666</v>
+        <v>0.2912163652661123</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>0.1840552814785316</v>
+        <v>0.295919219229083</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0.1861490511662801</v>
+        <v>0.296779974413089</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>0.1856019473611825</v>
+        <v>0.2903943302640095</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.1831249891196447</v>
+        <v>0.2809291321877625</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>χ_рк_вт_i</t>
+          <t>v_рк_к_i</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr"/>
       <c r="C59" s="2" t="n">
-        <v>0.08362861622820945</v>
+        <v>39.54339464197052</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>-0.02934600574898777</v>
+        <v>38.34588757448704</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>-0.01408791050229788</v>
+        <v>37.2587280915807</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.01881035473710999</v>
+        <v>36.03874995978816</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.05380301173347936</v>
+        <v>34.89815727748316</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>0.09033769334085054</v>
+        <v>33.71610631975087</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.1253258337755137</v>
+        <v>32.56760154310536</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.1568318317597444</v>
+        <v>31.49089757502536</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0.1892099494493825</v>
+        <v>30.29462025863446</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>0.2169293165146731</v>
+        <v>29.17042160359454</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>0.2415236126856925</v>
+        <v>28.0432568729264</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.2622222190975284</v>
+        <v>26.92445228005211</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>χ_на_вт_i</t>
+          <t>v_на_к_i</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr"/>
       <c r="C60" s="2" t="n">
-        <v>0.1311754370300218</v>
+        <v>56.59019450008793</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0.1752420406957827</v>
+        <v>54.1113380830797</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>0.1980025412553746</v>
+        <v>51.56825052584809</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.2188824231340344</v>
+        <v>48.89358313125041</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.2373622652090115</v>
+        <v>46.15299448472333</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>0.2524901077420542</v>
+        <v>43.38513031450641</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.2659715218280022</v>
+        <v>40.53525878638788</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.276000958407535</v>
+        <v>37.66392937342557</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0.2823931334832808</v>
+        <v>34.77727832185135</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>0.2850176377811779</v>
+        <v>31.88119935810246</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>0.2805642346665991</v>
+        <v>29.07226872304961</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.2730493272905801</v>
+        <v>26.33414299342228</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>v_рк_вт_i</t>
+          <t>t_вт_рк_i</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr"/>
       <c r="C61" s="2" t="n">
-        <v>74.74324140004022</v>
+        <v>0.02243038496141303</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>69.6742708472452</v>
+        <v>0.02359059260035254</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>65.05875905893463</v>
+        <v>0.02359883362154009</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>60.31772204613338</v>
+        <v>0.0245692832369308</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>55.87620136108077</v>
+        <v>0.02450272786805347</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>51.53566229292001</v>
+        <v>0.02444551360357999</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>47.43548673295959</v>
+        <v>0.02362133291748071</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>43.63130682283349</v>
+        <v>0.02168347496162342</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>39.86865643884803</v>
+        <v>0.02021257073006909</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>36.4099090165288</v>
+        <v>0.01754844622765307</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>33.15148827827766</v>
+        <v>0.01425299822435255</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>30.09950153588676</v>
+        <v>0.01016524593672233</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>v_на_вт_i</t>
+          <t>t_вт_на_i</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr"/>
       <c r="C62" s="2" t="n">
-        <v>59.57417215444337</v>
+        <v>0.02272330439172211</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>55.4043974438888</v>
+        <v>0.02098791246007154</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>52.59530914034876</v>
+        <v>0.01966055231252826</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>49.76073697678891</v>
+        <v>0.01903955717418168</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>46.90518155271934</v>
+        <v>0.01836338193992195</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>44.05108303875345</v>
+        <v>0.01735796413339145</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>41.11489059347205</v>
+        <v>0.01648339776006898</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>38.16506348578071</v>
+        <v>0.01545003789132032</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>35.20259770341047</v>
+        <v>0.01434708495495242</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>32.23097857175508</v>
+        <v>0.01323990197472734</v>
       </c>
       <c r="M62" s="2" t="n">
-        <v>29.35747908621037</v>
+        <v>0.0117261775699369</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>26.55867081032476</v>
+        <v>0.01002716522040984</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>R_сл_рк_вт_i</t>
+          <t>bt_1вт_i_отн</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr"/>
       <c r="C63" s="2" t="n">
-        <v>18.9896496176594</v>
+        <v>2.471396026616342</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>-51.37751858490998</v>
+        <v>2.230954006775791</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>-100.9732691660246</v>
+        <v>2.10411669333848</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>70.80958729862108</v>
+        <v>1.892360688471095</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>22.96456600172329</v>
+        <v>1.760182471694519</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>12.53902116719294</v>
+        <v>1.617486444664623</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>8.161437225371769</v>
+        <v>1.511505958374118</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>5.771028823729717</v>
+        <v>1.457019608311988</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>4.115006952408685</v>
+        <v>1.344619992343144</v>
       </c>
       <c r="L63" s="2" t="n">
-        <v>2.961287237846502</v>
+        <v>1.277810461176449</v>
       </c>
       <c r="M63" s="2" t="n">
-        <v>2.050659783077384</v>
+        <v>1.212978369819622</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>1.281036917387719</v>
+        <v>1.15350396245685</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>R_сл_на_вт_i</t>
+          <t>bt_2вт_i_отн</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr"/>
       <c r="C64" s="2" t="n">
-        <v>11.31026382302569</v>
+        <v>2.279086207578047</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>5.444917708362168</v>
+        <v>1.586963961284126</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>4.222982368393026</v>
+        <v>1.484570468483345</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>3.511191348359</v>
+        <v>1.409012510814416</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>3.011500500323452</v>
+        <v>1.358776638334208</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>2.634245650464841</v>
+        <v>1.337543176814893</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>2.314092659541661</v>
+        <v>1.303391690025634</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>2.044360584565208</v>
+        <v>1.274806367479403</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>1.807640860458127</v>
+        <v>1.241961739999457</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>1.591379048684799</v>
+        <v>1.195820997076961</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>1.401610061190252</v>
+        <v>1.170600419578624</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>1.206362818688264</v>
+        <v>1.14669152474503</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>S_1_i</t>
+          <t>i_рк_вт_i</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr"/>
       <c r="C65" s="2" t="n">
-        <v>0.01385859106727777</v>
+        <v>3.678490066540854</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0.01315738177099296</v>
+        <v>3.077385016939478</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.01241367494159997</v>
+        <v>2.760291733346201</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.01162348643536992</v>
+        <v>2.230901721177736</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.01078231802551213</v>
+        <v>1.900456179236298</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>0.009885071721663821</v>
+        <v>1.543716111661558</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>0.008925946362377693</v>
+        <v>1.278764895935294</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.007898312048856842</v>
+        <v>1.142549020779971</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>0.00679455667507519</v>
+        <v>0.8615499808578603</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>0.005605897041771868</v>
+        <v>0.6945261529411217</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>0.004322144637804282</v>
+        <v>0.5324459245490543</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.002931412866839401</v>
+        <v>0.383759906142126</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>S_2_i</t>
+          <t>i_на_вт_i</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr"/>
       <c r="C66" s="2" t="n">
-        <v>0.01294709240744288</v>
+        <v>0.6977155189451179</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0.008326765174179901</v>
+        <v>-1.032590096789685</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>0.007296868839312849</v>
+        <v>-1.288573828791638</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0.006706743564697088</v>
+        <v>-1.477468722963961</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.006237933595193562</v>
+        <v>-1.603058404164481</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>0.005804256622503843</v>
+        <v>-1.656142057962767</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>0.005371080915965266</v>
+        <v>-1.741520774935915</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.004923951670413299</v>
+        <v>-1.812984081301493</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>0.004454632648643186</v>
+        <v>-1.895095650001357</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>0.00395813819515492</v>
+        <v>-2.010447507307597</v>
       </c>
       <c r="M66" s="2" t="n">
-        <v>0.003431667095855395</v>
+        <v>-2.07349895105344</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.002874516343865525</v>
+        <v>-2.133271188137424</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>S_в_РК_i</t>
+          <t>m_рк_вт_i</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr"/>
       <c r="C67" s="2" t="n">
-        <v>0.05348065161085038</v>
+        <v>0.2444953355682234</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>0.04935244672483962</v>
+        <v>0.2760752532782931</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0.04502393831156841</v>
+        <v>0.2824543186837005</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>0.0403932297369132</v>
+        <v>0.2859874013401232</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.03570359291219267</v>
+        <v>0.288707758774392</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>0.03095986565509889</v>
+        <v>0.2911450660861047</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.02629641552912036</v>
+        <v>0.2935143251639874</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.02179981936945496</v>
+        <v>0.2959195017249108</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>0.0174220548346053</v>
+        <v>0.2984378036069403</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>0.01330970194045197</v>
+        <v>0.3011421125314475</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>0.009454337808190653</v>
+        <v>0.3041113325474636</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.005880451855633163</v>
+        <v>0.3074309813694824</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>S_в_НА_i</t>
+          <t>m_на_вт_i</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr"/>
       <c r="C68" s="2" t="n">
-        <v>0.04465635870911464</v>
+        <v>0.2663549579009676</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>0.02741770449389811</v>
+        <v>0.2679208643185232</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0.02318550569353218</v>
+        <v>0.2698777984725082</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.0204784656919946</v>
+        <v>0.2722579294732932</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.01822035692341738</v>
+        <v>0.275103499313716</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>0.01614278537928499</v>
+        <v>0.2784695412248092</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0.01412746963743333</v>
+        <v>0.2824253772273643</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.0121706120674842</v>
+        <v>0.2870486147946897</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>0.01027183699361799</v>
+        <v>0.2924220028884709</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>0.008444034212239363</v>
+        <v>0.2986248932311759</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>0.00672959614882052</v>
+        <v>0.3057143940942084</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.00514094589581024</v>
+        <v>0.3131505681731242</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>S_ср_РК_i</t>
+          <t>θ_рк_вт_i</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr"/>
       <c r="C69" s="2" t="n">
-        <v>0.04448146661709266</v>
+        <v>0.1672572324564189</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>0.04080380248333932</v>
+        <v>-0.05869201149797553</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0.0372905260295658</v>
+        <v>-0.02817582100459576</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.03366047207473166</v>
+        <v>0.03762070947421998</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.0300558749697196</v>
+        <v>0.1076060234669587</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>0.02641565437523911</v>
+        <v>0.1806753866817011</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0.02280380767342325</v>
+        <v>0.2506516675510275</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.01925557442008509</v>
+        <v>0.3136636635194889</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>0.01570097082549171</v>
+        <v>0.378419898898765</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>0.01225179121567093</v>
+        <v>0.4338586330293461</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>0.008895152825414362</v>
+        <v>0.4830472253713849</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.005656269385850665</v>
+        <v>0.5244444381950567</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>S_ср_НА_i</t>
+          <t>θ_на_вт_i</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr"/>
       <c r="C70" s="2" t="n">
-        <v>0.04008746233962627</v>
+        <v>0.2623508740600435</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0.0255432593625421</v>
+        <v>0.3504840813915654</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0.02168935847875152</v>
+        <v>0.3960050825107493</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>0.0191741161370407</v>
+        <v>0.4377648462680688</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.01706723427804866</v>
+        <v>0.474724530418023</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>0.01513339634946587</v>
+        <v>0.5049802154841083</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0.0132654841102659</v>
+        <v>0.5319430436560044</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.0114580375728913</v>
+        <v>0.5520019168150699</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>0.009706961431880611</v>
+        <v>0.5647862669665616</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>0.008019610838336058</v>
+        <v>0.5700352755623559</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>0.006431329457920825</v>
+        <v>0.5611284693331983</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.004949255210666078</v>
+        <v>0.5460986545811601</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>S_к_РК_i</t>
+          <t>δ_рк_вт_i</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr"/>
       <c r="C71" s="2" t="n">
-        <v>0.03529297818838117</v>
+        <v>0.06428751765653345</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>0.0326517455312112</v>
+        <v>-0.02420202926285983</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>0.03006171193335206</v>
+        <v>-0.01154409016165329</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>0.02735388853024765</v>
+        <v>0.0148004814087846</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.02467509740809998</v>
+        <v>0.04121676326293985</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>0.02194795422776095</v>
+        <v>0.06690040585460004</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>0.01921914512347143</v>
+        <v>0.0904492212768311</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.01650314711364222</v>
+        <v>0.1120393281474088</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>0.01370996279618971</v>
+        <v>0.1309566577428124</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>0.01092945770959476</v>
+        <v>0.1476906343689841</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>0.008128018298888534</v>
+        <v>0.1617889007592458</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.005309553953316647</v>
+        <v>0.1731636218328381</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>S_к_НА_i</t>
+          <t>δ_на_вт_i</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr"/>
       <c r="C72" s="2" t="n">
-        <v>0.04323053019914518</v>
+        <v>0.1054930082770162</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.02698397035490908</v>
+        <v>0.1182928146079504</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>0.02286398367976868</v>
+        <v>0.1302171923699162</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>0.02021385051689902</v>
+        <v>0.1414747208230928</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.01799499497206569</v>
+        <v>0.1522340578875385</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>0.01594775050048612</v>
+        <v>0.1626319868588671</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>0.01396300280667979</v>
+        <v>0.1715166656621255</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.01203470518695078</v>
+        <v>0.1789032183371666</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0.01016347391261594</v>
+        <v>0.1840552814785316</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>0.008362116810762451</v>
+        <v>0.1861490511662801</v>
       </c>
       <c r="M72" s="2" t="n">
-        <v>0.006669958596379822</v>
+        <v>0.1856019473611825</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.005100603145579266</v>
+        <v>0.1831249891196447</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>Length_all_compressor</t>
+          <t>χ_рк_вт_i</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr"/>
       <c r="C73" s="2" t="n">
+        <v>0.08362861622820945</v>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>-0.02934600574898777</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>-0.01408791050229788</v>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>0.01881035473710999</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>0.05380301173347936</v>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>0.09033769334085054</v>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>0.1253258337755137</v>
+      </c>
+      <c r="J73" s="2" t="n">
+        <v>0.1568318317597444</v>
+      </c>
+      <c r="K73" s="2" t="n">
+        <v>0.1892099494493825</v>
+      </c>
+      <c r="L73" s="2" t="n">
+        <v>0.2169293165146731</v>
+      </c>
+      <c r="M73" s="2" t="n">
+        <v>0.2415236126856925</v>
+      </c>
+      <c r="N73" s="2" t="n">
+        <v>0.2622222190975284</v>
+      </c>
+    </row>
+    <row r="74" ht="15" customHeight="1">
+      <c r="A74" s="1" t="inlineStr">
+        <is>
+          <t>χ_на_вт_i</t>
+        </is>
+      </c>
+      <c r="B74" s="1" t="inlineStr"/>
+      <c r="C74" s="2" t="n">
+        <v>0.1311754370300218</v>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>0.1752420406957827</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>0.1980025412553746</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>0.2188824231340344</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>0.2373622652090115</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>0.2524901077420542</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>0.2659715218280022</v>
+      </c>
+      <c r="J74" s="2" t="n">
+        <v>0.276000958407535</v>
+      </c>
+      <c r="K74" s="2" t="n">
+        <v>0.2823931334832808</v>
+      </c>
+      <c r="L74" s="2" t="n">
+        <v>0.2850176377811779</v>
+      </c>
+      <c r="M74" s="2" t="n">
+        <v>0.2805642346665991</v>
+      </c>
+      <c r="N74" s="2" t="n">
+        <v>0.2730493272905801</v>
+      </c>
+    </row>
+    <row r="75" ht="15" customHeight="1">
+      <c r="A75" s="1" t="inlineStr">
+        <is>
+          <t>v_рк_вт_i</t>
+        </is>
+      </c>
+      <c r="B75" s="1" t="inlineStr"/>
+      <c r="C75" s="2" t="n">
+        <v>74.74324140004022</v>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>69.6742708472452</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>65.05875905893463</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>60.31772204613338</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>55.87620136108077</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>51.53566229292001</v>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>47.43548673295959</v>
+      </c>
+      <c r="J75" s="2" t="n">
+        <v>43.63130682283349</v>
+      </c>
+      <c r="K75" s="2" t="n">
+        <v>39.86865643884803</v>
+      </c>
+      <c r="L75" s="2" t="n">
+        <v>36.4099090165288</v>
+      </c>
+      <c r="M75" s="2" t="n">
+        <v>33.15148827827766</v>
+      </c>
+      <c r="N75" s="2" t="n">
+        <v>30.09950153588676</v>
+      </c>
+    </row>
+    <row r="76" ht="15" customHeight="1">
+      <c r="A76" s="1" t="inlineStr">
+        <is>
+          <t>v_на_вт_i</t>
+        </is>
+      </c>
+      <c r="B76" s="1" t="inlineStr"/>
+      <c r="C76" s="2" t="n">
+        <v>59.57417215444337</v>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>55.4043974438888</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>52.59530914034876</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>49.76073697678891</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>46.90518155271934</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>44.05108303875345</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>41.11489059347205</v>
+      </c>
+      <c r="J76" s="2" t="n">
+        <v>38.16506348578071</v>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>35.20259770341047</v>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>32.23097857175508</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>29.35747908621037</v>
+      </c>
+      <c r="N76" s="2" t="n">
+        <v>26.55867081032476</v>
+      </c>
+    </row>
+    <row r="77" ht="15" customHeight="1">
+      <c r="A77" s="1" t="inlineStr">
+        <is>
+          <t>R_сл_рк_вт_i</t>
+        </is>
+      </c>
+      <c r="B77" s="1" t="inlineStr"/>
+      <c r="C77" s="2" t="n">
+        <v>18.9896496176594</v>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>-51.37751858490998</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>-100.9732691660246</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>70.80958729862108</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>22.96456600172329</v>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>12.53902116719294</v>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>8.161437225371769</v>
+      </c>
+      <c r="J77" s="2" t="n">
+        <v>5.771028823729717</v>
+      </c>
+      <c r="K77" s="2" t="n">
+        <v>4.115006952408685</v>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>2.961287237846502</v>
+      </c>
+      <c r="M77" s="2" t="n">
+        <v>2.050659783077384</v>
+      </c>
+      <c r="N77" s="2" t="n">
+        <v>1.281036917387719</v>
+      </c>
+    </row>
+    <row r="78" ht="15" customHeight="1">
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>R_сл_на_вт_i</t>
+        </is>
+      </c>
+      <c r="B78" s="1" t="inlineStr"/>
+      <c r="C78" s="2" t="n">
+        <v>11.31026382302569</v>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>5.444917708362168</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>4.222982368393026</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>3.511191348359</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>3.011500500323452</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>2.634245650464841</v>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>2.314092659541661</v>
+      </c>
+      <c r="J78" s="2" t="n">
+        <v>2.044360584565208</v>
+      </c>
+      <c r="K78" s="2" t="n">
+        <v>1.807640860458127</v>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>1.591379048684799</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>1.401610061190252</v>
+      </c>
+      <c r="N78" s="2" t="n">
+        <v>1.206362818688264</v>
+      </c>
+    </row>
+    <row r="79" ht="15" customHeight="1">
+      <c r="A79" s="1" t="inlineStr">
+        <is>
+          <t>S_1_i</t>
+        </is>
+      </c>
+      <c r="B79" s="1" t="inlineStr"/>
+      <c r="C79" s="2" t="n">
+        <v>0.01385859106727777</v>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>0.01315738177099296</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>0.01241367494159997</v>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>0.01162348643536992</v>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>0.01078231802551213</v>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>0.009885071721663821</v>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>0.008925946362377693</v>
+      </c>
+      <c r="J79" s="2" t="n">
+        <v>0.007898312048856842</v>
+      </c>
+      <c r="K79" s="2" t="n">
+        <v>0.00679455667507519</v>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>0.005605897041771868</v>
+      </c>
+      <c r="M79" s="2" t="n">
+        <v>0.004322144637804282</v>
+      </c>
+      <c r="N79" s="2" t="n">
+        <v>0.002931412866839401</v>
+      </c>
+    </row>
+    <row r="80" ht="15" customHeight="1">
+      <c r="A80" s="1" t="inlineStr">
+        <is>
+          <t>S_2_i</t>
+        </is>
+      </c>
+      <c r="B80" s="1" t="inlineStr"/>
+      <c r="C80" s="2" t="n">
+        <v>0.01294709240744288</v>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>0.008326765174179901</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>0.007296868839312849</v>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>0.006706743564697088</v>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>0.006237933595193562</v>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>0.005804256622503843</v>
+      </c>
+      <c r="I80" s="2" t="n">
+        <v>0.005371080915965266</v>
+      </c>
+      <c r="J80" s="2" t="n">
+        <v>0.004923951670413299</v>
+      </c>
+      <c r="K80" s="2" t="n">
+        <v>0.004454632648643186</v>
+      </c>
+      <c r="L80" s="2" t="n">
+        <v>0.00395813819515492</v>
+      </c>
+      <c r="M80" s="2" t="n">
+        <v>0.003431667095855395</v>
+      </c>
+      <c r="N80" s="2" t="n">
+        <v>0.002874516343865525</v>
+      </c>
+    </row>
+    <row r="81" ht="15" customHeight="1">
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>S_в_РК_i</t>
+        </is>
+      </c>
+      <c r="B81" s="1" t="inlineStr"/>
+      <c r="C81" s="2" t="n">
+        <v>0.05348065161085038</v>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>0.04935244672483962</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>0.04502393831156841</v>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>0.0403932297369132</v>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>0.03570359291219267</v>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>0.03095986565509889</v>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>0.02629641552912036</v>
+      </c>
+      <c r="J81" s="2" t="n">
+        <v>0.02179981936945496</v>
+      </c>
+      <c r="K81" s="2" t="n">
+        <v>0.0174220548346053</v>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>0.01330970194045197</v>
+      </c>
+      <c r="M81" s="2" t="n">
+        <v>0.009454337808190653</v>
+      </c>
+      <c r="N81" s="2" t="n">
+        <v>0.005880451855633163</v>
+      </c>
+    </row>
+    <row r="82" ht="15" customHeight="1">
+      <c r="A82" s="1" t="inlineStr">
+        <is>
+          <t>S_в_НА_i</t>
+        </is>
+      </c>
+      <c r="B82" s="1" t="inlineStr"/>
+      <c r="C82" s="2" t="n">
+        <v>0.04465635870911464</v>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>0.02741770449389811</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>0.02318550569353218</v>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>0.0204784656919946</v>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>0.01822035692341738</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>0.01614278537928499</v>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>0.01412746963743333</v>
+      </c>
+      <c r="J82" s="2" t="n">
+        <v>0.0121706120674842</v>
+      </c>
+      <c r="K82" s="2" t="n">
+        <v>0.01027183699361799</v>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>0.008444034212239363</v>
+      </c>
+      <c r="M82" s="2" t="n">
+        <v>0.00672959614882052</v>
+      </c>
+      <c r="N82" s="2" t="n">
+        <v>0.00514094589581024</v>
+      </c>
+    </row>
+    <row r="83" ht="15" customHeight="1">
+      <c r="A83" s="1" t="inlineStr">
+        <is>
+          <t>S_ср_РК_i</t>
+        </is>
+      </c>
+      <c r="B83" s="1" t="inlineStr"/>
+      <c r="C83" s="2" t="n">
+        <v>0.04448146661709266</v>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>0.04080380248333932</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>0.0372905260295658</v>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>0.03366047207473166</v>
+      </c>
+      <c r="G83" s="2" t="n">
+        <v>0.0300558749697196</v>
+      </c>
+      <c r="H83" s="2" t="n">
+        <v>0.02641565437523911</v>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>0.02280380767342325</v>
+      </c>
+      <c r="J83" s="2" t="n">
+        <v>0.01925557442008509</v>
+      </c>
+      <c r="K83" s="2" t="n">
+        <v>0.01570097082549171</v>
+      </c>
+      <c r="L83" s="2" t="n">
+        <v>0.01225179121567093</v>
+      </c>
+      <c r="M83" s="2" t="n">
+        <v>0.008895152825414362</v>
+      </c>
+      <c r="N83" s="2" t="n">
+        <v>0.005656269385850665</v>
+      </c>
+    </row>
+    <row r="84" ht="15" customHeight="1">
+      <c r="A84" s="1" t="inlineStr">
+        <is>
+          <t>S_ср_НА_i</t>
+        </is>
+      </c>
+      <c r="B84" s="1" t="inlineStr"/>
+      <c r="C84" s="2" t="n">
+        <v>0.04008746233962627</v>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>0.0255432593625421</v>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>0.02168935847875152</v>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>0.0191741161370407</v>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>0.01706723427804866</v>
+      </c>
+      <c r="H84" s="2" t="n">
+        <v>0.01513339634946587</v>
+      </c>
+      <c r="I84" s="2" t="n">
+        <v>0.0132654841102659</v>
+      </c>
+      <c r="J84" s="2" t="n">
+        <v>0.0114580375728913</v>
+      </c>
+      <c r="K84" s="2" t="n">
+        <v>0.009706961431880611</v>
+      </c>
+      <c r="L84" s="2" t="n">
+        <v>0.008019610838336058</v>
+      </c>
+      <c r="M84" s="2" t="n">
+        <v>0.006431329457920825</v>
+      </c>
+      <c r="N84" s="2" t="n">
+        <v>0.004949255210666078</v>
+      </c>
+    </row>
+    <row r="85" ht="15" customHeight="1">
+      <c r="A85" s="1" t="inlineStr">
+        <is>
+          <t>S_к_РК_i</t>
+        </is>
+      </c>
+      <c r="B85" s="1" t="inlineStr"/>
+      <c r="C85" s="2" t="n">
+        <v>0.03529297818838117</v>
+      </c>
+      <c r="D85" s="2" t="n">
+        <v>0.0326517455312112</v>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>0.03006171193335206</v>
+      </c>
+      <c r="F85" s="2" t="n">
+        <v>0.02735388853024765</v>
+      </c>
+      <c r="G85" s="2" t="n">
+        <v>0.02467509740809998</v>
+      </c>
+      <c r="H85" s="2" t="n">
+        <v>0.02194795422776095</v>
+      </c>
+      <c r="I85" s="2" t="n">
+        <v>0.01921914512347143</v>
+      </c>
+      <c r="J85" s="2" t="n">
+        <v>0.01650314711364222</v>
+      </c>
+      <c r="K85" s="2" t="n">
+        <v>0.01370996279618971</v>
+      </c>
+      <c r="L85" s="2" t="n">
+        <v>0.01092945770959476</v>
+      </c>
+      <c r="M85" s="2" t="n">
+        <v>0.008128018298888534</v>
+      </c>
+      <c r="N85" s="2" t="n">
+        <v>0.005309553953316647</v>
+      </c>
+    </row>
+    <row r="86" ht="15" customHeight="1">
+      <c r="A86" s="1" t="inlineStr">
+        <is>
+          <t>S_к_НА_i</t>
+        </is>
+      </c>
+      <c r="B86" s="1" t="inlineStr"/>
+      <c r="C86" s="2" t="n">
+        <v>0.04323053019914518</v>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>0.02698397035490908</v>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>0.02286398367976868</v>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>0.02021385051689902</v>
+      </c>
+      <c r="G86" s="2" t="n">
+        <v>0.01799499497206569</v>
+      </c>
+      <c r="H86" s="2" t="n">
+        <v>0.01594775050048612</v>
+      </c>
+      <c r="I86" s="2" t="n">
+        <v>0.01396300280667979</v>
+      </c>
+      <c r="J86" s="2" t="n">
+        <v>0.01203470518695078</v>
+      </c>
+      <c r="K86" s="2" t="n">
+        <v>0.01016347391261594</v>
+      </c>
+      <c r="L86" s="2" t="n">
+        <v>0.008362116810762451</v>
+      </c>
+      <c r="M86" s="2" t="n">
+        <v>0.006669958596379822</v>
+      </c>
+      <c r="N86" s="2" t="n">
+        <v>0.005100603145579266</v>
+      </c>
+    </row>
+    <row r="87" ht="15" customHeight="1">
+      <c r="A87" s="1" t="inlineStr">
+        <is>
+          <t>Length_all_compressor</t>
+        </is>
+      </c>
+      <c r="B87" s="1" t="inlineStr"/>
+      <c r="C87" s="2" t="n">
         <v>0.7365946188039367</v>
       </c>
-      <c r="D73" s="1" t="inlineStr"/>
-      <c r="E73" s="1" t="inlineStr"/>
-      <c r="F73" s="1" t="inlineStr"/>
-      <c r="G73" s="1" t="inlineStr"/>
-      <c r="H73" s="1" t="inlineStr"/>
-      <c r="I73" s="1" t="inlineStr"/>
-      <c r="J73" s="1" t="inlineStr"/>
-      <c r="K73" s="1" t="inlineStr"/>
-      <c r="L73" s="1" t="inlineStr"/>
-      <c r="M73" s="1" t="inlineStr"/>
-      <c r="N73" s="1" t="inlineStr"/>
+      <c r="D87" s="1" t="inlineStr"/>
+      <c r="E87" s="1" t="inlineStr"/>
+      <c r="F87" s="1" t="inlineStr"/>
+      <c r="G87" s="1" t="inlineStr"/>
+      <c r="H87" s="1" t="inlineStr"/>
+      <c r="I87" s="1" t="inlineStr"/>
+      <c r="J87" s="1" t="inlineStr"/>
+      <c r="K87" s="1" t="inlineStr"/>
+      <c r="L87" s="1" t="inlineStr"/>
+      <c r="M87" s="1" t="inlineStr"/>
+      <c r="N87" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
changes in calculations by steps of compressor
</commit_message>
<xml_diff>
--- a/results/Профилирование_лопаток.xlsx
+++ b/results/Профилирование_лопаток.xlsx
@@ -429,12 +429,12 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
@@ -713,49 +713,49 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.5001636199179899</v>
+        <v>0.5009381928937913</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.5617100530871115</v>
+        <v>0.5619445913362097</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.5786865325542744</v>
+        <v>0.5788430143500115</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.5886622106352932</v>
+        <v>0.588788042896121</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.5963033137274103</v>
+        <v>0.5964130578426809</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.6029262608455921</v>
+        <v>0.603026388575261</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.609061965975974</v>
+        <v>0.6091558089400462</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>0.6149218274125312</v>
+        <v>0.6150115322162666</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>0.6206230137327287</v>
+        <v>0.6207100273692308</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0.6262289932332992</v>
+        <v>0.6263143456511029</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0.6317654130017214</v>
+        <v>0.631849952496621</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.6372454088562733</v>
+        <v>0.6373298173379243</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>0.6426697333096638</v>
+        <v>0.6427545913547572</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>0.6480299855930918</v>
+        <v>0.6481157962010724</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>0.6533088632224319</v>
+        <v>0.6533960776906537</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -827,49 +827,49 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.3195543453030364</v>
+        <v>0.3211034912546391</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.4426472116412798</v>
+        <v>0.443116288139476</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.4766001705756054</v>
+        <v>0.4769131341670796</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.4965515267376431</v>
+        <v>0.4968031912592987</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.5118337329218774</v>
+        <v>0.5120532211524186</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0.5250796271582407</v>
+        <v>0.5252798826175787</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0.5373510374190045</v>
+        <v>0.537538723347149</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>0.5490707602921192</v>
+        <v>0.54925016989959</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0.560473132932514</v>
+        <v>0.5606471602055181</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>0.5716850919336551</v>
+        <v>0.5718557967692626</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0.5827579314704996</v>
+        <v>0.5829270104602986</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.5937179231796033</v>
+        <v>0.5938867401429052</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>0.6045665720863843</v>
+        <v>0.604736288176571</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>0.6152870766532401</v>
+        <v>0.6154586978692015</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>0.6258448319119204</v>
+        <v>0.626019260848364</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -884,49 +884,49 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.05348029644731106</v>
+        <v>0.05347988022802827</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.05060676323739891</v>
+        <v>0.05060693192612765</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.04753301551061671</v>
+        <v>0.04753332832998856</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.04427214776847856</v>
+        <v>0.04427254892416915</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.04085938848479383</v>
+        <v>0.04085985463305541</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.03733295319982487</v>
+        <v>0.03733346837255656</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0.03373235555441111</v>
+        <v>0.03373290630729443</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0.03015722502249987</v>
+        <v>0.03015779401962254</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0.02662024572341182</v>
+        <v>0.02662081694295447</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>0.02304055589828181</v>
+        <v>0.02304112091977756</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>0.01958188562076119</v>
+        <v>0.01958242589493833</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.01619614885663912</v>
+        <v>0.0161966503741525</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>0.01292913946988257</v>
+        <v>0.01292958534235631</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>0.009764542459919865</v>
+        <v>0.009764917296766951</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>0.006721373732741089</v>
+        <v>0.006721660281119007</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
@@ -941,49 +941,49 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.04452797092663265</v>
+        <v>0.04437525304713333</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.02911522331264094</v>
+        <v>0.02910092532496663</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.02500816934311377</v>
+        <v>0.02501269180249618</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.02261280764116443</v>
+        <v>0.02262529958492056</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.02073668558350001</v>
+        <v>0.02075382689188481</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0.01907548196630301</v>
+        <v>0.01909548304204345</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.01749803524396536</v>
+        <v>0.01751971322713502</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0.01595701889384122</v>
+        <v>0.01597938431123609</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>0.01444924048389688</v>
+        <v>0.01447131067056159</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>0.01294626907285786</v>
+        <v>0.01296724538909818</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0.01146670852973583</v>
+        <v>0.01148575897070705</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.01000035726654358</v>
+        <v>0.01002920574158626</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>0.008579654270020231</v>
+        <v>0.008592823756558501</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>0.007206817239764161</v>
+        <v>0.00721614809988272</v>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>0.005887264029587563</v>
+        <v>0.005898890257028502</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
@@ -998,49 +998,49 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.04448020987657037</v>
+        <v>0.04447872578469382</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.04186394409874142</v>
+        <v>0.04186408438557271</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.03931724706798685</v>
+        <v>0.03931766343598594</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.03673074266682043</v>
+        <v>0.03673126683686326</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.03409232457246877</v>
+        <v>0.03409290159483412</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0.03140138672752691</v>
+        <v>0.03140199028321476</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.02866196877270612</v>
+        <v>0.02866258360820718</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0.02593253872788959</v>
+        <v>0.02593314109349731</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0.02320153751691592</v>
+        <v>0.02320211076010172</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>0.02038017349037437</v>
+        <v>0.0203807239600046</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0.01759544927006901</v>
+        <v>0.01759595626207825</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.01479496235224498</v>
+        <v>0.01479541909653592</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>0.01201274727308245</v>
+        <v>0.01201314073259318</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>0.009230495125408049</v>
+        <v>0.009230817698799113</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>0.006465082432865896</v>
+        <v>0.006465323550020442</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
@@ -1055,49 +1055,49 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.04001686526877036</v>
+        <v>0.0399336197082567</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.02707720376682778</v>
+        <v>0.027082465917497</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.02338158219782631</v>
+        <v>0.02339961722668475</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.02117262765891408</v>
+        <v>0.02119600220118516</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0.01942528113643191</v>
+        <v>0.01945158425099778</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0.01787492022552809</v>
+        <v>0.01790274194357312</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.01640596156846623</v>
+        <v>0.01643431324499545</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.01497588439128392</v>
+        <v>0.01500391865706821</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>0.01358167057566953</v>
+        <v>0.01360853750374109</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0.01219563163415452</v>
+        <v>0.01222064711370299</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>0.01083319806857282</v>
+        <v>0.01085565109038657</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.00948234891135669</v>
+        <v>0.009513430312522246</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>0.008171162389595714</v>
+        <v>0.008186774648133876</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>0.006899240008938476</v>
+        <v>0.006910661345394523</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>0.005668965999215133</v>
+        <v>0.00568214129664112</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -1112,49 +1112,49 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.03529414824668107</v>
+        <v>0.03529557343950659</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.03346157666592845</v>
+        <v>0.03346296508831367</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.03159593607532506</v>
+        <v>0.03159728509910138</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.02969284747215544</v>
+        <v>0.02969415410293409</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.02774885426324433</v>
+        <v>0.02775011511049226</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0.02576079492675613</v>
+        <v>0.02576200616523388</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0.02372649425892189</v>
+        <v>0.02372765158043555</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>0.02169651776215099</v>
+        <v>0.02169760760902936</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>0.01964899080885401</v>
+        <v>0.01965000249008469</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>0.01748552901654696</v>
+        <v>0.01748646599040068</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0.01532167683016455</v>
+        <v>0.01532252323631826</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.0130940194351212</v>
+        <v>0.01309476783030983</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>0.01082418213674616</v>
+        <v>0.0108248199652255</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>0.008481553687055197</v>
+        <v>0.008482070866848957</v>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>0.006069041746897686</v>
+        <v>0.006069425061761733</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -1169,49 +1169,49 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.04312667151729712</v>
+        <v>0.04300265915208532</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.02862233861657726</v>
+        <v>0.02861308194131834</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.02464680623967282</v>
+        <v>0.02465436912570533</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.02230605686053166</v>
+        <v>0.02232088599011457</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.02046837576334395</v>
+        <v>0.02048744138815947</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>0.01883683474810338</v>
+        <v>0.01885848384928689</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.01728602466129522</v>
+        <v>0.01730913418957931</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>0.01577052895767529</v>
+        <v>0.01579414305739371</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>0.01428469864772943</v>
+        <v>0.01430787772541313</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>0.01280456983293463</v>
+        <v>0.01282652202922495</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0.01134616071996539</v>
+        <v>0.01136607536486715</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.00990165258060334</v>
+        <v>0.009929654288552294</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>0.008500126935404936</v>
+        <v>0.008513956839925068</v>
       </c>
       <c r="P13" s="2" t="n">
-        <v>0.007144918104593149</v>
+        <v>0.007154825821260083</v>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>0.005841798328744522</v>
+        <v>0.005853380867601016</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
@@ -1283,49 +1283,49 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.01290066247249668</v>
+        <v>0.01284533583136801</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.008754620694546451</v>
+        <v>0.008737375235053947</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.007733815301414316</v>
+        <v>0.007721960619919079</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.007196147179503915</v>
+        <v>0.007186316534126742</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.006812062968188142</v>
+        <v>0.006803212636311481</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>0.00648721947394594</v>
+        <v>0.006478875496473524</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0.006181976599738744</v>
+        <v>0.006173886689042857</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>0.005879559564322505</v>
+        <v>0.005871550206846132</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>0.005569433407427283</v>
+        <v>0.005561376589232649</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>0.005244605894196547</v>
+        <v>0.00523639893094619</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0.004900748153122187</v>
+        <v>0.004892294203632236</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.004534113091319795</v>
+        <v>0.004525320541147819</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>0.00414164795905212</v>
+        <v>0.004132424258498496</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>0.003720785106801318</v>
+        <v>0.003711033901348967</v>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>0.003269527536965649</v>
+        <v>0.00325914486217734</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
@@ -1340,49 +1340,49 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>65.88480884808848</v>
+        <v>65.91625916259161</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>59.43919439194391</v>
+        <v>59.54544545445454</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>57.80717807178072</v>
+        <v>57.92617926179262</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>56.94611946119461</v>
+        <v>57.07022070220702</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>56.33156331563315</v>
+        <v>56.45821458214582</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>55.8130581305813</v>
+        <v>55.94140941409414</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>55.32770327703277</v>
+        <v>55.45690456904569</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>54.84574845748458</v>
+        <v>54.97579975799758</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>54.34679346793467</v>
+        <v>54.47684476844768</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>53.81213812138121</v>
+        <v>53.94303943039431</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>53.22818228182282</v>
+        <v>53.35908359083591</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>52.57622576225762</v>
+        <v>52.70712707127071</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>51.83756837568376</v>
+        <v>51.96846968469684</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>50.99180991809918</v>
+        <v>51.12271122711227</v>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>50.01515015150152</v>
+        <v>50.14520145201452</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
@@ -1397,49 +1397,49 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>22.74314486148478</v>
+        <v>22.75759304962766</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>19.81033854880426</v>
+        <v>19.8582625963552</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>19.07566438082045</v>
+        <v>19.12914909098895</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>18.68901599763496</v>
+        <v>18.74470603621865</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>18.4133981175232</v>
+        <v>18.47017797056738</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>18.18104712967699</v>
+        <v>18.23854877988621</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>17.96368594671666</v>
+        <v>18.0215359146327</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>17.74795509772907</v>
+        <v>17.80615882297755</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>17.52470474593576</v>
+        <v>17.58288688297654</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>17.28555432812008</v>
+        <v>17.34410087785628</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>17.02440161411968</v>
+        <v>17.08294001320597</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>16.73284667432172</v>
+        <v>16.79138789542323</v>
       </c>
       <c r="O17" s="2" t="n">
-        <v>16.40245103743367</v>
+        <v>16.46101148265325</v>
       </c>
       <c r="P17" s="2" t="n">
-        <v>16.02393781276411</v>
+        <v>16.08254240220031</v>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>15.58635987583843</v>
+        <v>15.64466566168751</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1454,7 +1454,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.5967325673256733</v>
+        <v>0.5977528775287753</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>0.5</v>
@@ -1463,40 +1463,40 @@
         <v>0.5</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.5237714377143772</v>
+        <v>0.5288371883718838</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.5918279182791828</v>
+        <v>0.5968578685786858</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>0.6659883598835988</v>
+        <v>0.670928809288093</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.7434424344243442</v>
+        <v>0.748239682396824</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0.8230803308033081</v>
+        <v>0.8276985769857699</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0.903989139891399</v>
+        <v>0.9084283842838429</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>0.985649756497565</v>
+        <v>0.9898562985629857</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>1.067560975609756</v>
+        <v>1.071570615706157</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1.149364793647937</v>
+        <v>1.153159631596316</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>1.230774807748078</v>
+        <v>1.234336943369434</v>
       </c>
       <c r="P18" s="2" t="n">
-        <v>1.311558315583156</v>
+        <v>1.314887748877489</v>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>1.39169741697417</v>
+        <v>1.394829948299483</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -1511,49 +1511,49 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.360461113243105</v>
+        <v>1.359268994132519</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>1.277218463666814</v>
+        <v>1.276816256101269</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>1.258127592297547</v>
+        <v>1.257855855586862</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1.24348201792478</v>
+        <v>1.243263164380322</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>1.224940931476805</v>
+        <v>1.224751236999864</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>1.199674230278176</v>
+        <v>1.199503573189725</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>1.166091699143498</v>
+        <v>1.165935355979127</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>1.163886000384814</v>
+        <v>1.163736118354602</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>1.182013720855483</v>
+        <v>1.181865457369071</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>1.140273478874963</v>
+        <v>1.140132674049013</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>1.138318454526145</v>
+        <v>1.138178792777726</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>1.124064206434387</v>
+        <v>1.123926134919388</v>
       </c>
       <c r="O19" s="2" t="n">
-        <v>1.125502489526477</v>
+        <v>1.12536318529928</v>
       </c>
       <c r="P19" s="2" t="n">
-        <v>1.114655248939401</v>
+        <v>1.11451547034251</v>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>1.102462436158852</v>
+        <v>1.102321704294059</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
@@ -1568,49 +1568,49 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>65.92305923059232</v>
+        <v>66.07946079460794</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>60.66745667456674</v>
+        <v>60.90120901209012</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>59.16379163791638</v>
+        <v>59.41454414544145</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>58.28318283182831</v>
+        <v>58.54158541585416</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>57.59637596375964</v>
+        <v>57.8590285902859</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>56.97671976719767</v>
+        <v>57.24362243622436</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>56.36811368113681</v>
+        <v>56.63756637566375</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>55.74505745057451</v>
+        <v>56.01706017060171</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>55.08545085450854</v>
+        <v>55.35915359153591</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>54.37144371443715</v>
+        <v>54.64684646846469</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>53.58433584335843</v>
+        <v>53.86228862288623</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>52.70457704577046</v>
+        <v>52.98337983379834</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>51.70836708367084</v>
+        <v>51.98801988019881</v>
       </c>
       <c r="P20" s="2" t="n">
-        <v>50.56850568505685</v>
+        <v>50.84985849858499</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>49.25609256092561</v>
+        <v>49.53829538295383</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -1625,49 +1625,49 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>22.76071716398198</v>
+        <v>22.83258962360599</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>20.36511320949262</v>
+        <v>20.47089229358808</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>19.68617556802523</v>
+        <v>19.79922190857446</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>19.28967943368313</v>
+        <v>19.40594676766502</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>18.98095010819886</v>
+        <v>19.09896690558236</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>18.70274671634997</v>
+        <v>18.82253919235903</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>18.42978317932242</v>
+        <v>18.55060258665135</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>18.15058638052806</v>
+        <v>18.27244488309833</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>17.85523772386471</v>
+        <v>17.97776712120652</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>17.53573236940483</v>
+        <v>17.65894957364337</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>17.18367422312499</v>
+        <v>17.30798415698666</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>16.79024749909142</v>
+        <v>16.91492804853464</v>
       </c>
       <c r="O21" s="2" t="n">
-        <v>16.34464596821867</v>
+        <v>16.46975710705444</v>
       </c>
       <c r="P21" s="2" t="n">
-        <v>15.83435933575202</v>
+        <v>15.96037585383293</v>
       </c>
       <c r="Q21" s="2" t="n">
-        <v>15.24576220617891</v>
+        <v>15.37245159470422</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -1682,7 +1682,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.5995965959659597</v>
+        <v>0.5969115691156912</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>0.5</v>
@@ -1694,37 +1694,37 @@
         <v>0.5</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0.5424055240552406</v>
+        <v>0.5445535455354553</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>0.6196447964479644</v>
+        <v>0.6214706147061471</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0.7019140191401914</v>
+        <v>0.7033639336393365</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>0.7876379763797638</v>
+        <v>0.7887119871198712</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0.8756889568895689</v>
+        <v>0.8763691636916369</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>0.9652256522565226</v>
+        <v>0.9655120551205512</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>1.055639456394564</v>
+        <v>1.05549625496255</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>1.146285962859629</v>
+        <v>1.14580265802658</v>
       </c>
       <c r="O22" s="2" t="n">
-        <v>1.236842968429684</v>
+        <v>1.235983759837598</v>
       </c>
       <c r="P22" s="2" t="n">
-        <v>1.327041970419704</v>
+        <v>1.325771057710577</v>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>1.416918769187692</v>
+        <v>1.415236152361524</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
@@ -1739,49 +1739,49 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.359088961273341</v>
+        <v>1.352074472445295</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>1.281255586487429</v>
+        <v>1.2783289962116</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>1.240045201516039</v>
+        <v>1.237876993184842</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>1.230215889373667</v>
+        <v>1.228319070463965</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>1.209724973243711</v>
+        <v>1.207966186119128</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>1.195630675385311</v>
+        <v>1.193922970751948</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>1.180794306973175</v>
+        <v>1.179090978669131</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>1.162064338786814</v>
+        <v>1.160331887392207</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>1.160014029326455</v>
+        <v>1.158190643726329</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>1.147287997135767</v>
+        <v>1.145351226953136</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>1.142278198656699</v>
+        <v>1.14016782590582</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>1.120744603278987</v>
+        <v>1.136473114810535</v>
       </c>
       <c r="O23" s="2" t="n">
-        <v>1.113967164851394</v>
+        <v>1.111348723153137</v>
       </c>
       <c r="P23" s="2" t="n">
-        <v>1.109786737780181</v>
+        <v>1.106739473390241</v>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>1.095018876527833</v>
+        <v>1.104092932501829</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
@@ -1796,49 +1796,49 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.9011527831077626</v>
+        <v>0.8981724853312972</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.6930461591670356</v>
+        <v>0.6920406402531715</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.6453189807438686</v>
+        <v>0.6446396389671555</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.6087050448119491</v>
+        <v>0.6081579109508056</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.5623523286920129</v>
+        <v>0.5618780924996591</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0.4991855756954389</v>
+        <v>0.4987589329743125</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0.415229247858746</v>
+        <v>0.4148383899478186</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0.4097150009620343</v>
+        <v>0.4093402958865061</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0.4550343021387065</v>
+        <v>0.4546636434226786</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>0.3506836971874072</v>
+        <v>0.3503316851225313</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0.3457961363153633</v>
+        <v>0.3454469819443162</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.3101605160859672</v>
+        <v>0.3098153372984708</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>0.3137562238161928</v>
+        <v>0.3134079632482006</v>
       </c>
       <c r="P24" s="2" t="n">
-        <v>0.2866381223485037</v>
+        <v>0.2862886758562744</v>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>0.2561560903971294</v>
+        <v>0.2558042607351485</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
@@ -1853,49 +1853,49 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>-1.602277596816648</v>
+        <v>-1.619813818886762</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>-1.796861033781428</v>
+        <v>-1.804177509471</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>-1.899886996209901</v>
+        <v>-1.905307517037895</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>-1.924460276565831</v>
+        <v>-1.929202323840088</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>-1.975687566890723</v>
+        <v>-1.98008453470218</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>-2.010923311536721</v>
+        <v>-2.01519257312013</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>-2.048014232567063</v>
+        <v>-2.052272553327172</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>-2.094839153032966</v>
+        <v>-2.099170281519481</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>-2.099964926683862</v>
+        <v>-2.104523390684178</v>
       </c>
       <c r="L25" s="2" t="n">
-        <v>-2.131780007160582</v>
+        <v>-2.136621932617161</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>-2.144304503358252</v>
+        <v>-2.14958043523545</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-2.198138491802532</v>
+        <v>-2.158817212973662</v>
       </c>
       <c r="O25" s="2" t="n">
-        <v>-2.215082087871515</v>
+        <v>-2.221628192117157</v>
       </c>
       <c r="P25" s="2" t="n">
-        <v>-2.225533155549547</v>
+        <v>-2.233151316524398</v>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>-2.262452808680418</v>
+        <v>-2.239767668745428</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
@@ -1939,49 +1939,49 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.2782311443946953</v>
+        <v>0.2781671965720997</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.2911219906853548</v>
+        <v>0.2909087228200907</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.294385619831479</v>
+        <v>0.2941473546432335</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.2961078670481653</v>
+        <v>0.2958596296124711</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.2973376243936491</v>
+        <v>0.2970841059727802</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>0.2983732755101661</v>
+        <v>0.2981165733981956</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.2993445840843663</v>
+        <v>0.2990857729840223</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.3003080621646955</v>
+        <v>0.3000478502071238</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0.3013068803947239</v>
+        <v>0.3010457531766011</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0.3023754883343238</v>
+        <v>0.3021138018217254</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0.303544169499859</v>
+        <v>0.3032822352737538</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.3048482616462355</v>
+        <v>0.304586347768892</v>
       </c>
       <c r="O27" s="2" t="n">
-        <v>0.3063245995180726</v>
+        <v>0.306062964026375</v>
       </c>
       <c r="P27" s="2" t="n">
-        <v>0.3080163716791252</v>
+        <v>0.3077552796434658</v>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>0.3099700757544458</v>
+        <v>0.3097098328783951</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -1996,49 +1996,49 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.2781534450104553</v>
+        <v>0.277841673535937</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.2886656287518554</v>
+        <v>0.2881976304386023</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.2916730163450347</v>
+        <v>0.2911715125014595</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.2934338068009301</v>
+        <v>0.292916800707715</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.2948080497448895</v>
+        <v>0.2942814885309308</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>0.2960467900355973</v>
+        <v>0.2955133667865897</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0.2972632962476837</v>
+        <v>0.2967243629298101</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.2985096870027703</v>
+        <v>0.2979661051671418</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0.2998287835063569</v>
+        <v>0.2992811104249428</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0.3012574702446295</v>
+        <v>0.3007060905665759</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0.302830881781959</v>
+        <v>0.3022761314021425</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.3045911045540071</v>
+        <v>0.3040332909317357</v>
       </c>
       <c r="O28" s="2" t="n">
-        <v>0.3065837738017492</v>
+        <v>0.3060232542672205</v>
       </c>
       <c r="P28" s="2" t="n">
-        <v>0.3088629848981053</v>
+        <v>0.308300239407172</v>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>0.3114881723821596</v>
+        <v>0.3109239263046714</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -2053,49 +2053,49 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.2904139482802001</v>
+        <v>0.2912341491002388</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.1916412719578368</v>
+        <v>0.1941330461990847</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.1960534755270549</v>
+        <v>0.1988390766094632</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.218148573062621</v>
+        <v>0.2210510909446292</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.2466431898372687</v>
+        <v>0.2496084805690395</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>0.2784778608869841</v>
+        <v>0.2814837897989076</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0.3124574800377362</v>
+        <v>0.3154951679505159</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.3433936941249157</v>
+        <v>0.3464422654199729</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0.3715195186914556</v>
+        <v>0.374565437278188</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>0.4062844069665942</v>
+        <v>0.4093487516994832</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0.434905186835059</v>
+        <v>0.4379688224100076</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.4635307849368263</v>
+        <v>0.4665970625846961</v>
       </c>
       <c r="O29" s="2" t="n">
-        <v>0.4876791190147885</v>
+        <v>0.490739911805946</v>
       </c>
       <c r="P29" s="2" t="n">
-        <v>0.510832411291076</v>
+        <v>0.5138918532883772</v>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>0.5308248173918085</v>
+        <v>0.5338823653246009</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2110,49 +2110,49 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.3495540892005352</v>
+        <v>0.3497060542988462</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.2375943919195203</v>
+        <v>0.2395045853283123</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.2408830653897533</v>
+        <v>0.2431517271677378</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.2624785754916061</v>
+        <v>0.2648904640700067</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.2925939224278827</v>
+        <v>0.2950920935257041</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>0.3254921187345331</v>
+        <v>0.3280597699736482</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0.3600055881847862</v>
+        <v>0.3626461795081406</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.3956335418450313</v>
+        <v>0.3983595320457717</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0.4289623756143955</v>
+        <v>0.4317869929485038</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>0.4627786707355405</v>
+        <v>0.4657256923206325</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>0.4939909330973987</v>
+        <v>0.4970823891447421</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.5254642748184707</v>
+        <v>0.5259371335060461</v>
       </c>
       <c r="O30" s="2" t="n">
-        <v>0.5517676975664716</v>
+        <v>0.5552398047649175</v>
       </c>
       <c r="P30" s="2" t="n">
-        <v>0.5738228037633274</v>
+        <v>0.5775337149146863</v>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>0.5930428921694032</v>
+        <v>0.5948017898152202</v>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
@@ -2167,49 +2167,49 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.1452069741401001</v>
+        <v>0.1456170745501194</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.09582063597891839</v>
+        <v>0.09706652309954236</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.09802673776352744</v>
+        <v>0.09941953830473159</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.1090742865313105</v>
+        <v>0.1105255454723146</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.1233215949186344</v>
+        <v>0.1248042402845198</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>0.139238930443492</v>
+        <v>0.1407418948994538</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.1562287400188681</v>
+        <v>0.1577475839752579</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.1716968470624579</v>
+        <v>0.1732211327099864</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>0.1857597593457278</v>
+        <v>0.187282718639094</v>
       </c>
       <c r="L31" s="2" t="n">
-        <v>0.2031422034832971</v>
+        <v>0.2046743758497416</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>0.2174525934175295</v>
+        <v>0.2189844112050038</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.2317653924684132</v>
+        <v>0.233298531292348</v>
       </c>
       <c r="O31" s="2" t="n">
-        <v>0.2438395595073942</v>
+        <v>0.245369955902973</v>
       </c>
       <c r="P31" s="2" t="n">
-        <v>0.255416205645538</v>
+        <v>0.2569459266441886</v>
       </c>
       <c r="Q31" s="2" t="n">
-        <v>0.2654124086959043</v>
+        <v>0.2669411826623004</v>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
@@ -2224,49 +2224,49 @@
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.1747770446002676</v>
+        <v>0.1748530271494231</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.1187971959597601</v>
+        <v>0.1197522926641562</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.1204415326948766</v>
+        <v>0.1215758635838689</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0.131239287745803</v>
+        <v>0.1324452320350033</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.1462969612139414</v>
+        <v>0.147546046762852</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>0.1627460593672665</v>
+        <v>0.1640298849868241</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.1800027940923931</v>
+        <v>0.1813230897540703</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.1978167709225157</v>
+        <v>0.1991797660228859</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>0.2144811878071977</v>
+        <v>0.2158934964742519</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>0.2313893353677703</v>
+        <v>0.2328628461603162</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>0.2469954665486994</v>
+        <v>0.248541194572371</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.2627321374092353</v>
+        <v>0.262968566753023</v>
       </c>
       <c r="O32" s="2" t="n">
-        <v>0.2758838487832358</v>
+        <v>0.2776199023824588</v>
       </c>
       <c r="P32" s="2" t="n">
-        <v>0.2869114018816637</v>
+        <v>0.2887668574573432</v>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>0.2965214460847016</v>
+        <v>0.2974008949076101</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -2281,49 +2281,49 @@
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>53.35933937060781</v>
+        <v>53.35676917324136</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>51.38307563229338</v>
+        <v>51.38331600050014</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>49.62034267307361</v>
+        <v>49.6210561318381</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>47.87513253624866</v>
+        <v>47.87603666132853</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>46.1194012614794</v>
+        <v>46.12040967065293</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>44.34351387073093</v>
+        <v>44.34459019246577</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>42.54414854421805</v>
+        <v>42.54527653026351</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>40.81945430879651</v>
+        <v>40.82060388936851</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>39.14514053867467</v>
+        <v>39.14629283925201</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>37.32867714368869</v>
+        <v>37.32985730399026</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>35.61649935046696</v>
+        <v>35.61768201388339</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>33.88568939496494</v>
+        <v>33.88687735500139</v>
       </c>
       <c r="O33" s="2" t="n">
-        <v>32.20757612848312</v>
+        <v>32.2087582643107</v>
       </c>
       <c r="P33" s="2" t="n">
-        <v>30.51764160718717</v>
+        <v>30.51882188169359</v>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>28.84501685044005</v>
+        <v>28.84619379474446</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2338,49 +2338,49 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>50.84864576114282</v>
+        <v>51.00499045019128</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>50.6444775113062</v>
+        <v>50.79622034876635</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>49.09733449906353</v>
+        <v>49.25019699119846</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>47.35407348435245</v>
+        <v>47.50816996137173</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>45.47136696642195</v>
+        <v>45.62632515477396</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>43.5392539067577</v>
+        <v>43.69442680346505</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>41.56424187793456</v>
+        <v>41.71891401667401</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>39.55194153833671</v>
+        <v>39.70535686343437</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>37.5643630870023</v>
+        <v>37.71565552666295</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>35.54496344673632</v>
+        <v>35.69336044340334</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>33.54761660778107</v>
+        <v>33.69226638153408</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>31.5225247030722</v>
+        <v>31.70639800418256</v>
       </c>
       <c r="O34" s="2" t="n">
-        <v>29.55319076553586</v>
+        <v>29.68800129019249</v>
       </c>
       <c r="P34" s="2" t="n">
-        <v>27.61711713941265</v>
+        <v>27.74570958097211</v>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>25.68796579656799</v>
+        <v>25.84011645995972</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2566,49 +2566,49 @@
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.0516026498899867</v>
+        <v>0.05138134332547203</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.0350184827781858</v>
+        <v>0.03494950094021579</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.03093526120565726</v>
+        <v>0.03088784247967631</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.02878458871801566</v>
+        <v>0.02874526613650697</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.02724825187275257</v>
+        <v>0.02721285054524593</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>0.02594887789578376</v>
+        <v>0.0259155019858941</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.02472790639895497</v>
+        <v>0.02469554675617143</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.02351823825729002</v>
+        <v>0.02348620082738453</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>0.02227773362970913</v>
+        <v>0.0222455063569306</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>0.02097842357678619</v>
+        <v>0.02094559572378476</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>0.01960299261248875</v>
+        <v>0.01956917681452894</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.01813645236527918</v>
+        <v>0.01810128216459127</v>
       </c>
       <c r="O38" s="2" t="n">
-        <v>0.01656659183620848</v>
+        <v>0.01652969703399398</v>
       </c>
       <c r="P38" s="2" t="n">
-        <v>0.01488314042720527</v>
+        <v>0.01484413560539587</v>
       </c>
       <c r="Q38" s="2" t="n">
-        <v>0.0130781101478626</v>
+        <v>0.01303657944870936</v>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
@@ -2623,49 +2623,49 @@
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>10.9366596591929</v>
+        <v>10.90585888251</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>16.01902252432823</v>
+        <v>15.81341224301587</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>15.08372003305326</v>
+        <v>14.87240751702662</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>13.00711119647705</v>
+        <v>12.83632114622654</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>10.9876341637178</v>
+        <v>10.85710382652865</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>9.243357392703798</v>
+        <v>9.144648972380121</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>7.773023913836975</v>
+        <v>7.698182951486129</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>6.619305116283704</v>
+        <v>6.561057711412545</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>5.668023774427132</v>
+        <v>5.621932286777939</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>4.739709931777243</v>
+        <v>4.70422907586592</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>3.980522458340657</v>
+        <v>3.952678441076787</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>3.280082715156502</v>
+        <v>3.258527523147615</v>
       </c>
       <c r="O39" s="2" t="n">
-        <v>2.647979140849933</v>
+        <v>2.631463536177982</v>
       </c>
       <c r="P39" s="2" t="n">
-        <v>2.038800894940752</v>
+        <v>2.026663026633166</v>
       </c>
       <c r="Q39" s="2" t="n">
-        <v>1.446444900407079</v>
+        <v>1.438161160060052</v>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
@@ -2680,49 +2680,49 @@
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>8.458257897784941</v>
+        <v>8.418323479605016</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>8.444697240221616</v>
+        <v>8.360843510124257</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>7.358181064817534</v>
+        <v>7.278353976740703</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>6.283320029589359</v>
+        <v>6.21760357876926</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>5.335761983340662</v>
+        <v>5.283717328421937</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>4.567739432691304</v>
+        <v>4.526159718314659</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>3.935513919724886</v>
+        <v>3.901745127058179</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>3.405925757708602</v>
+        <v>3.378011033584674</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>2.975606178441053</v>
+        <v>2.951864378307122</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>2.597307255232921</v>
+        <v>2.576833440792933</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>2.273669709406926</v>
+        <v>2.255631623425026</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>1.977576530667574</v>
+        <v>1.971967079201872</v>
       </c>
       <c r="O40" s="2" t="n">
-        <v>1.720288203131946</v>
+        <v>1.705723499013519</v>
       </c>
       <c r="P40" s="2" t="n">
-        <v>1.486076695840159</v>
+        <v>1.472658477526947</v>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>1.263523887202407</v>
+        <v>1.255786967331678</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
@@ -2737,49 +2737,49 @@
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>0.04074674662105197</v>
+        <v>0.04078248272299415</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.04195048959377978</v>
+        <v>0.04196370434117381</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.04102376136360771</v>
+        <v>0.04103262379559733</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.03982637929620157</v>
+        <v>0.03983338999556241</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.03861314758136208</v>
+        <v>0.038619128143465</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>0.0374484657596978</v>
+        <v>0.03745379366890653</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0.03635172759635227</v>
+        <v>0.03635660208968813</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.03408560362043529</v>
+        <v>0.03408999363582712</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>0.03109334083821417</v>
+        <v>0.03109724145743279</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>0.02947469723992853</v>
+        <v>0.02947833732472679</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0.02654282930051913</v>
+        <v>0.02654608627382738</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.02360741543891134</v>
+        <v>0.02361031555086139</v>
       </c>
       <c r="O41" s="2" t="n">
-        <v>0.02002526708248775</v>
+        <v>0.02002774593055366</v>
       </c>
       <c r="P41" s="2" t="n">
-        <v>0.01630754643516592</v>
+        <v>0.01630959167008648</v>
       </c>
       <c r="Q41" s="2" t="n">
-        <v>0.0121552844746468</v>
+        <v>0.01215683632275478</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
@@ -2794,49 +2794,49 @@
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0.03796855935143479</v>
+        <v>0.03800185890097182</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.02733137958382622</v>
+        <v>0.02733998919197687</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.02494688191030198</v>
+        <v>0.02495227122705243</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.02339799783651842</v>
+        <v>0.02340211662239292</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.02252433608912788</v>
+        <v>0.02252782475035458</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>0.02170308811073396</v>
+        <v>0.0217061758762981</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.02094175611528989</v>
+        <v>0.02094456424732034</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.02023832714963345</v>
+        <v>0.02024093372127235</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>0.01920471051772052</v>
+        <v>0.01920711972370849</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>0.01828522884328899</v>
+        <v>0.01828748704404347</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>0.01716131204774944</v>
+        <v>0.01716341784945736</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.01618250251860858</v>
+        <v>0.01592759382399379</v>
       </c>
       <c r="O42" s="2" t="n">
-        <v>0.01487170570096517</v>
+        <v>0.01487354661019059</v>
       </c>
       <c r="P42" s="2" t="n">
-        <v>0.01341081121312987</v>
+        <v>0.01341249314974217</v>
       </c>
       <c r="Q42" s="2" t="n">
-        <v>0.01194327369892622</v>
+        <v>0.01180750194566413</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
@@ -2941,7 +2941,7 @@
         <v>116</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="O44" s="2" t="n">
         <v>136</v>
@@ -2950,7 +2950,7 @@
         <v>152</v>
       </c>
       <c r="Q44" s="2" t="n">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
@@ -3055,7 +3055,7 @@
         <v>0.01843716486403236</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.01724767035667543</v>
+        <v>0.01697389781133138</v>
       </c>
       <c r="O46" s="2" t="n">
         <v>0.01572581708990995</v>
@@ -3064,7 +3064,7 @@
         <v>0.01407046792255101</v>
       </c>
       <c r="Q46" s="2" t="n">
-        <v>0.01243436700132415</v>
+        <v>0.01229144324268824</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
@@ -3136,49 +3136,49 @@
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>1.061628459046452</v>
+        <v>1.057075488461347</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>1.080660140202337</v>
+        <v>1.078531380850761</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>1.070368645529548</v>
+        <v>1.068727944416228</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>1.07670786921854</v>
+        <v>1.075236980286856</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>1.070202109757892</v>
+        <v>1.068811687518595</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>1.067699713608353</v>
+        <v>1.066326419180219</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>1.063709522493508</v>
+        <v>1.062317521908501</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>1.055659573246514</v>
+        <v>1.054221514017249</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>1.062475808204731</v>
+        <v>1.060938816235048</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>1.059362211486601</v>
+        <v>1.057704480302623</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>1.063232484877906</v>
+        <v>1.061398374362044</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>1.051530553995065</v>
+        <v>1.066418707464309</v>
       </c>
       <c r="O48" s="2" t="n">
-        <v>1.053464614365761</v>
+        <v>1.051118484940272</v>
       </c>
       <c r="P48" s="2" t="n">
-        <v>1.057757319026454</v>
+        <v>1.054985213505578</v>
       </c>
       <c r="Q48" s="2" t="n">
-        <v>1.0517712840927</v>
+        <v>1.060622352583728</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
@@ -3250,49 +3250,49 @@
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>-2.345928852383871</v>
+        <v>-2.357311278846633</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>-2.298349649494156</v>
+        <v>-2.303671547873098</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>-2.32407838617613</v>
+        <v>-2.32818013895943</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>-2.30823032695365</v>
+        <v>-2.311907549282859</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>-2.324494725605269</v>
+        <v>-2.327970781203512</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>-2.330750715979118</v>
+        <v>-2.334183952049453</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>-2.34072619376623</v>
+        <v>-2.344206195228748</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>-2.360851066883716</v>
+        <v>-2.364446214956878</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>-2.343810479488172</v>
+        <v>-2.347652959412381</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>-2.351594471283497</v>
+        <v>-2.355738799243444</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>-2.341918787805235</v>
+        <v>-2.34650406409489</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-2.371173615012338</v>
+        <v>-2.333953231339227</v>
       </c>
       <c r="O50" s="2" t="n">
-        <v>-2.366338464085598</v>
+        <v>-2.372203787649321</v>
       </c>
       <c r="P50" s="2" t="n">
-        <v>-2.355606702433866</v>
+        <v>-2.362536966236055</v>
       </c>
       <c r="Q50" s="2" t="n">
-        <v>-2.37057178976825</v>
+        <v>-2.348444118540681</v>
       </c>
     </row>
     <row r="51" ht="30" customHeight="1">
@@ -3307,49 +3307,49 @@
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>0.3176095213652849</v>
+        <v>0.3173006382047701</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>0.3179200855650576</v>
+        <v>0.3176113022404495</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0.318230418867067</v>
+        <v>0.3179217563220058</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>0.3185335230500181</v>
+        <v>0.3182250045306538</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.3188249400168262</v>
+        <v>0.3185165901510365</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>0.3191002082184362</v>
+        <v>0.3187920527813159</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>0.3193582377635946</v>
+        <v>0.3190503032947515</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.319598513298731</v>
+        <v>0.3192908273743471</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0.3198246105861322</v>
+        <v>0.3195172021318117</v>
       </c>
       <c r="L51" s="2" t="n">
-        <v>0.3200420163464603</v>
+        <v>0.319734916477971</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>0.3202600192180161</v>
+        <v>0.3199532623648659</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.3204936635127881</v>
+        <v>0.3201872891209281</v>
       </c>
       <c r="O51" s="2" t="n">
-        <v>0.3207624130389822</v>
+        <v>0.3204564681314989</v>
       </c>
       <c r="P51" s="2" t="n">
-        <v>0.3210943081874975</v>
+        <v>0.3207888515240575</v>
       </c>
       <c r="Q51" s="2" t="n">
-        <v>0.3215255233993043</v>
+        <v>0.3212206323758896</v>
       </c>
     </row>
     <row r="52" ht="30" customHeight="1">
@@ -3421,49 +3421,49 @@
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>0.1698965375383986</v>
+        <v>0.1737171085455128</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>0.1883833902871027</v>
+        <v>0.1921854632746524</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.2070862547859797</v>
+        <v>0.210874088624505</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0.2263019162537689</v>
+        <v>0.2300796950091716</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.2462915644251765</v>
+        <v>0.2500636244277133</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>0.2673499451646901</v>
+        <v>0.2711209925840055</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.2897581104690655</v>
+        <v>0.2935335559587714</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.3089741139134963</v>
+        <v>0.3127343357993995</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0.3258732342397151</v>
+        <v>0.3296058102779497</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>0.3501409914471718</v>
+        <v>0.353881788343289</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0.3694959824157375</v>
+        <v>0.3732205404482752</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.3902439354768183</v>
+        <v>0.3939596163909047</v>
       </c>
       <c r="O53" s="2" t="n">
-        <v>0.4083141054527459</v>
+        <v>0.4120112947882481</v>
       </c>
       <c r="P53" s="2" t="n">
-        <v>0.4272210271933259</v>
+        <v>0.4309072937974451</v>
       </c>
       <c r="Q53" s="2" t="n">
-        <v>0.4450113611693607</v>
+        <v>0.4486878124043132</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
@@ -3478,49 +3478,49 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>0.3636236830873243</v>
+        <v>0.3609457115181305</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>0.3940699550525534</v>
+        <v>0.3910121589041948</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.4268664268894479</v>
+        <v>0.4236566283461362</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>0.4562342718001332</v>
+        <v>0.4529278512852163</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.4857934672082915</v>
+        <v>0.4824115285556035</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>0.5129814566049137</v>
+        <v>0.5095506140891612</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.5381208667926274</v>
+        <v>0.5346643540036551</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.5610876312798708</v>
+        <v>0.5576283429501668</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0.5781803888561092</v>
+        <v>0.5747535128897914</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>0.5926193539275433</v>
+        <v>0.5892468124058294</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0.6008088973299066</v>
+        <v>0.5975237122270933</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.6058106626833105</v>
+        <v>0.5996652385437593</v>
       </c>
       <c r="O54" s="2" t="n">
-        <v>0.6017265230227838</v>
+        <v>0.5986998906738616</v>
       </c>
       <c r="P54" s="2" t="n">
-        <v>0.5897955340580403</v>
+        <v>0.5869554415245498</v>
       </c>
       <c r="Q54" s="2" t="n">
-        <v>0.5758528641222752</v>
+        <v>0.5710371829011919</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
@@ -3535,49 +3535,49 @@
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>0.05562671853027708</v>
+        <v>0.05682231685729708</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>0.06216126583194667</v>
+        <v>0.0633542505743461</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.06867572282136881</v>
+        <v>0.06986404750469015</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>0.07520061782934841</v>
+        <v>0.07638192977577055</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.08174269946628178</v>
+        <v>0.08291435584145446</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>0.08830085131058422</v>
+        <v>0.08945988504334802</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>0.09484282342809748</v>
+        <v>0.09598595004238103</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.1015380751663378</v>
+        <v>0.1026748527692</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>0.1084425531441556</v>
+        <v>0.1095792356290587</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>0.1149848122162595</v>
+        <v>0.1161017602681656</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>0.1218070734474477</v>
+        <v>0.1229170540849989</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.1284425117023587</v>
+        <v>0.1295415151967718</v>
       </c>
       <c r="O55" s="2" t="n">
-        <v>0.1351216271196396</v>
+        <v>0.1362150753442319</v>
       </c>
       <c r="P55" s="2" t="n">
-        <v>0.1413932783163229</v>
+        <v>0.1424776190355522</v>
       </c>
       <c r="Q55" s="2" t="n">
-        <v>0.1472374559040594</v>
+        <v>0.1483130813753793</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
@@ -3592,49 +3592,49 @@
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>0.09968542647845208</v>
+        <v>0.09873886284363749</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>0.1094611116294252</v>
+        <v>0.1085047170526714</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.1186100613858937</v>
+        <v>0.1176279235584212</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.1279111690365455</v>
+        <v>0.1268974052708382</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.1367318916492712</v>
+        <v>0.1356917756232247</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>0.1453639962070348</v>
+        <v>0.144298905884079</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.1535774069325275</v>
+        <v>0.1524910577754558</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.1611503102091336</v>
+        <v>0.1600476429986036</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0.1684995994016883</v>
+        <v>0.1673797036520552</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>0.174656962810124</v>
+        <v>0.1735270757987532</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>0.1799138290401008</v>
+        <v>0.1787756748849112</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.1832452134458469</v>
+        <v>0.1826659205952031</v>
       </c>
       <c r="O56" s="2" t="n">
-        <v>0.1853228224540481</v>
+        <v>0.1841852256638633</v>
       </c>
       <c r="P56" s="2" t="n">
-        <v>0.1854429752797969</v>
+        <v>0.1843080086621809</v>
       </c>
       <c r="Q56" s="2" t="n">
-        <v>0.184006134738683</v>
+        <v>0.1832335064599259</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
@@ -3649,49 +3649,49 @@
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>0.08494826876919929</v>
+        <v>0.08685855427275639</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>0.09419169514355137</v>
+        <v>0.09609273163732619</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.1035431273929898</v>
+        <v>0.1054370443122525</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.1131509581268844</v>
+        <v>0.1150398475045858</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.1231457822125883</v>
+        <v>0.1250318122138567</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>0.133674972582345</v>
+        <v>0.1355604962920027</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.1448790552345327</v>
+        <v>0.1467667779793857</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.1544870569567482</v>
+        <v>0.1563671678996997</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0.1629366171198576</v>
+        <v>0.1648029051389749</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>0.1750704957235859</v>
+        <v>0.1769408941716445</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>0.1847479912078688</v>
+        <v>0.1866102702241376</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.1951219677384092</v>
+        <v>0.1969798081954524</v>
       </c>
       <c r="O57" s="2" t="n">
-        <v>0.2041570527263729</v>
+        <v>0.206005647394124</v>
       </c>
       <c r="P57" s="2" t="n">
-        <v>0.2136105135966629</v>
+        <v>0.2154536468987226</v>
       </c>
       <c r="Q57" s="2" t="n">
-        <v>0.2225056805846804</v>
+        <v>0.2243439062021566</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
@@ -3706,49 +3706,49 @@
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>0.1818118415436621</v>
+        <v>0.1804728557590653</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>0.1970349775262767</v>
+        <v>0.1955060794520974</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.2134332134447239</v>
+        <v>0.2118283141730681</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0.2281171359000666</v>
+        <v>0.2264639256426082</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.2428967336041457</v>
+        <v>0.2412057642778018</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>0.2564907283024568</v>
+        <v>0.2547753070445806</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.2690604333963137</v>
+        <v>0.2673321770018275</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.2805438156399354</v>
+        <v>0.2788141714750834</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>0.2890901944280546</v>
+        <v>0.2873767564448957</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0.2963096769637716</v>
+        <v>0.2946234062029147</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>0.3004044486649533</v>
+        <v>0.2987618561135467</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.3029053313416553</v>
+        <v>0.2998326192718797</v>
       </c>
       <c r="O58" s="2" t="n">
-        <v>0.3008632615113919</v>
+        <v>0.2993499453369308</v>
       </c>
       <c r="P58" s="2" t="n">
-        <v>0.2948977670290202</v>
+        <v>0.2934777207622749</v>
       </c>
       <c r="Q58" s="2" t="n">
-        <v>0.2879264320611376</v>
+        <v>0.2855185914505959</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
@@ -3763,49 +3763,49 @@
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>39.54496291353914</v>
+        <v>39.54687319904271</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>38.64673621985121</v>
+        <v>38.64863725634498</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>37.74647387474349</v>
+        <v>37.74836779166276</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>36.83926729732154</v>
+        <v>36.84115618669924</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>35.92113438425852</v>
+        <v>35.92302041425979</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>34.98804897313749</v>
+        <v>34.98993449684714</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>34.03688062117565</v>
+        <v>34.03876834392051</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>33.15465738462369</v>
+        <v>33.15653749556665</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>32.31857361999521</v>
+        <v>32.32043990801433</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>31.34969046228904</v>
+        <v>31.3515608607371</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>30.47098621212547</v>
+        <v>30.47284849114174</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>29.56686489945214</v>
+        <v>29.56872273990918</v>
       </c>
       <c r="O59" s="2" t="n">
-        <v>28.70194360956346</v>
+        <v>28.70379220423122</v>
       </c>
       <c r="P59" s="2" t="n">
-        <v>27.81392435857617</v>
+        <v>27.81576749187823</v>
       </c>
       <c r="Q59" s="2" t="n">
-        <v>26.92915224627476</v>
+        <v>26.93099047189223</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
@@ -3820,49 +3820,49 @@
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>56.69352265537425</v>
+        <v>56.81748671774152</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>54.82033976456226</v>
+        <v>54.95465707283512</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>52.81821614195854</v>
+        <v>52.95761261992859</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>50.79873545786026</v>
+        <v>50.94181738031107</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>48.69280482531953</v>
+        <v>48.83865014039614</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>46.54551612353002</v>
+        <v>46.69319038385163</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>44.35077565348564</v>
+        <v>44.49933864148981</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>42.11075743378222</v>
+        <v>42.25923260463952</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>39.88208220037828</v>
+        <v>40.02939842969723</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>37.61615579534509</v>
+        <v>37.76130120215889</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>35.3660009789853</v>
+        <v>35.50789998136179</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>33.08981995091819</v>
+        <v>33.26833551173312</v>
       </c>
       <c r="O60" s="2" t="n">
-        <v>30.86976974185301</v>
+        <v>31.00215740679556</v>
       </c>
       <c r="P60" s="2" t="n">
-        <v>28.6898373527907</v>
+        <v>28.81589740113847</v>
       </c>
       <c r="Q60" s="2" t="n">
-        <v>26.53120828165639</v>
+        <v>26.67933006955999</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
@@ -3934,49 +3934,49 @@
         </is>
       </c>
       <c r="C62" s="2" t="n">
-        <v>0.02281612690060716</v>
+        <v>0.0229267356629002</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>0.02106995800339774</v>
+        <v>0.02109228599249933</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0.02023356208891843</v>
+        <v>0.02024684863107812</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0.01949953285659719</v>
+        <v>0.01950941569925222</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.01914253684770012</v>
+        <v>0.01915074568832652</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>0.01874529885488633</v>
+        <v>0.01875244795806698</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>0.01834932686472172</v>
+        <v>0.01835573591616782</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.01796829861286129</v>
+        <v>0.01797416977853643</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>0.01726253212701217</v>
+        <v>0.01726789215448662</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>0.01662964523134793</v>
+        <v>0.01663461083373197</v>
       </c>
       <c r="M62" s="2" t="n">
-        <v>0.01578265548559401</v>
+        <v>0.01578723460035461</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.01504209569165831</v>
+        <v>0.01480754142775668</v>
       </c>
       <c r="O62" s="2" t="n">
-        <v>0.01396545515788639</v>
+        <v>0.01396937559040203</v>
       </c>
       <c r="P62" s="2" t="n">
-        <v>0.01271698263067473</v>
+        <v>0.01272052976193305</v>
       </c>
       <c r="Q62" s="2" t="n">
-        <v>0.01143110189663737</v>
+        <v>0.01130285925797088</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
@@ -4048,49 +4048,49 @@
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>2.261674389995328</v>
+        <v>2.24111029502629</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>1.662010089082224</v>
+        <v>1.656980232140047</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>1.528908309357944</v>
+        <v>1.525562967476563</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>1.476168117959662</v>
+        <v>1.473404769247331</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>1.423439959371232</v>
+        <v>1.42098124992771</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>1.384287233650568</v>
+        <v>1.381979677738324</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>1.347619265886895</v>
+        <v>1.345385816671043</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>1.308873965421312</v>
+        <v>1.306664013791068</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>1.290525252367192</v>
+        <v>1.288258355907711</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>1.261507583892441</v>
+        <v>1.259157544059335</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>1.242059210529042</v>
+        <v>1.23955697814799</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>1.205713135792432</v>
+        <v>1.222436705843719</v>
       </c>
       <c r="O64" s="2" t="n">
-        <v>1.186255059281273</v>
+        <v>1.183281022621447</v>
       </c>
       <c r="P64" s="2" t="n">
-        <v>1.17033583039624</v>
+        <v>1.166943192084487</v>
       </c>
       <c r="Q64" s="2" t="n">
-        <v>1.144081320079013</v>
+        <v>1.153387753591274</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
@@ -4162,49 +4162,49 @@
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>0.6541859749883205</v>
+        <v>0.602775737565725</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>-0.8449747772944399</v>
+        <v>-0.8575494196498834</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>-1.177729226605141</v>
+        <v>-1.186092581308593</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>-1.309579705100846</v>
+        <v>-1.316488076881673</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>-1.441400101571921</v>
+        <v>-1.447546875180725</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>-1.539281915873579</v>
+        <v>-1.54505080565419</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>-1.630951835282762</v>
+        <v>-1.636535458322393</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>-1.72781508644672</v>
+        <v>-1.73333996552233</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>-1.773686869082021</v>
+        <v>-1.779354110230722</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>-1.846231040268896</v>
+        <v>-1.852106139851663</v>
       </c>
       <c r="M66" s="2" t="n">
-        <v>-1.894851973677396</v>
+        <v>-1.901107554630026</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-1.985717160518919</v>
+        <v>-1.943908235390702</v>
       </c>
       <c r="O66" s="2" t="n">
-        <v>-2.034362351796817</v>
+        <v>-2.041797443446383</v>
       </c>
       <c r="P66" s="2" t="n">
-        <v>-2.0741604240094</v>
+        <v>-2.082642019788783</v>
       </c>
       <c r="Q66" s="2" t="n">
-        <v>-2.139796699802467</v>
+        <v>-2.116530616021816</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
@@ -4219,49 +4219,49 @@
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>0.244768588559608</v>
+        <v>0.2450886420156227</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>0.2735230086193629</v>
+        <v>0.273420185033782</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0.280181275064998</v>
+        <v>0.2800164308751246</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>0.2836920511433934</v>
+        <v>0.28350192241841</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.2862045683136525</v>
+        <v>0.2860001002345475</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>0.2883050376207305</v>
+        <v>0.2880909792836339</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.2902332234196005</v>
+        <v>0.290011986028923</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.2920880812699925</v>
+        <v>0.2918612110201229</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>0.2939349466203122</v>
+        <v>0.2937034924039966</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>0.2958192807537868</v>
+        <v>0.2955840094789561</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>0.2977750424397602</v>
+        <v>0.2975366063925467</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.2998386802528163</v>
+        <v>0.2995976361698822</v>
       </c>
       <c r="O67" s="2" t="n">
-        <v>0.3020458779246915</v>
+        <v>0.3018027454215164</v>
       </c>
       <c r="P67" s="2" t="n">
-        <v>0.3044371728435766</v>
+        <v>0.3041924635356923</v>
       </c>
       <c r="Q67" s="2" t="n">
-        <v>0.3070551938599419</v>
+        <v>0.3068094564057059</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
@@ -4333,49 +4333,49 @@
         </is>
       </c>
       <c r="C69" s="2" t="n">
-        <v>0.1644673404247142</v>
+        <v>0.1611981582144354</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>-0.05558343842748145</v>
+        <v>-0.05448512024119608</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>-0.0469585307628413</v>
+        <v>-0.0451762325450814</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>-0.004883830027398508</v>
+        <v>-0.002812489733490704</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.04776910885093914</v>
+        <v>0.05001107298489656</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>0.104682471344049</v>
+        <v>0.1070446558962952</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0.1632558691814683</v>
+        <v>0.1657143961281069</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.2181738540494817</v>
+        <v>0.2207034825152581</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>0.2691873373494308</v>
+        <v>0.2717704906125423</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>0.3245696290177395</v>
+        <v>0.3272157718516041</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>0.3725843529927163</v>
+        <v>0.3752750194101367</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.4187289468505993</v>
+        <v>0.4214629667741911</v>
       </c>
       <c r="O69" s="2" t="n">
-        <v>0.458802591764033</v>
+        <v>0.4615701955891656</v>
       </c>
       <c r="P69" s="2" t="n">
-        <v>0.4960957823619158</v>
+        <v>0.4988973546970896</v>
       </c>
       <c r="Q69" s="2" t="n">
-        <v>0.5286492929786418</v>
+        <v>0.5314816569981683</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
@@ -4390,49 +4390,49 @@
         </is>
       </c>
       <c r="C70" s="2" t="n">
-        <v>0.2640853098699804</v>
+        <v>0.2625353735500591</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0.3373292157659991</v>
+        <v>0.3346307234501876</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0.3781921815468364</v>
+        <v>0.3752575132771734</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>0.4115220998204198</v>
+        <v>0.4084555841463008</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.4438299371417339</v>
+        <v>0.4406672250073639</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>0.4733531619917389</v>
+        <v>0.4701257702030213</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0.5007078174389558</v>
+        <v>0.4974411632014777</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.525876616658009</v>
+        <v>0.5225947904479865</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>0.5453712343993459</v>
+        <v>0.5421086928977191</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>0.5622779405222017</v>
+        <v>0.5590573194275863</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>0.5731421064021958</v>
+        <v>0.569996012285054</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.5808563655327604</v>
+        <v>0.5749638861872786</v>
       </c>
       <c r="O70" s="2" t="n">
-        <v>0.5797354623106791</v>
+        <v>0.5768230445364327</v>
       </c>
       <c r="P70" s="2" t="n">
-        <v>0.570897633136825</v>
+        <v>0.5681590952860041</v>
       </c>
       <c r="Q70" s="2" t="n">
-        <v>0.5600013512482378</v>
+        <v>0.5553434743256773</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
@@ -4447,49 +4447,49 @@
         </is>
       </c>
       <c r="C71" s="2" t="n">
-        <v>0.0632858365372804</v>
+        <v>0.06210898514394837</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>-0.02314522082282575</v>
+        <v>-0.02267934676145549</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>-0.01939746277424421</v>
+        <v>-0.0186502580610428</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>-0.001977159295452177</v>
+        <v>-0.001137839239642961</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.01886361044271688</v>
+        <v>0.01973483391768834</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>0.04019290773057611</v>
+        <v>0.04106935464220979</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>0.06075836299402841</v>
+        <v>0.0616263323072546</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.0798357643341111</v>
+        <v>0.08069869548884291</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>0.09781014477568209</v>
+        <v>0.09867098433210125</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>0.1142743122442787</v>
+        <v>0.1151143391676647</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>0.1294667719525114</v>
+        <v>0.1302973171202928</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.1430065098041257</v>
+        <v>0.1438245312790599</v>
       </c>
       <c r="O71" s="2" t="n">
-        <v>0.155282651889511</v>
+        <v>0.1560936038052568</v>
       </c>
       <c r="P71" s="2" t="n">
-        <v>0.1657087788932929</v>
+        <v>0.1665106258748914</v>
       </c>
       <c r="Q71" s="2" t="n">
-        <v>0.1744031482123807</v>
+        <v>0.175197231139362</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
@@ -4504,49 +4504,49 @@
         </is>
       </c>
       <c r="C72" s="2" t="n">
-        <v>0.1056701971133371</v>
+        <v>0.1045713408724083</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.1162017712538874</v>
+        <v>0.1150976454708926</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>0.1255931951687216</v>
+        <v>0.1244822150738495</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>0.1350929521424367</v>
+        <v>0.1339607258952853</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.1440692913792906</v>
+        <v>0.1429190678330644</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>0.1527316394404971</v>
+        <v>0.1515638087565276</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>0.160843661665733</v>
+        <v>0.1596618350910941</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.1681788119795944</v>
+        <v>0.1669881090547966</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0.175166669052629</v>
+        <v>0.1739657870063144</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>0.180835550594171</v>
+        <v>0.179632208016393</v>
       </c>
       <c r="M72" s="2" t="n">
-        <v>0.1855015478898817</v>
+        <v>0.1842973697817023</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.1881375687333493</v>
+        <v>0.1875160889632148</v>
       </c>
       <c r="O72" s="2" t="n">
-        <v>0.1894692258255292</v>
+        <v>0.1882809266221269</v>
       </c>
       <c r="P72" s="2" t="n">
-        <v>0.1888119077973828</v>
+        <v>0.1876336418572714</v>
       </c>
       <c r="Q72" s="2" t="n">
-        <v>0.1866283596815477</v>
+        <v>0.1858272746503072</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
@@ -4561,49 +4561,49 @@
         </is>
       </c>
       <c r="C73" s="2" t="n">
-        <v>0.0822336702123571</v>
+        <v>0.08059907910721771</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>-0.02779171921374073</v>
+        <v>-0.02724256012059804</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>-0.02347926538142065</v>
+        <v>-0.0225881162725407</v>
       </c>
       <c r="F73" s="2" t="n">
-        <v>-0.002441915013699254</v>
+        <v>-0.001406244866745352</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>0.02388455442546957</v>
+        <v>0.02500553649244828</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>0.05234123567202452</v>
+        <v>0.05352232794814759</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>0.08162793459073414</v>
+        <v>0.08285719806405345</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.1090869270247409</v>
+        <v>0.1103517412576291</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>0.1345936686747154</v>
+        <v>0.1358852453062711</v>
       </c>
       <c r="L73" s="2" t="n">
-        <v>0.1622848145088698</v>
+        <v>0.163607885925802</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>0.1862921764963582</v>
+        <v>0.1876375097050683</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.2093644734252997</v>
+        <v>0.2107314833870955</v>
       </c>
       <c r="O73" s="2" t="n">
-        <v>0.2294012958820165</v>
+        <v>0.2307850977945828</v>
       </c>
       <c r="P73" s="2" t="n">
-        <v>0.2480478911809579</v>
+        <v>0.2494486773485448</v>
       </c>
       <c r="Q73" s="2" t="n">
-        <v>0.2643246464893209</v>
+        <v>0.2657408284990841</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
@@ -4618,49 +4618,49 @@
         </is>
       </c>
       <c r="C74" s="2" t="n">
-        <v>0.1320426549349902</v>
+        <v>0.1312676867750295</v>
       </c>
       <c r="D74" s="2" t="n">
-        <v>0.1686646078829995</v>
+        <v>0.1673153617250938</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>0.1890960907734182</v>
+        <v>0.1876287566385867</v>
       </c>
       <c r="F74" s="2" t="n">
-        <v>0.2057610499102099</v>
+        <v>0.2042277920731504</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.2219149685708669</v>
+        <v>0.2203336125036819</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>0.2366765809958695</v>
+        <v>0.2350628851015106</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>0.2503539087194779</v>
+        <v>0.2487205816007388</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.2629383083290045</v>
+        <v>0.2612973952239933</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>0.2726856171996729</v>
+        <v>0.2710543464488596</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>0.2811389702611009</v>
+        <v>0.2795286597137931</v>
       </c>
       <c r="M74" s="2" t="n">
-        <v>0.2865710532010979</v>
+        <v>0.284998006142527</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.2904281827663802</v>
+        <v>0.2874819430936393</v>
       </c>
       <c r="O74" s="2" t="n">
-        <v>0.2898677311553395</v>
+        <v>0.2884115222682164</v>
       </c>
       <c r="P74" s="2" t="n">
-        <v>0.2854488165684125</v>
+        <v>0.284079547643002</v>
       </c>
       <c r="Q74" s="2" t="n">
-        <v>0.2800006756241189</v>
+        <v>0.2776717371628387</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
@@ -4675,49 +4675,49 @@
         </is>
       </c>
       <c r="C75" s="2" t="n">
-        <v>74.74184645402445</v>
+        <v>74.74021186291931</v>
       </c>
       <c r="D75" s="2" t="n">
-        <v>70.8232109466645</v>
+        <v>70.82376010575764</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>67.06509808052596</v>
+        <v>67.06598922963484</v>
       </c>
       <c r="F75" s="2" t="n">
-        <v>63.37572698492632</v>
+        <v>63.37676265507328</v>
       </c>
       <c r="G75" s="2" t="n">
-        <v>59.7523664767103</v>
+        <v>59.75348745877728</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>56.20040973870197</v>
+        <v>56.20159083097809</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>52.72827832480113</v>
+        <v>52.72950758827445</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>49.47906609025372</v>
+        <v>49.48033090448661</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>46.41115574374071</v>
+        <v>46.41244732037226</v>
       </c>
       <c r="L75" s="2" t="n">
-        <v>43.27831062414885</v>
+        <v>43.27963369556578</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>40.39867082198991</v>
+        <v>40.40001615519862</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>37.61412831964161</v>
+        <v>37.61549532960341</v>
       </c>
       <c r="O75" s="2" t="n">
-        <v>35.00494650926174</v>
+        <v>35.0063303111743</v>
       </c>
       <c r="P75" s="2" t="n">
-        <v>32.49211625961495</v>
+        <v>32.49351704578254</v>
       </c>
       <c r="Q75" s="2" t="n">
-        <v>30.10373850058883</v>
+        <v>30.10515468259859</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
@@ -4732,49 +4732,49 @@
         </is>
       </c>
       <c r="C76" s="2" t="n">
-        <v>59.64386829613776</v>
+        <v>59.72836856516984</v>
       </c>
       <c r="D76" s="2" t="n">
-        <v>56.2453442671187</v>
+        <v>56.37258848333133</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>53.94022817885823</v>
+        <v>54.07550062004495</v>
       </c>
       <c r="F76" s="2" t="n">
-        <v>51.7750299937232</v>
+        <v>51.9150007191428</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>49.5549176843196</v>
+        <v>49.6982018946448</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>47.31717077632896</v>
+        <v>47.46261110830381</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>45.04184348729227</v>
+        <v>45.18839778299508</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>42.72618790690829</v>
+        <v>42.87282207782296</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>40.43580123355604</v>
+        <v>40.58137486888285</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>38.10634851965703</v>
+        <v>38.24983911506154</v>
       </c>
       <c r="M76" s="2" t="n">
-        <v>35.79923439764929</v>
+        <v>35.93953264085562</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>33.46279925683634</v>
+        <v>33.64602983150341</v>
       </c>
       <c r="O76" s="2" t="n">
-        <v>31.19075032378574</v>
+        <v>31.32162532792979</v>
       </c>
       <c r="P76" s="2" t="n">
-        <v>28.96183468075457</v>
+        <v>29.08639417446647</v>
       </c>
       <c r="Q76" s="2" t="n">
-        <v>26.75405761518516</v>
+        <v>26.90339671779109</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
@@ -4789,49 +4789,49 @@
         </is>
       </c>
       <c r="C77" s="2" t="n">
-        <v>19.31177457394332</v>
+        <v>19.70342710686125</v>
       </c>
       <c r="D77" s="2" t="n">
-        <v>-55.2305619856029</v>
+        <v>-56.34390679770192</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>-62.97501920067582</v>
+        <v>-65.4595171766683</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>-580.9950424636048</v>
+        <v>-1008.88582802312</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>56.73170779469048</v>
+        <v>54.18846208924776</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>24.58929547102723</v>
+        <v>24.04667671920015</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>14.87687572023246</v>
+        <v>14.65616360491454</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>10.41841433107436</v>
+        <v>10.29900214450413</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>7.822729452881926</v>
+        <v>7.74837527366673</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>5.932991281335901</v>
+        <v>5.885012236440789</v>
       </c>
       <c r="M77" s="2" t="n">
-        <v>4.646327050001036</v>
+        <v>4.613013689672324</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>3.631032829875893</v>
+        <v>3.607478514185594</v>
       </c>
       <c r="O77" s="2" t="n">
-        <v>2.814639040383788</v>
+        <v>2.797762378721892</v>
       </c>
       <c r="P77" s="2" t="n">
-        <v>2.099363506365515</v>
+        <v>2.087574544533808</v>
       </c>
       <c r="Q77" s="2" t="n">
-        <v>1.452397341416213</v>
+        <v>1.444657302497473</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
@@ -4846,49 +4846,49 @@
         </is>
       </c>
       <c r="C78" s="2" t="n">
-        <v>11.19568774568605</v>
+        <v>11.21348583952843</v>
       </c>
       <c r="D78" s="2" t="n">
-        <v>5.947940682837526</v>
+        <v>5.984094124247088</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>4.686673097443435</v>
+        <v>4.716084589474976</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>4.007655953973131</v>
+        <v>4.032227694017815</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>3.517594475112175</v>
+        <v>3.538237561611895</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>3.140922115062723</v>
+        <v>3.158416634966211</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>2.82961266414643</v>
+        <v>2.84446714610457</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>2.562389124764259</v>
+        <v>2.574967973955494</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>2.340469852843322</v>
+        <v>2.351149129934989</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>2.137697157297684</v>
+        <v>2.14664749637807</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>1.959677037981139</v>
+        <v>1.967094224323015</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>1.788990682557818</v>
+        <v>1.803820115334921</v>
       </c>
       <c r="O78" s="2" t="n">
-        <v>1.637298222993616</v>
+        <v>1.641900207103614</v>
       </c>
       <c r="P78" s="2" t="n">
-        <v>1.493691006015827</v>
+        <v>1.496957124228334</v>
       </c>
       <c r="Q78" s="2" t="n">
-        <v>1.338074446389007</v>
+        <v>1.34501248340014</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
@@ -4960,49 +4960,49 @@
         </is>
       </c>
       <c r="C80" s="2" t="n">
-        <v>0.01290066247249668</v>
+        <v>0.01284533583136801</v>
       </c>
       <c r="D80" s="2" t="n">
-        <v>0.008754620694546451</v>
+        <v>0.008737375235053947</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>0.007733815301414316</v>
+        <v>0.007721960619919079</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>0.007196147179503915</v>
+        <v>0.007186316534126742</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.006812062968188142</v>
+        <v>0.006803212636311481</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>0.00648721947394594</v>
+        <v>0.006478875496473524</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>0.006181976599738744</v>
+        <v>0.006173886689042857</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.005879559564322505</v>
+        <v>0.005871550206846132</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0.005569433407427283</v>
+        <v>0.005561376589232649</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>0.005244605894196547</v>
+        <v>0.00523639893094619</v>
       </c>
       <c r="M80" s="2" t="n">
-        <v>0.004900748153122187</v>
+        <v>0.004892294203632236</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.004534113091319795</v>
+        <v>0.004525320541147819</v>
       </c>
       <c r="O80" s="2" t="n">
-        <v>0.00414164795905212</v>
+        <v>0.004132424258498496</v>
       </c>
       <c r="P80" s="2" t="n">
-        <v>0.003720785106801318</v>
+        <v>0.003711033901348967</v>
       </c>
       <c r="Q80" s="2" t="n">
-        <v>0.003269527536965649</v>
+        <v>0.00325914486217734</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
@@ -5017,49 +5017,49 @@
         </is>
       </c>
       <c r="C81" s="2" t="n">
-        <v>0.05348029644731106</v>
+        <v>0.05347988022802827</v>
       </c>
       <c r="D81" s="2" t="n">
-        <v>0.05060676323739891</v>
+        <v>0.05060693192612765</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>0.04753301551061671</v>
+        <v>0.04753332832998856</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>0.04427214776847856</v>
+        <v>0.04427254892416915</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>0.04085938848479383</v>
+        <v>0.04085985463305541</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>0.03733295319982487</v>
+        <v>0.03733346837255656</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>0.03373235555441111</v>
+        <v>0.03373290630729443</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.03015722502249987</v>
+        <v>0.03015779401962254</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>0.02662024572341182</v>
+        <v>0.02662081694295447</v>
       </c>
       <c r="L81" s="2" t="n">
-        <v>0.02304055589828181</v>
+        <v>0.02304112091977756</v>
       </c>
       <c r="M81" s="2" t="n">
-        <v>0.01958188562076119</v>
+        <v>0.01958242589493833</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.01619614885663912</v>
+        <v>0.0161966503741525</v>
       </c>
       <c r="O81" s="2" t="n">
-        <v>0.01292913946988257</v>
+        <v>0.01292958534235631</v>
       </c>
       <c r="P81" s="2" t="n">
-        <v>0.009764542459919865</v>
+        <v>0.009764917296766951</v>
       </c>
       <c r="Q81" s="2" t="n">
-        <v>0.006721373732741089</v>
+        <v>0.006721660281119007</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
@@ -5074,49 +5074,49 @@
         </is>
       </c>
       <c r="C82" s="2" t="n">
-        <v>0.04452797092663265</v>
+        <v>0.04437525304713333</v>
       </c>
       <c r="D82" s="2" t="n">
-        <v>0.02911522331264094</v>
+        <v>0.02910092532496663</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>0.02500816934311377</v>
+        <v>0.02501269180249618</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>0.02261280764116443</v>
+        <v>0.02262529958492056</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>0.02073668558350001</v>
+        <v>0.02075382689188481</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>0.01907548196630301</v>
+        <v>0.01909548304204345</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>0.01749803524396536</v>
+        <v>0.01751971322713502</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.01595701889384122</v>
+        <v>0.01597938431123609</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>0.01444924048389688</v>
+        <v>0.01447131067056159</v>
       </c>
       <c r="L82" s="2" t="n">
-        <v>0.01294626907285786</v>
+        <v>0.01296724538909818</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>0.01146670852973583</v>
+        <v>0.01148575897070705</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.01000035726654358</v>
+        <v>0.01002920574158626</v>
       </c>
       <c r="O82" s="2" t="n">
-        <v>0.008579654270020231</v>
+        <v>0.008592823756558501</v>
       </c>
       <c r="P82" s="2" t="n">
-        <v>0.007206817239764161</v>
+        <v>0.00721614809988272</v>
       </c>
       <c r="Q82" s="2" t="n">
-        <v>0.005887264029587563</v>
+        <v>0.005898890257028502</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
@@ -5131,49 +5131,49 @@
         </is>
       </c>
       <c r="C83" s="2" t="n">
-        <v>0.04448020987657037</v>
+        <v>0.04447872578469382</v>
       </c>
       <c r="D83" s="2" t="n">
-        <v>0.04186394409874142</v>
+        <v>0.04186408438557271</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>0.03931724706798685</v>
+        <v>0.03931766343598594</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>0.03673074266682043</v>
+        <v>0.03673126683686326</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>0.03409232457246877</v>
+        <v>0.03409290159483412</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>0.03140138672752691</v>
+        <v>0.03140199028321476</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>0.02866196877270612</v>
+        <v>0.02866258360820718</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.02593253872788959</v>
+        <v>0.02593314109349731</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>0.02320153751691592</v>
+        <v>0.02320211076010172</v>
       </c>
       <c r="L83" s="2" t="n">
-        <v>0.02038017349037437</v>
+        <v>0.0203807239600046</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>0.01759544927006901</v>
+        <v>0.01759595626207825</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.01479496235224498</v>
+        <v>0.01479541909653592</v>
       </c>
       <c r="O83" s="2" t="n">
-        <v>0.01201274727308245</v>
+        <v>0.01201314073259318</v>
       </c>
       <c r="P83" s="2" t="n">
-        <v>0.009230495125408049</v>
+        <v>0.009230817698799113</v>
       </c>
       <c r="Q83" s="2" t="n">
-        <v>0.006465082432865896</v>
+        <v>0.006465323550020442</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
@@ -5188,49 +5188,49 @@
         </is>
       </c>
       <c r="C84" s="2" t="n">
-        <v>0.04001686526877036</v>
+        <v>0.0399336197082567</v>
       </c>
       <c r="D84" s="2" t="n">
-        <v>0.02707720376682778</v>
+        <v>0.027082465917497</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>0.02338158219782631</v>
+        <v>0.02339961722668475</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>0.02117262765891408</v>
+        <v>0.02119600220118516</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>0.01942528113643191</v>
+        <v>0.01945158425099778</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>0.01787492022552809</v>
+        <v>0.01790274194357312</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>0.01640596156846623</v>
+        <v>0.01643431324499545</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.01497588439128392</v>
+        <v>0.01500391865706821</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>0.01358167057566953</v>
+        <v>0.01360853750374109</v>
       </c>
       <c r="L84" s="2" t="n">
-        <v>0.01219563163415452</v>
+        <v>0.01222064711370299</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>0.01083319806857282</v>
+        <v>0.01085565109038657</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.00948234891135669</v>
+        <v>0.009513430312522246</v>
       </c>
       <c r="O84" s="2" t="n">
-        <v>0.008171162389595714</v>
+        <v>0.008186774648133876</v>
       </c>
       <c r="P84" s="2" t="n">
-        <v>0.006899240008938476</v>
+        <v>0.006910661345394523</v>
       </c>
       <c r="Q84" s="2" t="n">
-        <v>0.005668965999215133</v>
+        <v>0.00568214129664112</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
@@ -5245,49 +5245,49 @@
         </is>
       </c>
       <c r="C85" s="2" t="n">
-        <v>0.03529414824668107</v>
+        <v>0.03529557343950659</v>
       </c>
       <c r="D85" s="2" t="n">
-        <v>0.03346157666592845</v>
+        <v>0.03346296508831367</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>0.03159593607532506</v>
+        <v>0.03159728509910138</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>0.02969284747215544</v>
+        <v>0.02969415410293409</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>0.02774885426324433</v>
+        <v>0.02775011511049226</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>0.02576079492675613</v>
+        <v>0.02576200616523388</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>0.02372649425892189</v>
+        <v>0.02372765158043555</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.02169651776215099</v>
+        <v>0.02169760760902936</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>0.01964899080885401</v>
+        <v>0.01965000249008469</v>
       </c>
       <c r="L85" s="2" t="n">
-        <v>0.01748552901654696</v>
+        <v>0.01748646599040068</v>
       </c>
       <c r="M85" s="2" t="n">
-        <v>0.01532167683016455</v>
+        <v>0.01532252323631826</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0130940194351212</v>
+        <v>0.01309476783030983</v>
       </c>
       <c r="O85" s="2" t="n">
-        <v>0.01082418213674616</v>
+        <v>0.0108248199652255</v>
       </c>
       <c r="P85" s="2" t="n">
-        <v>0.008481553687055197</v>
+        <v>0.008482070866848957</v>
       </c>
       <c r="Q85" s="2" t="n">
-        <v>0.006069041746897686</v>
+        <v>0.006069425061761733</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
@@ -5302,49 +5302,49 @@
         </is>
       </c>
       <c r="C86" s="2" t="n">
-        <v>0.04312667151729712</v>
+        <v>0.04300265915208532</v>
       </c>
       <c r="D86" s="2" t="n">
-        <v>0.02862233861657726</v>
+        <v>0.02861308194131834</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>0.02464680623967282</v>
+        <v>0.02465436912570533</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>0.02230605686053166</v>
+        <v>0.02232088599011457</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>0.02046837576334395</v>
+        <v>0.02048744138815947</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>0.01883683474810338</v>
+        <v>0.01885848384928689</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>0.01728602466129522</v>
+        <v>0.01730913418957931</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.01577052895767529</v>
+        <v>0.01579414305739371</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>0.01428469864772943</v>
+        <v>0.01430787772541313</v>
       </c>
       <c r="L86" s="2" t="n">
-        <v>0.01280456983293463</v>
+        <v>0.01282652202922495</v>
       </c>
       <c r="M86" s="2" t="n">
-        <v>0.01134616071996539</v>
+        <v>0.01136607536486715</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.00990165258060334</v>
+        <v>0.009929654288552294</v>
       </c>
       <c r="O86" s="2" t="n">
-        <v>0.008500126935404936</v>
+        <v>0.008513956839925068</v>
       </c>
       <c r="P86" s="2" t="n">
-        <v>0.007144918104593149</v>
+        <v>0.007154825821260083</v>
       </c>
       <c r="Q86" s="2" t="n">
-        <v>0.005841798328744522</v>
+        <v>0.005853380867601016</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
@@ -5359,7 +5359,7 @@
         </is>
       </c>
       <c r="C87" s="2" t="n">
-        <v>0.9526391023487388</v>
+        <v>0.9525107926014297</v>
       </c>
       <c r="D87" s="1" t="inlineStr"/>
       <c r="E87" s="1" t="inlineStr"/>

</xml_diff>